<commit_message>
chocs à moyenne 0
</commit_message>
<xml_diff>
--- a/all_shocks.xlsx
+++ b/all_shocks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\emanu\OneDrive\Matlab\cdc_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE137D5-EB3F-4AE8-BA0A-7AB3B5ECB4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C61C937-F1AF-4F2D-8EDE-DE420304E3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3750" yWindow="2085" windowWidth="21600" windowHeight="11835" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="7935" windowWidth="28800" windowHeight="8265" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_pop_shocks_norm2000" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="117">
   <si>
     <t>P_Q_1</t>
   </si>
@@ -338,6 +338,54 @@
   </si>
   <si>
     <t>Ce choc resultent du modele CDC complet une fois qu'on exogenise la population normalisée des cohortes</t>
+  </si>
+  <si>
+    <t>mig_NQ_2</t>
+  </si>
+  <si>
+    <t>mig_NQ_3</t>
+  </si>
+  <si>
+    <t>mig_NQ_4</t>
+  </si>
+  <si>
+    <t>mig_NQ_5</t>
+  </si>
+  <si>
+    <t>mig_NQ_6</t>
+  </si>
+  <si>
+    <t>mig_NQ_7</t>
+  </si>
+  <si>
+    <t>mig_NQ_8</t>
+  </si>
+  <si>
+    <t>mig_NQ_9</t>
+  </si>
+  <si>
+    <t>mig_NQ_10</t>
+  </si>
+  <si>
+    <t>mig_NQ_11</t>
+  </si>
+  <si>
+    <t>mig_NQ_12</t>
+  </si>
+  <si>
+    <t>mig_NQ_13</t>
+  </si>
+  <si>
+    <t>mig_NQ_14</t>
+  </si>
+  <si>
+    <t>mig_NQ_15</t>
+  </si>
+  <si>
+    <t>mig_NQ_16</t>
+  </si>
+  <si>
+    <t>mig_NQ_17</t>
   </si>
 </sst>
 </file>
@@ -5551,7 +5599,7 @@
         <v>18</v>
       </c>
       <c r="D6">
-        <v>-0.15967272058620607</v>
+        <v>0.2753267546775866</v>
       </c>
       <c r="E6">
         <v>2.214154581450245E-3</v>
@@ -5685,7 +5733,7 @@
         <v>18</v>
       </c>
       <c r="D7">
-        <v>-0.24565717190814917</v>
+        <v>0.18944091200051794</v>
       </c>
       <c r="E7">
         <v>-8.798052235841184E-3</v>
@@ -5694,7 +5742,7 @@
         <v>2.4929074421023954E-3</v>
       </c>
       <c r="G7">
-        <v>-2.1373270782093393E-2</v>
+        <v>-2.137327078209339E-2</v>
       </c>
       <c r="H7">
         <v>-8.6453951054279478E-3</v>
@@ -5718,7 +5766,7 @@
         <v>3.3933903565056878E-2</v>
       </c>
       <c r="O7">
-        <v>3.0383907874593656E-2</v>
+        <v>3.038390787459366E-2</v>
       </c>
       <c r="P7">
         <v>4.7839256681225573E-2</v>
@@ -5730,40 +5778,40 @@
         <v>3.9490915288615258E-2</v>
       </c>
       <c r="S7">
-        <v>3.6536510565018603E-2</v>
+        <v>3.6536510565018609E-2</v>
       </c>
       <c r="T7">
-        <v>4.2142916628999709E-2</v>
+        <v>4.2142916628999716E-2</v>
       </c>
       <c r="U7">
-        <v>4.6470535159674135E-2</v>
+        <v>4.6470535159674142E-2</v>
       </c>
       <c r="V7">
         <v>7.4841309368095077E-2</v>
       </c>
       <c r="W7">
-        <v>5.4583454125459951E-2</v>
+        <v>5.4583454125459945E-2</v>
       </c>
       <c r="X7">
-        <v>5.5003826390571886E-2</v>
+        <v>5.5003826390571879E-2</v>
       </c>
       <c r="Y7">
         <v>6.5383546651785807E-2</v>
       </c>
       <c r="Z7">
-        <v>6.1813519294937391E-2</v>
+        <v>6.1813519294937606E-2</v>
       </c>
       <c r="AA7">
         <v>6.5356164722600418E-2</v>
       </c>
       <c r="AB7">
-        <v>6.3794944403975595E-2</v>
+        <v>6.3794944403975373E-2</v>
       </c>
       <c r="AC7">
-        <v>6.1654781829491911E-2</v>
+        <v>6.1654781829491904E-2</v>
       </c>
       <c r="AD7">
-        <v>6.2307356539842318E-2</v>
+        <v>6.2307356539842311E-2</v>
       </c>
       <c r="AE7">
         <v>6.3362208607063986E-2</v>
@@ -5775,25 +5823,25 @@
         <v>6.4188713044355028E-2</v>
       </c>
       <c r="AH7">
-        <v>6.1814578816645427E-2</v>
+        <v>6.181457881664542E-2</v>
       </c>
       <c r="AI7">
-        <v>6.0425638744489363E-2</v>
+        <v>6.0425638744489356E-2</v>
       </c>
       <c r="AJ7">
-        <v>6.0816741782236616E-2</v>
+        <v>6.0816741782236609E-2</v>
       </c>
       <c r="AK7">
-        <v>6.1455653716094405E-2</v>
+        <v>6.1455653716094398E-2</v>
       </c>
       <c r="AL7">
-        <v>6.1922434122747338E-2</v>
+        <v>6.1922434122747332E-2</v>
       </c>
       <c r="AM7">
-        <v>6.1888309307405409E-2</v>
+        <v>6.1888309307405402E-2</v>
       </c>
       <c r="AN7">
-        <v>6.115230770110347E-2</v>
+        <v>6.1152307701103463E-2</v>
       </c>
       <c r="AO7">
         <v>6.0103532554758754E-2</v>
@@ -5819,7 +5867,7 @@
         <v>18</v>
       </c>
       <c r="D8">
-        <v>-0.26155473045267985</v>
+        <v>0.17236558985102601</v>
       </c>
       <c r="E8">
         <v>-7.236851580176909E-4</v>
@@ -5870,25 +5918,25 @@
         <v>2.6039029199987899E-2</v>
       </c>
       <c r="U8">
-        <v>3.6717245073956788E-2</v>
+        <v>3.6717245073956781E-2</v>
       </c>
       <c r="V8">
         <v>6.2434500490324389E-2</v>
       </c>
       <c r="W8">
-        <v>4.6318139893231074E-2</v>
+        <v>4.6318139893231067E-2</v>
       </c>
       <c r="X8">
         <v>5.135931795910563E-2</v>
       </c>
       <c r="Y8">
-        <v>6.3306729060164532E-2</v>
+        <v>6.3306729060164546E-2</v>
       </c>
       <c r="Z8">
         <v>6.4793987221842819E-2</v>
       </c>
       <c r="AA8">
-        <v>6.7801677319718298E-2</v>
+        <v>6.7801677319718312E-2</v>
       </c>
       <c r="AB8">
         <v>6.6660882767059615E-2</v>
@@ -5900,16 +5948,16 @@
         <v>6.3914424269086556E-2</v>
       </c>
       <c r="AE8">
-        <v>6.4829697214101589E-2</v>
+        <v>6.4829697214101478E-2</v>
       </c>
       <c r="AF8">
         <v>6.615753944350633E-2</v>
       </c>
       <c r="AG8">
-        <v>6.7667415928057237E-2</v>
+        <v>6.7667415928057251E-2</v>
       </c>
       <c r="AH8">
-        <v>6.7112657448067367E-2</v>
+        <v>6.7112657448067381E-2</v>
       </c>
       <c r="AI8">
         <v>6.4605800891545329E-2</v>
@@ -5953,67 +6001,67 @@
         <v>18</v>
       </c>
       <c r="D9">
-        <v>-0.30679603837354075</v>
+        <v>0.1254070895445526</v>
       </c>
       <c r="E9">
-        <v>-5.9408663182357775E-3</v>
+        <v>-5.940866318235774E-3</v>
       </c>
       <c r="F9">
-        <v>-5.2210796294517928E-4</v>
+        <v>-5.2210796294517581E-4</v>
       </c>
       <c r="G9">
-        <v>-1.1217645657931173E-2</v>
+        <v>-1.1217645657931166E-2</v>
       </c>
       <c r="H9">
         <v>4.7936319832520939E-3</v>
       </c>
       <c r="I9">
-        <v>1.2300780327542872E-2</v>
+        <v>1.2300780327542877E-2</v>
       </c>
       <c r="J9">
         <v>3.6018982593929265E-3</v>
       </c>
       <c r="K9">
-        <v>-1.0632310666801502E-2</v>
+        <v>-1.0632310666801495E-2</v>
       </c>
       <c r="L9">
-        <v>-6.1418031984663245E-2</v>
+        <v>-6.1418031984663238E-2</v>
       </c>
       <c r="M9">
         <v>8.3506772794188819E-2</v>
       </c>
       <c r="N9">
-        <v>4.2098509327472035E-2</v>
+        <v>4.2098509327472042E-2</v>
       </c>
       <c r="O9">
-        <v>2.1277843934306522E-2</v>
+        <v>2.1277843934306526E-2</v>
       </c>
       <c r="P9">
-        <v>3.2427341011736256E-2</v>
+        <v>3.2427341011736263E-2</v>
       </c>
       <c r="Q9">
-        <v>4.1599468865491242E-2</v>
+        <v>4.1599468865491249E-2</v>
       </c>
       <c r="R9">
         <v>3.3459220219192877E-2</v>
       </c>
       <c r="S9">
-        <v>2.251123900569283E-2</v>
+        <v>2.2511239005692834E-2</v>
       </c>
       <c r="T9">
-        <v>2.258295303613609E-2</v>
+        <v>2.2582953036136093E-2</v>
       </c>
       <c r="U9">
         <v>2.5075531682969145E-2</v>
       </c>
       <c r="V9">
-        <v>5.4937600323355464E-2</v>
+        <v>5.4937600323355457E-2</v>
       </c>
       <c r="W9">
-        <v>4.1640307135442069E-2</v>
+        <v>4.1640307135442062E-2</v>
       </c>
       <c r="X9">
-        <v>4.4439142707816327E-2</v>
+        <v>4.443914270781632E-2</v>
       </c>
       <c r="Y9">
         <v>5.5212886244188714E-2</v>
@@ -6022,34 +6070,34 @@
         <v>5.618081009162032E-2</v>
       </c>
       <c r="AA9">
-        <v>5.4722622480382489E-2</v>
+        <v>5.4722622480382482E-2</v>
       </c>
       <c r="AB9">
-        <v>5.1066943946999489E-2</v>
+        <v>5.1066943946999482E-2</v>
       </c>
       <c r="AC9">
-        <v>5.2200109377753524E-2</v>
+        <v>5.2200109377753517E-2</v>
       </c>
       <c r="AD9">
-        <v>5.225936691619102E-2</v>
+        <v>5.2259366916191013E-2</v>
       </c>
       <c r="AE9">
         <v>5.0570034717299019E-2</v>
       </c>
       <c r="AF9">
-        <v>5.1734782894280885E-2</v>
+        <v>5.1734782894280879E-2</v>
       </c>
       <c r="AG9">
         <v>5.3243420655319153E-2</v>
       </c>
       <c r="AH9">
-        <v>5.4949081267275469E-2</v>
+        <v>5.4949081267275462E-2</v>
       </c>
       <c r="AI9">
         <v>5.4397351488425262E-2</v>
       </c>
       <c r="AJ9">
-        <v>5.1711484709427748E-2</v>
+        <v>5.1711484709427637E-2</v>
       </c>
       <c r="AK9">
         <v>5.0164603436464762E-2</v>
@@ -6061,7 +6109,7 @@
         <v>5.1499939203650348E-2</v>
       </c>
       <c r="AN9">
-        <v>5.2104933092651941E-2</v>
+        <v>5.210493309265183E-2</v>
       </c>
       <c r="AO9">
         <v>5.2116584423815705E-2</v>
@@ -6087,124 +6135,124 @@
         <v>18</v>
       </c>
       <c r="D10">
-        <v>-0.37443848101655242</v>
+        <v>5.5486024490896124E-2</v>
       </c>
       <c r="E10">
-        <v>-1.2702194956710489E-2</v>
+        <v>-1.2702194956710565E-2</v>
       </c>
       <c r="F10">
-        <v>-5.3741464852489762E-3</v>
+        <v>-5.374146485249056E-3</v>
       </c>
       <c r="G10">
-        <v>1.3202308870674251E-2</v>
+        <v>1.3202308870674173E-2</v>
       </c>
       <c r="H10">
-        <v>2.0226923364166038E-2</v>
+        <v>2.0226923364166066E-2</v>
       </c>
       <c r="I10">
-        <v>3.8681168096839601E-3</v>
+        <v>3.8681168096838768E-3</v>
       </c>
       <c r="J10">
-        <v>-1.4069022719456793E-3</v>
+        <v>-1.4069022719457626E-3</v>
       </c>
       <c r="K10">
-        <v>-1.0746652435382701E-2</v>
+        <v>-1.0746652435382781E-2</v>
       </c>
       <c r="L10">
-        <v>-3.8672715018868549E-2</v>
+        <v>-3.8672715018868625E-2</v>
       </c>
       <c r="M10">
-        <v>4.6242670608277851E-2</v>
+        <v>4.6242670608277768E-2</v>
       </c>
       <c r="N10">
-        <v>3.2087587651180735E-2</v>
+        <v>3.2087587651180645E-2</v>
       </c>
       <c r="O10">
-        <v>2.0549004741740859E-2</v>
+        <v>2.0549004741740769E-2</v>
       </c>
       <c r="P10">
-        <v>2.8630609697237797E-2</v>
+        <v>2.8630609697237724E-2</v>
       </c>
       <c r="Q10">
-        <v>2.5809721325159296E-2</v>
+        <v>2.5809721325159334E-2</v>
       </c>
       <c r="R10">
-        <v>2.6436049586985234E-2</v>
+        <v>2.6436049586985248E-2</v>
       </c>
       <c r="S10">
-        <v>1.878120487739502E-2</v>
+        <v>1.8781204877395034E-2</v>
       </c>
       <c r="T10">
-        <v>1.9427291127762467E-2</v>
+        <v>1.942729112776248E-2</v>
       </c>
       <c r="U10">
-        <v>1.8842827998864428E-2</v>
+        <v>1.8842827998864345E-2</v>
       </c>
       <c r="V10">
-        <v>3.9848805662785737E-2</v>
+        <v>3.9848805662785751E-2</v>
       </c>
       <c r="W10">
-        <v>3.68354748338462E-2</v>
+        <v>3.6835474833846187E-2</v>
       </c>
       <c r="X10">
-        <v>4.1295026842261835E-2</v>
+        <v>4.1295026842261828E-2</v>
       </c>
       <c r="Y10">
-        <v>4.8146828548922833E-2</v>
+        <v>4.814682854892282E-2</v>
       </c>
       <c r="Z10">
-        <v>4.8803883237712682E-2</v>
+        <v>4.8803883237712661E-2</v>
       </c>
       <c r="AA10">
-        <v>4.8887690302795057E-2</v>
+        <v>4.8887690302795037E-2</v>
       </c>
       <c r="AB10">
-        <v>4.338826851800804E-2</v>
+        <v>4.3388268518008033E-2</v>
       </c>
       <c r="AC10">
-        <v>4.3315476262297384E-2</v>
+        <v>4.331547626229737E-2</v>
       </c>
       <c r="AD10">
-        <v>4.4697988409070813E-2</v>
+        <v>4.4697988409070799E-2</v>
       </c>
       <c r="AE10">
-        <v>4.4708888724039456E-2</v>
+        <v>4.4708888724039442E-2</v>
       </c>
       <c r="AF10">
-        <v>4.304110553234166E-2</v>
+        <v>4.3041105532341653E-2</v>
       </c>
       <c r="AG10">
         <v>4.4448454850834609E-2</v>
       </c>
       <c r="AH10">
-        <v>4.6217389546187496E-2</v>
+        <v>4.6217389546187489E-2</v>
       </c>
       <c r="AI10">
-        <v>4.820173184352728E-2</v>
+        <v>4.8201731843527273E-2</v>
       </c>
       <c r="AJ10">
-        <v>4.7693422755138895E-2</v>
+        <v>4.7693422755138881E-2</v>
       </c>
       <c r="AK10">
-        <v>4.4825064135562552E-2</v>
+        <v>4.4825064135562545E-2</v>
       </c>
       <c r="AL10">
         <v>4.3202834678336549E-2</v>
       </c>
       <c r="AM10">
-        <v>4.3856471237945248E-2</v>
+        <v>4.3856471237945255E-2</v>
       </c>
       <c r="AN10">
         <v>4.4819082596581759E-2</v>
       </c>
       <c r="AO10">
-        <v>4.5550537967718151E-2</v>
+        <v>4.5550537967718262E-2</v>
       </c>
       <c r="AP10">
         <v>4.5619038144155709E-2</v>
       </c>
       <c r="AQ10">
-        <v>4.4756495508269233E-2</v>
+        <v>4.475649550826924E-2</v>
       </c>
       <c r="AR10" t="s">
         <v>81</v>
@@ -6221,34 +6269,34 @@
         <v>18</v>
       </c>
       <c r="D11">
-        <v>-0.39477406481363475</v>
+        <v>3.2263302252500826E-2</v>
       </c>
       <c r="E11">
-        <v>-9.4274541427797065E-3</v>
+        <v>-9.4274541427796996E-3</v>
       </c>
       <c r="F11">
-        <v>-9.8165612929002333E-3</v>
+        <v>-9.8165612929002263E-3</v>
       </c>
       <c r="G11">
-        <v>-2.3487080085657086E-3</v>
+        <v>-2.3487080085657017E-3</v>
       </c>
       <c r="H11">
-        <v>-8.6583804029078115E-3</v>
+        <v>-8.6583804029078046E-3</v>
       </c>
       <c r="I11">
-        <v>-5.4340259083950626E-3</v>
+        <v>-5.4340259083950557E-3</v>
       </c>
       <c r="J11">
-        <v>-6.5539401508452333E-3</v>
+        <v>-6.5539401508452264E-3</v>
       </c>
       <c r="K11">
-        <v>-1.3651670884479744E-2</v>
+        <v>-1.3651670884479737E-2</v>
       </c>
       <c r="L11">
         <v>-3.5139292967922203E-2</v>
       </c>
       <c r="M11">
-        <v>2.4831739846267381E-2</v>
+        <v>2.4831739846267388E-2</v>
       </c>
       <c r="N11">
         <v>1.6870479800516897E-2</v>
@@ -6260,10 +6308,10 @@
         <v>2.3562270899732257E-2</v>
       </c>
       <c r="Q11">
-        <v>2.2503835982026071E-2</v>
+        <v>2.2503835982026078E-2</v>
       </c>
       <c r="R11">
-        <v>1.6627122488387241E-2</v>
+        <v>1.6627122488387248E-2</v>
       </c>
       <c r="S11">
         <v>1.6294200651658847E-2</v>
@@ -6278,34 +6326,34 @@
         <v>3.3677227950180105E-2</v>
       </c>
       <c r="W11">
-        <v>3.0801701882456865E-2</v>
+        <v>3.0801701882456869E-2</v>
       </c>
       <c r="X11">
-        <v>4.3793562001004115E-2</v>
+        <v>4.3793562001004108E-2</v>
       </c>
       <c r="Y11">
-        <v>4.6527981823540863E-2</v>
+        <v>4.6527981823540857E-2</v>
       </c>
       <c r="Z11">
-        <v>4.5534778306406586E-2</v>
+        <v>4.5534778306406579E-2</v>
       </c>
       <c r="AA11">
-        <v>4.701621914579298E-2</v>
+        <v>4.7016219145792973E-2</v>
       </c>
       <c r="AB11">
-        <v>4.2204248431996404E-2</v>
+        <v>4.2204248431996397E-2</v>
       </c>
       <c r="AC11">
-        <v>4.2186777917608574E-2</v>
+        <v>4.2186777917608567E-2</v>
       </c>
       <c r="AD11">
-        <v>4.2399357228157984E-2</v>
+        <v>4.2399357228157977E-2</v>
       </c>
       <c r="AE11">
-        <v>4.3862301147063319E-2</v>
+        <v>4.3862301147063312E-2</v>
       </c>
       <c r="AF11">
-        <v>4.4074140935555138E-2</v>
+        <v>4.4074140935555131E-2</v>
       </c>
       <c r="AG11">
         <v>4.2516374851200488E-2</v>
@@ -6314,13 +6362,13 @@
         <v>4.4270114989099794E-2</v>
       </c>
       <c r="AI11">
-        <v>4.6403055946117232E-2</v>
+        <v>4.6403055946117225E-2</v>
       </c>
       <c r="AJ11">
-        <v>4.876923028997978E-2</v>
+        <v>4.8769230289979773E-2</v>
       </c>
       <c r="AK11">
-        <v>4.8383908285399811E-2</v>
+        <v>4.8383908285399804E-2</v>
       </c>
       <c r="AL11">
         <v>4.5371764879791519E-2</v>
@@ -6335,7 +6383,7 @@
         <v>4.5740860162084528E-2</v>
       </c>
       <c r="AP11">
-        <v>4.6658586496614217E-2</v>
+        <v>4.6658586496614106E-2</v>
       </c>
       <c r="AQ11">
         <v>4.6827914600688213E-2</v>
@@ -6355,64 +6403,64 @@
         <v>18</v>
       </c>
       <c r="D12">
-        <v>-0.44667298808583028</v>
+        <v>-2.4362696747206626E-2</v>
       </c>
       <c r="E12">
-        <v>-1.9744143023249609E-2</v>
+        <v>-1.9744143023249595E-2</v>
       </c>
       <c r="F12">
-        <v>-1.5694522694105643E-2</v>
+        <v>-1.569452269410563E-2</v>
       </c>
       <c r="G12">
-        <v>-1.3803534801163191E-2</v>
+        <v>-1.3803534801163177E-2</v>
       </c>
       <c r="H12">
-        <v>-5.6008504068616946E-3</v>
+        <v>-5.6008504068616807E-3</v>
       </c>
       <c r="I12">
-        <v>-1.1072434743251085E-2</v>
+        <v>-1.1072434743251078E-2</v>
       </c>
       <c r="J12">
-        <v>-1.1630240244701988E-2</v>
+        <v>-1.1630240244701981E-2</v>
       </c>
       <c r="K12">
-        <v>-1.5827651241563205E-2</v>
+        <v>-1.5827651241563198E-2</v>
       </c>
       <c r="L12">
-        <v>-3.310727451521616E-2</v>
+        <v>-3.3107274515216153E-2</v>
       </c>
       <c r="M12">
-        <v>1.6949583156538335E-2</v>
+        <v>1.6949583156538345E-2</v>
       </c>
       <c r="N12">
-        <v>1.1694021451363834E-2</v>
+        <v>1.1694021451363851E-2</v>
       </c>
       <c r="O12">
-        <v>6.6070355231971356E-3</v>
+        <v>6.607035523197146E-3</v>
       </c>
       <c r="P12">
-        <v>1.6179132674044194E-2</v>
+        <v>1.617913267404409E-2</v>
       </c>
       <c r="Q12">
-        <v>1.9926990479983864E-2</v>
+        <v>1.992699047998376E-2</v>
       </c>
       <c r="R12">
-        <v>1.1600062759427765E-2</v>
+        <v>1.1600062759427779E-2</v>
       </c>
       <c r="S12">
-        <v>1.1348239910148161E-2</v>
+        <v>1.1348239910148179E-2</v>
       </c>
       <c r="T12">
-        <v>1.7647398240613066E-2</v>
+        <v>1.7647398240613069E-2</v>
       </c>
       <c r="U12">
-        <v>2.0410556529964541E-2</v>
+        <v>2.0410556529964433E-2</v>
       </c>
       <c r="V12">
-        <v>3.4731058335620346E-2</v>
+        <v>3.4731058335620353E-2</v>
       </c>
       <c r="W12">
-        <v>2.7111581932348916E-2</v>
+        <v>2.7111581932348923E-2</v>
       </c>
       <c r="X12">
         <v>3.7972505161053161E-2</v>
@@ -6436,31 +6484,31 @@
         <v>4.9972656292513504E-2</v>
       </c>
       <c r="AE12">
-        <v>5.0367205191953639E-2</v>
+        <v>5.0367205191953632E-2</v>
       </c>
       <c r="AF12">
         <v>5.2324027316411989E-2</v>
       </c>
       <c r="AG12">
-        <v>5.2839647456881682E-2</v>
+        <v>5.2839647456881675E-2</v>
       </c>
       <c r="AH12">
-        <v>5.128470322715855E-2</v>
+        <v>5.1284703227158661E-2</v>
       </c>
       <c r="AI12">
-        <v>5.3524444794866115E-2</v>
+        <v>5.3524444794866108E-2</v>
       </c>
       <c r="AJ12">
-        <v>5.6196092357453091E-2</v>
+        <v>5.6196092357453084E-2</v>
       </c>
       <c r="AK12">
         <v>5.9140392258269989E-2</v>
       </c>
       <c r="AL12">
-        <v>5.8861085693118813E-2</v>
+        <v>5.8861085693118806E-2</v>
       </c>
       <c r="AM12">
-        <v>5.5482472390448505E-2</v>
+        <v>5.5482472390448616E-2</v>
       </c>
       <c r="AN12">
         <v>5.3666018053928059E-2</v>
@@ -6472,7 +6520,7 @@
         <v>5.6281623903386695E-2</v>
       </c>
       <c r="AQ12">
-        <v>5.7466221853147585E-2</v>
+        <v>5.7466221853147696E-2</v>
       </c>
       <c r="AR12" t="s">
         <v>81</v>
@@ -6489,73 +6537,73 @@
         <v>18</v>
       </c>
       <c r="D13">
-        <v>-0.49360419959189489</v>
+        <v>-7.7681981575542222E-2</v>
       </c>
       <c r="E13">
-        <v>-2.3277271395060535E-2</v>
+        <v>-2.3277271395060518E-2</v>
       </c>
       <c r="F13">
-        <v>-2.4987170380011477E-2</v>
+        <v>-2.4987170380011459E-2</v>
       </c>
       <c r="G13">
-        <v>-2.2380335949466271E-3</v>
+        <v>-2.2380335949466045E-3</v>
       </c>
       <c r="H13">
-        <v>-3.774767171564504E-3</v>
+        <v>-3.7747671715644814E-3</v>
       </c>
       <c r="I13">
-        <v>-1.8837995105936929E-2</v>
+        <v>-1.8837995105936915E-2</v>
       </c>
       <c r="J13">
-        <v>-1.8099542588297497E-2</v>
+        <v>-1.8099542588297483E-2</v>
       </c>
       <c r="K13">
-        <v>-2.3618017476338245E-2</v>
+        <v>-2.3618017476338342E-2</v>
       </c>
       <c r="L13">
-        <v>-3.6927158134320411E-2</v>
+        <v>-3.6927158134320508E-2</v>
       </c>
       <c r="M13">
-        <v>7.065565109499676E-3</v>
+        <v>7.0655651094995806E-3</v>
       </c>
       <c r="N13">
-        <v>3.7115214991423826E-3</v>
+        <v>3.7115214991422867E-3</v>
       </c>
       <c r="O13">
-        <v>4.6446070404598111E-4</v>
+        <v>4.6446070404588478E-4</v>
       </c>
       <c r="P13">
-        <v>8.1538935903364002E-3</v>
+        <v>8.153893590336303E-3</v>
       </c>
       <c r="Q13">
-        <v>9.2240250353885916E-3</v>
+        <v>9.2240250353885986E-3</v>
       </c>
       <c r="R13">
-        <v>6.9506092481375487E-3</v>
+        <v>6.9506092481375547E-3</v>
       </c>
       <c r="S13">
-        <v>8.2444176885352813E-3</v>
+        <v>8.2444176885351841E-3</v>
       </c>
       <c r="T13">
-        <v>1.2443883907405744E-2</v>
+        <v>1.2443883907405643E-2</v>
       </c>
       <c r="U13">
-        <v>1.7292850567156161E-2</v>
+        <v>1.7292850567156171E-2</v>
       </c>
       <c r="V13">
-        <v>3.1521434602123012E-2</v>
+        <v>3.1521434602123026E-2</v>
       </c>
       <c r="W13">
-        <v>2.7082537533778685E-2</v>
+        <v>2.7082537533778699E-2</v>
       </c>
       <c r="X13">
-        <v>3.2384978759609814E-2</v>
+        <v>3.2384978759609821E-2</v>
       </c>
       <c r="Y13">
-        <v>4.1678498616248873E-2</v>
+        <v>4.167849861624888E-2</v>
       </c>
       <c r="Z13">
-        <v>4.6740050040789204E-2</v>
+        <v>4.6740050040789197E-2</v>
       </c>
       <c r="AA13">
         <v>5.1460424840708799E-2</v>
@@ -6573,28 +6621,28 @@
         <v>5.9285298673382406E-2</v>
       </c>
       <c r="AF13">
-        <v>6.0157936055520139E-2</v>
+        <v>6.0157936055520132E-2</v>
       </c>
       <c r="AG13">
-        <v>6.2814644599020003E-2</v>
+        <v>6.2814644599019989E-2</v>
       </c>
       <c r="AH13">
-        <v>6.3767816462993926E-2</v>
+        <v>6.3767816462993912E-2</v>
       </c>
       <c r="AI13">
-        <v>6.2263152718157105E-2</v>
+        <v>6.2263152718157112E-2</v>
       </c>
       <c r="AJ13">
-        <v>6.5180589669482064E-2</v>
+        <v>6.518058966948205E-2</v>
       </c>
       <c r="AK13">
-        <v>6.8591157893913263E-2</v>
+        <v>6.8591157893913249E-2</v>
       </c>
       <c r="AL13">
         <v>7.2326527671071963E-2</v>
       </c>
       <c r="AM13">
-        <v>7.2218810292072361E-2</v>
+        <v>7.2218810292072347E-2</v>
       </c>
       <c r="AN13">
         <v>6.839029681186129E-2</v>
@@ -6623,82 +6671,82 @@
         <v>18</v>
       </c>
       <c r="D14">
-        <v>-0.56305776842292055</v>
+        <v>-0.15514258183260632</v>
       </c>
       <c r="E14">
-        <v>-3.7199091661566056E-2</v>
+        <v>-3.7199091661566021E-2</v>
       </c>
       <c r="F14">
-        <v>-3.6004194110941704E-2</v>
+        <v>-3.6004194110941669E-2</v>
       </c>
       <c r="G14">
-        <v>-3.4009631774868723E-2</v>
+        <v>-3.4009631774868689E-2</v>
       </c>
       <c r="H14">
-        <v>-3.8667025253932251E-2</v>
+        <v>-3.8667025253932216E-2</v>
       </c>
       <c r="I14">
-        <v>-3.3762485938915753E-2</v>
+        <v>-3.3762485938915718E-2</v>
       </c>
       <c r="J14">
-        <v>-3.1649879133818698E-2</v>
+        <v>-3.1649879133818677E-2</v>
       </c>
       <c r="K14">
-        <v>-3.4137274010349966E-2</v>
+        <v>-3.4137274010349945E-2</v>
       </c>
       <c r="L14">
-        <v>-4.3899557951590937E-2</v>
+        <v>-4.3899557951590965E-2</v>
       </c>
       <c r="M14">
-        <v>-1.0537820685555289E-2</v>
+        <v>-1.053782068555531E-2</v>
       </c>
       <c r="N14">
-        <v>-8.743488884343488E-3</v>
+        <v>-8.7434888843435209E-3</v>
       </c>
       <c r="O14">
-        <v>-1.0566105072038125E-2</v>
+        <v>-1.0566105072038159E-2</v>
       </c>
       <c r="P14">
-        <v>-3.0381415838877518E-3</v>
+        <v>-3.038141583887672E-3</v>
       </c>
       <c r="Q14">
-        <v>-2.3588494353154466E-3</v>
+        <v>-2.3588494353154938E-3</v>
       </c>
       <c r="R14">
-        <v>-5.0283536279328092E-3</v>
+        <v>-5.0283536279328639E-3</v>
       </c>
       <c r="S14">
-        <v>1.1611979587263163E-3</v>
+        <v>1.1611979587262615E-3</v>
       </c>
       <c r="T14">
-        <v>3.9062506038237202E-3</v>
+        <v>3.9062506038237974E-3</v>
       </c>
       <c r="U14">
-        <v>1.1517652170845723E-2</v>
+        <v>1.1517652170845801E-2</v>
       </c>
       <c r="V14">
-        <v>2.7024673757968055E-2</v>
+        <v>2.702467375796799E-2</v>
       </c>
       <c r="W14">
-        <v>2.26823134521991E-2</v>
+        <v>2.2682313452199031E-2</v>
       </c>
       <c r="X14">
-        <v>3.1198898782945052E-2</v>
+        <v>3.1198898782944989E-2</v>
       </c>
       <c r="Y14">
-        <v>3.4877454123141513E-2</v>
+        <v>3.4877454123141451E-2</v>
       </c>
       <c r="Z14">
-        <v>3.6961729073535926E-2</v>
+        <v>3.6961729073535843E-2</v>
       </c>
       <c r="AA14">
-        <v>5.4339186864002284E-2</v>
+        <v>5.4339186864002277E-2</v>
       </c>
       <c r="AB14">
-        <v>5.2703664240623435E-2</v>
+        <v>5.2703664240623428E-2</v>
       </c>
       <c r="AC14">
-        <v>5.7869015600664361E-2</v>
+        <v>5.7869015600664347E-2</v>
       </c>
       <c r="AD14">
         <v>6.3396858649342386E-2</v>
@@ -6707,37 +6755,37 @@
         <v>6.6801046139085857E-2</v>
       </c>
       <c r="AF14">
-        <v>6.7031310904129712E-2</v>
+        <v>6.7031310904129698E-2</v>
       </c>
       <c r="AG14">
-        <v>6.8527730407746401E-2</v>
+        <v>6.8527730407746498E-2</v>
       </c>
       <c r="AH14">
-        <v>7.2040010733636403E-2</v>
+        <v>7.2040010733636389E-2</v>
       </c>
       <c r="AI14">
-        <v>7.3528539983840902E-2</v>
+        <v>7.3528539983840888E-2</v>
       </c>
       <c r="AJ14">
         <v>7.2081871265615161E-2</v>
       </c>
       <c r="AK14">
-        <v>7.5831399120298792E-2</v>
+        <v>7.5831399120298779E-2</v>
       </c>
       <c r="AL14">
-        <v>8.0163584725834722E-2</v>
+        <v>8.0163584725834708E-2</v>
       </c>
       <c r="AM14">
         <v>8.4886327220696195E-2</v>
       </c>
       <c r="AN14">
-        <v>8.500565772529188E-2</v>
+        <v>8.5005657725291867E-2</v>
       </c>
       <c r="AO14">
         <v>8.0633336811407608E-2</v>
       </c>
       <c r="AP14">
-        <v>7.8429760642341417E-2</v>
+        <v>7.8429760642341431E-2</v>
       </c>
       <c r="AQ14">
         <v>8.0404472206152766E-2</v>
@@ -6757,103 +6805,103 @@
         <v>18</v>
       </c>
       <c r="D15">
-        <v>-0.63283476123326854</v>
+        <v>-0.2336411048282977</v>
       </c>
       <c r="E15">
-        <v>-5.2037642757123095E-2</v>
+        <v>-5.2037642757123061E-2</v>
       </c>
       <c r="F15">
-        <v>-5.2427197860636612E-2</v>
+        <v>-5.2427197860636578E-2</v>
       </c>
       <c r="G15">
-        <v>-4.6107837924667675E-2</v>
+        <v>-4.610783792466764E-2</v>
       </c>
       <c r="H15">
-        <v>-4.2071983317046716E-2</v>
+        <v>-4.2071983317046681E-2</v>
       </c>
       <c r="I15">
-        <v>-4.6706357299421478E-2</v>
+        <v>-4.6706357299421457E-2</v>
       </c>
       <c r="J15">
-        <v>-4.8835170295939825E-2</v>
+        <v>-4.8835170295939805E-2</v>
       </c>
       <c r="K15">
-        <v>-5.0145710164612917E-2</v>
+        <v>-5.0145710164612882E-2</v>
       </c>
       <c r="L15">
-        <v>-5.7982793637873037E-2</v>
+        <v>-5.7982793637873002E-2</v>
       </c>
       <c r="M15">
-        <v>-3.4758791616538803E-2</v>
+        <v>-3.4758791616538838E-2</v>
       </c>
       <c r="N15">
-        <v>-3.0807569915452276E-2</v>
+        <v>-3.0807569915452259E-2</v>
       </c>
       <c r="O15">
-        <v>-2.9071464908344197E-2</v>
+        <v>-2.9071464908344179E-2</v>
       </c>
       <c r="P15">
-        <v>-2.0415995927386105E-2</v>
+        <v>-2.0415995927386087E-2</v>
       </c>
       <c r="Q15">
-        <v>-1.6114372976254815E-2</v>
+        <v>-1.6114372976254867E-2</v>
       </c>
       <c r="R15">
         <v>-2.4037370796022736E-2</v>
       </c>
       <c r="S15">
-        <v>-1.6994802059183682E-2</v>
+        <v>-1.6994802059183634E-2</v>
       </c>
       <c r="T15">
-        <v>-8.9083952660905519E-3</v>
+        <v>-8.9083952660904964E-3</v>
       </c>
       <c r="U15">
-        <v>-3.1001449426675612E-3</v>
+        <v>-3.1001449426676072E-3</v>
       </c>
       <c r="V15">
-        <v>1.2822225808479706E-2</v>
+        <v>1.2822225808479715E-2</v>
       </c>
       <c r="W15">
-        <v>1.4650831894722605E-2</v>
+        <v>1.4650831894722638E-2</v>
       </c>
       <c r="X15">
-        <v>2.2492956868268577E-2</v>
+        <v>2.2492956868268608E-2</v>
       </c>
       <c r="Y15">
-        <v>3.0610684006430411E-2</v>
+        <v>3.0610684006430446E-2</v>
       </c>
       <c r="Z15">
-        <v>2.9085253769752462E-2</v>
+        <v>2.9085253769752503E-2</v>
       </c>
       <c r="AA15">
-        <v>4.001302546674855E-2</v>
+        <v>4.0013025466748578E-2</v>
       </c>
       <c r="AB15">
-        <v>4.8993111566340397E-2</v>
+        <v>4.8993111566340293E-2</v>
       </c>
       <c r="AC15">
-        <v>5.1938305422385589E-2</v>
+        <v>5.1938305422385485E-2</v>
       </c>
       <c r="AD15">
-        <v>5.7929186365458019E-2</v>
+        <v>5.7929186365457908E-2</v>
       </c>
       <c r="AE15">
-        <v>6.4747300591034784E-2</v>
+        <v>6.474730059103477E-2</v>
       </c>
       <c r="AF15">
-        <v>6.9432461292525838E-2</v>
+        <v>6.9432461292525824E-2</v>
       </c>
       <c r="AG15">
-        <v>7.050681580248791E-2</v>
+        <v>7.0506815802488021E-2</v>
       </c>
       <c r="AH15">
-        <v>7.3059685358416948E-2</v>
+        <v>7.3059685358416837E-2</v>
       </c>
       <c r="AI15">
         <v>7.7627298958828972E-2</v>
       </c>
       <c r="AJ15">
-        <v>7.9937592374988709E-2</v>
+        <v>7.9937592374988597E-2</v>
       </c>
       <c r="AK15">
         <v>7.8913323318595643E-2</v>
@@ -6862,10 +6910,10 @@
         <v>8.3707308737051955E-2</v>
       </c>
       <c r="AM15">
-        <v>8.9127787434477745E-2</v>
+        <v>8.9127787434477634E-2</v>
       </c>
       <c r="AN15">
-        <v>9.5003213782684559E-2</v>
+        <v>9.5003213782684545E-2</v>
       </c>
       <c r="AO15">
         <v>9.5569887732861181E-2</v>
@@ -6874,7 +6922,7 @@
         <v>9.0922408542367827E-2</v>
       </c>
       <c r="AQ15">
-        <v>8.8734932072262088E-2</v>
+        <v>8.8734932072262102E-2</v>
       </c>
       <c r="AR15" t="s">
         <v>81</v>
@@ -6891,7 +6939,7 @@
         <v>18</v>
       </c>
       <c r="D16">
-        <v>-0.71421675204726509</v>
+        <v>-0.32390276212599578</v>
       </c>
       <c r="E16">
         <v>-6.3095807121780478E-2</v>
@@ -6915,64 +6963,64 @@
         <v>-6.2601565455874586E-2</v>
       </c>
       <c r="L16">
-        <v>-7.1900696615017926E-2</v>
+        <v>-7.1900696615017939E-2</v>
       </c>
       <c r="M16">
         <v>-5.6389295960481069E-2</v>
       </c>
       <c r="N16">
-        <v>-5.351963079214133E-2</v>
+        <v>-5.3519630792141344E-2</v>
       </c>
       <c r="O16">
-        <v>-5.2387330617470411E-2</v>
+        <v>-5.2387330617470425E-2</v>
       </c>
       <c r="P16">
-        <v>-4.4351996998709224E-2</v>
+        <v>-4.4351996998709238E-2</v>
       </c>
       <c r="Q16">
-        <v>-3.9156312930785579E-2</v>
+        <v>-3.9156312930785607E-2</v>
       </c>
       <c r="R16">
-        <v>-4.3064026664249626E-2</v>
+        <v>-4.3064026664249654E-2</v>
       </c>
       <c r="S16">
-        <v>-4.3426805538880016E-2</v>
+        <v>-4.3426805538880002E-2</v>
       </c>
       <c r="T16">
-        <v>-3.7189685831258229E-2</v>
+        <v>-3.718968583125825E-2</v>
       </c>
       <c r="U16">
-        <v>-2.7270322534959895E-2</v>
+        <v>-2.7270322534959875E-2</v>
       </c>
       <c r="V16">
-        <v>-9.3583961450495259E-3</v>
+        <v>-9.3583961450494982E-3</v>
       </c>
       <c r="W16">
-        <v>-3.1568683343509846E-3</v>
+        <v>-3.1568683343509494E-3</v>
       </c>
       <c r="X16">
-        <v>1.2758384819101104E-3</v>
+        <v>1.2758384819101709E-3</v>
       </c>
       <c r="Y16">
-        <v>1.2176445807687578E-2</v>
+        <v>1.2176445807687631E-2</v>
       </c>
       <c r="Z16">
-        <v>1.5351071580688228E-2</v>
+        <v>1.5351071580688288E-2</v>
       </c>
       <c r="AA16">
-        <v>2.2716677505166219E-2</v>
+        <v>2.2716677505166288E-2</v>
       </c>
       <c r="AB16">
-        <v>2.7638269636964211E-2</v>
+        <v>2.7638269636964242E-2</v>
       </c>
       <c r="AC16">
-        <v>3.8452279376099879E-2</v>
+        <v>3.8452279376099886E-2</v>
       </c>
       <c r="AD16">
-        <v>4.1301010444640657E-2</v>
+        <v>4.1301010444640664E-2</v>
       </c>
       <c r="AE16">
-        <v>4.796399875360681E-2</v>
+        <v>4.7963998753606824E-2</v>
       </c>
       <c r="AF16">
         <v>5.6287149449450694E-2</v>
@@ -6981,19 +7029,19 @@
         <v>6.2829846873620823E-2</v>
       </c>
       <c r="AH16">
-        <v>6.5683415624833055E-2</v>
+        <v>6.5683415624833069E-2</v>
       </c>
       <c r="AI16">
         <v>7.0191718917387874E-2</v>
       </c>
       <c r="AJ16">
-        <v>7.61950887609011E-2</v>
+        <v>7.6195088760901114E-2</v>
       </c>
       <c r="AK16">
-        <v>7.9951042190502433E-2</v>
+        <v>7.9951042190502447E-2</v>
       </c>
       <c r="AL16">
-        <v>8.0218701882241145E-2</v>
+        <v>8.0218701882241158E-2</v>
       </c>
       <c r="AM16">
         <v>8.6397575908968266E-2</v>
@@ -7002,7 +7050,7 @@
         <v>9.3151961142697096E-2</v>
       </c>
       <c r="AO16">
-        <v>0.10040439131758706</v>
+        <v>0.10040439131758705</v>
       </c>
       <c r="AP16">
         <v>0.10193129163395233</v>
@@ -7025,28 +7073,28 @@
         <v>18</v>
       </c>
       <c r="D17">
-        <v>-0.77912343740203005</v>
+        <v>-0.39596462147111655</v>
       </c>
       <c r="E17">
-        <v>-5.7882462110618434E-2</v>
+        <v>-5.7882462110618427E-2</v>
       </c>
       <c r="F17">
-        <v>-5.8502182241174393E-2</v>
+        <v>-5.8502182241174386E-2</v>
       </c>
       <c r="G17">
-        <v>-5.5487365748173013E-2</v>
+        <v>-5.5487365748173006E-2</v>
       </c>
       <c r="H17">
-        <v>-5.8398778806590008E-2</v>
+        <v>-5.8398778806590002E-2</v>
       </c>
       <c r="I17">
-        <v>-6.1221379632603525E-2</v>
+        <v>-6.1221379632603518E-2</v>
       </c>
       <c r="J17">
         <v>-6.3109714086543131E-2</v>
       </c>
       <c r="K17">
-        <v>-6.1028222051366966E-2</v>
+        <v>-6.1028222051366959E-2</v>
       </c>
       <c r="L17">
         <v>-7.1770928129587075E-2</v>
@@ -7058,82 +7106,82 @@
         <v>-6.0416401237069629E-2</v>
       </c>
       <c r="O17">
-        <v>-6.7543286206199607E-2</v>
+        <v>-6.7543286206199593E-2</v>
       </c>
       <c r="P17">
-        <v>-6.2255815915461143E-2</v>
+        <v>-6.225581591546115E-2</v>
       </c>
       <c r="Q17">
-        <v>-6.1660531178651529E-2</v>
+        <v>-6.1660531178651536E-2</v>
       </c>
       <c r="R17">
-        <v>-6.2259141649635114E-2</v>
+        <v>-6.225914164963512E-2</v>
       </c>
       <c r="S17">
-        <v>-6.1028771065346432E-2</v>
+        <v>-6.1028771065346439E-2</v>
       </c>
       <c r="T17">
-        <v>-6.3646586060022228E-2</v>
+        <v>-6.3646586060022242E-2</v>
       </c>
       <c r="U17">
-        <v>-6.226801879858819E-2</v>
+        <v>-6.2268018798588183E-2</v>
       </c>
       <c r="V17">
-        <v>-4.7715992430325829E-2</v>
+        <v>-4.7715992430325822E-2</v>
       </c>
       <c r="W17">
-        <v>-3.5240744956108086E-2</v>
+        <v>-3.5240744956108051E-2</v>
       </c>
       <c r="X17">
-        <v>-2.6376491651412051E-2</v>
+        <v>-2.637649165141203E-2</v>
       </c>
       <c r="Y17">
-        <v>-2.5943043178616038E-2</v>
+        <v>-2.5943043178616034E-2</v>
       </c>
       <c r="Z17">
-        <v>-2.1897463176828752E-2</v>
+        <v>-2.1897463176828762E-2</v>
       </c>
       <c r="AA17">
-        <v>-9.9024715330879587E-3</v>
+        <v>-9.9024715330879691E-3</v>
       </c>
       <c r="AB17">
-        <v>-4.5045624943921558E-3</v>
+        <v>-4.5045624943921515E-3</v>
       </c>
       <c r="AC17">
-        <v>1.8896324776878221E-3</v>
+        <v>1.8896324776877553E-3</v>
       </c>
       <c r="AD17">
-        <v>4.3655702827180981E-3</v>
+        <v>4.365570282718125E-3</v>
       </c>
       <c r="AE17">
-        <v>7.3417494248764065E-3</v>
+        <v>7.3417494248764334E-3</v>
       </c>
       <c r="AF17">
-        <v>1.5324723570639284E-2</v>
+        <v>1.5324723570639296E-2</v>
       </c>
       <c r="AG17">
-        <v>2.5357244804214626E-2</v>
+        <v>2.535724480421463E-2</v>
       </c>
       <c r="AH17">
         <v>3.4700380701019759E-2</v>
       </c>
       <c r="AI17">
-        <v>4.1054146586258708E-2</v>
+        <v>4.1054146586258715E-2</v>
       </c>
       <c r="AJ17">
-        <v>4.902412598894966E-2</v>
+        <v>4.9024125988949674E-2</v>
       </c>
       <c r="AK17">
-        <v>5.7071189215417747E-2</v>
+        <v>5.7071189215417754E-2</v>
       </c>
       <c r="AL17">
         <v>6.3365854611260194E-2</v>
       </c>
       <c r="AM17">
-        <v>6.6576855081792993E-2</v>
+        <v>6.6576855081793007E-2</v>
       </c>
       <c r="AN17">
-        <v>7.460381519617397E-2</v>
+        <v>7.4603815196173984E-2</v>
       </c>
       <c r="AO17">
         <v>8.2989221957588052E-2</v>
@@ -7159,7 +7207,7 @@
         <v>18</v>
       </c>
       <c r="D18">
-        <v>-0.81696434357021708</v>
+        <v>-0.43927762026361944</v>
       </c>
       <c r="E18">
         <v>-3.8499867934799592E-2</v>
@@ -7195,10 +7243,10 @@
         <v>-5.2025480713557004E-2</v>
       </c>
       <c r="P18">
-        <v>-5.694144674551474E-2</v>
+        <v>-5.6941446745514747E-2</v>
       </c>
       <c r="Q18">
-        <v>-6.0921105529923733E-2</v>
+        <v>-6.0921105529923726E-2</v>
       </c>
       <c r="R18">
         <v>-6.3235788810306268E-2</v>
@@ -7216,64 +7264,64 @@
         <v>-7.2324230884668841E-2</v>
       </c>
       <c r="W18">
-        <v>-7.1012069490101068E-2</v>
+        <v>-7.101206949010104E-2</v>
       </c>
       <c r="X18">
-        <v>-6.0751002163581883E-2</v>
+        <v>-6.0751002163581862E-2</v>
       </c>
       <c r="Y18">
-        <v>-5.2671560158189842E-2</v>
+        <v>-5.2671560158189815E-2</v>
       </c>
       <c r="Z18">
-        <v>-6.893749032213195E-2</v>
+        <v>-6.8937490322132006E-2</v>
       </c>
       <c r="AA18">
-        <v>-6.1465805543283215E-2</v>
+        <v>-6.1465805543283208E-2</v>
       </c>
       <c r="AB18">
-        <v>-5.52906917100826E-2</v>
+        <v>-5.5290691710082628E-2</v>
       </c>
       <c r="AC18">
-        <v>-4.4809964072162457E-2</v>
+        <v>-4.480996407216245E-2</v>
       </c>
       <c r="AD18">
-        <v>-4.4386436561787701E-2</v>
+        <v>-4.4386436561787687E-2</v>
       </c>
       <c r="AE18">
-        <v>-5.7069717185191403E-2</v>
+        <v>-5.7069717185191375E-2</v>
       </c>
       <c r="AF18">
-        <v>-5.4037897288023128E-2</v>
+        <v>-5.40378972880231E-2</v>
       </c>
       <c r="AG18">
-        <v>-4.6904188690595455E-2</v>
+        <v>-4.6904188690595414E-2</v>
       </c>
       <c r="AH18">
-        <v>-3.8415503548994284E-2</v>
+        <v>-3.8415503548994263E-2</v>
       </c>
       <c r="AI18">
-        <v>-2.8105353051253543E-2</v>
+        <v>-2.8105353051253508E-2</v>
       </c>
       <c r="AJ18">
-        <v>-1.8604447039354849E-2</v>
+        <v>-1.8604447039354832E-2</v>
       </c>
       <c r="AK18">
-        <v>-6.8676179986192631E-3</v>
+        <v>-6.8676179986192449E-3</v>
       </c>
       <c r="AL18">
-        <v>1.7731315482683724E-3</v>
+        <v>1.7731315482683941E-3</v>
       </c>
       <c r="AM18">
-        <v>1.0506404215373924E-2</v>
+        <v>1.0506404215373947E-2</v>
       </c>
       <c r="AN18">
-        <v>1.8258941888178518E-2</v>
+        <v>1.8258941888178549E-2</v>
       </c>
       <c r="AO18">
-        <v>2.7482244375284862E-2</v>
+        <v>2.7482244375284886E-2</v>
       </c>
       <c r="AP18">
-        <v>3.6363293737241287E-2</v>
+        <v>3.6363293737241308E-2</v>
       </c>
       <c r="AQ18">
         <v>4.5797794273245998E-2</v>
@@ -7293,7 +7341,7 @@
         <v>18</v>
       </c>
       <c r="D19">
-        <v>-0.82743038255087886</v>
+        <v>-0.45322080250298341</v>
       </c>
       <c r="E19">
         <v>-1.4391441276768537E-2</v>
@@ -7362,55 +7410,55 @@
         <v>-6.9499559313150217E-2</v>
       </c>
       <c r="AA19">
-        <v>-9.323917844778061E-2</v>
+        <v>-9.3239178447780624E-2</v>
       </c>
       <c r="AB19">
-        <v>-9.7383452624637865E-2</v>
+        <v>-9.7383452624637892E-2</v>
       </c>
       <c r="AC19">
         <v>-9.5190578088595504E-2</v>
       </c>
       <c r="AD19">
-        <v>-9.0152375335023113E-2</v>
+        <v>-9.0152375335023141E-2</v>
       </c>
       <c r="AE19">
-        <v>-0.102576641790045</v>
+        <v>-0.10257664179004501</v>
       </c>
       <c r="AF19">
-        <v>-0.13417950705034012</v>
+        <v>-0.13417950705034015</v>
       </c>
       <c r="AG19">
-        <v>-0.13293766279002708</v>
+        <v>-0.13293766279002711</v>
       </c>
       <c r="AH19">
-        <v>-0.1335880302465654</v>
+        <v>-0.13358803024656543</v>
       </c>
       <c r="AI19">
         <v>-0.13557314433976142</v>
       </c>
       <c r="AJ19">
-        <v>-0.13226872978540294</v>
+        <v>-0.13226872978540297</v>
       </c>
       <c r="AK19">
-        <v>-0.12459140471888019</v>
+        <v>-0.12459140471888018</v>
       </c>
       <c r="AL19">
-        <v>-0.11535101057565567</v>
+        <v>-0.11535101057565568</v>
       </c>
       <c r="AM19">
-        <v>-0.11302040291566937</v>
+        <v>-0.11302040291566935</v>
       </c>
       <c r="AN19">
-        <v>-0.10699752375611601</v>
+        <v>-0.106997523756116</v>
       </c>
       <c r="AO19">
-        <v>-9.653127121046276E-2</v>
+        <v>-9.6531271210462746E-2</v>
       </c>
       <c r="AP19">
-        <v>-9.2826748981408774E-2</v>
+        <v>-9.2826748981408719E-2</v>
       </c>
       <c r="AQ19">
-        <v>-9.0435411379077096E-2</v>
+        <v>-9.0435411379077069E-2</v>
       </c>
       <c r="AR19" t="s">
         <v>81</v>
@@ -7427,7 +7475,7 @@
         <v>18</v>
       </c>
       <c r="D20">
-        <v>-0.82593455233002355</v>
+        <v>-0.454063972031513</v>
       </c>
       <c r="E20">
         <v>-2.978950400279384E-3</v>
@@ -7561,7 +7609,7 @@
         <v>18</v>
       </c>
       <c r="D21">
-        <v>-0.82237107008060717</v>
+        <v>-0.452291760434334</v>
       </c>
       <c r="E21">
         <v>-3.3334425406091809E-4</v>
@@ -7691,7 +7739,7 @@
     </row>
     <row r="24" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="B24" t="s">
         <v>17</v>
@@ -7700,7 +7748,7 @@
         <v>18</v>
       </c>
       <c r="D24">
-        <v>-0.15967272058620607</v>
+        <v>0.2753267546775866</v>
       </c>
       <c r="E24">
         <v>2.214154581450245E-3</v>
@@ -7825,7 +7873,7 @@
     </row>
     <row r="25" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>65</v>
+        <v>102</v>
       </c>
       <c r="B25" t="s">
         <v>17</v>
@@ -7834,7 +7882,7 @@
         <v>18</v>
       </c>
       <c r="D25">
-        <v>-0.24565717190814917</v>
+        <v>0.18944091200051794</v>
       </c>
       <c r="E25">
         <v>-8.798052235841184E-3</v>
@@ -7843,7 +7891,7 @@
         <v>2.4929074421023954E-3</v>
       </c>
       <c r="G25">
-        <v>-2.1373270782093393E-2</v>
+        <v>-2.137327078209339E-2</v>
       </c>
       <c r="H25">
         <v>-8.6453951054279478E-3</v>
@@ -7867,7 +7915,7 @@
         <v>3.3933903565056878E-2</v>
       </c>
       <c r="O25">
-        <v>3.0383907874593656E-2</v>
+        <v>3.038390787459366E-2</v>
       </c>
       <c r="P25">
         <v>4.7839256681225573E-2</v>
@@ -7879,40 +7927,40 @@
         <v>3.9490915288615258E-2</v>
       </c>
       <c r="S25">
-        <v>3.6536510565018603E-2</v>
+        <v>3.6536510565018609E-2</v>
       </c>
       <c r="T25">
-        <v>4.2142916628999709E-2</v>
+        <v>4.2142916628999716E-2</v>
       </c>
       <c r="U25">
-        <v>4.6470535159674135E-2</v>
+        <v>4.6470535159674142E-2</v>
       </c>
       <c r="V25">
         <v>7.4841309368095077E-2</v>
       </c>
       <c r="W25">
-        <v>5.4583454125459951E-2</v>
+        <v>5.4583454125459945E-2</v>
       </c>
       <c r="X25">
-        <v>5.5003826390571886E-2</v>
+        <v>5.5003826390571879E-2</v>
       </c>
       <c r="Y25">
         <v>6.5383546651785807E-2</v>
       </c>
       <c r="Z25">
-        <v>6.1813519294937391E-2</v>
+        <v>6.1813519294937606E-2</v>
       </c>
       <c r="AA25">
         <v>6.5356164722600418E-2</v>
       </c>
       <c r="AB25">
-        <v>6.3794944403975595E-2</v>
+        <v>6.3794944403975373E-2</v>
       </c>
       <c r="AC25">
-        <v>6.1654781829491911E-2</v>
+        <v>6.1654781829491904E-2</v>
       </c>
       <c r="AD25">
-        <v>6.2307356539842318E-2</v>
+        <v>6.2307356539842311E-2</v>
       </c>
       <c r="AE25">
         <v>6.3362208607063986E-2</v>
@@ -7924,25 +7972,25 @@
         <v>6.4188713044355028E-2</v>
       </c>
       <c r="AH25">
-        <v>6.1814578816645427E-2</v>
+        <v>6.181457881664542E-2</v>
       </c>
       <c r="AI25">
-        <v>6.0425638744489363E-2</v>
+        <v>6.0425638744489356E-2</v>
       </c>
       <c r="AJ25">
-        <v>6.0816741782236616E-2</v>
+        <v>6.0816741782236609E-2</v>
       </c>
       <c r="AK25">
-        <v>6.1455653716094405E-2</v>
+        <v>6.1455653716094398E-2</v>
       </c>
       <c r="AL25">
-        <v>6.1922434122747338E-2</v>
+        <v>6.1922434122747332E-2</v>
       </c>
       <c r="AM25">
-        <v>6.1888309307405409E-2</v>
+        <v>6.1888309307405402E-2</v>
       </c>
       <c r="AN25">
-        <v>6.115230770110347E-2</v>
+        <v>6.1152307701103463E-2</v>
       </c>
       <c r="AO25">
         <v>6.0103532554758754E-2</v>
@@ -7959,7 +8007,7 @@
     </row>
     <row r="26" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="B26" t="s">
         <v>17</v>
@@ -7968,7 +8016,7 @@
         <v>18</v>
       </c>
       <c r="D26">
-        <v>-0.26155473045267985</v>
+        <v>0.17236558985102601</v>
       </c>
       <c r="E26">
         <v>-7.236851580176909E-4</v>
@@ -8019,25 +8067,25 @@
         <v>2.6039029199987899E-2</v>
       </c>
       <c r="U26">
-        <v>3.6717245073956788E-2</v>
+        <v>3.6717245073956781E-2</v>
       </c>
       <c r="V26">
         <v>6.2434500490324389E-2</v>
       </c>
       <c r="W26">
-        <v>4.6318139893231074E-2</v>
+        <v>4.6318139893231067E-2</v>
       </c>
       <c r="X26">
         <v>5.135931795910563E-2</v>
       </c>
       <c r="Y26">
-        <v>6.3306729060164532E-2</v>
+        <v>6.3306729060164546E-2</v>
       </c>
       <c r="Z26">
         <v>6.4793987221842819E-2</v>
       </c>
       <c r="AA26">
-        <v>6.7801677319718298E-2</v>
+        <v>6.7801677319718312E-2</v>
       </c>
       <c r="AB26">
         <v>6.6660882767059615E-2</v>
@@ -8049,16 +8097,16 @@
         <v>6.3914424269086556E-2</v>
       </c>
       <c r="AE26">
-        <v>6.4829697214101589E-2</v>
+        <v>6.4829697214101478E-2</v>
       </c>
       <c r="AF26">
         <v>6.615753944350633E-2</v>
       </c>
       <c r="AG26">
-        <v>6.7667415928057237E-2</v>
+        <v>6.7667415928057251E-2</v>
       </c>
       <c r="AH26">
-        <v>6.7112657448067367E-2</v>
+        <v>6.7112657448067381E-2</v>
       </c>
       <c r="AI26">
         <v>6.4605800891545329E-2</v>
@@ -8093,7 +8141,7 @@
     </row>
     <row r="27" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="B27" t="s">
         <v>17</v>
@@ -8102,67 +8150,67 @@
         <v>18</v>
       </c>
       <c r="D27">
-        <v>-0.30679603837354075</v>
+        <v>0.1254070895445526</v>
       </c>
       <c r="E27">
-        <v>-5.9408663182357775E-3</v>
+        <v>-5.940866318235774E-3</v>
       </c>
       <c r="F27">
-        <v>-5.2210796294517928E-4</v>
+        <v>-5.2210796294517581E-4</v>
       </c>
       <c r="G27">
-        <v>-1.1217645657931173E-2</v>
+        <v>-1.1217645657931166E-2</v>
       </c>
       <c r="H27">
         <v>4.7936319832520939E-3</v>
       </c>
       <c r="I27">
-        <v>1.2300780327542872E-2</v>
+        <v>1.2300780327542877E-2</v>
       </c>
       <c r="J27">
         <v>3.6018982593929265E-3</v>
       </c>
       <c r="K27">
-        <v>-1.0632310666801502E-2</v>
+        <v>-1.0632310666801495E-2</v>
       </c>
       <c r="L27">
-        <v>-6.1418031984663245E-2</v>
+        <v>-6.1418031984663238E-2</v>
       </c>
       <c r="M27">
         <v>8.3506772794188819E-2</v>
       </c>
       <c r="N27">
-        <v>4.2098509327472035E-2</v>
+        <v>4.2098509327472042E-2</v>
       </c>
       <c r="O27">
-        <v>2.1277843934306522E-2</v>
+        <v>2.1277843934306526E-2</v>
       </c>
       <c r="P27">
-        <v>3.2427341011736256E-2</v>
+        <v>3.2427341011736263E-2</v>
       </c>
       <c r="Q27">
-        <v>4.1599468865491242E-2</v>
+        <v>4.1599468865491249E-2</v>
       </c>
       <c r="R27">
         <v>3.3459220219192877E-2</v>
       </c>
       <c r="S27">
-        <v>2.251123900569283E-2</v>
+        <v>2.2511239005692834E-2</v>
       </c>
       <c r="T27">
-        <v>2.258295303613609E-2</v>
+        <v>2.2582953036136093E-2</v>
       </c>
       <c r="U27">
         <v>2.5075531682969145E-2</v>
       </c>
       <c r="V27">
-        <v>5.4937600323355464E-2</v>
+        <v>5.4937600323355457E-2</v>
       </c>
       <c r="W27">
-        <v>4.1640307135442069E-2</v>
+        <v>4.1640307135442062E-2</v>
       </c>
       <c r="X27">
-        <v>4.4439142707816327E-2</v>
+        <v>4.443914270781632E-2</v>
       </c>
       <c r="Y27">
         <v>5.5212886244188714E-2</v>
@@ -8171,34 +8219,34 @@
         <v>5.618081009162032E-2</v>
       </c>
       <c r="AA27">
-        <v>5.4722622480382489E-2</v>
+        <v>5.4722622480382482E-2</v>
       </c>
       <c r="AB27">
-        <v>5.1066943946999489E-2</v>
+        <v>5.1066943946999482E-2</v>
       </c>
       <c r="AC27">
-        <v>5.2200109377753524E-2</v>
+        <v>5.2200109377753517E-2</v>
       </c>
       <c r="AD27">
-        <v>5.225936691619102E-2</v>
+        <v>5.2259366916191013E-2</v>
       </c>
       <c r="AE27">
         <v>5.0570034717299019E-2</v>
       </c>
       <c r="AF27">
-        <v>5.1734782894280885E-2</v>
+        <v>5.1734782894280879E-2</v>
       </c>
       <c r="AG27">
         <v>5.3243420655319153E-2</v>
       </c>
       <c r="AH27">
-        <v>5.4949081267275469E-2</v>
+        <v>5.4949081267275462E-2</v>
       </c>
       <c r="AI27">
         <v>5.4397351488425262E-2</v>
       </c>
       <c r="AJ27">
-        <v>5.1711484709427748E-2</v>
+        <v>5.1711484709427637E-2</v>
       </c>
       <c r="AK27">
         <v>5.0164603436464762E-2</v>
@@ -8210,7 +8258,7 @@
         <v>5.1499939203650348E-2</v>
       </c>
       <c r="AN27">
-        <v>5.2104933092651941E-2</v>
+        <v>5.210493309265183E-2</v>
       </c>
       <c r="AO27">
         <v>5.2116584423815705E-2</v>
@@ -8227,7 +8275,7 @@
     </row>
     <row r="28" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>68</v>
+        <v>105</v>
       </c>
       <c r="B28" t="s">
         <v>17</v>
@@ -8236,124 +8284,124 @@
         <v>18</v>
       </c>
       <c r="D28">
-        <v>-0.37443848101655242</v>
+        <v>5.5486024490896124E-2</v>
       </c>
       <c r="E28">
-        <v>-1.2702194956710489E-2</v>
+        <v>-1.2702194956710565E-2</v>
       </c>
       <c r="F28">
-        <v>-5.3741464852489762E-3</v>
+        <v>-5.374146485249056E-3</v>
       </c>
       <c r="G28">
-        <v>1.3202308870674251E-2</v>
+        <v>1.3202308870674173E-2</v>
       </c>
       <c r="H28">
-        <v>2.0226923364166038E-2</v>
+        <v>2.0226923364166066E-2</v>
       </c>
       <c r="I28">
-        <v>3.8681168096839601E-3</v>
+        <v>3.8681168096838768E-3</v>
       </c>
       <c r="J28">
-        <v>-1.4069022719456793E-3</v>
+        <v>-1.4069022719457626E-3</v>
       </c>
       <c r="K28">
-        <v>-1.0746652435382701E-2</v>
+        <v>-1.0746652435382781E-2</v>
       </c>
       <c r="L28">
-        <v>-3.8672715018868549E-2</v>
+        <v>-3.8672715018868625E-2</v>
       </c>
       <c r="M28">
-        <v>4.6242670608277851E-2</v>
+        <v>4.6242670608277768E-2</v>
       </c>
       <c r="N28">
-        <v>3.2087587651180735E-2</v>
+        <v>3.2087587651180645E-2</v>
       </c>
       <c r="O28">
-        <v>2.0549004741740859E-2</v>
+        <v>2.0549004741740769E-2</v>
       </c>
       <c r="P28">
-        <v>2.8630609697237797E-2</v>
+        <v>2.8630609697237724E-2</v>
       </c>
       <c r="Q28">
-        <v>2.5809721325159296E-2</v>
+        <v>2.5809721325159334E-2</v>
       </c>
       <c r="R28">
-        <v>2.6436049586985234E-2</v>
+        <v>2.6436049586985248E-2</v>
       </c>
       <c r="S28">
-        <v>1.878120487739502E-2</v>
+        <v>1.8781204877395034E-2</v>
       </c>
       <c r="T28">
-        <v>1.9427291127762467E-2</v>
+        <v>1.942729112776248E-2</v>
       </c>
       <c r="U28">
-        <v>1.8842827998864428E-2</v>
+        <v>1.8842827998864345E-2</v>
       </c>
       <c r="V28">
-        <v>3.9848805662785737E-2</v>
+        <v>3.9848805662785751E-2</v>
       </c>
       <c r="W28">
-        <v>3.68354748338462E-2</v>
+        <v>3.6835474833846187E-2</v>
       </c>
       <c r="X28">
-        <v>4.1295026842261835E-2</v>
+        <v>4.1295026842261828E-2</v>
       </c>
       <c r="Y28">
-        <v>4.8146828548922833E-2</v>
+        <v>4.814682854892282E-2</v>
       </c>
       <c r="Z28">
-        <v>4.8803883237712682E-2</v>
+        <v>4.8803883237712661E-2</v>
       </c>
       <c r="AA28">
-        <v>4.8887690302795057E-2</v>
+        <v>4.8887690302795037E-2</v>
       </c>
       <c r="AB28">
-        <v>4.338826851800804E-2</v>
+        <v>4.3388268518008033E-2</v>
       </c>
       <c r="AC28">
-        <v>4.3315476262297384E-2</v>
+        <v>4.331547626229737E-2</v>
       </c>
       <c r="AD28">
-        <v>4.4697988409070813E-2</v>
+        <v>4.4697988409070799E-2</v>
       </c>
       <c r="AE28">
-        <v>4.4708888724039456E-2</v>
+        <v>4.4708888724039442E-2</v>
       </c>
       <c r="AF28">
-        <v>4.304110553234166E-2</v>
+        <v>4.3041105532341653E-2</v>
       </c>
       <c r="AG28">
         <v>4.4448454850834609E-2</v>
       </c>
       <c r="AH28">
-        <v>4.6217389546187496E-2</v>
+        <v>4.6217389546187489E-2</v>
       </c>
       <c r="AI28">
-        <v>4.820173184352728E-2</v>
+        <v>4.8201731843527273E-2</v>
       </c>
       <c r="AJ28">
-        <v>4.7693422755138895E-2</v>
+        <v>4.7693422755138881E-2</v>
       </c>
       <c r="AK28">
-        <v>4.4825064135562552E-2</v>
+        <v>4.4825064135562545E-2</v>
       </c>
       <c r="AL28">
         <v>4.3202834678336549E-2</v>
       </c>
       <c r="AM28">
-        <v>4.3856471237945248E-2</v>
+        <v>4.3856471237945255E-2</v>
       </c>
       <c r="AN28">
         <v>4.4819082596581759E-2</v>
       </c>
       <c r="AO28">
-        <v>4.5550537967718151E-2</v>
+        <v>4.5550537967718262E-2</v>
       </c>
       <c r="AP28">
         <v>4.5619038144155709E-2</v>
       </c>
       <c r="AQ28">
-        <v>4.4756495508269233E-2</v>
+        <v>4.475649550826924E-2</v>
       </c>
       <c r="AR28" t="s">
         <v>81</v>
@@ -8361,7 +8409,7 @@
     </row>
     <row r="29" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>69</v>
+        <v>106</v>
       </c>
       <c r="B29" t="s">
         <v>17</v>
@@ -8370,34 +8418,34 @@
         <v>18</v>
       </c>
       <c r="D29">
-        <v>-0.39477406481363475</v>
+        <v>3.2263302252500826E-2</v>
       </c>
       <c r="E29">
-        <v>-9.4274541427797065E-3</v>
+        <v>-9.4274541427796996E-3</v>
       </c>
       <c r="F29">
-        <v>-9.8165612929002333E-3</v>
+        <v>-9.8165612929002263E-3</v>
       </c>
       <c r="G29">
-        <v>-2.3487080085657086E-3</v>
+        <v>-2.3487080085657017E-3</v>
       </c>
       <c r="H29">
-        <v>-8.6583804029078115E-3</v>
+        <v>-8.6583804029078046E-3</v>
       </c>
       <c r="I29">
-        <v>-5.4340259083950626E-3</v>
+        <v>-5.4340259083950557E-3</v>
       </c>
       <c r="J29">
-        <v>-6.5539401508452333E-3</v>
+        <v>-6.5539401508452264E-3</v>
       </c>
       <c r="K29">
-        <v>-1.3651670884479744E-2</v>
+        <v>-1.3651670884479737E-2</v>
       </c>
       <c r="L29">
         <v>-3.5139292967922203E-2</v>
       </c>
       <c r="M29">
-        <v>2.4831739846267381E-2</v>
+        <v>2.4831739846267388E-2</v>
       </c>
       <c r="N29">
         <v>1.6870479800516897E-2</v>
@@ -8409,10 +8457,10 @@
         <v>2.3562270899732257E-2</v>
       </c>
       <c r="Q29">
-        <v>2.2503835982026071E-2</v>
+        <v>2.2503835982026078E-2</v>
       </c>
       <c r="R29">
-        <v>1.6627122488387241E-2</v>
+        <v>1.6627122488387248E-2</v>
       </c>
       <c r="S29">
         <v>1.6294200651658847E-2</v>
@@ -8427,34 +8475,34 @@
         <v>3.3677227950180105E-2</v>
       </c>
       <c r="W29">
-        <v>3.0801701882456865E-2</v>
+        <v>3.0801701882456869E-2</v>
       </c>
       <c r="X29">
-        <v>4.3793562001004115E-2</v>
+        <v>4.3793562001004108E-2</v>
       </c>
       <c r="Y29">
-        <v>4.6527981823540863E-2</v>
+        <v>4.6527981823540857E-2</v>
       </c>
       <c r="Z29">
-        <v>4.5534778306406586E-2</v>
+        <v>4.5534778306406579E-2</v>
       </c>
       <c r="AA29">
-        <v>4.701621914579298E-2</v>
+        <v>4.7016219145792973E-2</v>
       </c>
       <c r="AB29">
-        <v>4.2204248431996404E-2</v>
+        <v>4.2204248431996397E-2</v>
       </c>
       <c r="AC29">
-        <v>4.2186777917608574E-2</v>
+        <v>4.2186777917608567E-2</v>
       </c>
       <c r="AD29">
-        <v>4.2399357228157984E-2</v>
+        <v>4.2399357228157977E-2</v>
       </c>
       <c r="AE29">
-        <v>4.3862301147063319E-2</v>
+        <v>4.3862301147063312E-2</v>
       </c>
       <c r="AF29">
-        <v>4.4074140935555138E-2</v>
+        <v>4.4074140935555131E-2</v>
       </c>
       <c r="AG29">
         <v>4.2516374851200488E-2</v>
@@ -8463,13 +8511,13 @@
         <v>4.4270114989099794E-2</v>
       </c>
       <c r="AI29">
-        <v>4.6403055946117232E-2</v>
+        <v>4.6403055946117225E-2</v>
       </c>
       <c r="AJ29">
-        <v>4.876923028997978E-2</v>
+        <v>4.8769230289979773E-2</v>
       </c>
       <c r="AK29">
-        <v>4.8383908285399811E-2</v>
+        <v>4.8383908285399804E-2</v>
       </c>
       <c r="AL29">
         <v>4.5371764879791519E-2</v>
@@ -8484,7 +8532,7 @@
         <v>4.5740860162084528E-2</v>
       </c>
       <c r="AP29">
-        <v>4.6658586496614217E-2</v>
+        <v>4.6658586496614106E-2</v>
       </c>
       <c r="AQ29">
         <v>4.6827914600688213E-2</v>
@@ -8495,7 +8543,7 @@
     </row>
     <row r="30" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>70</v>
+        <v>107</v>
       </c>
       <c r="B30" t="s">
         <v>17</v>
@@ -8504,64 +8552,64 @@
         <v>18</v>
       </c>
       <c r="D30">
-        <v>-0.44667298808583028</v>
+        <v>-2.4362696747206626E-2</v>
       </c>
       <c r="E30">
-        <v>-1.9744143023249609E-2</v>
+        <v>-1.9744143023249595E-2</v>
       </c>
       <c r="F30">
-        <v>-1.5694522694105643E-2</v>
+        <v>-1.569452269410563E-2</v>
       </c>
       <c r="G30">
-        <v>-1.3803534801163191E-2</v>
+        <v>-1.3803534801163177E-2</v>
       </c>
       <c r="H30">
-        <v>-5.6008504068616946E-3</v>
+        <v>-5.6008504068616807E-3</v>
       </c>
       <c r="I30">
-        <v>-1.1072434743251085E-2</v>
+        <v>-1.1072434743251078E-2</v>
       </c>
       <c r="J30">
-        <v>-1.1630240244701988E-2</v>
+        <v>-1.1630240244701981E-2</v>
       </c>
       <c r="K30">
-        <v>-1.5827651241563205E-2</v>
+        <v>-1.5827651241563198E-2</v>
       </c>
       <c r="L30">
-        <v>-3.310727451521616E-2</v>
+        <v>-3.3107274515216153E-2</v>
       </c>
       <c r="M30">
-        <v>1.6949583156538335E-2</v>
+        <v>1.6949583156538345E-2</v>
       </c>
       <c r="N30">
-        <v>1.1694021451363834E-2</v>
+        <v>1.1694021451363851E-2</v>
       </c>
       <c r="O30">
-        <v>6.6070355231971356E-3</v>
+        <v>6.607035523197146E-3</v>
       </c>
       <c r="P30">
-        <v>1.6179132674044194E-2</v>
+        <v>1.617913267404409E-2</v>
       </c>
       <c r="Q30">
-        <v>1.9926990479983864E-2</v>
+        <v>1.992699047998376E-2</v>
       </c>
       <c r="R30">
-        <v>1.1600062759427765E-2</v>
+        <v>1.1600062759427779E-2</v>
       </c>
       <c r="S30">
-        <v>1.1348239910148161E-2</v>
+        <v>1.1348239910148179E-2</v>
       </c>
       <c r="T30">
-        <v>1.7647398240613066E-2</v>
+        <v>1.7647398240613069E-2</v>
       </c>
       <c r="U30">
-        <v>2.0410556529964541E-2</v>
+        <v>2.0410556529964433E-2</v>
       </c>
       <c r="V30">
-        <v>3.4731058335620346E-2</v>
+        <v>3.4731058335620353E-2</v>
       </c>
       <c r="W30">
-        <v>2.7111581932348916E-2</v>
+        <v>2.7111581932348923E-2</v>
       </c>
       <c r="X30">
         <v>3.7972505161053161E-2</v>
@@ -8585,31 +8633,31 @@
         <v>4.9972656292513504E-2</v>
       </c>
       <c r="AE30">
-        <v>5.0367205191953639E-2</v>
+        <v>5.0367205191953632E-2</v>
       </c>
       <c r="AF30">
         <v>5.2324027316411989E-2</v>
       </c>
       <c r="AG30">
-        <v>5.2839647456881682E-2</v>
+        <v>5.2839647456881675E-2</v>
       </c>
       <c r="AH30">
-        <v>5.128470322715855E-2</v>
+        <v>5.1284703227158661E-2</v>
       </c>
       <c r="AI30">
-        <v>5.3524444794866115E-2</v>
+        <v>5.3524444794866108E-2</v>
       </c>
       <c r="AJ30">
-        <v>5.6196092357453091E-2</v>
+        <v>5.6196092357453084E-2</v>
       </c>
       <c r="AK30">
         <v>5.9140392258269989E-2</v>
       </c>
       <c r="AL30">
-        <v>5.8861085693118813E-2</v>
+        <v>5.8861085693118806E-2</v>
       </c>
       <c r="AM30">
-        <v>5.5482472390448505E-2</v>
+        <v>5.5482472390448616E-2</v>
       </c>
       <c r="AN30">
         <v>5.3666018053928059E-2</v>
@@ -8621,7 +8669,7 @@
         <v>5.6281623903386695E-2</v>
       </c>
       <c r="AQ30">
-        <v>5.7466221853147585E-2</v>
+        <v>5.7466221853147696E-2</v>
       </c>
       <c r="AR30" t="s">
         <v>81</v>
@@ -8629,7 +8677,7 @@
     </row>
     <row r="31" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>108</v>
       </c>
       <c r="B31" t="s">
         <v>17</v>
@@ -8638,73 +8686,73 @@
         <v>18</v>
       </c>
       <c r="D31">
-        <v>-0.49360419959189489</v>
+        <v>-7.7681981575542222E-2</v>
       </c>
       <c r="E31">
-        <v>-2.3277271395060535E-2</v>
+        <v>-2.3277271395060518E-2</v>
       </c>
       <c r="F31">
-        <v>-2.4987170380011477E-2</v>
+        <v>-2.4987170380011459E-2</v>
       </c>
       <c r="G31">
-        <v>-2.2380335949466271E-3</v>
+        <v>-2.2380335949466045E-3</v>
       </c>
       <c r="H31">
-        <v>-3.774767171564504E-3</v>
+        <v>-3.7747671715644814E-3</v>
       </c>
       <c r="I31">
-        <v>-1.8837995105936929E-2</v>
+        <v>-1.8837995105936915E-2</v>
       </c>
       <c r="J31">
-        <v>-1.8099542588297497E-2</v>
+        <v>-1.8099542588297483E-2</v>
       </c>
       <c r="K31">
-        <v>-2.3618017476338245E-2</v>
+        <v>-2.3618017476338342E-2</v>
       </c>
       <c r="L31">
-        <v>-3.6927158134320411E-2</v>
+        <v>-3.6927158134320508E-2</v>
       </c>
       <c r="M31">
-        <v>7.065565109499676E-3</v>
+        <v>7.0655651094995806E-3</v>
       </c>
       <c r="N31">
-        <v>3.7115214991423826E-3</v>
+        <v>3.7115214991422867E-3</v>
       </c>
       <c r="O31">
-        <v>4.6446070404598111E-4</v>
+        <v>4.6446070404588478E-4</v>
       </c>
       <c r="P31">
-        <v>8.1538935903364002E-3</v>
+        <v>8.153893590336303E-3</v>
       </c>
       <c r="Q31">
-        <v>9.2240250353885916E-3</v>
+        <v>9.2240250353885986E-3</v>
       </c>
       <c r="R31">
-        <v>6.9506092481375487E-3</v>
+        <v>6.9506092481375547E-3</v>
       </c>
       <c r="S31">
-        <v>8.2444176885352813E-3</v>
+        <v>8.2444176885351841E-3</v>
       </c>
       <c r="T31">
-        <v>1.2443883907405744E-2</v>
+        <v>1.2443883907405643E-2</v>
       </c>
       <c r="U31">
-        <v>1.7292850567156161E-2</v>
+        <v>1.7292850567156171E-2</v>
       </c>
       <c r="V31">
-        <v>3.1521434602123012E-2</v>
+        <v>3.1521434602123026E-2</v>
       </c>
       <c r="W31">
-        <v>2.7082537533778685E-2</v>
+        <v>2.7082537533778699E-2</v>
       </c>
       <c r="X31">
-        <v>3.2384978759609814E-2</v>
+        <v>3.2384978759609821E-2</v>
       </c>
       <c r="Y31">
-        <v>4.1678498616248873E-2</v>
+        <v>4.167849861624888E-2</v>
       </c>
       <c r="Z31">
-        <v>4.6740050040789204E-2</v>
+        <v>4.6740050040789197E-2</v>
       </c>
       <c r="AA31">
         <v>5.1460424840708799E-2</v>
@@ -8722,28 +8770,28 @@
         <v>5.9285298673382406E-2</v>
       </c>
       <c r="AF31">
-        <v>6.0157936055520139E-2</v>
+        <v>6.0157936055520132E-2</v>
       </c>
       <c r="AG31">
-        <v>6.2814644599020003E-2</v>
+        <v>6.2814644599019989E-2</v>
       </c>
       <c r="AH31">
-        <v>6.3767816462993926E-2</v>
+        <v>6.3767816462993912E-2</v>
       </c>
       <c r="AI31">
-        <v>6.2263152718157105E-2</v>
+        <v>6.2263152718157112E-2</v>
       </c>
       <c r="AJ31">
-        <v>6.5180589669482064E-2</v>
+        <v>6.518058966948205E-2</v>
       </c>
       <c r="AK31">
-        <v>6.8591157893913263E-2</v>
+        <v>6.8591157893913249E-2</v>
       </c>
       <c r="AL31">
         <v>7.2326527671071963E-2</v>
       </c>
       <c r="AM31">
-        <v>7.2218810292072361E-2</v>
+        <v>7.2218810292072347E-2</v>
       </c>
       <c r="AN31">
         <v>6.839029681186129E-2</v>
@@ -8763,7 +8811,7 @@
     </row>
     <row r="32" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>72</v>
+        <v>109</v>
       </c>
       <c r="B32" t="s">
         <v>17</v>
@@ -8772,82 +8820,82 @@
         <v>18</v>
       </c>
       <c r="D32">
-        <v>-0.56305776842292055</v>
+        <v>-0.15514258183260632</v>
       </c>
       <c r="E32">
-        <v>-3.7199091661566056E-2</v>
+        <v>-3.7199091661566021E-2</v>
       </c>
       <c r="F32">
-        <v>-3.6004194110941704E-2</v>
+        <v>-3.6004194110941669E-2</v>
       </c>
       <c r="G32">
-        <v>-3.4009631774868723E-2</v>
+        <v>-3.4009631774868689E-2</v>
       </c>
       <c r="H32">
-        <v>-3.8667025253932251E-2</v>
+        <v>-3.8667025253932216E-2</v>
       </c>
       <c r="I32">
-        <v>-3.3762485938915753E-2</v>
+        <v>-3.3762485938915718E-2</v>
       </c>
       <c r="J32">
-        <v>-3.1649879133818698E-2</v>
+        <v>-3.1649879133818677E-2</v>
       </c>
       <c r="K32">
-        <v>-3.4137274010349966E-2</v>
+        <v>-3.4137274010349945E-2</v>
       </c>
       <c r="L32">
-        <v>-4.3899557951590937E-2</v>
+        <v>-4.3899557951590965E-2</v>
       </c>
       <c r="M32">
-        <v>-1.0537820685555289E-2</v>
+        <v>-1.053782068555531E-2</v>
       </c>
       <c r="N32">
-        <v>-8.743488884343488E-3</v>
+        <v>-8.7434888843435209E-3</v>
       </c>
       <c r="O32">
-        <v>-1.0566105072038125E-2</v>
+        <v>-1.0566105072038159E-2</v>
       </c>
       <c r="P32">
-        <v>-3.0381415838877518E-3</v>
+        <v>-3.038141583887672E-3</v>
       </c>
       <c r="Q32">
-        <v>-2.3588494353154466E-3</v>
+        <v>-2.3588494353154938E-3</v>
       </c>
       <c r="R32">
-        <v>-5.0283536279328092E-3</v>
+        <v>-5.0283536279328639E-3</v>
       </c>
       <c r="S32">
-        <v>1.1611979587263163E-3</v>
+        <v>1.1611979587262615E-3</v>
       </c>
       <c r="T32">
-        <v>3.9062506038237202E-3</v>
+        <v>3.9062506038237974E-3</v>
       </c>
       <c r="U32">
-        <v>1.1517652170845723E-2</v>
+        <v>1.1517652170845801E-2</v>
       </c>
       <c r="V32">
-        <v>2.7024673757968055E-2</v>
+        <v>2.702467375796799E-2</v>
       </c>
       <c r="W32">
-        <v>2.26823134521991E-2</v>
+        <v>2.2682313452199031E-2</v>
       </c>
       <c r="X32">
-        <v>3.1198898782945052E-2</v>
+        <v>3.1198898782944989E-2</v>
       </c>
       <c r="Y32">
-        <v>3.4877454123141513E-2</v>
+        <v>3.4877454123141451E-2</v>
       </c>
       <c r="Z32">
-        <v>3.6961729073535926E-2</v>
+        <v>3.6961729073535843E-2</v>
       </c>
       <c r="AA32">
-        <v>5.4339186864002284E-2</v>
+        <v>5.4339186864002277E-2</v>
       </c>
       <c r="AB32">
-        <v>5.2703664240623435E-2</v>
+        <v>5.2703664240623428E-2</v>
       </c>
       <c r="AC32">
-        <v>5.7869015600664361E-2</v>
+        <v>5.7869015600664347E-2</v>
       </c>
       <c r="AD32">
         <v>6.3396858649342386E-2</v>
@@ -8856,37 +8904,37 @@
         <v>6.6801046139085857E-2</v>
       </c>
       <c r="AF32">
-        <v>6.7031310904129712E-2</v>
+        <v>6.7031310904129698E-2</v>
       </c>
       <c r="AG32">
-        <v>6.8527730407746401E-2</v>
+        <v>6.8527730407746498E-2</v>
       </c>
       <c r="AH32">
-        <v>7.2040010733636403E-2</v>
+        <v>7.2040010733636389E-2</v>
       </c>
       <c r="AI32">
-        <v>7.3528539983840902E-2</v>
+        <v>7.3528539983840888E-2</v>
       </c>
       <c r="AJ32">
         <v>7.2081871265615161E-2</v>
       </c>
       <c r="AK32">
-        <v>7.5831399120298792E-2</v>
+        <v>7.5831399120298779E-2</v>
       </c>
       <c r="AL32">
-        <v>8.0163584725834722E-2</v>
+        <v>8.0163584725834708E-2</v>
       </c>
       <c r="AM32">
         <v>8.4886327220696195E-2</v>
       </c>
       <c r="AN32">
-        <v>8.500565772529188E-2</v>
+        <v>8.5005657725291867E-2</v>
       </c>
       <c r="AO32">
         <v>8.0633336811407608E-2</v>
       </c>
       <c r="AP32">
-        <v>7.8429760642341417E-2</v>
+        <v>7.8429760642341431E-2</v>
       </c>
       <c r="AQ32">
         <v>8.0404472206152766E-2</v>
@@ -8897,7 +8945,7 @@
     </row>
     <row r="33" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>73</v>
+        <v>110</v>
       </c>
       <c r="B33" t="s">
         <v>17</v>
@@ -8906,103 +8954,103 @@
         <v>18</v>
       </c>
       <c r="D33">
-        <v>-0.63283476123326854</v>
+        <v>-0.2336411048282977</v>
       </c>
       <c r="E33">
-        <v>-5.2037642757123095E-2</v>
+        <v>-5.2037642757123061E-2</v>
       </c>
       <c r="F33">
-        <v>-5.2427197860636612E-2</v>
+        <v>-5.2427197860636578E-2</v>
       </c>
       <c r="G33">
-        <v>-4.6107837924667675E-2</v>
+        <v>-4.610783792466764E-2</v>
       </c>
       <c r="H33">
-        <v>-4.2071983317046716E-2</v>
+        <v>-4.2071983317046681E-2</v>
       </c>
       <c r="I33">
-        <v>-4.6706357299421478E-2</v>
+        <v>-4.6706357299421457E-2</v>
       </c>
       <c r="J33">
-        <v>-4.8835170295939825E-2</v>
+        <v>-4.8835170295939805E-2</v>
       </c>
       <c r="K33">
-        <v>-5.0145710164612917E-2</v>
+        <v>-5.0145710164612882E-2</v>
       </c>
       <c r="L33">
-        <v>-5.7982793637873037E-2</v>
+        <v>-5.7982793637873002E-2</v>
       </c>
       <c r="M33">
-        <v>-3.4758791616538803E-2</v>
+        <v>-3.4758791616538838E-2</v>
       </c>
       <c r="N33">
-        <v>-3.0807569915452276E-2</v>
+        <v>-3.0807569915452259E-2</v>
       </c>
       <c r="O33">
-        <v>-2.9071464908344197E-2</v>
+        <v>-2.9071464908344179E-2</v>
       </c>
       <c r="P33">
-        <v>-2.0415995927386105E-2</v>
+        <v>-2.0415995927386087E-2</v>
       </c>
       <c r="Q33">
-        <v>-1.6114372976254815E-2</v>
+        <v>-1.6114372976254867E-2</v>
       </c>
       <c r="R33">
         <v>-2.4037370796022736E-2</v>
       </c>
       <c r="S33">
-        <v>-1.6994802059183682E-2</v>
+        <v>-1.6994802059183634E-2</v>
       </c>
       <c r="T33">
-        <v>-8.9083952660905519E-3</v>
+        <v>-8.9083952660904964E-3</v>
       </c>
       <c r="U33">
-        <v>-3.1001449426675612E-3</v>
+        <v>-3.1001449426676072E-3</v>
       </c>
       <c r="V33">
-        <v>1.2822225808479706E-2</v>
+        <v>1.2822225808479715E-2</v>
       </c>
       <c r="W33">
-        <v>1.4650831894722605E-2</v>
+        <v>1.4650831894722638E-2</v>
       </c>
       <c r="X33">
-        <v>2.2492956868268577E-2</v>
+        <v>2.2492956868268608E-2</v>
       </c>
       <c r="Y33">
-        <v>3.0610684006430411E-2</v>
+        <v>3.0610684006430446E-2</v>
       </c>
       <c r="Z33">
-        <v>2.9085253769752462E-2</v>
+        <v>2.9085253769752503E-2</v>
       </c>
       <c r="AA33">
-        <v>4.001302546674855E-2</v>
+        <v>4.0013025466748578E-2</v>
       </c>
       <c r="AB33">
-        <v>4.8993111566340397E-2</v>
+        <v>4.8993111566340293E-2</v>
       </c>
       <c r="AC33">
-        <v>5.1938305422385589E-2</v>
+        <v>5.1938305422385485E-2</v>
       </c>
       <c r="AD33">
-        <v>5.7929186365458019E-2</v>
+        <v>5.7929186365457908E-2</v>
       </c>
       <c r="AE33">
-        <v>6.4747300591034784E-2</v>
+        <v>6.474730059103477E-2</v>
       </c>
       <c r="AF33">
-        <v>6.9432461292525838E-2</v>
+        <v>6.9432461292525824E-2</v>
       </c>
       <c r="AG33">
-        <v>7.050681580248791E-2</v>
+        <v>7.0506815802488021E-2</v>
       </c>
       <c r="AH33">
-        <v>7.3059685358416948E-2</v>
+        <v>7.3059685358416837E-2</v>
       </c>
       <c r="AI33">
         <v>7.7627298958828972E-2</v>
       </c>
       <c r="AJ33">
-        <v>7.9937592374988709E-2</v>
+        <v>7.9937592374988597E-2</v>
       </c>
       <c r="AK33">
         <v>7.8913323318595643E-2</v>
@@ -9011,10 +9059,10 @@
         <v>8.3707308737051955E-2</v>
       </c>
       <c r="AM33">
-        <v>8.9127787434477745E-2</v>
+        <v>8.9127787434477634E-2</v>
       </c>
       <c r="AN33">
-        <v>9.5003213782684559E-2</v>
+        <v>9.5003213782684545E-2</v>
       </c>
       <c r="AO33">
         <v>9.5569887732861181E-2</v>
@@ -9023,7 +9071,7 @@
         <v>9.0922408542367827E-2</v>
       </c>
       <c r="AQ33">
-        <v>8.8734932072262088E-2</v>
+        <v>8.8734932072262102E-2</v>
       </c>
       <c r="AR33" t="s">
         <v>81</v>
@@ -9031,7 +9079,7 @@
     </row>
     <row r="34" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>74</v>
+        <v>111</v>
       </c>
       <c r="B34" t="s">
         <v>17</v>
@@ -9040,7 +9088,7 @@
         <v>18</v>
       </c>
       <c r="D34">
-        <v>-0.71421675204726509</v>
+        <v>-0.32390276212599578</v>
       </c>
       <c r="E34">
         <v>-6.3095807121780478E-2</v>
@@ -9064,64 +9112,64 @@
         <v>-6.2601565455874586E-2</v>
       </c>
       <c r="L34">
-        <v>-7.1900696615017926E-2</v>
+        <v>-7.1900696615017939E-2</v>
       </c>
       <c r="M34">
         <v>-5.6389295960481069E-2</v>
       </c>
       <c r="N34">
-        <v>-5.351963079214133E-2</v>
+        <v>-5.3519630792141344E-2</v>
       </c>
       <c r="O34">
-        <v>-5.2387330617470411E-2</v>
+        <v>-5.2387330617470425E-2</v>
       </c>
       <c r="P34">
-        <v>-4.4351996998709224E-2</v>
+        <v>-4.4351996998709238E-2</v>
       </c>
       <c r="Q34">
-        <v>-3.9156312930785579E-2</v>
+        <v>-3.9156312930785607E-2</v>
       </c>
       <c r="R34">
-        <v>-4.3064026664249626E-2</v>
+        <v>-4.3064026664249654E-2</v>
       </c>
       <c r="S34">
-        <v>-4.3426805538880016E-2</v>
+        <v>-4.3426805538880002E-2</v>
       </c>
       <c r="T34">
-        <v>-3.7189685831258229E-2</v>
+        <v>-3.718968583125825E-2</v>
       </c>
       <c r="U34">
-        <v>-2.7270322534959895E-2</v>
+        <v>-2.7270322534959875E-2</v>
       </c>
       <c r="V34">
-        <v>-9.3583961450495259E-3</v>
+        <v>-9.3583961450494982E-3</v>
       </c>
       <c r="W34">
-        <v>-3.1568683343509846E-3</v>
+        <v>-3.1568683343509494E-3</v>
       </c>
       <c r="X34">
-        <v>1.2758384819101104E-3</v>
+        <v>1.2758384819101709E-3</v>
       </c>
       <c r="Y34">
-        <v>1.2176445807687578E-2</v>
+        <v>1.2176445807687631E-2</v>
       </c>
       <c r="Z34">
-        <v>1.5351071580688228E-2</v>
+        <v>1.5351071580688288E-2</v>
       </c>
       <c r="AA34">
-        <v>2.2716677505166219E-2</v>
+        <v>2.2716677505166288E-2</v>
       </c>
       <c r="AB34">
-        <v>2.7638269636964211E-2</v>
+        <v>2.7638269636964242E-2</v>
       </c>
       <c r="AC34">
-        <v>3.8452279376099879E-2</v>
+        <v>3.8452279376099886E-2</v>
       </c>
       <c r="AD34">
-        <v>4.1301010444640657E-2</v>
+        <v>4.1301010444640664E-2</v>
       </c>
       <c r="AE34">
-        <v>4.796399875360681E-2</v>
+        <v>4.7963998753606824E-2</v>
       </c>
       <c r="AF34">
         <v>5.6287149449450694E-2</v>
@@ -9130,19 +9178,19 @@
         <v>6.2829846873620823E-2</v>
       </c>
       <c r="AH34">
-        <v>6.5683415624833055E-2</v>
+        <v>6.5683415624833069E-2</v>
       </c>
       <c r="AI34">
         <v>7.0191718917387874E-2</v>
       </c>
       <c r="AJ34">
-        <v>7.61950887609011E-2</v>
+        <v>7.6195088760901114E-2</v>
       </c>
       <c r="AK34">
-        <v>7.9951042190502433E-2</v>
+        <v>7.9951042190502447E-2</v>
       </c>
       <c r="AL34">
-        <v>8.0218701882241145E-2</v>
+        <v>8.0218701882241158E-2</v>
       </c>
       <c r="AM34">
         <v>8.6397575908968266E-2</v>
@@ -9151,7 +9199,7 @@
         <v>9.3151961142697096E-2</v>
       </c>
       <c r="AO34">
-        <v>0.10040439131758706</v>
+        <v>0.10040439131758705</v>
       </c>
       <c r="AP34">
         <v>0.10193129163395233</v>
@@ -9165,7 +9213,7 @@
     </row>
     <row r="35" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="B35" t="s">
         <v>17</v>
@@ -9174,28 +9222,28 @@
         <v>18</v>
       </c>
       <c r="D35">
-        <v>-0.77912343740203005</v>
+        <v>-0.39596462147111655</v>
       </c>
       <c r="E35">
-        <v>-5.7882462110618434E-2</v>
+        <v>-5.7882462110618427E-2</v>
       </c>
       <c r="F35">
-        <v>-5.8502182241174393E-2</v>
+        <v>-5.8502182241174386E-2</v>
       </c>
       <c r="G35">
-        <v>-5.5487365748173013E-2</v>
+        <v>-5.5487365748173006E-2</v>
       </c>
       <c r="H35">
-        <v>-5.8398778806590008E-2</v>
+        <v>-5.8398778806590002E-2</v>
       </c>
       <c r="I35">
-        <v>-6.1221379632603525E-2</v>
+        <v>-6.1221379632603518E-2</v>
       </c>
       <c r="J35">
         <v>-6.3109714086543131E-2</v>
       </c>
       <c r="K35">
-        <v>-6.1028222051366966E-2</v>
+        <v>-6.1028222051366959E-2</v>
       </c>
       <c r="L35">
         <v>-7.1770928129587075E-2</v>
@@ -9207,82 +9255,82 @@
         <v>-6.0416401237069629E-2</v>
       </c>
       <c r="O35">
-        <v>-6.7543286206199607E-2</v>
+        <v>-6.7543286206199593E-2</v>
       </c>
       <c r="P35">
-        <v>-6.2255815915461143E-2</v>
+        <v>-6.225581591546115E-2</v>
       </c>
       <c r="Q35">
-        <v>-6.1660531178651529E-2</v>
+        <v>-6.1660531178651536E-2</v>
       </c>
       <c r="R35">
-        <v>-6.2259141649635114E-2</v>
+        <v>-6.225914164963512E-2</v>
       </c>
       <c r="S35">
-        <v>-6.1028771065346432E-2</v>
+        <v>-6.1028771065346439E-2</v>
       </c>
       <c r="T35">
-        <v>-6.3646586060022228E-2</v>
+        <v>-6.3646586060022242E-2</v>
       </c>
       <c r="U35">
-        <v>-6.226801879858819E-2</v>
+        <v>-6.2268018798588183E-2</v>
       </c>
       <c r="V35">
-        <v>-4.7715992430325829E-2</v>
+        <v>-4.7715992430325822E-2</v>
       </c>
       <c r="W35">
-        <v>-3.5240744956108086E-2</v>
+        <v>-3.5240744956108051E-2</v>
       </c>
       <c r="X35">
-        <v>-2.6376491651412051E-2</v>
+        <v>-2.637649165141203E-2</v>
       </c>
       <c r="Y35">
-        <v>-2.5943043178616038E-2</v>
+        <v>-2.5943043178616034E-2</v>
       </c>
       <c r="Z35">
-        <v>-2.1897463176828752E-2</v>
+        <v>-2.1897463176828762E-2</v>
       </c>
       <c r="AA35">
-        <v>-9.9024715330879587E-3</v>
+        <v>-9.9024715330879691E-3</v>
       </c>
       <c r="AB35">
-        <v>-4.5045624943921558E-3</v>
+        <v>-4.5045624943921515E-3</v>
       </c>
       <c r="AC35">
-        <v>1.8896324776878221E-3</v>
+        <v>1.8896324776877553E-3</v>
       </c>
       <c r="AD35">
-        <v>4.3655702827180981E-3</v>
+        <v>4.365570282718125E-3</v>
       </c>
       <c r="AE35">
-        <v>7.3417494248764065E-3</v>
+        <v>7.3417494248764334E-3</v>
       </c>
       <c r="AF35">
-        <v>1.5324723570639284E-2</v>
+        <v>1.5324723570639296E-2</v>
       </c>
       <c r="AG35">
-        <v>2.5357244804214626E-2</v>
+        <v>2.535724480421463E-2</v>
       </c>
       <c r="AH35">
         <v>3.4700380701019759E-2</v>
       </c>
       <c r="AI35">
-        <v>4.1054146586258708E-2</v>
+        <v>4.1054146586258715E-2</v>
       </c>
       <c r="AJ35">
-        <v>4.902412598894966E-2</v>
+        <v>4.9024125988949674E-2</v>
       </c>
       <c r="AK35">
-        <v>5.7071189215417747E-2</v>
+        <v>5.7071189215417754E-2</v>
       </c>
       <c r="AL35">
         <v>6.3365854611260194E-2</v>
       </c>
       <c r="AM35">
-        <v>6.6576855081792993E-2</v>
+        <v>6.6576855081793007E-2</v>
       </c>
       <c r="AN35">
-        <v>7.460381519617397E-2</v>
+        <v>7.4603815196173984E-2</v>
       </c>
       <c r="AO35">
         <v>8.2989221957588052E-2</v>
@@ -9299,7 +9347,7 @@
     </row>
     <row r="36" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>76</v>
+        <v>113</v>
       </c>
       <c r="B36" t="s">
         <v>17</v>
@@ -9308,7 +9356,7 @@
         <v>18</v>
       </c>
       <c r="D36">
-        <v>-0.81696434357021708</v>
+        <v>-0.43927762026361944</v>
       </c>
       <c r="E36">
         <v>-3.8499867934799592E-2</v>
@@ -9344,10 +9392,10 @@
         <v>-5.2025480713557004E-2</v>
       </c>
       <c r="P36">
-        <v>-5.694144674551474E-2</v>
+        <v>-5.6941446745514747E-2</v>
       </c>
       <c r="Q36">
-        <v>-6.0921105529923733E-2</v>
+        <v>-6.0921105529923726E-2</v>
       </c>
       <c r="R36">
         <v>-6.3235788810306268E-2</v>
@@ -9365,64 +9413,64 @@
         <v>-7.2324230884668841E-2</v>
       </c>
       <c r="W36">
-        <v>-7.1012069490101068E-2</v>
+        <v>-7.101206949010104E-2</v>
       </c>
       <c r="X36">
-        <v>-6.0751002163581883E-2</v>
+        <v>-6.0751002163581862E-2</v>
       </c>
       <c r="Y36">
-        <v>-5.2671560158189842E-2</v>
+        <v>-5.2671560158189815E-2</v>
       </c>
       <c r="Z36">
-        <v>-6.893749032213195E-2</v>
+        <v>-6.8937490322132006E-2</v>
       </c>
       <c r="AA36">
-        <v>-6.1465805543283215E-2</v>
+        <v>-6.1465805543283208E-2</v>
       </c>
       <c r="AB36">
-        <v>-5.52906917100826E-2</v>
+        <v>-5.5290691710082628E-2</v>
       </c>
       <c r="AC36">
-        <v>-4.4809964072162457E-2</v>
+        <v>-4.480996407216245E-2</v>
       </c>
       <c r="AD36">
-        <v>-4.4386436561787701E-2</v>
+        <v>-4.4386436561787687E-2</v>
       </c>
       <c r="AE36">
-        <v>-5.7069717185191403E-2</v>
+        <v>-5.7069717185191375E-2</v>
       </c>
       <c r="AF36">
-        <v>-5.4037897288023128E-2</v>
+        <v>-5.40378972880231E-2</v>
       </c>
       <c r="AG36">
-        <v>-4.6904188690595455E-2</v>
+        <v>-4.6904188690595414E-2</v>
       </c>
       <c r="AH36">
-        <v>-3.8415503548994284E-2</v>
+        <v>-3.8415503548994263E-2</v>
       </c>
       <c r="AI36">
-        <v>-2.8105353051253543E-2</v>
+        <v>-2.8105353051253508E-2</v>
       </c>
       <c r="AJ36">
-        <v>-1.8604447039354849E-2</v>
+        <v>-1.8604447039354832E-2</v>
       </c>
       <c r="AK36">
-        <v>-6.8676179986192631E-3</v>
+        <v>-6.8676179986192449E-3</v>
       </c>
       <c r="AL36">
-        <v>1.7731315482683724E-3</v>
+        <v>1.7731315482683941E-3</v>
       </c>
       <c r="AM36">
-        <v>1.0506404215373924E-2</v>
+        <v>1.0506404215373947E-2</v>
       </c>
       <c r="AN36">
-        <v>1.8258941888178518E-2</v>
+        <v>1.8258941888178549E-2</v>
       </c>
       <c r="AO36">
-        <v>2.7482244375284862E-2</v>
+        <v>2.7482244375284886E-2</v>
       </c>
       <c r="AP36">
-        <v>3.6363293737241287E-2</v>
+        <v>3.6363293737241308E-2</v>
       </c>
       <c r="AQ36">
         <v>4.5797794273245998E-2</v>
@@ -9433,7 +9481,7 @@
     </row>
     <row r="37" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>77</v>
+        <v>114</v>
       </c>
       <c r="B37" t="s">
         <v>17</v>
@@ -9442,7 +9490,7 @@
         <v>18</v>
       </c>
       <c r="D37">
-        <v>-0.82743038255087886</v>
+        <v>-0.45322080250298341</v>
       </c>
       <c r="E37">
         <v>-1.4391441276768537E-2</v>
@@ -9511,55 +9559,55 @@
         <v>-6.9499559313150217E-2</v>
       </c>
       <c r="AA37">
-        <v>-9.323917844778061E-2</v>
+        <v>-9.3239178447780624E-2</v>
       </c>
       <c r="AB37">
-        <v>-9.7383452624637865E-2</v>
+        <v>-9.7383452624637892E-2</v>
       </c>
       <c r="AC37">
         <v>-9.5190578088595504E-2</v>
       </c>
       <c r="AD37">
-        <v>-9.0152375335023113E-2</v>
+        <v>-9.0152375335023141E-2</v>
       </c>
       <c r="AE37">
-        <v>-0.102576641790045</v>
+        <v>-0.10257664179004501</v>
       </c>
       <c r="AF37">
-        <v>-0.13417950705034012</v>
+        <v>-0.13417950705034015</v>
       </c>
       <c r="AG37">
-        <v>-0.13293766279002708</v>
+        <v>-0.13293766279002711</v>
       </c>
       <c r="AH37">
-        <v>-0.1335880302465654</v>
+        <v>-0.13358803024656543</v>
       </c>
       <c r="AI37">
         <v>-0.13557314433976142</v>
       </c>
       <c r="AJ37">
-        <v>-0.13226872978540294</v>
+        <v>-0.13226872978540297</v>
       </c>
       <c r="AK37">
-        <v>-0.12459140471888019</v>
+        <v>-0.12459140471888018</v>
       </c>
       <c r="AL37">
-        <v>-0.11535101057565567</v>
+        <v>-0.11535101057565568</v>
       </c>
       <c r="AM37">
-        <v>-0.11302040291566937</v>
+        <v>-0.11302040291566935</v>
       </c>
       <c r="AN37">
-        <v>-0.10699752375611601</v>
+        <v>-0.106997523756116</v>
       </c>
       <c r="AO37">
-        <v>-9.653127121046276E-2</v>
+        <v>-9.6531271210462746E-2</v>
       </c>
       <c r="AP37">
-        <v>-9.2826748981408774E-2</v>
+        <v>-9.2826748981408719E-2</v>
       </c>
       <c r="AQ37">
-        <v>-9.0435411379077096E-2</v>
+        <v>-9.0435411379077069E-2</v>
       </c>
       <c r="AR37" t="s">
         <v>81</v>
@@ -9567,7 +9615,7 @@
     </row>
     <row r="38" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="B38" t="s">
         <v>17</v>
@@ -9576,7 +9624,7 @@
         <v>18</v>
       </c>
       <c r="D38">
-        <v>-0.82593455233002355</v>
+        <v>-0.454063972031513</v>
       </c>
       <c r="E38">
         <v>-2.978950400279384E-3</v>
@@ -9701,7 +9749,7 @@
     </row>
     <row r="39" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="B39" t="s">
         <v>17</v>
@@ -9710,7 +9758,7 @@
         <v>18</v>
       </c>
       <c r="D39">
-        <v>-0.82237107008060717</v>
+        <v>-0.452291760434334</v>
       </c>
       <c r="E39">
         <v>-3.3334425406091809E-4</v>

</xml_diff>

<commit_message>
linear solver pour les chocs migratoires
</commit_message>
<xml_diff>
--- a/all_shocks.xlsx
+++ b/all_shocks.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\emanu\OneDrive\Matlab\cdc_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67CF5976-DA50-458E-A81C-A6B3EAE312F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{805979DB-7382-40C6-8002-035900C8F5AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_pop_shocks_norm2000" sheetId="1" r:id="rId1"/>
     <sheet name="1_popshocks_values" sheetId="3" r:id="rId2"/>
-    <sheet name="2_mig_shocks" sheetId="2" r:id="rId3"/>
+    <sheet name="2_mig_shocks_vieux" sheetId="2" r:id="rId3"/>
+    <sheet name="2_mig_shocks_renorm" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="121">
   <si>
     <t>=</t>
   </si>
@@ -20946,4 +20947,4448 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AA2E4BB-BE47-467E-8717-D1D74DF6029F}">
+  <dimension ref="A1:AR39"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AC3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AE3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AF3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AG3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AH3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AI3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AJ3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AL3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AO3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AQ3" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>-0.44726131189217022</v>
+      </c>
+      <c r="E6">
+        <v>-0.36914315052464836</v>
+      </c>
+      <c r="F6">
+        <v>-0.37300933490262422</v>
+      </c>
+      <c r="G6">
+        <v>-0.37252326236856126</v>
+      </c>
+      <c r="H6">
+        <v>-0.35442939666455564</v>
+      </c>
+      <c r="I6">
+        <v>-0.3325867631175855</v>
+      </c>
+      <c r="J6">
+        <v>-0.33589175986139724</v>
+      </c>
+      <c r="K6">
+        <v>-0.3405174763785298</v>
+      </c>
+      <c r="L6">
+        <v>-0.36332093854591141</v>
+      </c>
+      <c r="M6">
+        <v>-0.3411407980530059</v>
+      </c>
+      <c r="N6">
+        <v>-0.32796983850718536</v>
+      </c>
+      <c r="O6">
+        <v>-0.35816074040762857</v>
+      </c>
+      <c r="P6">
+        <v>-0.39199561409953987</v>
+      </c>
+      <c r="Q6">
+        <v>-0.4471368803890074</v>
+      </c>
+      <c r="R6">
+        <v>-0.48084828304877447</v>
+      </c>
+      <c r="S6">
+        <v>-0.46652123327721062</v>
+      </c>
+      <c r="T6">
+        <v>-0.46390298605986258</v>
+      </c>
+      <c r="U6">
+        <v>-0.45153292834668868</v>
+      </c>
+      <c r="V6">
+        <v>-0.43592860767132346</v>
+      </c>
+      <c r="W6">
+        <v>-0.43672168946432383</v>
+      </c>
+      <c r="X6">
+        <v>-0.43261945944728797</v>
+      </c>
+      <c r="Y6">
+        <v>-0.43758192652992484</v>
+      </c>
+      <c r="Z6">
+        <v>-0.44440202423966135</v>
+      </c>
+      <c r="AA6">
+        <v>-0.45149807951239551</v>
+      </c>
+      <c r="AB6">
+        <v>-0.46292639152740389</v>
+      </c>
+      <c r="AC6">
+        <v>-0.45248147114409781</v>
+      </c>
+      <c r="AD6">
+        <v>-0.43772372803985582</v>
+      </c>
+      <c r="AE6">
+        <v>-0.41783594159099446</v>
+      </c>
+      <c r="AF6">
+        <v>-0.40655877800291129</v>
+      </c>
+      <c r="AG6">
+        <v>-0.41091630005462393</v>
+      </c>
+      <c r="AH6">
+        <v>-0.41843819002776772</v>
+      </c>
+      <c r="AI6">
+        <v>-0.41756202764977474</v>
+      </c>
+      <c r="AJ6">
+        <v>-0.40971265710146298</v>
+      </c>
+      <c r="AK6">
+        <v>-0.39789833865400437</v>
+      </c>
+      <c r="AL6">
+        <v>-0.38746318626010229</v>
+      </c>
+      <c r="AM6">
+        <v>-0.3821398646666968</v>
+      </c>
+      <c r="AN6">
+        <v>-0.38192233664322683</v>
+      </c>
+      <c r="AO6">
+        <v>-0.38234125283036119</v>
+      </c>
+      <c r="AP6">
+        <v>-0.37912346563453064</v>
+      </c>
+      <c r="AQ6">
+        <v>-0.37207387365439981</v>
+      </c>
+      <c r="AR6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>-0.47880771499948205</v>
+      </c>
+      <c r="E7">
+        <v>-6.4627396979410889E-4</v>
+      </c>
+      <c r="F7">
+        <v>1.8312026495126421E-4</v>
+      </c>
+      <c r="G7">
+        <v>-1.5700047159400432E-3</v>
+      </c>
+      <c r="H7">
+        <v>-6.3505995688339922E-4</v>
+      </c>
+      <c r="I7">
+        <v>2.6919206285099251E-3</v>
+      </c>
+      <c r="J7">
+        <v>1.6692021167747373E-3</v>
+      </c>
+      <c r="K7">
+        <v>-8.6455450690969826E-5</v>
+      </c>
+      <c r="L7">
+        <v>-8.303486742639421E-3</v>
+      </c>
+      <c r="M7">
+        <v>6.1311684188237736E-3</v>
+      </c>
+      <c r="N7">
+        <v>2.492665390036175E-3</v>
+      </c>
+      <c r="O7">
+        <v>2.2318949756262585E-3</v>
+      </c>
+      <c r="P7">
+        <v>3.5715495223050397E-3</v>
+      </c>
+      <c r="Q7">
+        <v>3.4555337579774137E-3</v>
+      </c>
+      <c r="R7">
+        <v>2.9008637925752034E-3</v>
+      </c>
+      <c r="S7">
+        <v>2.6838434061236538E-3</v>
+      </c>
+      <c r="T7">
+        <v>3.0956704666160739E-3</v>
+      </c>
+      <c r="U7">
+        <v>3.4135617514798877E-3</v>
+      </c>
+      <c r="V7">
+        <v>5.4975792200159801E-3</v>
+      </c>
+      <c r="W7">
+        <v>4.0095088043512472E-3</v>
+      </c>
+      <c r="X7">
+        <v>4.0403876502772551E-3</v>
+      </c>
+      <c r="Y7">
+        <v>4.8028451673184924E-3</v>
+      </c>
+      <c r="Z7">
+        <v>4.5406036708912634E-3</v>
+      </c>
+      <c r="AA7">
+        <v>4.8008342744096932E-3</v>
+      </c>
+      <c r="AB7">
+        <v>4.6861521274530471E-3</v>
+      </c>
+      <c r="AC7">
+        <v>4.5289433363621123E-3</v>
+      </c>
+      <c r="AD7">
+        <v>4.57687873561341E-3</v>
+      </c>
+      <c r="AE7">
+        <v>4.6543657206043476E-3</v>
+      </c>
+      <c r="AF7">
+        <v>4.7555844295341099E-3</v>
+      </c>
+      <c r="AG7">
+        <v>4.7150777167476177E-3</v>
+      </c>
+      <c r="AH7">
+        <v>4.5406817779693465E-3</v>
+      </c>
+      <c r="AI7">
+        <v>4.4386551399621665E-3</v>
+      </c>
+      <c r="AJ7">
+        <v>4.467384214106751E-3</v>
+      </c>
+      <c r="AK7">
+        <v>4.5143161269602938E-3</v>
+      </c>
+      <c r="AL7">
+        <v>4.5486035792373647E-3</v>
+      </c>
+      <c r="AM7">
+        <v>4.546098008672228E-3</v>
+      </c>
+      <c r="AN7">
+        <v>4.4920337440940705E-3</v>
+      </c>
+      <c r="AO7">
+        <v>4.4149938224959939E-3</v>
+      </c>
+      <c r="AP7">
+        <v>4.3658186224450057E-3</v>
+      </c>
+      <c r="AQ7">
+        <v>4.3638484198814664E-3</v>
+      </c>
+      <c r="AR7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>-0.47872825914897399</v>
+      </c>
+      <c r="E8">
+        <v>-5.3159446124939613E-5</v>
+      </c>
+      <c r="F8">
+        <v>5.0888083150180119E-5</v>
+      </c>
+      <c r="G8">
+        <v>-7.0412999249941377E-4</v>
+      </c>
+      <c r="H8">
+        <v>-1.8870197301190661E-4</v>
+      </c>
+      <c r="I8">
+        <v>1.934859810363565E-3</v>
+      </c>
+      <c r="J8">
+        <v>1.0598391742976387E-3</v>
+      </c>
+      <c r="K8">
+        <v>-3.4627662091551992E-4</v>
+      </c>
+      <c r="L8">
+        <v>-6.9977922497858058E-3</v>
+      </c>
+      <c r="M8">
+        <v>7.588370611202544E-3</v>
+      </c>
+      <c r="N8">
+        <v>3.2845330520310245E-3</v>
+      </c>
+      <c r="O8">
+        <v>1.7133420005925881E-3</v>
+      </c>
+      <c r="P8">
+        <v>3.2920311670212032E-3</v>
+      </c>
+      <c r="Q8">
+        <v>3.4552685786040649E-3</v>
+      </c>
+      <c r="R8">
+        <v>2.7702768133184841E-3</v>
+      </c>
+      <c r="S8">
+        <v>1.7574502021153182E-3</v>
+      </c>
+      <c r="T8">
+        <v>1.9127355944216773E-3</v>
+      </c>
+      <c r="U8">
+        <v>2.6971190458636718E-3</v>
+      </c>
+      <c r="V8">
+        <v>4.5862193011654839E-3</v>
+      </c>
+      <c r="W8">
+        <v>3.4023674734629528E-3</v>
+      </c>
+      <c r="X8">
+        <v>3.7726743049525391E-3</v>
+      </c>
+      <c r="Y8">
+        <v>4.6502891450257433E-3</v>
+      </c>
+      <c r="Z8">
+        <v>4.7595381535229242E-3</v>
+      </c>
+      <c r="AA8">
+        <v>4.9804731047050632E-3</v>
+      </c>
+      <c r="AB8">
+        <v>4.8966742190908463E-3</v>
+      </c>
+      <c r="AC8">
+        <v>4.835644269742867E-3</v>
+      </c>
+      <c r="AD8">
+        <v>4.6949291268807425E-3</v>
+      </c>
+      <c r="AE8">
+        <v>4.7621613869786028E-3</v>
+      </c>
+      <c r="AF8">
+        <v>4.8596996696590455E-3</v>
+      </c>
+      <c r="AG8">
+        <v>4.9706111034334977E-3</v>
+      </c>
+      <c r="AH8">
+        <v>4.9298593550914926E-3</v>
+      </c>
+      <c r="AI8">
+        <v>4.7457154038292315E-3</v>
+      </c>
+      <c r="AJ8">
+        <v>4.6387628960360416E-3</v>
+      </c>
+      <c r="AK8">
+        <v>4.6714550160493196E-3</v>
+      </c>
+      <c r="AL8">
+        <v>4.7233514406865851E-3</v>
+      </c>
+      <c r="AM8">
+        <v>4.7616394041393173E-3</v>
+      </c>
+      <c r="AN8">
+        <v>4.7604381944313379E-3</v>
+      </c>
+      <c r="AO8">
+        <v>4.7036793708022384E-3</v>
+      </c>
+      <c r="AP8">
+        <v>4.6222036243005471E-3</v>
+      </c>
+      <c r="AQ8">
+        <v>4.5705513897718042E-3</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>-0.48023304445544734</v>
+      </c>
+      <c r="E9">
+        <v>-4.3639452705629411E-4</v>
+      </c>
+      <c r="F9">
+        <v>-3.8351879539655354E-5</v>
+      </c>
+      <c r="G9">
+        <v>-8.240093634657164E-4</v>
+      </c>
+      <c r="H9">
+        <v>3.5212347230745289E-4</v>
+      </c>
+      <c r="I9">
+        <v>9.0357224249476564E-4</v>
+      </c>
+      <c r="J9">
+        <v>2.6458229105325026E-4</v>
+      </c>
+      <c r="K9">
+        <v>-7.8101204498864929E-4</v>
+      </c>
+      <c r="L9">
+        <v>-4.5115521179441842E-3</v>
+      </c>
+      <c r="M9">
+        <v>6.134114311951655E-3</v>
+      </c>
+      <c r="N9">
+        <v>3.092407832651356E-3</v>
+      </c>
+      <c r="O9">
+        <v>1.5629952349722198E-3</v>
+      </c>
+      <c r="P9">
+        <v>2.3688418161338931E-3</v>
+      </c>
+      <c r="Q9">
+        <v>2.9486138349620328E-3</v>
+      </c>
+      <c r="R9">
+        <v>2.4577969624251517E-3</v>
+      </c>
+      <c r="S9">
+        <v>1.6535966698173477E-3</v>
+      </c>
+      <c r="T9">
+        <v>1.6588644538443331E-3</v>
+      </c>
+      <c r="U9">
+        <v>1.841960035304735E-3</v>
+      </c>
+      <c r="V9">
+        <v>4.035523325018997E-3</v>
+      </c>
+      <c r="W9">
+        <v>3.058749930472171E-3</v>
+      </c>
+      <c r="X9">
+        <v>3.264342585644342E-3</v>
+      </c>
+      <c r="Y9">
+        <v>4.0557442544742472E-3</v>
+      </c>
+      <c r="Z9">
+        <v>4.1268448420505588E-3</v>
+      </c>
+      <c r="AA9">
+        <v>4.0197311931188251E-3</v>
+      </c>
+      <c r="AB9">
+        <v>3.7511977156240439E-3</v>
+      </c>
+      <c r="AC9">
+        <v>3.8344358745150964E-3</v>
+      </c>
+      <c r="AD9">
+        <v>3.8387898041483126E-3</v>
+      </c>
+      <c r="AE9">
+        <v>3.7146966706816387E-3</v>
+      </c>
+      <c r="AF9">
+        <v>3.8002551304623933E-3</v>
+      </c>
+      <c r="AG9">
+        <v>3.9110739527127292E-3</v>
+      </c>
+      <c r="AH9">
+        <v>4.0363656872483E-3</v>
+      </c>
+      <c r="AI9">
+        <v>3.9958378264378092E-3</v>
+      </c>
+      <c r="AJ9">
+        <v>3.7985432340723602E-3</v>
+      </c>
+      <c r="AK9">
+        <v>3.6849148403184095E-3</v>
+      </c>
+      <c r="AL9">
+        <v>3.723572386509777E-3</v>
+      </c>
+      <c r="AM9">
+        <v>3.7830049458139614E-3</v>
+      </c>
+      <c r="AN9">
+        <v>3.8274449440508507E-3</v>
+      </c>
+      <c r="AO9">
+        <v>3.8283012458907306E-3</v>
+      </c>
+      <c r="AP9">
+        <v>3.7680738524394908E-3</v>
+      </c>
+      <c r="AQ9">
+        <v>3.6804563481211972E-3</v>
+      </c>
+      <c r="AR9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>-0.4827887915091037</v>
+      </c>
+      <c r="E10">
+        <v>-9.3305878912203211E-4</v>
+      </c>
+      <c r="F10">
+        <v>-3.9476648597719377E-4</v>
+      </c>
+      <c r="G10">
+        <v>9.6979470390512468E-4</v>
+      </c>
+      <c r="H10">
+        <v>1.4857990543022392E-3</v>
+      </c>
+      <c r="I10">
+        <v>2.8413810071137302E-4</v>
+      </c>
+      <c r="J10">
+        <v>-1.0334559595664983E-4</v>
+      </c>
+      <c r="K10">
+        <v>-7.894111737963283E-4</v>
+      </c>
+      <c r="L10">
+        <v>-2.8407615835654432E-3</v>
+      </c>
+      <c r="M10">
+        <v>3.3968240278848261E-3</v>
+      </c>
+      <c r="N10">
+        <v>2.3570413477065344E-3</v>
+      </c>
+      <c r="O10">
+        <v>1.5094581776927685E-3</v>
+      </c>
+      <c r="P10">
+        <v>2.1125915897757253E-3</v>
+      </c>
+      <c r="Q10">
+        <v>1.9084614321338567E-3</v>
+      </c>
+      <c r="R10">
+        <v>1.9418997467842147E-3</v>
+      </c>
+      <c r="S10">
+        <v>1.3796007075831396E-3</v>
+      </c>
+      <c r="T10">
+        <v>1.4270607882068131E-3</v>
+      </c>
+      <c r="U10">
+        <v>1.3841283584009045E-3</v>
+      </c>
+      <c r="V10">
+        <v>2.9271538241418815E-3</v>
+      </c>
+      <c r="W10">
+        <v>2.7058040595424604E-3</v>
+      </c>
+      <c r="X10">
+        <v>3.0333876344351141E-3</v>
+      </c>
+      <c r="Y10">
+        <v>3.5366971368161471E-3</v>
+      </c>
+      <c r="Z10">
+        <v>3.5849620568428331E-3</v>
+      </c>
+      <c r="AA10">
+        <v>3.5911178332263538E-3</v>
+      </c>
+      <c r="AB10">
+        <v>3.1871496164249113E-3</v>
+      </c>
+      <c r="AC10">
+        <v>3.1818022912238897E-3</v>
+      </c>
+      <c r="AD10">
+        <v>3.2833576772886008E-3</v>
+      </c>
+      <c r="AE10">
+        <v>3.2841576486102309E-3</v>
+      </c>
+      <c r="AF10">
+        <v>3.1616482061682105E-3</v>
+      </c>
+      <c r="AG10">
+        <v>3.2650272767845157E-3</v>
+      </c>
+      <c r="AH10">
+        <v>3.3949676435666709E-3</v>
+      </c>
+      <c r="AI10">
+        <v>3.5407298414859567E-3</v>
+      </c>
+      <c r="AJ10">
+        <v>3.5033909035794286E-3</v>
+      </c>
+      <c r="AK10">
+        <v>3.2926918956808771E-3</v>
+      </c>
+      <c r="AL10">
+        <v>3.1735287858333239E-3</v>
+      </c>
+      <c r="AM10">
+        <v>3.2215423000871435E-3</v>
+      </c>
+      <c r="AN10">
+        <v>3.292251469204921E-3</v>
+      </c>
+      <c r="AO10">
+        <v>3.345982329356012E-3</v>
+      </c>
+      <c r="AP10">
+        <v>3.3510137443018007E-3</v>
+      </c>
+      <c r="AQ10">
+        <v>3.2876550610315691E-3</v>
+      </c>
+      <c r="AR10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>-0.48122513474749917</v>
+      </c>
+      <c r="E11">
+        <v>-6.9250784800500842E-4</v>
+      </c>
+      <c r="F11">
+        <v>-7.2108933922543361E-4</v>
+      </c>
+      <c r="G11">
+        <v>-1.7252818368934664E-4</v>
+      </c>
+      <c r="H11">
+        <v>-6.3601395281320805E-4</v>
+      </c>
+      <c r="I11">
+        <v>-3.9916462106276418E-4</v>
+      </c>
+      <c r="J11">
+        <v>-4.8142949975665816E-4</v>
+      </c>
+      <c r="K11">
+        <v>-1.0028043989358526E-3</v>
+      </c>
+      <c r="L11">
+        <v>-2.5812088772941277E-3</v>
+      </c>
+      <c r="M11">
+        <v>1.8240523753960125E-3</v>
+      </c>
+      <c r="N11">
+        <v>1.2392455903026955E-3</v>
+      </c>
+      <c r="O11">
+        <v>9.1508063954931496E-4</v>
+      </c>
+      <c r="P11">
+        <v>1.8266515949459383E-3</v>
+      </c>
+      <c r="Q11">
+        <v>1.6440489266426606E-3</v>
+      </c>
+      <c r="R11">
+        <v>1.2213701768027385E-3</v>
+      </c>
+      <c r="S11">
+        <v>1.1969144506278062E-3</v>
+      </c>
+      <c r="T11">
+        <v>1.2197740889111075E-3</v>
+      </c>
+      <c r="U11">
+        <v>1.273255678725993E-3</v>
+      </c>
+      <c r="V11">
+        <v>2.4738097868804987E-3</v>
+      </c>
+      <c r="W11">
+        <v>2.262584166552839E-3</v>
+      </c>
+      <c r="X11">
+        <v>3.2169208956970285E-3</v>
+      </c>
+      <c r="Y11">
+        <v>3.4177816179182252E-3</v>
+      </c>
+      <c r="Z11">
+        <v>3.3448249670005037E-3</v>
+      </c>
+      <c r="AA11">
+        <v>3.4536461093880866E-3</v>
+      </c>
+      <c r="AB11">
+        <v>3.1001760098184339E-3</v>
+      </c>
+      <c r="AC11">
+        <v>3.0988927970268532E-3</v>
+      </c>
+      <c r="AD11">
+        <v>3.1145081655162277E-3</v>
+      </c>
+      <c r="AE11">
+        <v>3.2219700726250911E-3</v>
+      </c>
+      <c r="AF11">
+        <v>3.23753089180423E-3</v>
+      </c>
+      <c r="AG11">
+        <v>3.1231030976869856E-3</v>
+      </c>
+      <c r="AH11">
+        <v>3.2519266498872157E-3</v>
+      </c>
+      <c r="AI11">
+        <v>3.408605062526826E-3</v>
+      </c>
+      <c r="AJ11">
+        <v>3.5824161462768567E-3</v>
+      </c>
+      <c r="AK11">
+        <v>3.5541118943258621E-3</v>
+      </c>
+      <c r="AL11">
+        <v>3.3328496453527423E-3</v>
+      </c>
+      <c r="AM11">
+        <v>3.2109406821726472E-3</v>
+      </c>
+      <c r="AN11">
+        <v>3.2731859843662114E-3</v>
+      </c>
+      <c r="AO11">
+        <v>3.3599629452635282E-3</v>
+      </c>
+      <c r="AP11">
+        <v>3.427376166149132E-3</v>
+      </c>
+      <c r="AQ11">
+        <v>3.4398137263500494E-3</v>
+      </c>
+      <c r="AR11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>-0.48003154174720664</v>
+      </c>
+      <c r="E12">
+        <v>-1.450334737728487E-3</v>
+      </c>
+      <c r="F12">
+        <v>-1.1528640951902203E-3</v>
+      </c>
+      <c r="G12">
+        <v>-1.0139597323016725E-3</v>
+      </c>
+      <c r="H12">
+        <v>-4.1141794567517431E-4</v>
+      </c>
+      <c r="I12">
+        <v>-8.1334240700015048E-4</v>
+      </c>
+      <c r="J12">
+        <v>-8.5431658771822905E-4</v>
+      </c>
+      <c r="K12">
+        <v>-1.1626440656327675E-3</v>
+      </c>
+      <c r="L12">
+        <v>-2.43194361383825E-3</v>
+      </c>
+      <c r="M12">
+        <v>1.2450565408889114E-3</v>
+      </c>
+      <c r="N12">
+        <v>8.5900126009885724E-4</v>
+      </c>
+      <c r="O12">
+        <v>4.8532935517886511E-4</v>
+      </c>
+      <c r="P12">
+        <v>1.2033349275739624E-3</v>
+      </c>
+      <c r="Q12">
+        <v>1.3738142284016042E-3</v>
+      </c>
+      <c r="R12">
+        <v>8.5210026992715848E-4</v>
+      </c>
+      <c r="S12">
+        <v>8.3360156583511813E-4</v>
+      </c>
+      <c r="T12">
+        <v>1.2963156906844464E-3</v>
+      </c>
+      <c r="U12">
+        <v>1.4992877190453946E-3</v>
+      </c>
+      <c r="V12">
+        <v>2.5512208341338383E-3</v>
+      </c>
+      <c r="W12">
+        <v>1.9915218097699694E-3</v>
+      </c>
+      <c r="X12">
+        <v>2.7893266793266314E-3</v>
+      </c>
+      <c r="Y12">
+        <v>3.8895022470258334E-3</v>
+      </c>
+      <c r="Z12">
+        <v>3.4715106376480009E-3</v>
+      </c>
+      <c r="AA12">
+        <v>3.6600328521652625E-3</v>
+      </c>
+      <c r="AB12">
+        <v>3.5086239902280547E-3</v>
+      </c>
+      <c r="AC12">
+        <v>3.6971730467271757E-3</v>
+      </c>
+      <c r="AD12">
+        <v>3.6708151967850822E-3</v>
+      </c>
+      <c r="AE12">
+        <v>3.6997970643742328E-3</v>
+      </c>
+      <c r="AF12">
+        <v>3.8435386097986357E-3</v>
+      </c>
+      <c r="AG12">
+        <v>3.8814152138405E-3</v>
+      </c>
+      <c r="AH12">
+        <v>3.7671939015503364E-3</v>
+      </c>
+      <c r="AI12">
+        <v>3.931717232402987E-3</v>
+      </c>
+      <c r="AJ12">
+        <v>4.1279671577751365E-3</v>
+      </c>
+      <c r="AK12">
+        <v>4.3442449969414709E-3</v>
+      </c>
+      <c r="AL12">
+        <v>4.3237287584966255E-3</v>
+      </c>
+      <c r="AM12">
+        <v>4.0755477010931962E-3</v>
+      </c>
+      <c r="AN12">
+        <v>3.9421162005892629E-3</v>
+      </c>
+      <c r="AO12">
+        <v>4.0240406716185451E-3</v>
+      </c>
+      <c r="AP12">
+        <v>4.1342505921941886E-3</v>
+      </c>
+      <c r="AQ12">
+        <v>4.2212661305847665E-3</v>
+      </c>
+      <c r="AR12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>-0.47671406557554208</v>
+      </c>
+      <c r="E13">
+        <v>-1.7098659653945747E-3</v>
+      </c>
+      <c r="F13">
+        <v>-1.8354693796918675E-3</v>
+      </c>
+      <c r="G13">
+        <v>-1.6439814433139022E-4</v>
+      </c>
+      <c r="H13">
+        <v>-2.7728107600588636E-4</v>
+      </c>
+      <c r="I13">
+        <v>-1.3837728688707585E-3</v>
+      </c>
+      <c r="J13">
+        <v>-1.329528114448808E-3</v>
+      </c>
+      <c r="K13">
+        <v>-1.7348961874466551E-3</v>
+      </c>
+      <c r="L13">
+        <v>-2.712538629090766E-3</v>
+      </c>
+      <c r="M13">
+        <v>5.1901192337694413E-4</v>
+      </c>
+      <c r="N13">
+        <v>2.7263569268209942E-4</v>
+      </c>
+      <c r="O13">
+        <v>3.4117418769241681E-5</v>
+      </c>
+      <c r="P13">
+        <v>6.0493111728621152E-4</v>
+      </c>
+      <c r="Q13">
+        <v>6.6381839077489513E-4</v>
+      </c>
+      <c r="R13">
+        <v>5.1056718228953413E-4</v>
+      </c>
+      <c r="S13">
+        <v>6.0560566792888793E-4</v>
+      </c>
+      <c r="T13">
+        <v>9.1408372590306985E-4</v>
+      </c>
+      <c r="U13">
+        <v>1.2702720208886409E-3</v>
+      </c>
+      <c r="V13">
+        <v>2.3154534243786662E-3</v>
+      </c>
+      <c r="W13">
+        <v>1.9893879099134315E-3</v>
+      </c>
+      <c r="X13">
+        <v>2.3788866607457604E-3</v>
+      </c>
+      <c r="Y13">
+        <v>3.0615555283495244E-3</v>
+      </c>
+      <c r="Z13">
+        <v>3.4333596317617787E-3</v>
+      </c>
+      <c r="AA13">
+        <v>3.7801013399258454E-3</v>
+      </c>
+      <c r="AB13">
+        <v>3.7801072901120225E-3</v>
+      </c>
+      <c r="AC13">
+        <v>4.1677908944367514E-3</v>
+      </c>
+      <c r="AD13">
+        <v>4.3730065770713478E-3</v>
+      </c>
+      <c r="AE13">
+        <v>4.3548898152495075E-3</v>
+      </c>
+      <c r="AF13">
+        <v>4.4189907254966188E-3</v>
+      </c>
+      <c r="AG13">
+        <v>4.6141428370075066E-3</v>
+      </c>
+      <c r="AH13">
+        <v>4.6841592435456492E-3</v>
+      </c>
+      <c r="AI13">
+        <v>4.573632742059297E-3</v>
+      </c>
+      <c r="AJ13">
+        <v>4.7879370161840185E-3</v>
+      </c>
+      <c r="AK13">
+        <v>5.0384650218069371E-3</v>
+      </c>
+      <c r="AL13">
+        <v>5.3128523035827491E-3</v>
+      </c>
+      <c r="AM13">
+        <v>5.3049396703973573E-3</v>
+      </c>
+      <c r="AN13">
+        <v>5.0237100054028594E-3</v>
+      </c>
+      <c r="AO13">
+        <v>4.8773403591650388E-3</v>
+      </c>
+      <c r="AP13">
+        <v>4.9870990495839984E-3</v>
+      </c>
+      <c r="AQ13">
+        <v>5.1301242250866297E-3</v>
+      </c>
+      <c r="AR13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>-0.47333654983260626</v>
+      </c>
+      <c r="E14">
+        <v>-2.7325144384951483E-3</v>
+      </c>
+      <c r="F14">
+        <v>-2.6447414233570221E-3</v>
+      </c>
+      <c r="G14">
+        <v>-2.4982279448358957E-3</v>
+      </c>
+      <c r="H14">
+        <v>-2.8403443420224606E-3</v>
+      </c>
+      <c r="I14">
+        <v>-2.480072873055239E-3</v>
+      </c>
+      <c r="J14">
+        <v>-2.3248894493110295E-3</v>
+      </c>
+      <c r="K14">
+        <v>-2.5076044603681846E-3</v>
+      </c>
+      <c r="L14">
+        <v>-3.224707639192359E-3</v>
+      </c>
+      <c r="M14">
+        <v>-7.7407130855550177E-4</v>
+      </c>
+      <c r="N14">
+        <v>-6.4226584115906205E-4</v>
+      </c>
+      <c r="O14">
+        <v>-7.7614945192422402E-4</v>
+      </c>
+      <c r="P14">
+        <v>-1.7087640009838534E-4</v>
+      </c>
+      <c r="Q14">
+        <v>-1.7868852626112819E-4</v>
+      </c>
+      <c r="R14">
+        <v>-3.6936482825578043E-4</v>
+      </c>
+      <c r="S14">
+        <v>8.5297883985091527E-5</v>
+      </c>
+      <c r="T14">
+        <v>2.8693882621100286E-4</v>
+      </c>
+      <c r="U14">
+        <v>8.4604653083242276E-4</v>
+      </c>
+      <c r="V14">
+        <v>1.9851376048860558E-3</v>
+      </c>
+      <c r="W14">
+        <v>1.6661635322137158E-3</v>
+      </c>
+      <c r="X14">
+        <v>2.2917611520406056E-3</v>
+      </c>
+      <c r="Y14">
+        <v>2.5619749858899477E-3</v>
+      </c>
+      <c r="Z14">
+        <v>2.715078811804883E-3</v>
+      </c>
+      <c r="AA14">
+        <v>3.9915650714220097E-3</v>
+      </c>
+      <c r="AB14">
+        <v>3.8714263748072519E-3</v>
+      </c>
+      <c r="AC14">
+        <v>4.2508537418281533E-3</v>
+      </c>
+      <c r="AD14">
+        <v>4.6569094560783286E-3</v>
+      </c>
+      <c r="AE14">
+        <v>4.9069695840325278E-3</v>
+      </c>
+      <c r="AF14">
+        <v>4.9238840993690025E-3</v>
+      </c>
+      <c r="AG14">
+        <v>5.033805466738539E-3</v>
+      </c>
+      <c r="AH14">
+        <v>5.2918058714209182E-3</v>
+      </c>
+      <c r="AI14">
+        <v>5.4011478690863535E-3</v>
+      </c>
+      <c r="AJ14">
+        <v>5.2948802667586725E-3</v>
+      </c>
+      <c r="AK14">
+        <v>5.5703082854008934E-3</v>
+      </c>
+      <c r="AL14">
+        <v>5.8885349099337403E-3</v>
+      </c>
+      <c r="AM14">
+        <v>6.2354506725634806E-3</v>
+      </c>
+      <c r="AN14">
+        <v>6.2442161141966213E-3</v>
+      </c>
+      <c r="AO14">
+        <v>5.9230421370876085E-3</v>
+      </c>
+      <c r="AP14">
+        <v>5.7611739534196849E-3</v>
+      </c>
+      <c r="AQ14">
+        <v>5.9062291576458814E-3</v>
+      </c>
+      <c r="AR14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>57</v>
+      </c>
+      <c r="B15" t="s">
+        <v>0</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>-0.46922614682829761</v>
+      </c>
+      <c r="E15">
+        <v>-3.8225017972868813E-3</v>
+      </c>
+      <c r="F15">
+        <v>-3.8511176792528912E-3</v>
+      </c>
+      <c r="G15">
+        <v>-3.3869195487313264E-3</v>
+      </c>
+      <c r="H15">
+        <v>-3.0904602475158027E-3</v>
+      </c>
+      <c r="I15">
+        <v>-3.4308840470465007E-3</v>
+      </c>
+      <c r="J15">
+        <v>-3.5872600856778347E-3</v>
+      </c>
+      <c r="K15">
+        <v>-3.6835273636638965E-3</v>
+      </c>
+      <c r="L15">
+        <v>-4.2592122504391816E-3</v>
+      </c>
+      <c r="M15">
+        <v>-2.5532582155671224E-3</v>
+      </c>
+      <c r="N15">
+        <v>-2.2630159069482736E-3</v>
+      </c>
+      <c r="O15">
+        <v>-2.1354875205431556E-3</v>
+      </c>
+      <c r="P15">
+        <v>-1.483743230543344E-3</v>
+      </c>
+      <c r="Q15">
+        <v>-1.2300954904311268E-3</v>
+      </c>
+      <c r="R15">
+        <v>-1.765701031080813E-3</v>
+      </c>
+      <c r="S15">
+        <v>-1.2483789202817897E-3</v>
+      </c>
+      <c r="T15">
+        <v>-6.5437972308440839E-4</v>
+      </c>
+      <c r="U15">
+        <v>-2.2772535217158163E-4</v>
+      </c>
+      <c r="V15">
+        <v>9.4187529684258697E-4</v>
+      </c>
+      <c r="W15">
+        <v>1.0761990535097521E-3</v>
+      </c>
+      <c r="X15">
+        <v>1.6522528209919063E-3</v>
+      </c>
+      <c r="Y15">
+        <v>2.2485538850229858E-3</v>
+      </c>
+      <c r="Z15">
+        <v>2.1365009932022838E-3</v>
+      </c>
+      <c r="AA15">
+        <v>2.9392161919400972E-3</v>
+      </c>
+      <c r="AB15">
+        <v>3.5988616855635036E-3</v>
+      </c>
+      <c r="AC15">
+        <v>3.8152045589892603E-3</v>
+      </c>
+      <c r="AD15">
+        <v>4.2552745189372021E-3</v>
+      </c>
+      <c r="AE15">
+        <v>4.7561092749863754E-3</v>
+      </c>
+      <c r="AF15">
+        <v>5.1002648481903723E-3</v>
+      </c>
+      <c r="AG15">
+        <v>5.1791823498448242E-3</v>
+      </c>
+      <c r="AH15">
+        <v>5.3667073763332129E-3</v>
+      </c>
+      <c r="AI15">
+        <v>5.7022284316892713E-3</v>
+      </c>
+      <c r="AJ15">
+        <v>5.8719343624971665E-3</v>
+      </c>
+      <c r="AK15">
+        <v>5.7966955060015923E-3</v>
+      </c>
+      <c r="AL15">
+        <v>6.1488443809375459E-3</v>
+      </c>
+      <c r="AM15">
+        <v>6.547014303586729E-3</v>
+      </c>
+      <c r="AN15">
+        <v>6.9786023773559802E-3</v>
+      </c>
+      <c r="AO15">
+        <v>7.0202280928007843E-3</v>
+      </c>
+      <c r="AP15">
+        <v>6.6788395172929227E-3</v>
+      </c>
+      <c r="AQ15">
+        <v>6.5181561088925033E-3</v>
+      </c>
+      <c r="AR15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" t="s">
+        <v>0</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>-0.46580074312599562</v>
+      </c>
+      <c r="E16">
+        <v>-4.6347963244698365E-3</v>
+      </c>
+      <c r="F16">
+        <v>-4.6530351509976309E-3</v>
+      </c>
+      <c r="G16">
+        <v>-4.5526697213157385E-3</v>
+      </c>
+      <c r="H16">
+        <v>-4.4441535597322668E-3</v>
+      </c>
+      <c r="I16">
+        <v>-4.4973629793343406E-3</v>
+      </c>
+      <c r="J16">
+        <v>-4.5068807682909218E-3</v>
+      </c>
+      <c r="K16">
+        <v>-4.5984910873528295E-3</v>
+      </c>
+      <c r="L16">
+        <v>-5.2815717251761818E-3</v>
+      </c>
+      <c r="M16">
+        <v>-4.1421596000414951E-3</v>
+      </c>
+      <c r="N16">
+        <v>-3.9313638760848924E-3</v>
+      </c>
+      <c r="O16">
+        <v>-3.8481888975432921E-3</v>
+      </c>
+      <c r="P16">
+        <v>-3.255247148021112E-3</v>
+      </c>
+      <c r="Q16">
+        <v>-2.890113533134675E-3</v>
+      </c>
+      <c r="R16">
+        <v>-3.1633324284907616E-3</v>
+      </c>
+      <c r="S16">
+        <v>-3.1899801155906293E-3</v>
+      </c>
+      <c r="T16">
+        <v>-2.7318237462555239E-3</v>
+      </c>
+      <c r="U16">
+        <v>-2.0031819978312271E-3</v>
+      </c>
+      <c r="V16">
+        <v>-6.874345707475471E-4</v>
+      </c>
+      <c r="W16">
+        <v>-2.3189254339839316E-4</v>
+      </c>
+      <c r="X16">
+        <v>9.3717840789708795E-5</v>
+      </c>
+      <c r="Y16">
+        <v>8.9443870661587432E-4</v>
+      </c>
+      <c r="Z16">
+        <v>1.1276352669762346E-3</v>
+      </c>
+      <c r="AA16">
+        <v>1.6686869296466122E-3</v>
+      </c>
+      <c r="AB16">
+        <v>2.0302098547785308E-3</v>
+      </c>
+      <c r="AC16">
+        <v>2.8245698318855039E-3</v>
+      </c>
+      <c r="AD16">
+        <v>3.0338277491364085E-3</v>
+      </c>
+      <c r="AE16">
+        <v>3.523266823841853E-3</v>
+      </c>
+      <c r="AF16">
+        <v>4.1346559081435474E-3</v>
+      </c>
+      <c r="AG16">
+        <v>4.6152596016577063E-3</v>
+      </c>
+      <c r="AH16">
+        <v>4.8248732562815588E-3</v>
+      </c>
+      <c r="AI16">
+        <v>5.1560371069968025E-3</v>
+      </c>
+      <c r="AJ16">
+        <v>5.5970230031713308E-3</v>
+      </c>
+      <c r="AK16">
+        <v>5.8729221667762066E-3</v>
+      </c>
+      <c r="AL16">
+        <v>5.892583392077988E-3</v>
+      </c>
+      <c r="AM16">
+        <v>6.3464615137763247E-3</v>
+      </c>
+      <c r="AN16">
+        <v>6.8426148763114369E-3</v>
+      </c>
+      <c r="AO16">
+        <v>7.3753528072630914E-3</v>
+      </c>
+      <c r="AP16">
+        <v>7.4875140062831136E-3</v>
+      </c>
+      <c r="AQ16">
+        <v>7.1815022250575344E-3</v>
+      </c>
+      <c r="AR16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>-0.46299133347111643</v>
+      </c>
+      <c r="E17">
+        <v>-4.2518415929578279E-3</v>
+      </c>
+      <c r="F17">
+        <v>-4.2973649919578194E-3</v>
+      </c>
+      <c r="G17">
+        <v>-4.0759065308804687E-3</v>
+      </c>
+      <c r="H17">
+        <v>-4.2897694640181006E-3</v>
+      </c>
+      <c r="I17">
+        <v>-4.4971072432772874E-3</v>
+      </c>
+      <c r="J17">
+        <v>-4.6358179102136132E-3</v>
+      </c>
+      <c r="K17">
+        <v>-4.482918420275539E-3</v>
+      </c>
+      <c r="L17">
+        <v>-5.2720398913033151E-3</v>
+      </c>
+      <c r="M17">
+        <v>-4.90472243618717E-3</v>
+      </c>
+      <c r="N17">
+        <v>-4.4379756244972146E-3</v>
+      </c>
+      <c r="O17">
+        <v>-4.961491959499631E-3</v>
+      </c>
+      <c r="P17">
+        <v>-4.5739158272504743E-3</v>
+      </c>
+      <c r="Q17">
+        <v>-4.5316604982063025E-3</v>
+      </c>
+      <c r="R17">
+        <v>-4.5733374856247178E-3</v>
+      </c>
+      <c r="S17">
+        <v>-4.4829587438070528E-3</v>
+      </c>
+      <c r="T17">
+        <v>-4.6752546350502522E-3</v>
+      </c>
+      <c r="U17">
+        <v>-4.5739894159584904E-3</v>
+      </c>
+      <c r="V17">
+        <v>-3.5050489756459635E-3</v>
+      </c>
+      <c r="W17">
+        <v>-2.5886618697923414E-3</v>
+      </c>
+      <c r="X17">
+        <v>-1.9375240396663496E-3</v>
+      </c>
+      <c r="Y17">
+        <v>-1.9056842230233406E-3</v>
+      </c>
+      <c r="Z17">
+        <v>-1.6085104008307649E-3</v>
+      </c>
+      <c r="AA17">
+        <v>-7.2740080405769847E-4</v>
+      </c>
+      <c r="AB17">
+        <v>-3.3088900843530888E-4</v>
+      </c>
+      <c r="AC17">
+        <v>1.3880602062171787E-4</v>
+      </c>
+      <c r="AD17">
+        <v>3.2067958366216454E-4</v>
+      </c>
+      <c r="AE17">
+        <v>5.3929908436184393E-4</v>
+      </c>
+      <c r="AF17">
+        <v>1.1257000385050397E-3</v>
+      </c>
+      <c r="AG17">
+        <v>1.8626545562051011E-3</v>
+      </c>
+      <c r="AH17">
+        <v>2.548967504293842E-3</v>
+      </c>
+      <c r="AI17">
+        <v>3.0156930015521333E-3</v>
+      </c>
+      <c r="AJ17">
+        <v>3.6011396080772307E-3</v>
+      </c>
+      <c r="AK17">
+        <v>4.1922489350655345E-3</v>
+      </c>
+      <c r="AL17">
+        <v>4.6546324246899418E-3</v>
+      </c>
+      <c r="AM17">
+        <v>4.8905014364045707E-3</v>
+      </c>
+      <c r="AN17">
+        <v>5.4801345306000337E-3</v>
+      </c>
+      <c r="AO17">
+        <v>6.0960963610020014E-3</v>
+      </c>
+      <c r="AP17">
+        <v>6.7489962565769335E-3</v>
+      </c>
+      <c r="AQ17">
+        <v>7.0033991602961865E-3</v>
+      </c>
+      <c r="AR17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>-0.45997612626361922</v>
+      </c>
+      <c r="E18">
+        <v>-2.8280648696995536E-3</v>
+      </c>
+      <c r="F18">
+        <v>-2.7777613547997348E-3</v>
+      </c>
+      <c r="G18">
+        <v>-2.8992729317079413E-3</v>
+      </c>
+      <c r="H18">
+        <v>-2.902550466579612E-3</v>
+      </c>
+      <c r="I18">
+        <v>-2.990897329596065E-3</v>
+      </c>
+      <c r="J18">
+        <v>-3.1530363004935169E-3</v>
+      </c>
+      <c r="K18">
+        <v>-3.1617454646445942E-3</v>
+      </c>
+      <c r="L18">
+        <v>-3.5183220881225274E-3</v>
+      </c>
+      <c r="M18">
+        <v>-3.5218176517475275E-3</v>
+      </c>
+      <c r="N18">
+        <v>-3.4364580888188723E-3</v>
+      </c>
+      <c r="O18">
+        <v>-3.8216088593286957E-3</v>
+      </c>
+      <c r="P18">
+        <v>-4.2034235322278568E-3</v>
+      </c>
+      <c r="Q18">
+        <v>-4.474359985212728E-3</v>
+      </c>
+      <c r="R18">
+        <v>-4.6450779681558307E-3</v>
+      </c>
+      <c r="S18">
+        <v>-4.7816297102924454E-3</v>
+      </c>
+      <c r="T18">
+        <v>-4.8926128790389711E-3</v>
+      </c>
+      <c r="U18">
+        <v>-5.520890232192821E-3</v>
+      </c>
+      <c r="V18">
+        <v>-5.3126840034615763E-3</v>
+      </c>
+      <c r="W18">
+        <v>-5.2162971277612269E-3</v>
+      </c>
+      <c r="X18">
+        <v>-4.4625549657682506E-3</v>
+      </c>
+      <c r="Y18">
+        <v>-3.869067654803271E-3</v>
+      </c>
+      <c r="Z18">
+        <v>-5.0639054102452064E-3</v>
+      </c>
+      <c r="AA18">
+        <v>-4.5150614785918752E-3</v>
+      </c>
+      <c r="AB18">
+        <v>-4.0614599039330845E-3</v>
+      </c>
+      <c r="AC18">
+        <v>-3.2915828275329462E-3</v>
+      </c>
+      <c r="AD18">
+        <v>-3.2604713470853475E-3</v>
+      </c>
+      <c r="AE18">
+        <v>-4.1921407980913261E-3</v>
+      </c>
+      <c r="AF18">
+        <v>-3.9694340804264372E-3</v>
+      </c>
+      <c r="AG18">
+        <v>-3.4454168487788039E-3</v>
+      </c>
+      <c r="AH18">
+        <v>-2.821868179392506E-3</v>
+      </c>
+      <c r="AI18">
+        <v>-2.0645199674011461E-3</v>
+      </c>
+      <c r="AJ18">
+        <v>-1.3666174998336333E-3</v>
+      </c>
+      <c r="AK18">
+        <v>-5.0447041027629203E-4</v>
+      </c>
+      <c r="AL18">
+        <v>1.3024756931018233E-4</v>
+      </c>
+      <c r="AM18">
+        <v>7.717637972144975E-4</v>
+      </c>
+      <c r="AN18">
+        <v>1.3412376673299642E-3</v>
+      </c>
+      <c r="AO18">
+        <v>2.0187487426246431E-3</v>
+      </c>
+      <c r="AP18">
+        <v>2.6711191724088645E-3</v>
+      </c>
+      <c r="AQ18">
+        <v>3.364145181511291E-3</v>
+      </c>
+      <c r="AR18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" t="s">
+        <v>0</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <v>-0.45706267950298318</v>
+      </c>
+      <c r="E19">
+        <v>-1.0571449703710711E-3</v>
+      </c>
+      <c r="F19">
+        <v>-1.0420372526225297E-3</v>
+      </c>
+      <c r="G19">
+        <v>-1.0831834292016618E-3</v>
+      </c>
+      <c r="H19">
+        <v>-1.1146743225792788E-3</v>
+      </c>
+      <c r="I19">
+        <v>-1.1583813347889049E-3</v>
+      </c>
+      <c r="J19">
+        <v>-1.2716324072058471E-3</v>
+      </c>
+      <c r="K19">
+        <v>-1.2921391135378157E-3</v>
+      </c>
+      <c r="L19">
+        <v>-1.5513781708056396E-3</v>
+      </c>
+      <c r="M19">
+        <v>-1.4810746453941537E-3</v>
+      </c>
+      <c r="N19">
+        <v>-1.5311291412434813E-3</v>
+      </c>
+      <c r="O19">
+        <v>-1.8517376341583014E-3</v>
+      </c>
+      <c r="P19">
+        <v>-2.0528633191080337E-3</v>
+      </c>
+      <c r="Q19">
+        <v>-2.5845364445012953E-3</v>
+      </c>
+      <c r="R19">
+        <v>-2.8608095050117743E-3</v>
+      </c>
+      <c r="S19">
+        <v>-3.2018081503859541E-3</v>
+      </c>
+      <c r="T19">
+        <v>-3.4751248687193703E-3</v>
+      </c>
+      <c r="U19">
+        <v>-3.8547752168035521E-3</v>
+      </c>
+      <c r="V19">
+        <v>-4.3357814658718796E-3</v>
+      </c>
+      <c r="W19">
+        <v>-4.9807372528715699E-3</v>
+      </c>
+      <c r="X19">
+        <v>-5.6674962378029936E-3</v>
+      </c>
+      <c r="Y19">
+        <v>-4.8984206311136758E-3</v>
+      </c>
+      <c r="Z19">
+        <v>-5.1051929667324525E-3</v>
+      </c>
+      <c r="AA19">
+        <v>-6.8490227580884078E-3</v>
+      </c>
+      <c r="AB19">
+        <v>-7.1534458198518336E-3</v>
+      </c>
+      <c r="AC19">
+        <v>-6.9923648856798915E-3</v>
+      </c>
+      <c r="AD19">
+        <v>-6.622276334814714E-3</v>
+      </c>
+      <c r="AE19">
+        <v>-7.5349189055119448E-3</v>
+      </c>
+      <c r="AF19">
+        <v>-9.8563548791290589E-3</v>
+      </c>
+      <c r="AG19">
+        <v>-9.7651334087855424E-3</v>
+      </c>
+      <c r="AH19">
+        <v>-9.8129069578811179E-3</v>
+      </c>
+      <c r="AI19">
+        <v>-9.9587263071218568E-3</v>
+      </c>
+      <c r="AJ19">
+        <v>-9.7159958675542835E-3</v>
+      </c>
+      <c r="AK19">
+        <v>-9.1520460244908231E-3</v>
+      </c>
+      <c r="AL19">
+        <v>-8.4732801191806373E-3</v>
+      </c>
+      <c r="AM19">
+        <v>-8.3020812828148993E-3</v>
+      </c>
+      <c r="AN19">
+        <v>-7.8596616087951432E-3</v>
+      </c>
+      <c r="AO19">
+        <v>-7.0908471903534664E-3</v>
+      </c>
+      <c r="AP19">
+        <v>-6.8187266301604765E-3</v>
+      </c>
+      <c r="AQ19">
+        <v>-6.6430668884595034E-3</v>
+      </c>
+      <c r="AR19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" t="s">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>-0.4544758345315128</v>
+      </c>
+      <c r="E20">
+        <v>-2.1882356822267024E-4</v>
+      </c>
+      <c r="F20">
+        <v>-2.2082520252508786E-4</v>
+      </c>
+      <c r="G20">
+        <v>-2.2670684913689287E-4</v>
+      </c>
+      <c r="H20">
+        <v>-2.3302216038983969E-4</v>
+      </c>
+      <c r="I20">
+        <v>-2.4746685234733334E-4</v>
+      </c>
+      <c r="J20">
+        <v>-2.6337800718589932E-4</v>
+      </c>
+      <c r="K20">
+        <v>-2.8856718161646144E-4</v>
+      </c>
+      <c r="L20">
+        <v>-3.4070605698777179E-4</v>
+      </c>
+      <c r="M20">
+        <v>-3.4621447970101249E-4</v>
+      </c>
+      <c r="N20">
+        <v>-3.3539299245144427E-4</v>
+      </c>
+      <c r="O20">
+        <v>-4.6215420676193331E-4</v>
+      </c>
+      <c r="P20">
+        <v>-5.5387382428051524E-4</v>
+      </c>
+      <c r="Q20">
+        <v>-6.9393367241260551E-4</v>
+      </c>
+      <c r="R20">
+        <v>-9.4502805750340535E-4</v>
+      </c>
+      <c r="S20">
+        <v>-1.1515967151416451E-3</v>
+      </c>
+      <c r="T20">
+        <v>-1.3517656613510898E-3</v>
+      </c>
+      <c r="U20">
+        <v>-1.5513056528376756E-3</v>
+      </c>
+      <c r="V20">
+        <v>-1.8505687481742417E-3</v>
+      </c>
+      <c r="W20">
+        <v>-2.4404485168751933E-3</v>
+      </c>
+      <c r="X20">
+        <v>-3.1720815884108133E-3</v>
+      </c>
+      <c r="Y20">
+        <v>-3.6883230642568154E-3</v>
+      </c>
+      <c r="Z20">
+        <v>-3.3911283599077913E-3</v>
+      </c>
+      <c r="AA20">
+        <v>-4.0599444211939506E-3</v>
+      </c>
+      <c r="AB20">
+        <v>-5.7932139829883211E-3</v>
+      </c>
+      <c r="AC20">
+        <v>-6.3008109814751689E-3</v>
+      </c>
+      <c r="AD20">
+        <v>-6.7282844595136782E-3</v>
+      </c>
+      <c r="AE20">
+        <v>-6.7710495719411901E-3</v>
+      </c>
+      <c r="AF20">
+        <v>-8.1776772164711686E-3</v>
+      </c>
+      <c r="AG20">
+        <v>-1.0691036382916963E-2</v>
+      </c>
+      <c r="AH20">
+        <v>-1.0837966058514725E-2</v>
+      </c>
+      <c r="AI20">
+        <v>-1.1478040554670443E-2</v>
+      </c>
+      <c r="AJ20">
+        <v>-1.2309522129443085E-2</v>
+      </c>
+      <c r="AK20">
+        <v>-1.2741534092863882E-2</v>
+      </c>
+      <c r="AL20">
+        <v>-1.256234783951421E-2</v>
+      </c>
+      <c r="AM20">
+        <v>-1.2612215720783637E-2</v>
+      </c>
+      <c r="AN20">
+        <v>-1.3070724969404923E-2</v>
+      </c>
+      <c r="AO20">
+        <v>-1.315612610941258E-2</v>
+      </c>
+      <c r="AP20">
+        <v>-1.268598063398213E-2</v>
+      </c>
+      <c r="AQ20">
+        <v>-1.3165227767042376E-2</v>
+      </c>
+      <c r="AR20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>-0.45231714383433369</v>
+      </c>
+      <c r="E21">
+        <v>-2.4486285907121541E-5</v>
+      </c>
+      <c r="F21">
+        <v>-2.5414501399534384E-5</v>
+      </c>
+      <c r="G21">
+        <v>-2.5643048990497963E-5</v>
+      </c>
+      <c r="H21">
+        <v>-2.611008635317047E-5</v>
+      </c>
+      <c r="I21">
+        <v>-2.7335182329835117E-5</v>
+      </c>
+      <c r="J21">
+        <v>-3.174009328571481E-5</v>
+      </c>
+      <c r="K21">
+        <v>-4.2384103439818688E-5</v>
+      </c>
+      <c r="L21">
+        <v>-4.7946899678796839E-5</v>
+      </c>
+      <c r="M21">
+        <v>-4.636176113270718E-5</v>
+      </c>
+      <c r="N21">
+        <v>-5.2182991936766676E-5</v>
+      </c>
+      <c r="O21">
+        <v>-7.7499295111194133E-5</v>
+      </c>
+      <c r="P21">
+        <v>-9.1649016949690854E-5</v>
+      </c>
+      <c r="Q21">
+        <v>-1.0658222541531925E-4</v>
+      </c>
+      <c r="R21">
+        <v>-1.3726566629967962E-4</v>
+      </c>
+      <c r="S21">
+        <v>-2.150102580149027E-4</v>
+      </c>
+      <c r="T21">
+        <v>-2.5834856054507416E-4</v>
+      </c>
+      <c r="U21">
+        <v>-3.2441576282388196E-4</v>
+      </c>
+      <c r="V21">
+        <v>-3.9785222209759441E-4</v>
+      </c>
+      <c r="W21">
+        <v>-5.5836115857749169E-4</v>
+      </c>
+      <c r="X21">
+        <v>-8.1512089676866184E-4</v>
+      </c>
+      <c r="Y21">
+        <v>-1.0725270413565746E-3</v>
+      </c>
+      <c r="Z21">
+        <v>-1.3088088358125805E-3</v>
+      </c>
+      <c r="AA21">
+        <v>-1.2830993519907796E-3</v>
+      </c>
+      <c r="AB21">
+        <v>-1.7437709560330639E-3</v>
+      </c>
+      <c r="AC21">
+        <v>-2.483157854851592E-3</v>
+      </c>
+      <c r="AD21">
+        <v>-2.8694146788614816E-3</v>
+      </c>
+      <c r="AE21">
+        <v>-3.1337977260460503E-3</v>
+      </c>
+      <c r="AF21">
+        <v>-3.2171327007279316E-3</v>
+      </c>
+      <c r="AG21">
+        <v>-4.0750963797110962E-3</v>
+      </c>
+      <c r="AH21">
+        <v>-5.2826286270493683E-3</v>
+      </c>
+      <c r="AI21">
+        <v>-5.3706295514880376E-3</v>
+      </c>
+      <c r="AJ21">
+        <v>-5.8732045004176725E-3</v>
+      </c>
+      <c r="AK21">
+        <v>-6.4531672280942476E-3</v>
+      </c>
+      <c r="AL21">
+        <v>-6.8213610465700514E-3</v>
+      </c>
+      <c r="AM21">
+        <v>-6.7551904750610126E-3</v>
+      </c>
+      <c r="AN21">
+        <v>-7.035663967127348E-3</v>
+      </c>
+      <c r="AO21">
+        <v>-7.3872938537746236E-3</v>
+      </c>
+      <c r="AP21">
+        <v>-7.4899764976742444E-3</v>
+      </c>
+      <c r="AQ21">
+        <v>-7.2454638997024867E-3</v>
+      </c>
+      <c r="AR21" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" t="s">
+        <v>0</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>-0.32180801969403589</v>
+      </c>
+      <c r="E24">
+        <v>-0.24835391559249614</v>
+      </c>
+      <c r="F24">
+        <v>-0.24106280321397716</v>
+      </c>
+      <c r="G24">
+        <v>-0.25204606578150579</v>
+      </c>
+      <c r="H24">
+        <v>-0.23647635633247516</v>
+      </c>
+      <c r="I24">
+        <v>-0.20380063737077947</v>
+      </c>
+      <c r="J24">
+        <v>-0.20358581062784248</v>
+      </c>
+      <c r="K24">
+        <v>-0.2129573704653433</v>
+      </c>
+      <c r="L24">
+        <v>-0.26268537140661191</v>
+      </c>
+      <c r="M24">
+        <v>-0.23550634104633489</v>
+      </c>
+      <c r="N24">
+        <v>-0.20065272573098819</v>
+      </c>
+      <c r="O24">
+        <v>-0.22820829269792009</v>
+      </c>
+      <c r="P24">
+        <v>-0.26095962894372471</v>
+      </c>
+      <c r="Q24">
+        <v>-0.31651067901876928</v>
+      </c>
+      <c r="R24">
+        <v>-0.33516575233036111</v>
+      </c>
+      <c r="S24">
+        <v>-0.29577657503756777</v>
+      </c>
+      <c r="T24">
+        <v>-0.29544165464999511</v>
+      </c>
+      <c r="U24">
+        <v>-0.28332722052968318</v>
+      </c>
+      <c r="V24">
+        <v>-0.26433955356375172</v>
+      </c>
+      <c r="W24">
+        <v>-0.26656667277197676</v>
+      </c>
+      <c r="X24">
+        <v>-0.26985882499920971</v>
+      </c>
+      <c r="Y24">
+        <v>-0.2778370240562813</v>
+      </c>
+      <c r="Z24">
+        <v>-0.28314950592105975</v>
+      </c>
+      <c r="AA24">
+        <v>-0.29142796441726215</v>
+      </c>
+      <c r="AB24">
+        <v>-0.30792782178134298</v>
+      </c>
+      <c r="AC24">
+        <v>-0.29609850403139792</v>
+      </c>
+      <c r="AD24">
+        <v>-0.27933588911271917</v>
+      </c>
+      <c r="AE24">
+        <v>-0.25733682873041347</v>
+      </c>
+      <c r="AF24">
+        <v>-0.24959548975679502</v>
+      </c>
+      <c r="AG24">
+        <v>-0.26204215611929976</v>
+      </c>
+      <c r="AH24">
+        <v>-0.27396811903430662</v>
+      </c>
+      <c r="AI24">
+        <v>-0.27229398784930742</v>
+      </c>
+      <c r="AJ24">
+        <v>-0.26343876284208384</v>
+      </c>
+      <c r="AK24">
+        <v>-0.25172374070099907</v>
+      </c>
+      <c r="AL24">
+        <v>-0.24271651795351434</v>
+      </c>
+      <c r="AM24">
+        <v>-0.24128398114117788</v>
+      </c>
+      <c r="AN24">
+        <v>-0.24557351815178197</v>
+      </c>
+      <c r="AO24">
+        <v>-0.24934086584961379</v>
+      </c>
+      <c r="AP24">
+        <v>-0.24794350263994924</v>
+      </c>
+      <c r="AQ24">
+        <v>-0.24229388427584642</v>
+      </c>
+      <c r="AR24" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" t="s">
+        <v>0</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>-0.40816927199948205</v>
+      </c>
+      <c r="E25">
+        <v>-1.5079719626350796E-3</v>
+      </c>
+      <c r="F25">
+        <v>4.2728031800165489E-4</v>
+      </c>
+      <c r="G25">
+        <v>-3.663345315116584E-3</v>
+      </c>
+      <c r="H25">
+        <v>-1.4818075439845257E-3</v>
+      </c>
+      <c r="I25">
+        <v>6.2811478108948937E-3</v>
+      </c>
+      <c r="J25">
+        <v>3.8948049391408501E-3</v>
+      </c>
+      <c r="K25">
+        <v>-2.0172908472759765E-4</v>
+      </c>
+      <c r="L25">
+        <v>-1.9374801743863967E-2</v>
+      </c>
+      <c r="M25">
+        <v>1.4306059354742662E-2</v>
+      </c>
+      <c r="N25">
+        <v>5.8162189431997247E-3</v>
+      </c>
+      <c r="O25">
+        <v>5.207754943127918E-3</v>
+      </c>
+      <c r="P25">
+        <v>8.3336142407887115E-3</v>
+      </c>
+      <c r="Q25">
+        <v>8.0629137465370038E-3</v>
+      </c>
+      <c r="R25">
+        <v>6.7686815380856857E-3</v>
+      </c>
+      <c r="S25">
+        <v>6.2623016142885346E-3</v>
+      </c>
+      <c r="T25">
+        <v>7.2232310556554213E-3</v>
+      </c>
+      <c r="U25">
+        <v>7.9649784090813358E-3</v>
+      </c>
+      <c r="V25">
+        <v>1.2827684813588591E-2</v>
+      </c>
+      <c r="W25">
+        <v>9.3555195434861793E-3</v>
+      </c>
+      <c r="X25">
+        <v>9.427570528352025E-3</v>
+      </c>
+      <c r="Y25">
+        <v>1.1206638379371359E-2</v>
+      </c>
+      <c r="Z25">
+        <v>1.0594741565412957E-2</v>
+      </c>
+      <c r="AA25">
+        <v>1.1201945995699458E-2</v>
+      </c>
+      <c r="AB25">
+        <v>1.0934354663839019E-2</v>
+      </c>
+      <c r="AC25">
+        <v>1.0567534462549988E-2</v>
+      </c>
+      <c r="AD25">
+        <v>1.0679385016649279E-2</v>
+      </c>
+      <c r="AE25">
+        <v>1.0860185025781843E-2</v>
+      </c>
+      <c r="AF25">
+        <v>1.1096365635797523E-2</v>
+      </c>
+      <c r="AG25">
+        <v>1.1001847016782751E-2</v>
+      </c>
+      <c r="AH25">
+        <v>1.0594924170671982E-2</v>
+      </c>
+      <c r="AI25">
+        <v>1.0356861670950179E-2</v>
+      </c>
+      <c r="AJ25">
+        <v>1.0423895532697791E-2</v>
+      </c>
+      <c r="AK25">
+        <v>1.0533404307279004E-2</v>
+      </c>
+      <c r="AL25">
+        <v>1.0613409985105071E-2</v>
+      </c>
+      <c r="AM25">
+        <v>1.0607560720017117E-2</v>
+      </c>
+      <c r="AN25">
+        <v>1.0481411747257918E-2</v>
+      </c>
+      <c r="AO25">
+        <v>1.0301652930195804E-2</v>
+      </c>
+      <c r="AP25">
+        <v>1.018690948548695E-2</v>
+      </c>
+      <c r="AQ25">
+        <v>1.0182312957646433E-2</v>
+      </c>
+      <c r="AR25" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>-0.409903193148974</v>
+      </c>
+      <c r="E26">
+        <v>-1.2403869571397941E-4</v>
+      </c>
+      <c r="F26">
+        <v>1.1873784877303173E-4</v>
+      </c>
+      <c r="G26">
+        <v>-1.6429716253436033E-3</v>
+      </c>
+      <c r="H26">
+        <v>-4.4030361560526421E-4</v>
+      </c>
+      <c r="I26">
+        <v>4.5146722122708649E-3</v>
+      </c>
+      <c r="J26">
+        <v>2.4729577400278702E-3</v>
+      </c>
+      <c r="K26">
+        <v>-8.0797844880275971E-4</v>
+      </c>
+      <c r="L26">
+        <v>-1.6328180273322002E-2</v>
+      </c>
+      <c r="M26">
+        <v>1.770619677138352E-2</v>
+      </c>
+      <c r="N26">
+        <v>7.6639084904716048E-3</v>
+      </c>
+      <c r="O26">
+        <v>3.997797691870919E-3</v>
+      </c>
+      <c r="P26">
+        <v>7.6814060563827891E-3</v>
+      </c>
+      <c r="Q26">
+        <v>8.0622943262543822E-3</v>
+      </c>
+      <c r="R26">
+        <v>6.4639792668091944E-3</v>
+      </c>
+      <c r="S26">
+        <v>4.1007181382692881E-3</v>
+      </c>
+      <c r="T26">
+        <v>4.4630497322280527E-3</v>
+      </c>
+      <c r="U26">
+        <v>6.2932797379492977E-3</v>
+      </c>
+      <c r="V26">
+        <v>1.0701177059874611E-2</v>
+      </c>
+      <c r="W26">
+        <v>7.9388580690142319E-3</v>
+      </c>
+      <c r="X26">
+        <v>8.802908342489979E-3</v>
+      </c>
+      <c r="Y26">
+        <v>1.0850675659815845E-2</v>
+      </c>
+      <c r="Z26">
+        <v>1.1105589334398425E-2</v>
+      </c>
+      <c r="AA26">
+        <v>1.1621103565734259E-2</v>
+      </c>
+      <c r="AB26">
+        <v>1.1425572844545262E-2</v>
+      </c>
+      <c r="AC26">
+        <v>1.1283169986555097E-2</v>
+      </c>
+      <c r="AD26">
+        <v>1.0954833641299289E-2</v>
+      </c>
+      <c r="AE26">
+        <v>1.1111709581527851E-2</v>
+      </c>
+      <c r="AF26">
+        <v>1.1339300514894346E-2</v>
+      </c>
+      <c r="AG26">
+        <v>1.1598090610410727E-2</v>
+      </c>
+      <c r="AH26">
+        <v>1.150300547139177E-2</v>
+      </c>
+      <c r="AI26">
+        <v>1.1073333966089949E-2</v>
+      </c>
+      <c r="AJ26">
+        <v>1.0823779757417495E-2</v>
+      </c>
+      <c r="AK26">
+        <v>1.0900062704114921E-2</v>
+      </c>
+      <c r="AL26">
+        <v>1.1021153706846198E-2</v>
+      </c>
+      <c r="AM26">
+        <v>1.1110491633479991E-2</v>
+      </c>
+      <c r="AN26">
+        <v>1.1107688775095659E-2</v>
+      </c>
+      <c r="AO26">
+        <v>1.097525186520526E-2</v>
+      </c>
+      <c r="AP26">
+        <v>1.0785140492433842E-2</v>
+      </c>
+      <c r="AQ26">
+        <v>1.0664619588045154E-2</v>
+      </c>
+      <c r="AR26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>-0.41621274645544737</v>
+      </c>
+      <c r="E27">
+        <v>-1.0182552034322945E-3</v>
+      </c>
+      <c r="F27">
+        <v>-8.9488705743212549E-5</v>
+      </c>
+      <c r="G27">
+        <v>-1.9226865674850102E-3</v>
+      </c>
+      <c r="H27">
+        <v>8.2162139583535909E-4</v>
+      </c>
+      <c r="I27">
+        <v>2.1083345921868446E-3</v>
+      </c>
+      <c r="J27">
+        <v>6.1735963957554318E-4</v>
+      </c>
+      <c r="K27">
+        <v>-1.8223614514897846E-3</v>
+      </c>
+      <c r="L27">
+        <v>-1.0526956262020326E-2</v>
+      </c>
+      <c r="M27">
+        <v>1.4312931767435755E-2</v>
+      </c>
+      <c r="N27">
+        <v>7.2156195699711323E-3</v>
+      </c>
+      <c r="O27">
+        <v>3.6469901753863887E-3</v>
+      </c>
+      <c r="P27">
+        <v>5.5272959174953451E-3</v>
+      </c>
+      <c r="Q27">
+        <v>6.8801002815780943E-3</v>
+      </c>
+      <c r="R27">
+        <v>5.7348579255082077E-3</v>
+      </c>
+      <c r="S27">
+        <v>3.8583912691222411E-3</v>
+      </c>
+      <c r="T27">
+        <v>3.870683431851929E-3</v>
+      </c>
+      <c r="U27">
+        <v>4.2979070955604937E-3</v>
+      </c>
+      <c r="V27">
+        <v>9.416219797926062E-3</v>
+      </c>
+      <c r="W27">
+        <v>7.1370838114025448E-3</v>
+      </c>
+      <c r="X27">
+        <v>7.6168006866538795E-3</v>
+      </c>
+      <c r="Y27">
+        <v>9.4634036201390326E-3</v>
+      </c>
+      <c r="Z27">
+        <v>9.6293049911503892E-3</v>
+      </c>
+      <c r="AA27">
+        <v>9.3793734374276183E-3</v>
+      </c>
+      <c r="AB27">
+        <v>8.7527949767569058E-3</v>
+      </c>
+      <c r="AC27">
+        <v>8.9470186940189822E-3</v>
+      </c>
+      <c r="AD27">
+        <v>8.9571742360450846E-3</v>
+      </c>
+      <c r="AE27">
+        <v>8.6676262052247099E-3</v>
+      </c>
+      <c r="AF27">
+        <v>8.8672629710788153E-3</v>
+      </c>
+      <c r="AG27">
+        <v>9.1258398896630899E-3</v>
+      </c>
+      <c r="AH27">
+        <v>9.4181878973640942E-3</v>
+      </c>
+      <c r="AI27">
+        <v>9.3236225818386087E-3</v>
+      </c>
+      <c r="AJ27">
+        <v>8.8632684934372707E-3</v>
+      </c>
+      <c r="AK27">
+        <v>8.5981352808932598E-3</v>
+      </c>
+      <c r="AL27">
+        <v>8.688335608071529E-3</v>
+      </c>
+      <c r="AM27">
+        <v>8.827009899931737E-3</v>
+      </c>
+      <c r="AN27">
+        <v>8.9307058826348928E-3</v>
+      </c>
+      <c r="AO27">
+        <v>8.932702880712684E-3</v>
+      </c>
+      <c r="AP27">
+        <v>8.7921726556920432E-3</v>
+      </c>
+      <c r="AQ27">
+        <v>8.5877317990998847E-3</v>
+      </c>
+      <c r="AR27" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>70</v>
+      </c>
+      <c r="B28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>-0.42588946850910375</v>
+      </c>
+      <c r="E28">
+        <v>-2.1771368115430234E-3</v>
+      </c>
+      <c r="F28">
+        <v>-9.2112083035511549E-4</v>
+      </c>
+      <c r="G28">
+        <v>2.2628552793705348E-3</v>
+      </c>
+      <c r="H28">
+        <v>3.4668631564467312E-3</v>
+      </c>
+      <c r="I28">
+        <v>6.6298952371429687E-4</v>
+      </c>
+      <c r="J28">
+        <v>-2.4114039056538639E-4</v>
+      </c>
+      <c r="K28">
+        <v>-1.841959405524729E-3</v>
+      </c>
+      <c r="L28">
+        <v>-6.6284440431901848E-3</v>
+      </c>
+      <c r="M28">
+        <v>7.9259223537857526E-3</v>
+      </c>
+      <c r="N28">
+        <v>5.4997634482404911E-3</v>
+      </c>
+      <c r="O28">
+        <v>3.5220684294871574E-3</v>
+      </c>
+      <c r="P28">
+        <v>4.9293807243475651E-3</v>
+      </c>
+      <c r="Q28">
+        <v>4.453077615495904E-3</v>
+      </c>
+      <c r="R28">
+        <v>4.5310974686461059E-3</v>
+      </c>
+      <c r="S28">
+        <v>3.2190702582109987E-3</v>
+      </c>
+      <c r="T28">
+        <v>3.3298081724826289E-3</v>
+      </c>
+      <c r="U28">
+        <v>3.2296308660102468E-3</v>
+      </c>
+      <c r="V28">
+        <v>6.8300242860726557E-3</v>
+      </c>
+      <c r="W28">
+        <v>6.3135431240617379E-3</v>
+      </c>
+      <c r="X28">
+        <v>7.0779041470153126E-3</v>
+      </c>
+      <c r="Y28">
+        <v>8.2522916971833338E-3</v>
+      </c>
+      <c r="Z28">
+        <v>8.3649101772453882E-3</v>
+      </c>
+      <c r="AA28">
+        <v>8.3792743221403065E-3</v>
+      </c>
+      <c r="AB28">
+        <v>7.4366821198623145E-3</v>
+      </c>
+      <c r="AC28">
+        <v>7.4242063313184059E-3</v>
+      </c>
+      <c r="AD28">
+        <v>7.6611656398231087E-3</v>
+      </c>
+      <c r="AE28">
+        <v>7.6630347872742033E-3</v>
+      </c>
+      <c r="AF28">
+        <v>7.377179481059315E-3</v>
+      </c>
+      <c r="AG28">
+        <v>7.6183966904427303E-3</v>
+      </c>
+      <c r="AH28">
+        <v>7.9215891980636277E-3</v>
+      </c>
+      <c r="AI28">
+        <v>8.2617026450046427E-3</v>
+      </c>
+      <c r="AJ28">
+        <v>8.1745791380935517E-3</v>
+      </c>
+      <c r="AK28">
+        <v>7.6829477417179604E-3</v>
+      </c>
+      <c r="AL28">
+        <v>7.4048998484819162E-3</v>
+      </c>
+      <c r="AM28">
+        <v>7.5169314114821861E-3</v>
+      </c>
+      <c r="AN28">
+        <v>7.6819220501992969E-3</v>
+      </c>
+      <c r="AO28">
+        <v>7.8072914946468175E-3</v>
+      </c>
+      <c r="AP28">
+        <v>7.8190320402959923E-3</v>
+      </c>
+      <c r="AQ28">
+        <v>7.6711944906110996E-3</v>
+      </c>
+      <c r="AR28" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" t="s">
+        <v>0</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1</v>
+      </c>
+      <c r="D29">
+        <v>-0.42694590074749916</v>
+      </c>
+      <c r="E29">
+        <v>-1.6158510297062945E-3</v>
+      </c>
+      <c r="F29">
+        <v>-1.6825434071647827E-3</v>
+      </c>
+      <c r="G29">
+        <v>-4.0256541159894299E-4</v>
+      </c>
+      <c r="H29">
+        <v>-1.4840325395545917E-3</v>
+      </c>
+      <c r="I29">
+        <v>-9.3138381649843227E-4</v>
+      </c>
+      <c r="J29">
+        <v>-1.1233358497749202E-3</v>
+      </c>
+      <c r="K29">
+        <v>-2.339875298202343E-3</v>
+      </c>
+      <c r="L29">
+        <v>-6.0228200470196502E-3</v>
+      </c>
+      <c r="M29">
+        <v>4.2561215085720749E-3</v>
+      </c>
+      <c r="N29">
+        <v>2.8915739760021486E-3</v>
+      </c>
+      <c r="O29">
+        <v>2.1351891419389979E-3</v>
+      </c>
+      <c r="P29">
+        <v>4.2621887045311002E-3</v>
+      </c>
+      <c r="Q29">
+        <v>3.8361138628514313E-3</v>
+      </c>
+      <c r="R29">
+        <v>2.8498633955303387E-3</v>
+      </c>
+      <c r="S29">
+        <v>2.7928010174461115E-3</v>
+      </c>
+      <c r="T29">
+        <v>2.8461385748112522E-3</v>
+      </c>
+      <c r="U29">
+        <v>2.9709292333512383E-3</v>
+      </c>
+      <c r="V29">
+        <v>5.7722247680171979E-3</v>
+      </c>
+      <c r="W29">
+        <v>5.2793636879378547E-3</v>
+      </c>
+      <c r="X29">
+        <v>7.5061494232930293E-3</v>
+      </c>
+      <c r="Y29">
+        <v>7.974824091466437E-3</v>
+      </c>
+      <c r="Z29">
+        <v>7.8045915556491097E-3</v>
+      </c>
+      <c r="AA29">
+        <v>8.0585069048962343E-3</v>
+      </c>
+      <c r="AB29">
+        <v>7.2337433732522771E-3</v>
+      </c>
+      <c r="AC29">
+        <v>7.2307491930625467E-3</v>
+      </c>
+      <c r="AD29">
+        <v>7.2671837535565054E-3</v>
+      </c>
+      <c r="AE29">
+        <v>7.5179311184302988E-3</v>
+      </c>
+      <c r="AF29">
+        <v>7.5542400298483914E-3</v>
+      </c>
+      <c r="AG29">
+        <v>7.2872405782788974E-3</v>
+      </c>
+      <c r="AH29">
+        <v>7.5878285504222265E-3</v>
+      </c>
+      <c r="AI29">
+        <v>7.9534130778585732E-3</v>
+      </c>
+      <c r="AJ29">
+        <v>8.3589710079793877E-3</v>
+      </c>
+      <c r="AK29">
+        <v>8.2929274711216472E-3</v>
+      </c>
+      <c r="AL29">
+        <v>7.7766504888135968E-3</v>
+      </c>
+      <c r="AM29">
+        <v>7.4921942413934683E-3</v>
+      </c>
+      <c r="AN29">
+        <v>7.6374329805304342E-3</v>
+      </c>
+      <c r="AO29">
+        <v>7.8399125899761279E-3</v>
+      </c>
+      <c r="AP29">
+        <v>7.9972097550333743E-3</v>
+      </c>
+      <c r="AQ29">
+        <v>8.0262326607979939E-3</v>
+      </c>
+      <c r="AR29" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>72</v>
+      </c>
+      <c r="B30" t="s">
+        <v>0</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1</v>
+      </c>
+      <c r="D30">
+        <v>-0.43186423374720662</v>
+      </c>
+      <c r="E30">
+        <v>-3.3841156803448014E-3</v>
+      </c>
+      <c r="F30">
+        <v>-2.6900165759548567E-3</v>
+      </c>
+      <c r="G30">
+        <v>-2.3659047497256447E-3</v>
+      </c>
+      <c r="H30">
+        <v>-9.5997716555379364E-4</v>
+      </c>
+      <c r="I30">
+        <v>-1.8977982624895917E-3</v>
+      </c>
+      <c r="J30">
+        <v>-1.9934053918534422E-3</v>
+      </c>
+      <c r="K30">
+        <v>-2.7128351941650419E-3</v>
+      </c>
+      <c r="L30">
+        <v>-5.674536037423461E-3</v>
+      </c>
+      <c r="M30">
+        <v>2.9051316364292479E-3</v>
+      </c>
+      <c r="N30">
+        <v>2.0043375248539053E-3</v>
+      </c>
+      <c r="O30">
+        <v>1.13243614157299E-3</v>
+      </c>
+      <c r="P30">
+        <v>2.8077802053609324E-3</v>
+      </c>
+      <c r="Q30">
+        <v>3.2055652816473379E-3</v>
+      </c>
+      <c r="R30">
+        <v>1.9882329836743984E-3</v>
+      </c>
+      <c r="S30">
+        <v>1.9450706125934136E-3</v>
+      </c>
+      <c r="T30">
+        <v>3.024737278263856E-3</v>
+      </c>
+      <c r="U30">
+        <v>3.4983379905950684E-3</v>
+      </c>
+      <c r="V30">
+        <v>5.9528505514463426E-3</v>
+      </c>
+      <c r="W30">
+        <v>4.6468839304850129E-3</v>
+      </c>
+      <c r="X30">
+        <v>6.5084289184287325E-3</v>
+      </c>
+      <c r="Y30">
+        <v>9.075504950748714E-3</v>
+      </c>
+      <c r="Z30">
+        <v>8.1001908211786877E-3</v>
+      </c>
+      <c r="AA30">
+        <v>8.5400779473638333E-3</v>
+      </c>
+      <c r="AB30">
+        <v>8.1867892489994043E-3</v>
+      </c>
+      <c r="AC30">
+        <v>8.6267370885192429E-3</v>
+      </c>
+      <c r="AD30">
+        <v>8.5652357514767186E-3</v>
+      </c>
+      <c r="AE30">
+        <v>8.6328617348296333E-3</v>
+      </c>
+      <c r="AF30">
+        <v>8.968257422863557E-3</v>
+      </c>
+      <c r="AG30">
+        <v>9.0566341861387789E-3</v>
+      </c>
+      <c r="AH30">
+        <v>8.7901197907951367E-3</v>
+      </c>
+      <c r="AI30">
+        <v>9.1740072294510533E-3</v>
+      </c>
+      <c r="AJ30">
+        <v>9.6319237014751979E-3</v>
+      </c>
+      <c r="AK30">
+        <v>1.013657199286333E-2</v>
+      </c>
+      <c r="AL30">
+        <v>1.0088699144180591E-2</v>
+      </c>
+      <c r="AM30">
+        <v>9.5096103640835428E-3</v>
+      </c>
+      <c r="AN30">
+        <v>9.1982724065090005E-3</v>
+      </c>
+      <c r="AO30">
+        <v>9.389428526088206E-3</v>
+      </c>
+      <c r="AP30">
+        <v>9.6465837151198386E-3</v>
+      </c>
+      <c r="AQ30">
+        <v>9.849621597009306E-3</v>
+      </c>
+      <c r="AR30" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>73</v>
+      </c>
+      <c r="B31" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <v>-0.43453364957554208</v>
+      </c>
+      <c r="E31">
+        <v>-3.9896875859208869E-3</v>
+      </c>
+      <c r="F31">
+        <v>-4.2827626031000654E-3</v>
+      </c>
+      <c r="G31">
+        <v>-3.8359605392562779E-4</v>
+      </c>
+      <c r="H31">
+        <v>-6.4698912686156351E-4</v>
+      </c>
+      <c r="I31">
+        <v>-3.2288024616695665E-3</v>
+      </c>
+      <c r="J31">
+        <v>-3.1022341913188867E-3</v>
+      </c>
+      <c r="K31">
+        <v>-4.0480917959517804E-3</v>
+      </c>
+      <c r="L31">
+        <v>-6.3292574426357939E-3</v>
+      </c>
+      <c r="M31">
+        <v>1.2110271545461293E-3</v>
+      </c>
+      <c r="N31">
+        <v>6.3614930816757731E-4</v>
+      </c>
+      <c r="O31">
+        <v>7.9607643794665783E-5</v>
+      </c>
+      <c r="P31">
+        <v>1.411504990820156E-3</v>
+      </c>
+      <c r="Q31">
+        <v>1.5489098613225005E-3</v>
+      </c>
+      <c r="R31">
+        <v>1.1913240920088386E-3</v>
+      </c>
+      <c r="S31">
+        <v>1.4130798413484191E-3</v>
+      </c>
+      <c r="T31">
+        <v>2.1328620018644662E-3</v>
+      </c>
+      <c r="U31">
+        <v>2.9639677658923058E-3</v>
+      </c>
+      <c r="V31">
+        <v>5.4027259649738757E-3</v>
+      </c>
+      <c r="W31">
+        <v>4.6419048655264028E-3</v>
+      </c>
+      <c r="X31">
+        <v>5.5507355669827674E-3</v>
+      </c>
+      <c r="Y31">
+        <v>7.143630232815501E-3</v>
+      </c>
+      <c r="Z31">
+        <v>8.0111728326868192E-3</v>
+      </c>
+      <c r="AA31">
+        <v>8.8202374093412916E-3</v>
+      </c>
+      <c r="AB31">
+        <v>8.8202483940802434E-3</v>
+      </c>
+      <c r="AC31">
+        <v>9.7248453446240335E-3</v>
+      </c>
+      <c r="AD31">
+        <v>1.0203681987923652E-2</v>
+      </c>
+      <c r="AE31">
+        <v>1.0161409543672728E-2</v>
+      </c>
+      <c r="AF31">
+        <v>1.0310977076644356E-2</v>
+      </c>
+      <c r="AG31">
+        <v>1.0766333003503104E-2</v>
+      </c>
+      <c r="AH31">
+        <v>1.0929705159211267E-2</v>
+      </c>
+      <c r="AI31">
+        <v>1.0671807473866646E-2</v>
+      </c>
+      <c r="AJ31">
+        <v>1.1171853088248307E-2</v>
+      </c>
+      <c r="AK31">
+        <v>1.1756418409458846E-2</v>
+      </c>
+      <c r="AL31">
+        <v>1.239665506693588E-2</v>
+      </c>
+      <c r="AM31">
+        <v>1.2378192847108116E-2</v>
+      </c>
+      <c r="AN31">
+        <v>1.1721991345939875E-2</v>
+      </c>
+      <c r="AO31">
+        <v>1.1380459529961084E-2</v>
+      </c>
+      <c r="AP31">
+        <v>1.1636564423786466E-2</v>
+      </c>
+      <c r="AQ31">
+        <v>1.1970290449473564E-2</v>
+      </c>
+      <c r="AR31" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="32" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>74</v>
+      </c>
+      <c r="B32" t="s">
+        <v>0</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1</v>
+      </c>
+      <c r="D32">
+        <v>-0.43970127483260618</v>
+      </c>
+      <c r="E32">
+        <v>-6.3758676898219568E-3</v>
+      </c>
+      <c r="F32">
+        <v>-6.1710640190068555E-3</v>
+      </c>
+      <c r="G32">
+        <v>-5.8291983293127791E-3</v>
+      </c>
+      <c r="H32">
+        <v>-6.6274685582406456E-3</v>
+      </c>
+      <c r="I32">
+        <v>-5.7868386414476336E-3</v>
+      </c>
+      <c r="J32">
+        <v>-5.4247404128997534E-3</v>
+      </c>
+      <c r="K32">
+        <v>-5.8510761677140755E-3</v>
+      </c>
+      <c r="L32">
+        <v>-7.5243162516370199E-3</v>
+      </c>
+      <c r="M32">
+        <v>-1.8061664178034009E-3</v>
+      </c>
+      <c r="N32">
+        <v>-1.4986210250522158E-3</v>
+      </c>
+      <c r="O32">
+        <v>-1.8110144189971145E-3</v>
+      </c>
+      <c r="P32">
+        <v>-3.9871123572216005E-4</v>
+      </c>
+      <c r="Q32">
+        <v>-4.169399257831774E-4</v>
+      </c>
+      <c r="R32">
+        <v>-8.6185229710411537E-4</v>
+      </c>
+      <c r="S32">
+        <v>1.9902679164651715E-4</v>
+      </c>
+      <c r="T32">
+        <v>6.695258654779157E-4</v>
+      </c>
+      <c r="U32">
+        <v>1.9741082074348215E-3</v>
+      </c>
+      <c r="V32">
+        <v>4.6319874425747587E-3</v>
+      </c>
+      <c r="W32">
+        <v>3.887713668687176E-3</v>
+      </c>
+      <c r="X32">
+        <v>5.347442750442688E-3</v>
+      </c>
+      <c r="Y32">
+        <v>5.977941664917219E-3</v>
+      </c>
+      <c r="Z32">
+        <v>6.3351836232259373E-3</v>
+      </c>
+      <c r="AA32">
+        <v>9.3136522289993806E-3</v>
+      </c>
+      <c r="AB32">
+        <v>9.0333272390577535E-3</v>
+      </c>
+      <c r="AC32">
+        <v>9.9186602729033346E-3</v>
+      </c>
+      <c r="AD32">
+        <v>1.0866123970660946E-2</v>
+      </c>
+      <c r="AE32">
+        <v>1.1449596331568612E-2</v>
+      </c>
+      <c r="AF32">
+        <v>1.1489062534020433E-2</v>
+      </c>
+      <c r="AG32">
+        <v>1.1745548026708741E-2</v>
+      </c>
+      <c r="AH32">
+        <v>1.2347547731156094E-2</v>
+      </c>
+      <c r="AI32">
+        <v>1.2602678632187003E-2</v>
+      </c>
+      <c r="AJ32">
+        <v>1.2354722497741166E-2</v>
+      </c>
+      <c r="AK32">
+        <v>1.2997384728283323E-2</v>
+      </c>
+      <c r="AL32">
+        <v>1.3739914487686133E-2</v>
+      </c>
+      <c r="AM32">
+        <v>1.4549385902648149E-2</v>
+      </c>
+      <c r="AN32">
+        <v>1.4569838901951571E-2</v>
+      </c>
+      <c r="AO32">
+        <v>1.3820429111233656E-2</v>
+      </c>
+      <c r="AP32">
+        <v>1.3442740464457592E-2</v>
+      </c>
+      <c r="AQ32">
+        <v>1.3781202003333104E-2</v>
+      </c>
+      <c r="AR32" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" t="s">
+        <v>0</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33">
+        <v>-0.44432319982829754</v>
+      </c>
+      <c r="E33">
+        <v>-8.9191718227017991E-3</v>
+      </c>
+      <c r="F33">
+        <v>-8.9859406601919267E-3</v>
+      </c>
+      <c r="G33">
+        <v>-7.9028123932760042E-3</v>
+      </c>
+      <c r="H33">
+        <v>-7.211072690439857E-3</v>
+      </c>
+      <c r="I33">
+        <v>-8.0053977011733668E-3</v>
+      </c>
+      <c r="J33">
+        <v>-8.3702726837856511E-3</v>
+      </c>
+      <c r="K33">
+        <v>-8.5948976980118053E-3</v>
+      </c>
+      <c r="L33">
+        <v>-9.938161251024924E-3</v>
+      </c>
+      <c r="M33">
+        <v>-5.9576037610547528E-3</v>
+      </c>
+      <c r="N33">
+        <v>-5.2803698205134975E-3</v>
+      </c>
+      <c r="O33">
+        <v>-4.9828036984713164E-3</v>
+      </c>
+      <c r="P33">
+        <v>-3.4620681293324185E-3</v>
+      </c>
+      <c r="Q33">
+        <v>-2.8702230690704766E-3</v>
+      </c>
+      <c r="R33">
+        <v>-4.1199681101561914E-3</v>
+      </c>
+      <c r="S33">
+        <v>-2.9128822978613522E-3</v>
+      </c>
+      <c r="T33">
+        <v>-1.5268848000998814E-3</v>
+      </c>
+      <c r="U33">
+        <v>-5.3136067119646802E-4</v>
+      </c>
+      <c r="V33">
+        <v>2.1977099506973463E-3</v>
+      </c>
+      <c r="W33">
+        <v>2.5111301248560425E-3</v>
+      </c>
+      <c r="X33">
+        <v>3.8552578780133295E-3</v>
+      </c>
+      <c r="Y33">
+        <v>5.2466241403223424E-3</v>
+      </c>
+      <c r="Z33">
+        <v>4.9851676884396512E-3</v>
+      </c>
+      <c r="AA33">
+        <v>6.8581708188279467E-3</v>
+      </c>
+      <c r="AB33">
+        <v>8.3973440458843251E-3</v>
+      </c>
+      <c r="AC33">
+        <v>8.902145229039482E-3</v>
+      </c>
+      <c r="AD33">
+        <v>9.928973248487849E-3</v>
+      </c>
+      <c r="AE33">
+        <v>1.1097587087871064E-2</v>
+      </c>
+      <c r="AF33">
+        <v>1.1900617350078468E-2</v>
+      </c>
+      <c r="AG33">
+        <v>1.2084760407702677E-2</v>
+      </c>
+      <c r="AH33">
+        <v>1.2522317028648089E-2</v>
+      </c>
+      <c r="AI33">
+        <v>1.3305199120177857E-2</v>
+      </c>
+      <c r="AJ33">
+        <v>1.3701180474859076E-2</v>
+      </c>
+      <c r="AK33">
+        <v>1.3525621589272396E-2</v>
+      </c>
+      <c r="AL33">
+        <v>1.4347304146918927E-2</v>
+      </c>
+      <c r="AM33">
+        <v>1.5276365375035683E-2</v>
+      </c>
+      <c r="AN33">
+        <v>1.6283404326733586E-2</v>
+      </c>
+      <c r="AO33">
+        <v>1.6380530662771398E-2</v>
+      </c>
+      <c r="AP33">
+        <v>1.5583960723146162E-2</v>
+      </c>
+      <c r="AQ33">
+        <v>1.5209029958383524E-2</v>
+      </c>
+      <c r="AR33" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="34" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B34" t="s">
+        <v>0</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>-0.45080115812599564</v>
+      </c>
+      <c r="E34">
+        <v>-1.0814523556398503E-2</v>
+      </c>
+      <c r="F34">
+        <v>-1.0857080440751732E-2</v>
+      </c>
+      <c r="G34">
+        <v>-1.0622896349736899E-2</v>
+      </c>
+      <c r="H34">
+        <v>-1.0369690772010831E-2</v>
+      </c>
+      <c r="I34">
+        <v>-1.0493848240901715E-2</v>
+      </c>
+      <c r="J34">
+        <v>-1.051605392531435E-2</v>
+      </c>
+      <c r="K34">
+        <v>-1.0729811914701681E-2</v>
+      </c>
+      <c r="L34">
+        <v>-1.232366827032072E-2</v>
+      </c>
+      <c r="M34">
+        <v>-9.6650383116729799E-3</v>
+      </c>
+      <c r="N34">
+        <v>-9.1731817992883879E-3</v>
+      </c>
+      <c r="O34">
+        <v>-8.9791077167225564E-3</v>
+      </c>
+      <c r="P34">
+        <v>-7.5955747671396789E-3</v>
+      </c>
+      <c r="Q34">
+        <v>-6.7435992439810466E-3</v>
+      </c>
+      <c r="R34">
+        <v>-7.3811079556000414E-3</v>
+      </c>
+      <c r="S34">
+        <v>-7.4432871812877832E-3</v>
+      </c>
+      <c r="T34">
+        <v>-6.3742556528392225E-3</v>
+      </c>
+      <c r="U34">
+        <v>-4.6740909507276829E-3</v>
+      </c>
+      <c r="V34">
+        <v>-1.6040147092895585E-3</v>
+      </c>
+      <c r="W34">
+        <v>-5.4108289038434787E-4</v>
+      </c>
+      <c r="X34">
+        <v>2.1867616254056532E-4</v>
+      </c>
+      <c r="Y34">
+        <v>2.0870234480727667E-3</v>
+      </c>
+      <c r="Z34">
+        <v>2.6311498236422093E-3</v>
+      </c>
+      <c r="AA34">
+        <v>3.8936033698730443E-3</v>
+      </c>
+      <c r="AB34">
+        <v>4.7371573278166546E-3</v>
+      </c>
+      <c r="AC34">
+        <v>6.5906617403683754E-3</v>
+      </c>
+      <c r="AD34">
+        <v>7.0789298364085651E-3</v>
+      </c>
+      <c r="AE34">
+        <v>8.2209552114190787E-3</v>
+      </c>
+      <c r="AF34">
+        <v>9.647531074789828E-3</v>
+      </c>
+      <c r="AG34">
+        <v>1.0768938692989394E-2</v>
+      </c>
+      <c r="AH34">
+        <v>1.1258035730625782E-2</v>
+      </c>
+      <c r="AI34">
+        <v>1.2030752715628146E-2</v>
+      </c>
+      <c r="AJ34">
+        <v>1.3059721051611572E-2</v>
+      </c>
+      <c r="AK34">
+        <v>1.3703484722477788E-2</v>
+      </c>
+      <c r="AL34">
+        <v>1.3749362159758194E-2</v>
+      </c>
+      <c r="AM34">
+        <v>1.4808411198811433E-2</v>
+      </c>
+      <c r="AN34">
+        <v>1.5966102534545945E-2</v>
+      </c>
+      <c r="AO34">
+        <v>1.7209158172735384E-2</v>
+      </c>
+      <c r="AP34">
+        <v>1.7470866592903589E-2</v>
+      </c>
+      <c r="AQ34">
+        <v>1.6756838613557923E-2</v>
+      </c>
+      <c r="AR34" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="35" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" t="s">
+        <v>0</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1</v>
+      </c>
+      <c r="D35">
+        <v>-0.45590615247111643</v>
+      </c>
+      <c r="E35">
+        <v>-9.9209637664135486E-3</v>
+      </c>
+      <c r="F35">
+        <v>-1.0027184265056333E-2</v>
+      </c>
+      <c r="G35">
+        <v>-9.5104487568517526E-3</v>
+      </c>
+      <c r="H35">
+        <v>-1.0009460798887593E-2</v>
+      </c>
+      <c r="I35">
+        <v>-1.04932502343138E-2</v>
+      </c>
+      <c r="J35">
+        <v>-1.0816907272367504E-2</v>
+      </c>
+      <c r="K35">
+        <v>-1.046014326446415E-2</v>
+      </c>
+      <c r="L35">
+        <v>-1.2301426696862183E-2</v>
+      </c>
+      <c r="M35">
+        <v>-1.1444351400615393E-2</v>
+      </c>
+      <c r="N35">
+        <v>-1.035527792577895E-2</v>
+      </c>
+      <c r="O35">
+        <v>-1.1576815572165833E-2</v>
+      </c>
+      <c r="P35">
+        <v>-1.0672468930250867E-2</v>
+      </c>
+      <c r="Q35">
+        <v>-1.05738752977666E-2</v>
+      </c>
+      <c r="R35">
+        <v>-1.0671120281660118E-2</v>
+      </c>
+      <c r="S35">
+        <v>-1.0460237537501804E-2</v>
+      </c>
+      <c r="T35">
+        <v>-1.0908927432271953E-2</v>
+      </c>
+      <c r="U35">
+        <v>-1.0672641921057768E-2</v>
+      </c>
+      <c r="V35">
+        <v>-8.1784478441498942E-3</v>
+      </c>
+      <c r="W35">
+        <v>-6.0402095113846199E-3</v>
+      </c>
+      <c r="X35">
+        <v>-4.5208900925547968E-3</v>
+      </c>
+      <c r="Y35">
+        <v>-4.4465974708758904E-3</v>
+      </c>
+      <c r="Z35">
+        <v>-3.753191169581227E-3</v>
+      </c>
+      <c r="AA35">
+        <v>-1.6972675428011397E-3</v>
+      </c>
+      <c r="AB35">
+        <v>-7.7207473586099473E-4</v>
+      </c>
+      <c r="AC35">
+        <v>3.2387952998669256E-4</v>
+      </c>
+      <c r="AD35">
+        <v>7.4825164569980451E-4</v>
+      </c>
+      <c r="AE35">
+        <v>1.2583640483083691E-3</v>
+      </c>
+      <c r="AF35">
+        <v>2.6266339413092421E-3</v>
+      </c>
+      <c r="AG35">
+        <v>4.3461923473238073E-3</v>
+      </c>
+      <c r="AH35">
+        <v>5.9475920776617675E-3</v>
+      </c>
+      <c r="AI35">
+        <v>7.0366175217523308E-3</v>
+      </c>
+      <c r="AJ35">
+        <v>8.4026591350254143E-3</v>
+      </c>
+      <c r="AK35">
+        <v>9.7819133303556072E-3</v>
+      </c>
+      <c r="AL35">
+        <v>1.0860809608097877E-2</v>
+      </c>
+      <c r="AM35">
+        <v>1.1411169734456106E-2</v>
+      </c>
+      <c r="AN35">
+        <v>1.2786979053269365E-2</v>
+      </c>
+      <c r="AO35">
+        <v>1.422422517567129E-2</v>
+      </c>
+      <c r="AP35">
+        <v>1.5747657463394182E-2</v>
+      </c>
+      <c r="AQ35">
+        <v>1.6341264040691139E-2</v>
+      </c>
+      <c r="AR35" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="36" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" t="s">
+        <v>0</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1</v>
+      </c>
+      <c r="D36">
+        <v>-0.45778815226361919</v>
+      </c>
+      <c r="E36">
+        <v>-6.5988184161977492E-3</v>
+      </c>
+      <c r="F36">
+        <v>-6.4814432147647372E-3</v>
+      </c>
+      <c r="G36">
+        <v>-6.7649716799555448E-3</v>
+      </c>
+      <c r="H36">
+        <v>-6.7726186482217621E-3</v>
+      </c>
+      <c r="I36">
+        <v>-6.9787612750279449E-3</v>
+      </c>
+      <c r="J36">
+        <v>-7.3570833678180958E-3</v>
+      </c>
+      <c r="K36">
+        <v>-7.3774060306054934E-3</v>
+      </c>
+      <c r="L36">
+        <v>-8.2094188722860451E-3</v>
+      </c>
+      <c r="M36">
+        <v>-8.2175745207442863E-3</v>
+      </c>
+      <c r="N36">
+        <v>-8.0184027667799529E-3</v>
+      </c>
+      <c r="O36">
+        <v>-8.9170873919991456E-3</v>
+      </c>
+      <c r="P36">
+        <v>-9.8079867358946138E-3</v>
+      </c>
+      <c r="Q36">
+        <v>-1.0440173751234905E-2</v>
+      </c>
+      <c r="R36">
+        <v>-1.0838516538798249E-2</v>
+      </c>
+      <c r="S36">
+        <v>-1.1157136044247895E-2</v>
+      </c>
+      <c r="T36">
+        <v>-1.1416096610626869E-2</v>
+      </c>
+      <c r="U36">
+        <v>-1.2882077488217791E-2</v>
+      </c>
+      <c r="V36">
+        <v>-1.23962619545116E-2</v>
+      </c>
+      <c r="W36">
+        <v>-1.2171359244544044E-2</v>
+      </c>
+      <c r="X36">
+        <v>-1.0412627812995123E-2</v>
+      </c>
+      <c r="Y36">
+        <v>-9.0278243016717052E-3</v>
+      </c>
+      <c r="Z36">
+        <v>-1.1815779397702952E-2</v>
+      </c>
+      <c r="AA36">
+        <v>-1.0535144063148871E-2</v>
+      </c>
+      <c r="AB36">
+        <v>-9.4767399484810833E-3</v>
+      </c>
+      <c r="AC36">
+        <v>-7.6803590380409292E-3</v>
+      </c>
+      <c r="AD36">
+        <v>-7.6077665300977593E-3</v>
+      </c>
+      <c r="AE36">
+        <v>-9.7816613562425325E-3</v>
+      </c>
+      <c r="AF36">
+        <v>-9.2620124019232586E-3</v>
+      </c>
+      <c r="AG36">
+        <v>-8.039305034049371E-3</v>
+      </c>
+      <c r="AH36">
+        <v>-6.5843582995107064E-3</v>
+      </c>
+      <c r="AI36">
+        <v>-4.8172144834719433E-3</v>
+      </c>
+      <c r="AJ36">
+        <v>-3.1887732198438434E-3</v>
+      </c>
+      <c r="AK36">
+        <v>-1.177098903745899E-3</v>
+      </c>
+      <c r="AL36">
+        <v>3.0391166172377693E-4</v>
+      </c>
+      <c r="AM36">
+        <v>1.8007822470658685E-3</v>
+      </c>
+      <c r="AN36">
+        <v>3.1295545571032868E-3</v>
+      </c>
+      <c r="AO36">
+        <v>4.7104139589932981E-3</v>
+      </c>
+      <c r="AP36">
+        <v>6.2326121225194653E-3</v>
+      </c>
+      <c r="AQ36">
+        <v>7.8496715306570763E-3</v>
+      </c>
+      <c r="AR36" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="37" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>79</v>
+      </c>
+      <c r="B37" t="s">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37">
+        <v>-0.45665656750298311</v>
+      </c>
+      <c r="E37">
+        <v>-2.4666714852504268E-3</v>
+      </c>
+      <c r="F37">
+        <v>-2.4314200350681325E-3</v>
+      </c>
+      <c r="G37">
+        <v>-2.5274267242783588E-3</v>
+      </c>
+      <c r="H37">
+        <v>-2.6009048649671684E-3</v>
+      </c>
+      <c r="I37">
+        <v>-2.7028901706483421E-3</v>
+      </c>
+      <c r="J37">
+        <v>-2.9671412834801902E-3</v>
+      </c>
+      <c r="K37">
+        <v>-3.0149933736907109E-3</v>
+      </c>
+      <c r="L37">
+        <v>-3.6198833424055388E-3</v>
+      </c>
+      <c r="M37">
+        <v>-3.4558399515352001E-3</v>
+      </c>
+      <c r="N37">
+        <v>-3.5726336629017252E-3</v>
+      </c>
+      <c r="O37">
+        <v>-4.3207214797026938E-3</v>
+      </c>
+      <c r="P37">
+        <v>-4.790015467392994E-3</v>
+      </c>
+      <c r="Q37">
+        <v>-6.0305855915541162E-3</v>
+      </c>
+      <c r="R37">
+        <v>-6.6752233994118448E-3</v>
+      </c>
+      <c r="S37">
+        <v>-7.470884852656956E-3</v>
+      </c>
+      <c r="T37">
+        <v>-8.1086250831529094E-3</v>
+      </c>
+      <c r="U37">
+        <v>-8.9944757269261877E-3</v>
+      </c>
+      <c r="V37">
+        <v>-1.0116823420367738E-2</v>
+      </c>
+      <c r="W37">
+        <v>-1.1621720421610637E-2</v>
+      </c>
+      <c r="X37">
+        <v>-1.3224159386450773E-2</v>
+      </c>
+      <c r="Y37">
+        <v>-1.1429650304175587E-2</v>
+      </c>
+      <c r="Z37">
+        <v>-1.1912117311850157E-2</v>
+      </c>
+      <c r="AA37">
+        <v>-1.5981051214488395E-2</v>
+      </c>
+      <c r="AB37">
+        <v>-1.6691373969128898E-2</v>
+      </c>
+      <c r="AC37">
+        <v>-1.631551828763772E-2</v>
+      </c>
+      <c r="AD37">
+        <v>-1.5451977725093158E-2</v>
+      </c>
+      <c r="AE37">
+        <v>-1.758147816900224E-2</v>
+      </c>
+      <c r="AF37">
+        <v>-2.29981607741091E-2</v>
+      </c>
+      <c r="AG37">
+        <v>-2.2785309732781867E-2</v>
+      </c>
+      <c r="AH37">
+        <v>-2.2896783122773712E-2</v>
+      </c>
+      <c r="AI37">
+        <v>-2.3237027439425517E-2</v>
+      </c>
+      <c r="AJ37">
+        <v>-2.2670656803242151E-2</v>
+      </c>
+      <c r="AK37">
+        <v>-2.1354774944863264E-2</v>
+      </c>
+      <c r="AL37">
+        <v>-1.977098511317793E-2</v>
+      </c>
+      <c r="AM37">
+        <v>-1.9371522547619313E-2</v>
+      </c>
+      <c r="AN37">
+        <v>-1.8339211364380936E-2</v>
+      </c>
+      <c r="AO37">
+        <v>-1.6545310777491384E-2</v>
+      </c>
+      <c r="AP37">
+        <v>-1.5910361526515537E-2</v>
+      </c>
+      <c r="AQ37">
+        <v>-1.5500489571315834E-2</v>
+      </c>
+      <c r="AR37" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>80</v>
+      </c>
+      <c r="B38" t="s">
+        <v>0</v>
+      </c>
+      <c r="C38" t="s">
+        <v>1</v>
+      </c>
+      <c r="D38">
+        <v>-0.4544322979315128</v>
+      </c>
+      <c r="E38">
+        <v>-5.1058732401432216E-4</v>
+      </c>
+      <c r="F38">
+        <v>-5.1525939014451794E-4</v>
+      </c>
+      <c r="G38">
+        <v>-5.2898240585952383E-4</v>
+      </c>
+      <c r="H38">
+        <v>-5.4371923395535315E-4</v>
+      </c>
+      <c r="I38">
+        <v>-5.7742369064911481E-4</v>
+      </c>
+      <c r="J38">
+        <v>-6.1454793251458639E-4</v>
+      </c>
+      <c r="K38">
+        <v>-6.7332461681746114E-4</v>
+      </c>
+      <c r="L38">
+        <v>-7.9498013992573835E-4</v>
+      </c>
+      <c r="M38">
+        <v>-8.0783336838291531E-4</v>
+      </c>
+      <c r="N38">
+        <v>-7.8258422451299436E-4</v>
+      </c>
+      <c r="O38">
+        <v>-1.0783616421569109E-3</v>
+      </c>
+      <c r="P38">
+        <v>-1.2923729811947782E-3</v>
+      </c>
+      <c r="Q38">
+        <v>-1.619178467124005E-3</v>
+      </c>
+      <c r="R38">
+        <v>-2.2050651341745664E-3</v>
+      </c>
+      <c r="S38">
+        <v>-2.6870577844113064E-3</v>
+      </c>
+      <c r="T38">
+        <v>-3.1541202098193666E-3</v>
+      </c>
+      <c r="U38">
+        <v>-3.6197133057016551E-3</v>
+      </c>
+      <c r="V38">
+        <v>-4.3179926878662567E-3</v>
+      </c>
+      <c r="W38">
+        <v>-5.694378872708683E-3</v>
+      </c>
+      <c r="X38">
+        <v>-7.4015249238778003E-3</v>
+      </c>
+      <c r="Y38">
+        <v>-8.6060875990128793E-3</v>
+      </c>
+      <c r="Z38">
+        <v>-7.9126317379460409E-3</v>
+      </c>
+      <c r="AA38">
+        <v>-9.4732027651996953E-3</v>
+      </c>
+      <c r="AB38">
+        <v>-1.3517499395478083E-2</v>
+      </c>
+      <c r="AC38">
+        <v>-1.4701891072522677E-2</v>
+      </c>
+      <c r="AD38">
+        <v>-1.5699329680991581E-2</v>
+      </c>
+      <c r="AE38">
+        <v>-1.5799115885448911E-2</v>
+      </c>
+      <c r="AF38">
+        <v>-1.9081245678720438E-2</v>
+      </c>
+      <c r="AG38">
+        <v>-2.4945752502265772E-2</v>
+      </c>
+      <c r="AH38">
+        <v>-2.5288587962913389E-2</v>
+      </c>
+      <c r="AI38">
+        <v>-2.6782095569690856E-2</v>
+      </c>
+      <c r="AJ38">
+        <v>-2.8722219577493435E-2</v>
+      </c>
+      <c r="AK38">
+        <v>-2.9730246941222616E-2</v>
+      </c>
+      <c r="AL38">
+        <v>-2.9312144350073399E-2</v>
+      </c>
+      <c r="AM38">
+        <v>-2.9428504174874304E-2</v>
+      </c>
+      <c r="AN38">
+        <v>-3.0498360421657045E-2</v>
+      </c>
+      <c r="AO38">
+        <v>-3.0697626371043119E-2</v>
+      </c>
+      <c r="AP38">
+        <v>-2.9600622261705678E-2</v>
+      </c>
+      <c r="AQ38">
+        <v>-3.0718864731891893E-2</v>
+      </c>
+      <c r="AR38" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>81</v>
+      </c>
+      <c r="B39" t="s">
+        <v>0</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>-0.45231446063433361</v>
+      </c>
+      <c r="E39">
+        <v>-5.7134618956733441E-5</v>
+      </c>
+      <c r="F39">
+        <v>-5.9300431025699485E-5</v>
+      </c>
+      <c r="G39">
+        <v>-5.9833766897887664E-5</v>
+      </c>
+      <c r="H39">
+        <v>-6.0923514077548813E-5</v>
+      </c>
+      <c r="I39">
+        <v>-6.378205802293202E-5</v>
+      </c>
+      <c r="J39">
+        <v>-7.4060272493292612E-5</v>
+      </c>
+      <c r="K39">
+        <v>-9.8896412505933284E-5</v>
+      </c>
+      <c r="L39">
+        <v>-1.1187579770455258E-4</v>
+      </c>
+      <c r="M39">
+        <v>-1.0817730557660665E-4</v>
+      </c>
+      <c r="N39">
+        <v>-1.2176020486598382E-4</v>
+      </c>
+      <c r="O39">
+        <v>-1.8083144187319711E-4</v>
+      </c>
+      <c r="P39">
+        <v>-2.1384675048402579E-4</v>
+      </c>
+      <c r="Q39">
+        <v>-2.4869107023739456E-4</v>
+      </c>
+      <c r="R39">
+        <v>-3.2028566563419014E-4</v>
+      </c>
+      <c r="S39">
+        <v>-5.0169074283423765E-4</v>
+      </c>
+      <c r="T39">
+        <v>-6.0281375620402367E-4</v>
+      </c>
+      <c r="U39">
+        <v>-7.5697023912268957E-4</v>
+      </c>
+      <c r="V39">
+        <v>-9.2832180329566194E-4</v>
+      </c>
+      <c r="W39">
+        <v>-1.3028444665454386E-3</v>
+      </c>
+      <c r="X39">
+        <v>-1.9019505815254245E-3</v>
+      </c>
+      <c r="Y39">
+        <v>-2.5025618815665562E-3</v>
+      </c>
+      <c r="Z39">
+        <v>-3.0538861278310292E-3</v>
+      </c>
+      <c r="AA39">
+        <v>-2.9938981546451249E-3</v>
+      </c>
+      <c r="AB39">
+        <v>-4.0687991715432914E-3</v>
+      </c>
+      <c r="AC39">
+        <v>-5.794035150385568E-3</v>
+      </c>
+      <c r="AD39">
+        <v>-6.6953007989423718E-3</v>
+      </c>
+      <c r="AE39">
+        <v>-7.3121965165059422E-3</v>
+      </c>
+      <c r="AF39">
+        <v>-7.5066429091649178E-3</v>
+      </c>
+      <c r="AG39">
+        <v>-9.5085584934587741E-3</v>
+      </c>
+      <c r="AH39">
+        <v>-1.232613324818288E-2</v>
+      </c>
+      <c r="AI39">
+        <v>-1.2531470227604924E-2</v>
+      </c>
+      <c r="AJ39">
+        <v>-1.3704143286042192E-2</v>
+      </c>
+      <c r="AK39">
+        <v>-1.5057390376488178E-2</v>
+      </c>
+      <c r="AL39">
+        <v>-1.591650761959823E-2</v>
+      </c>
+      <c r="AM39">
+        <v>-1.5762112049275079E-2</v>
+      </c>
+      <c r="AN39">
+        <v>-1.6416548589963942E-2</v>
+      </c>
+      <c r="AO39">
+        <v>-1.7237017562276191E-2</v>
+      </c>
+      <c r="AP39">
+        <v>-1.7476612376172262E-2</v>
+      </c>
+      <c r="AQ39">
+        <v>-1.6906082336107853E-2</v>
+      </c>
+      <c r="AR39" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chocs mig lineaires et plots populations
</commit_message>
<xml_diff>
--- a/all_shocks.xlsx
+++ b/all_shocks.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\emanu\OneDrive\Matlab\cdc_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{805979DB-7382-40C6-8002-035900C8F5AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BB2108-14DA-4585-ABA7-5B6A58511693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_pop_shocks_norm2000" sheetId="1" r:id="rId1"/>
     <sheet name="1_popshocks_values" sheetId="3" r:id="rId2"/>
     <sheet name="2_mig_shocks_vieux" sheetId="2" r:id="rId3"/>
     <sheet name="2_mig_shocks_renorm" sheetId="4" r:id="rId4"/>
+    <sheet name="3_med_chocs_probsurvie" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="158">
   <si>
     <t>=</t>
   </si>
@@ -401,12 +402,123 @@
   <si>
     <t>ppxpop</t>
   </si>
+  <si>
+    <t>survie qualifiés</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_1</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_2</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_3</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_4</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_5</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_6</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_7</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_8</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_9</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_10</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_11</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_12</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_13</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_14</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_15</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_16</t>
+  </si>
+  <si>
+    <t>bbBeta_Q_17</t>
+  </si>
+  <si>
+    <t>survie non qualifié</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_1</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_2</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_3</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_4</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_5</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_6</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_7</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_8</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_9</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_10</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_11</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_12</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_13</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_14</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_15</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_16</t>
+  </si>
+  <si>
+    <t>bbBeta_NQ_17</t>
+  </si>
+  <si>
+    <t>Ces chocs resultent des estimations sur les données des survie differenciées par niveau de qualification, ils sont passés ensuie au modele CDC complet avec les dynamiques demo des cohortes pour estimer en une fois chocs de santé et migratoires</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -427,6 +539,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -464,11 +581,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -25391,4 +25509,4785 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5B09A02-0DEB-47E6-AE34-AB582248ED4B}">
+  <dimension ref="A1:AR41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AC3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AE3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AF3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AG3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AH3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AI3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AJ3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AL3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AO3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AQ3" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.97383889999999995</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0.97533270000000005</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.95860509999999999</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0.90224629999999995</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0.97860950000000002</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0.98015459999999999</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0.98305229999999999</v>
+      </c>
+      <c r="K5" s="2">
+        <v>0.98505259999999994</v>
+      </c>
+      <c r="L5" s="2">
+        <v>0.95130680000000001</v>
+      </c>
+      <c r="M5" s="2">
+        <v>0.98782460000000005</v>
+      </c>
+      <c r="N5" s="2">
+        <v>0.99469269999999999</v>
+      </c>
+      <c r="O5" s="2">
+        <v>0.99581240000000004</v>
+      </c>
+      <c r="P5" s="2">
+        <v>0.9961795</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>0.99620310000000001</v>
+      </c>
+      <c r="R5" s="2">
+        <v>0.99629380000000001</v>
+      </c>
+      <c r="S5" s="2">
+        <v>0.99642750000000002</v>
+      </c>
+      <c r="T5" s="2">
+        <v>0.99630879999999999</v>
+      </c>
+      <c r="U5" s="2">
+        <v>0.99661160000000004</v>
+      </c>
+      <c r="V5" s="2">
+        <v>0.99674059999999998</v>
+      </c>
+      <c r="W5" s="2">
+        <v>0.99726700000000001</v>
+      </c>
+      <c r="X5" s="2">
+        <v>0.99814440000000004</v>
+      </c>
+      <c r="Y5" s="2">
+        <v>0.99843649999999995</v>
+      </c>
+      <c r="Z5" s="2">
+        <v>0.99866929999999998</v>
+      </c>
+      <c r="AA5" s="2">
+        <v>0.99882539999999997</v>
+      </c>
+      <c r="AB5" s="2">
+        <v>0.99892979999999998</v>
+      </c>
+      <c r="AC5" s="2">
+        <v>0.99903050000000004</v>
+      </c>
+      <c r="AD5" s="2">
+        <v>0.99911519999999998</v>
+      </c>
+      <c r="AE5" s="2">
+        <v>0.99919210000000003</v>
+      </c>
+      <c r="AF5" s="2">
+        <v>0.99926219999999999</v>
+      </c>
+      <c r="AG5" s="2">
+        <v>0.99932589999999999</v>
+      </c>
+      <c r="AH5" s="2">
+        <v>0.99938389999999999</v>
+      </c>
+      <c r="AI5" s="2">
+        <v>0.99943669999999996</v>
+      </c>
+      <c r="AJ5" s="2">
+        <v>0.99948479999999995</v>
+      </c>
+      <c r="AK5" s="2">
+        <v>0.99952870000000005</v>
+      </c>
+      <c r="AL5" s="2">
+        <v>0.99956860000000003</v>
+      </c>
+      <c r="AM5" s="2">
+        <v>0.99960510000000002</v>
+      </c>
+      <c r="AN5" s="2">
+        <v>0.99963829999999998</v>
+      </c>
+      <c r="AO5" s="2">
+        <v>0.99966849999999996</v>
+      </c>
+      <c r="AP5" s="2">
+        <v>0.99969620000000003</v>
+      </c>
+      <c r="AQ5" s="2">
+        <v>0.99972150000000004</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0.97343639999999998</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0.97425090000000003</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.96091910000000003</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0.91578079999999995</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0.97831590000000002</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0.98009299999999999</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0.98247119999999999</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0.98407690000000003</v>
+      </c>
+      <c r="L6" s="2">
+        <v>0.96266830000000003</v>
+      </c>
+      <c r="M6" s="2">
+        <v>0.98642669999999999</v>
+      </c>
+      <c r="N6" s="2">
+        <v>0.99359109999999995</v>
+      </c>
+      <c r="O6" s="2">
+        <v>0.99479470000000003</v>
+      </c>
+      <c r="P6" s="2">
+        <v>0.99543669999999995</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>0.99575480000000005</v>
+      </c>
+      <c r="R6" s="2">
+        <v>0.99594380000000005</v>
+      </c>
+      <c r="S6" s="2">
+        <v>0.99636789999999997</v>
+      </c>
+      <c r="T6" s="2">
+        <v>0.99632580000000004</v>
+      </c>
+      <c r="U6" s="2">
+        <v>0.99638289999999996</v>
+      </c>
+      <c r="V6" s="2">
+        <v>0.9961122</v>
+      </c>
+      <c r="W6" s="2">
+        <v>0.9968669</v>
+      </c>
+      <c r="X6" s="2">
+        <v>0.99794729999999998</v>
+      </c>
+      <c r="Y6" s="2">
+        <v>0.99828079999999997</v>
+      </c>
+      <c r="Z6" s="2">
+        <v>0.99843769999999998</v>
+      </c>
+      <c r="AA6" s="2">
+        <v>0.99856789999999995</v>
+      </c>
+      <c r="AB6" s="2">
+        <v>0.99863279999999999</v>
+      </c>
+      <c r="AC6" s="2">
+        <v>0.99874680000000005</v>
+      </c>
+      <c r="AD6" s="2">
+        <v>0.99885550000000001</v>
+      </c>
+      <c r="AE6" s="2">
+        <v>0.99895440000000002</v>
+      </c>
+      <c r="AF6" s="2">
+        <v>0.99904440000000005</v>
+      </c>
+      <c r="AG6" s="2">
+        <v>0.99912639999999997</v>
+      </c>
+      <c r="AH6" s="2">
+        <v>0.99920109999999995</v>
+      </c>
+      <c r="AI6" s="2">
+        <v>0.99926910000000002</v>
+      </c>
+      <c r="AJ6" s="2">
+        <v>0.99933110000000003</v>
+      </c>
+      <c r="AK6" s="2">
+        <v>0.99938760000000004</v>
+      </c>
+      <c r="AL6" s="2">
+        <v>0.99943910000000002</v>
+      </c>
+      <c r="AM6" s="2">
+        <v>0.99948610000000004</v>
+      </c>
+      <c r="AN6" s="2">
+        <v>0.99952909999999995</v>
+      </c>
+      <c r="AO6" s="2">
+        <v>0.99956820000000002</v>
+      </c>
+      <c r="AP6" s="2">
+        <v>0.99960389999999999</v>
+      </c>
+      <c r="AQ6" s="2">
+        <v>0.99963650000000004</v>
+      </c>
+      <c r="AR6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0.97053900000000004</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0.97105070000000004</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0.96356050000000004</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0.92695070000000002</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.97682440000000004</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0.97818369999999999</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0.98019100000000003</v>
+      </c>
+      <c r="K7" s="2">
+        <v>0.98134969999999999</v>
+      </c>
+      <c r="L7" s="2">
+        <v>0.96961470000000005</v>
+      </c>
+      <c r="M7" s="2">
+        <v>0.98747320000000005</v>
+      </c>
+      <c r="N7" s="2">
+        <v>0.9916587</v>
+      </c>
+      <c r="O7" s="2">
+        <v>0.99315129999999996</v>
+      </c>
+      <c r="P7" s="2">
+        <v>0.99385820000000002</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>0.99417129999999998</v>
+      </c>
+      <c r="R7" s="2">
+        <v>0.99463840000000003</v>
+      </c>
+      <c r="S7" s="2">
+        <v>0.9951913</v>
+      </c>
+      <c r="T7" s="2">
+        <v>0.99534860000000003</v>
+      </c>
+      <c r="U7" s="2">
+        <v>0.9954054</v>
+      </c>
+      <c r="V7" s="2">
+        <v>0.99519840000000004</v>
+      </c>
+      <c r="W7" s="2">
+        <v>0.99592309999999995</v>
+      </c>
+      <c r="X7" s="2">
+        <v>0.99728969999999995</v>
+      </c>
+      <c r="Y7" s="2">
+        <v>0.9977317</v>
+      </c>
+      <c r="Z7" s="2">
+        <v>0.99804369999999998</v>
+      </c>
+      <c r="AA7" s="2">
+        <v>0.99812190000000001</v>
+      </c>
+      <c r="AB7" s="2">
+        <v>0.99819749999999996</v>
+      </c>
+      <c r="AC7" s="2">
+        <v>0.99835910000000005</v>
+      </c>
+      <c r="AD7" s="2">
+        <v>0.99850000000000005</v>
+      </c>
+      <c r="AE7" s="2">
+        <v>0.99862839999999997</v>
+      </c>
+      <c r="AF7" s="2">
+        <v>0.99874529999999995</v>
+      </c>
+      <c r="AG7" s="2">
+        <v>0.99885190000000001</v>
+      </c>
+      <c r="AH7" s="2">
+        <v>0.99894899999999998</v>
+      </c>
+      <c r="AI7" s="2">
+        <v>0.99903759999999997</v>
+      </c>
+      <c r="AJ7" s="2">
+        <v>0.99911830000000001</v>
+      </c>
+      <c r="AK7" s="2">
+        <v>0.99919199999999997</v>
+      </c>
+      <c r="AL7" s="2">
+        <v>0.99925920000000001</v>
+      </c>
+      <c r="AM7" s="2">
+        <v>0.9993206</v>
+      </c>
+      <c r="AN7" s="2">
+        <v>0.99937670000000001</v>
+      </c>
+      <c r="AO7" s="2">
+        <v>0.99942790000000004</v>
+      </c>
+      <c r="AP7" s="2">
+        <v>0.99947459999999999</v>
+      </c>
+      <c r="AQ7" s="2">
+        <v>0.9995174</v>
+      </c>
+      <c r="AR7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0.96574420000000005</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0.96649779999999996</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.96407659999999995</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0.94629810000000003</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0.97275610000000001</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0.97344330000000001</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0.9754678</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0.97619579999999995</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0.96879029999999999</v>
+      </c>
+      <c r="M8" s="2">
+        <v>0.98469459999999998</v>
+      </c>
+      <c r="N8" s="2">
+        <v>0.98841199999999996</v>
+      </c>
+      <c r="O8" s="2">
+        <v>0.9900407</v>
+      </c>
+      <c r="P8" s="2">
+        <v>0.99089799999999995</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>0.99097650000000004</v>
+      </c>
+      <c r="R8" s="2">
+        <v>0.99146900000000004</v>
+      </c>
+      <c r="S8" s="2">
+        <v>0.99237909999999996</v>
+      </c>
+      <c r="T8" s="2">
+        <v>0.99299009999999999</v>
+      </c>
+      <c r="U8" s="2">
+        <v>0.9933805</v>
+      </c>
+      <c r="V8" s="2">
+        <v>0.99341699999999999</v>
+      </c>
+      <c r="W8" s="2">
+        <v>0.99402040000000003</v>
+      </c>
+      <c r="X8" s="2">
+        <v>0.99569470000000004</v>
+      </c>
+      <c r="Y8" s="2">
+        <v>0.99637529999999996</v>
+      </c>
+      <c r="Z8" s="2">
+        <v>0.99685469999999998</v>
+      </c>
+      <c r="AA8" s="2">
+        <v>0.99717630000000002</v>
+      </c>
+      <c r="AB8" s="2">
+        <v>0.99733459999999996</v>
+      </c>
+      <c r="AC8" s="2">
+        <v>0.99755530000000003</v>
+      </c>
+      <c r="AD8" s="2">
+        <v>0.99776069999999994</v>
+      </c>
+      <c r="AE8" s="2">
+        <v>0.9979481</v>
+      </c>
+      <c r="AF8" s="2">
+        <v>0.99811910000000004</v>
+      </c>
+      <c r="AG8" s="2">
+        <v>0.99827520000000003</v>
+      </c>
+      <c r="AH8" s="2">
+        <v>0.99841769999999996</v>
+      </c>
+      <c r="AI8" s="2">
+        <v>0.99854790000000004</v>
+      </c>
+      <c r="AJ8" s="2">
+        <v>0.99866679999999997</v>
+      </c>
+      <c r="AK8" s="2">
+        <v>0.99877550000000004</v>
+      </c>
+      <c r="AL8" s="2">
+        <v>0.99887499999999996</v>
+      </c>
+      <c r="AM8" s="2">
+        <v>0.99896589999999996</v>
+      </c>
+      <c r="AN8" s="2">
+        <v>0.99904910000000002</v>
+      </c>
+      <c r="AO8" s="2">
+        <v>0.99912529999999999</v>
+      </c>
+      <c r="AP8" s="2">
+        <v>0.99919500000000006</v>
+      </c>
+      <c r="AQ8" s="2">
+        <v>0.99925889999999995</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0.96117629999999998</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0.96060350000000005</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.96242490000000003</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0.95472650000000003</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0.96847419999999995</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0.96810010000000002</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0.96992120000000004</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0.97050479999999995</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0.96484800000000004</v>
+      </c>
+      <c r="M9" s="2">
+        <v>0.98031299999999999</v>
+      </c>
+      <c r="N9" s="2">
+        <v>0.98309530000000001</v>
+      </c>
+      <c r="O9" s="2">
+        <v>0.98540680000000003</v>
+      </c>
+      <c r="P9" s="2">
+        <v>0.98666690000000001</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>0.98663990000000001</v>
+      </c>
+      <c r="R9" s="2">
+        <v>0.9869829</v>
+      </c>
+      <c r="S9" s="2">
+        <v>0.9876355</v>
+      </c>
+      <c r="T9" s="2">
+        <v>0.98917449999999996</v>
+      </c>
+      <c r="U9" s="2">
+        <v>0.99008470000000004</v>
+      </c>
+      <c r="V9" s="2">
+        <v>0.99083149999999998</v>
+      </c>
+      <c r="W9" s="2">
+        <v>0.99107719999999999</v>
+      </c>
+      <c r="X9" s="2">
+        <v>0.99267519999999998</v>
+      </c>
+      <c r="Y9" s="2">
+        <v>0.99389340000000004</v>
+      </c>
+      <c r="Z9" s="2">
+        <v>0.99477990000000005</v>
+      </c>
+      <c r="AA9" s="2">
+        <v>0.9953303</v>
+      </c>
+      <c r="AB9" s="2">
+        <v>0.99574220000000002</v>
+      </c>
+      <c r="AC9" s="2">
+        <v>0.9961506</v>
+      </c>
+      <c r="AD9" s="2">
+        <v>0.99647149999999995</v>
+      </c>
+      <c r="AE9" s="2">
+        <v>0.99676450000000005</v>
+      </c>
+      <c r="AF9" s="2">
+        <v>0.99703200000000003</v>
+      </c>
+      <c r="AG9" s="2">
+        <v>0.99727639999999995</v>
+      </c>
+      <c r="AH9" s="2">
+        <v>0.99749960000000004</v>
+      </c>
+      <c r="AI9" s="2">
+        <v>0.99770360000000002</v>
+      </c>
+      <c r="AJ9" s="2">
+        <v>0.99789019999999995</v>
+      </c>
+      <c r="AK9" s="2">
+        <v>0.99806090000000003</v>
+      </c>
+      <c r="AL9" s="2">
+        <v>0.99821700000000002</v>
+      </c>
+      <c r="AM9" s="2">
+        <v>0.99835989999999997</v>
+      </c>
+      <c r="AN9" s="2">
+        <v>0.99849069999999995</v>
+      </c>
+      <c r="AO9" s="2">
+        <v>0.99861060000000001</v>
+      </c>
+      <c r="AP9" s="2">
+        <v>0.99872050000000001</v>
+      </c>
+      <c r="AQ9" s="2">
+        <v>0.99882110000000002</v>
+      </c>
+      <c r="AR9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0.95511630000000003</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0.95342879999999997</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.95630590000000004</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0.95289559999999995</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0.96129980000000004</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0.96072880000000005</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0.96205390000000002</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0.96215930000000005</v>
+      </c>
+      <c r="L10" s="2">
+        <v>0.95902030000000005</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0.97328559999999997</v>
+      </c>
+      <c r="N10" s="2">
+        <v>0.9750588</v>
+      </c>
+      <c r="O10" s="2">
+        <v>0.9778886</v>
+      </c>
+      <c r="P10" s="2">
+        <v>0.98006789999999999</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>0.98020090000000004</v>
+      </c>
+      <c r="R10" s="2">
+        <v>0.98119339999999999</v>
+      </c>
+      <c r="S10" s="2">
+        <v>0.98141900000000004</v>
+      </c>
+      <c r="T10" s="2">
+        <v>0.98306159999999998</v>
+      </c>
+      <c r="U10" s="2">
+        <v>0.98519089999999998</v>
+      </c>
+      <c r="V10" s="2">
+        <v>0.98709029999999998</v>
+      </c>
+      <c r="W10" s="2">
+        <v>0.98760079999999995</v>
+      </c>
+      <c r="X10" s="2">
+        <v>0.98826309999999995</v>
+      </c>
+      <c r="Y10" s="2">
+        <v>0.98947249999999998</v>
+      </c>
+      <c r="Z10" s="2">
+        <v>0.99102900000000005</v>
+      </c>
+      <c r="AA10" s="2">
+        <v>0.99200140000000003</v>
+      </c>
+      <c r="AB10" s="2">
+        <v>0.99259280000000005</v>
+      </c>
+      <c r="AC10" s="2">
+        <v>0.99329089999999998</v>
+      </c>
+      <c r="AD10" s="2">
+        <v>0.99384790000000001</v>
+      </c>
+      <c r="AE10" s="2">
+        <v>0.99435649999999998</v>
+      </c>
+      <c r="AF10" s="2">
+        <v>0.99482099999999996</v>
+      </c>
+      <c r="AG10" s="2">
+        <v>0.99524539999999995</v>
+      </c>
+      <c r="AH10" s="2">
+        <v>0.9956334</v>
+      </c>
+      <c r="AI10" s="2">
+        <v>0.99598810000000004</v>
+      </c>
+      <c r="AJ10" s="2">
+        <v>0.99631250000000005</v>
+      </c>
+      <c r="AK10" s="2">
+        <v>0.99660939999999998</v>
+      </c>
+      <c r="AL10" s="2">
+        <v>0.99688109999999996</v>
+      </c>
+      <c r="AM10" s="2">
+        <v>0.99712990000000001</v>
+      </c>
+      <c r="AN10" s="2">
+        <v>0.99735779999999996</v>
+      </c>
+      <c r="AO10" s="2">
+        <v>0.99756670000000003</v>
+      </c>
+      <c r="AP10" s="2">
+        <v>0.99775820000000004</v>
+      </c>
+      <c r="AQ10" s="2">
+        <v>0.99793370000000003</v>
+      </c>
+      <c r="AR10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2">
+        <v>0.94018400000000002</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0.93899089999999996</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.94209860000000001</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0.94032649999999995</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0.94725669999999995</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0.94710119999999998</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0.94870500000000002</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0.94881530000000003</v>
+      </c>
+      <c r="L11" s="2">
+        <v>0.94603199999999998</v>
+      </c>
+      <c r="M11" s="2">
+        <v>0.96205949999999996</v>
+      </c>
+      <c r="N11" s="2">
+        <v>0.96273640000000005</v>
+      </c>
+      <c r="O11" s="2">
+        <v>0.96588859999999999</v>
+      </c>
+      <c r="P11" s="2">
+        <v>0.96851580000000004</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>0.9700474</v>
+      </c>
+      <c r="R11" s="2">
+        <v>0.97154649999999998</v>
+      </c>
+      <c r="S11" s="2">
+        <v>0.97284789999999999</v>
+      </c>
+      <c r="T11" s="2">
+        <v>0.97437240000000003</v>
+      </c>
+      <c r="U11" s="2">
+        <v>0.97684139999999997</v>
+      </c>
+      <c r="V11" s="2">
+        <v>0.98076870000000005</v>
+      </c>
+      <c r="W11" s="2">
+        <v>0.98225019999999996</v>
+      </c>
+      <c r="X11" s="2">
+        <v>0.98303529999999995</v>
+      </c>
+      <c r="Y11" s="2">
+        <v>0.98374170000000005</v>
+      </c>
+      <c r="Z11" s="2">
+        <v>0.9851761</v>
+      </c>
+      <c r="AA11" s="2">
+        <v>0.98697290000000004</v>
+      </c>
+      <c r="AB11" s="2">
+        <v>0.9879966</v>
+      </c>
+      <c r="AC11" s="2">
+        <v>0.98911150000000003</v>
+      </c>
+      <c r="AD11" s="2">
+        <v>0.99001939999999999</v>
+      </c>
+      <c r="AE11" s="2">
+        <v>0.99084819999999996</v>
+      </c>
+      <c r="AF11" s="2">
+        <v>0.99160510000000002</v>
+      </c>
+      <c r="AG11" s="2">
+        <v>0.99229630000000002</v>
+      </c>
+      <c r="AH11" s="2">
+        <v>0.99292800000000003</v>
+      </c>
+      <c r="AI11" s="2">
+        <v>0.99350539999999998</v>
+      </c>
+      <c r="AJ11" s="2">
+        <v>0.99403319999999995</v>
+      </c>
+      <c r="AK11" s="2">
+        <v>0.99451610000000001</v>
+      </c>
+      <c r="AL11" s="2">
+        <v>0.9949578</v>
+      </c>
+      <c r="AM11" s="2">
+        <v>0.99536219999999997</v>
+      </c>
+      <c r="AN11" s="2">
+        <v>0.99573250000000002</v>
+      </c>
+      <c r="AO11" s="2">
+        <v>0.99607159999999995</v>
+      </c>
+      <c r="AP11" s="2">
+        <v>0.9963824</v>
+      </c>
+      <c r="AQ11" s="2">
+        <v>0.99666710000000003</v>
+      </c>
+      <c r="AR11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0.90949919999999995</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0.90736419999999995</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.91294059999999999</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0.91171190000000002</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0.91889969999999999</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.91866890000000001</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0.92155520000000002</v>
+      </c>
+      <c r="K12" s="2">
+        <v>0.92165059999999999</v>
+      </c>
+      <c r="L12" s="2">
+        <v>0.91794399999999998</v>
+      </c>
+      <c r="M12" s="2">
+        <v>0.93921209999999999</v>
+      </c>
+      <c r="N12" s="2">
+        <v>0.94115110000000002</v>
+      </c>
+      <c r="O12" s="2">
+        <v>0.94451490000000005</v>
+      </c>
+      <c r="P12" s="2">
+        <v>0.947322</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>0.94900770000000001</v>
+      </c>
+      <c r="R12" s="2">
+        <v>0.95414049999999995</v>
+      </c>
+      <c r="S12" s="2">
+        <v>0.95687599999999995</v>
+      </c>
+      <c r="T12" s="2">
+        <v>0.96018720000000002</v>
+      </c>
+      <c r="U12" s="2">
+        <v>0.96305419999999997</v>
+      </c>
+      <c r="V12" s="2">
+        <v>0.96872630000000004</v>
+      </c>
+      <c r="W12" s="2">
+        <v>0.97185429999999995</v>
+      </c>
+      <c r="X12" s="2">
+        <v>0.97570999999999997</v>
+      </c>
+      <c r="Y12" s="2">
+        <v>0.97708740000000005</v>
+      </c>
+      <c r="Z12" s="2">
+        <v>0.97780250000000002</v>
+      </c>
+      <c r="AA12" s="2">
+        <v>0.97911700000000002</v>
+      </c>
+      <c r="AB12" s="2">
+        <v>0.98088189999999997</v>
+      </c>
+      <c r="AC12" s="2">
+        <v>0.98274950000000005</v>
+      </c>
+      <c r="AD12" s="2">
+        <v>0.9841953</v>
+      </c>
+      <c r="AE12" s="2">
+        <v>0.98551469999999997</v>
+      </c>
+      <c r="AF12" s="2">
+        <v>0.98671909999999996</v>
+      </c>
+      <c r="AG12" s="2">
+        <v>0.98781890000000006</v>
+      </c>
+      <c r="AH12" s="2">
+        <v>0.98882340000000002</v>
+      </c>
+      <c r="AI12" s="2">
+        <v>0.98974119999999999</v>
+      </c>
+      <c r="AJ12" s="2">
+        <v>0.99058000000000002</v>
+      </c>
+      <c r="AK12" s="2">
+        <v>0.99134699999999998</v>
+      </c>
+      <c r="AL12" s="2">
+        <v>0.99204840000000005</v>
+      </c>
+      <c r="AM12" s="2">
+        <v>0.99269010000000002</v>
+      </c>
+      <c r="AN12" s="2">
+        <v>0.99327739999999998</v>
+      </c>
+      <c r="AO12" s="2">
+        <v>0.99381509999999995</v>
+      </c>
+      <c r="AP12" s="2">
+        <v>0.99430750000000001</v>
+      </c>
+      <c r="AQ12" s="2">
+        <v>0.9947587</v>
+      </c>
+      <c r="AR12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0.85988770000000003</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0.85550530000000002</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.86534849999999996</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0.86358210000000002</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0.87503909999999996</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0.87365360000000003</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0.87952410000000003</v>
+      </c>
+      <c r="K13" s="2">
+        <v>0.88041369999999997</v>
+      </c>
+      <c r="L13" s="2">
+        <v>0.87315889999999996</v>
+      </c>
+      <c r="M13" s="2">
+        <v>0.90284319999999996</v>
+      </c>
+      <c r="N13" s="2">
+        <v>0.90714779999999995</v>
+      </c>
+      <c r="O13" s="2">
+        <v>0.91269610000000001</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0.91607349999999999</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>0.91748149999999995</v>
+      </c>
+      <c r="R13" s="2">
+        <v>0.9248459</v>
+      </c>
+      <c r="S13" s="2">
+        <v>0.93206089999999997</v>
+      </c>
+      <c r="T13" s="2">
+        <v>0.9383416</v>
+      </c>
+      <c r="U13" s="2">
+        <v>0.94414439999999999</v>
+      </c>
+      <c r="V13" s="2">
+        <v>0.95133500000000004</v>
+      </c>
+      <c r="W13" s="2">
+        <v>0.95534819999999998</v>
+      </c>
+      <c r="X13" s="2">
+        <v>0.96306740000000002</v>
+      </c>
+      <c r="Y13" s="2">
+        <v>0.96648820000000002</v>
+      </c>
+      <c r="Z13" s="2">
+        <v>0.96811650000000005</v>
+      </c>
+      <c r="AA13" s="2">
+        <v>0.96827589999999997</v>
+      </c>
+      <c r="AB13" s="2">
+        <v>0.96982559999999995</v>
+      </c>
+      <c r="AC13" s="2">
+        <v>0.97294130000000001</v>
+      </c>
+      <c r="AD13" s="2">
+        <v>0.97522629999999999</v>
+      </c>
+      <c r="AE13" s="2">
+        <v>0.97731100000000004</v>
+      </c>
+      <c r="AF13" s="2">
+        <v>0.97921340000000001</v>
+      </c>
+      <c r="AG13" s="2">
+        <v>0.98094979999999998</v>
+      </c>
+      <c r="AH13" s="2">
+        <v>0.98253520000000005</v>
+      </c>
+      <c r="AI13" s="2">
+        <v>0.98398289999999999</v>
+      </c>
+      <c r="AJ13" s="2">
+        <v>0.9853054</v>
+      </c>
+      <c r="AK13" s="2">
+        <v>0.98651390000000005</v>
+      </c>
+      <c r="AL13" s="2">
+        <v>0.98761829999999995</v>
+      </c>
+      <c r="AM13" s="2">
+        <v>0.98862799999999995</v>
+      </c>
+      <c r="AN13" s="2">
+        <v>0.98955150000000003</v>
+      </c>
+      <c r="AO13" s="2">
+        <v>0.99039630000000001</v>
+      </c>
+      <c r="AP13" s="2">
+        <v>0.99116950000000004</v>
+      </c>
+      <c r="AQ13" s="2">
+        <v>0.99187720000000001</v>
+      </c>
+      <c r="AR13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0.78175380000000005</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0.77719050000000001</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0.78592839999999997</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0.78246020000000005</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0.80298449999999999</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0.80030610000000002</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0.80958169999999996</v>
+      </c>
+      <c r="K14" s="2">
+        <v>0.81160739999999998</v>
+      </c>
+      <c r="L14" s="2">
+        <v>0.79922459999999995</v>
+      </c>
+      <c r="M14" s="2">
+        <v>0.84030009999999999</v>
+      </c>
+      <c r="N14" s="2">
+        <v>0.84810759999999996</v>
+      </c>
+      <c r="O14" s="2">
+        <v>0.85859640000000004</v>
+      </c>
+      <c r="P14" s="2">
+        <v>0.86597880000000005</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>0.86633559999999998</v>
+      </c>
+      <c r="R14" s="2">
+        <v>0.8764651</v>
+      </c>
+      <c r="S14" s="2">
+        <v>0.88821470000000002</v>
+      </c>
+      <c r="T14" s="2">
+        <v>0.90101149999999997</v>
+      </c>
+      <c r="U14" s="2">
+        <v>0.91106710000000002</v>
+      </c>
+      <c r="V14" s="2">
+        <v>0.92433659999999995</v>
+      </c>
+      <c r="W14" s="2">
+        <v>0.9282437</v>
+      </c>
+      <c r="X14" s="2">
+        <v>0.94212439999999997</v>
+      </c>
+      <c r="Y14" s="2">
+        <v>0.95022359999999995</v>
+      </c>
+      <c r="Z14" s="2">
+        <v>0.95418510000000001</v>
+      </c>
+      <c r="AA14" s="2">
+        <v>0.95526339999999998</v>
+      </c>
+      <c r="AB14" s="2">
+        <v>0.95512160000000002</v>
+      </c>
+      <c r="AC14" s="2">
+        <v>0.95866189999999996</v>
+      </c>
+      <c r="AD14" s="2">
+        <v>0.96211930000000001</v>
+      </c>
+      <c r="AE14" s="2">
+        <v>0.96529880000000001</v>
+      </c>
+      <c r="AF14" s="2">
+        <v>0.96820220000000001</v>
+      </c>
+      <c r="AG14" s="2">
+        <v>0.97085359999999998</v>
+      </c>
+      <c r="AH14" s="2">
+        <v>0.97327549999999996</v>
+      </c>
+      <c r="AI14" s="2">
+        <v>0.97548809999999997</v>
+      </c>
+      <c r="AJ14" s="2">
+        <v>0.97750999999999999</v>
+      </c>
+      <c r="AK14" s="2">
+        <v>0.97935799999999995</v>
+      </c>
+      <c r="AL14" s="2">
+        <v>0.98104740000000001</v>
+      </c>
+      <c r="AM14" s="2">
+        <v>0.98259240000000003</v>
+      </c>
+      <c r="AN14" s="2">
+        <v>0.98400560000000004</v>
+      </c>
+      <c r="AO14" s="2">
+        <v>0.98529860000000002</v>
+      </c>
+      <c r="AP14" s="2">
+        <v>0.98648210000000003</v>
+      </c>
+      <c r="AQ14" s="2">
+        <v>0.98756560000000004</v>
+      </c>
+      <c r="AR14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" t="s">
+        <v>0</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0.65832939999999995</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0.65322970000000002</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0.66729470000000002</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0.66172949999999997</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0.68893199999999999</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0.68512280000000003</v>
+      </c>
+      <c r="J15" s="2">
+        <v>0.70182250000000002</v>
+      </c>
+      <c r="K15" s="2">
+        <v>0.70557150000000002</v>
+      </c>
+      <c r="L15" s="2">
+        <v>0.68410870000000001</v>
+      </c>
+      <c r="M15" s="2">
+        <v>0.74251560000000005</v>
+      </c>
+      <c r="N15" s="2">
+        <v>0.75022100000000003</v>
+      </c>
+      <c r="O15" s="2">
+        <v>0.7675054</v>
+      </c>
+      <c r="P15" s="2">
+        <v>0.7819815</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>0.78842420000000002</v>
+      </c>
+      <c r="R15" s="2">
+        <v>0.79946669999999997</v>
+      </c>
+      <c r="S15" s="2">
+        <v>0.81449629999999995</v>
+      </c>
+      <c r="T15" s="2">
+        <v>0.83255579999999996</v>
+      </c>
+      <c r="U15" s="2">
+        <v>0.8531569</v>
+      </c>
+      <c r="V15" s="2">
+        <v>0.87701379999999995</v>
+      </c>
+      <c r="W15" s="2">
+        <v>0.88493569999999999</v>
+      </c>
+      <c r="X15" s="2">
+        <v>0.90277320000000005</v>
+      </c>
+      <c r="Y15" s="2">
+        <v>0.91674250000000002</v>
+      </c>
+      <c r="Z15" s="2">
+        <v>0.92673430000000001</v>
+      </c>
+      <c r="AA15" s="2">
+        <v>0.93017130000000003</v>
+      </c>
+      <c r="AB15" s="2">
+        <v>0.93030230000000003</v>
+      </c>
+      <c r="AC15" s="2">
+        <v>0.93383709999999998</v>
+      </c>
+      <c r="AD15" s="2">
+        <v>0.93756790000000001</v>
+      </c>
+      <c r="AE15" s="2">
+        <v>0.94270189999999998</v>
+      </c>
+      <c r="AF15" s="2">
+        <v>0.94743480000000002</v>
+      </c>
+      <c r="AG15" s="2">
+        <v>0.95176510000000003</v>
+      </c>
+      <c r="AH15" s="2">
+        <v>0.9557272</v>
+      </c>
+      <c r="AI15" s="2">
+        <v>0.9593526</v>
+      </c>
+      <c r="AJ15" s="2">
+        <v>0.96267029999999998</v>
+      </c>
+      <c r="AK15" s="2">
+        <v>0.96570679999999998</v>
+      </c>
+      <c r="AL15" s="2">
+        <v>0.96848619999999996</v>
+      </c>
+      <c r="AM15" s="2">
+        <v>0.97103110000000004</v>
+      </c>
+      <c r="AN15" s="2">
+        <v>0.97336140000000004</v>
+      </c>
+      <c r="AO15" s="2">
+        <v>0.97549609999999998</v>
+      </c>
+      <c r="AP15" s="2">
+        <v>0.97745170000000003</v>
+      </c>
+      <c r="AQ15" s="2">
+        <v>0.97924389999999994</v>
+      </c>
+      <c r="AR15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" t="s">
+        <v>0</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0.51280899999999996</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0.50715149999999998</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.52165870000000003</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0.51307499999999995</v>
+      </c>
+      <c r="H16" s="2">
+        <v>0.54590559999999999</v>
+      </c>
+      <c r="I16" s="2">
+        <v>0.53332650000000004</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0.56400450000000002</v>
+      </c>
+      <c r="K16" s="2">
+        <v>0.56743200000000005</v>
+      </c>
+      <c r="L16" s="2">
+        <v>0.52429680000000001</v>
+      </c>
+      <c r="M16" s="2">
+        <v>0.60505549999999997</v>
+      </c>
+      <c r="N16" s="2">
+        <v>0.61620459999999999</v>
+      </c>
+      <c r="O16" s="2">
+        <v>0.63815520000000003</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0.65645659999999995</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>0.67202989999999996</v>
+      </c>
+      <c r="R16" s="2">
+        <v>0.68807799999999997</v>
+      </c>
+      <c r="S16" s="2">
+        <v>0.7052718</v>
+      </c>
+      <c r="T16" s="2">
+        <v>0.72555700000000001</v>
+      </c>
+      <c r="U16" s="2">
+        <v>0.75388840000000001</v>
+      </c>
+      <c r="V16" s="2">
+        <v>0.79734269999999996</v>
+      </c>
+      <c r="W16" s="2">
+        <v>0.8110406</v>
+      </c>
+      <c r="X16" s="2">
+        <v>0.83872000000000002</v>
+      </c>
+      <c r="Y16" s="2">
+        <v>0.85856710000000003</v>
+      </c>
+      <c r="Z16" s="2">
+        <v>0.87571390000000005</v>
+      </c>
+      <c r="AA16" s="2">
+        <v>0.88502559999999997</v>
+      </c>
+      <c r="AB16" s="2">
+        <v>0.88686100000000001</v>
+      </c>
+      <c r="AC16" s="2">
+        <v>0.89319999999999999</v>
+      </c>
+      <c r="AD16" s="2">
+        <v>0.8958564</v>
+      </c>
+      <c r="AE16" s="2">
+        <v>0.90168009999999998</v>
+      </c>
+      <c r="AF16" s="2">
+        <v>0.90986820000000002</v>
+      </c>
+      <c r="AG16" s="2">
+        <v>0.91742959999999996</v>
+      </c>
+      <c r="AH16" s="2">
+        <v>0.92435449999999997</v>
+      </c>
+      <c r="AI16" s="2">
+        <v>0.93069460000000004</v>
+      </c>
+      <c r="AJ16" s="2">
+        <v>0.93649850000000001</v>
+      </c>
+      <c r="AK16" s="2">
+        <v>0.94181040000000005</v>
+      </c>
+      <c r="AL16" s="2">
+        <v>0.94667190000000001</v>
+      </c>
+      <c r="AM16" s="2">
+        <v>0.95112070000000004</v>
+      </c>
+      <c r="AN16" s="2">
+        <v>0.95519189999999998</v>
+      </c>
+      <c r="AO16" s="2">
+        <v>0.95891749999999998</v>
+      </c>
+      <c r="AP16" s="2">
+        <v>0.96232689999999999</v>
+      </c>
+      <c r="AQ16" s="2">
+        <v>0.96544719999999995</v>
+      </c>
+      <c r="AR16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17" s="2">
+        <v>0.34479989999999999</v>
+      </c>
+      <c r="E17" s="2">
+        <v>0.34020689999999998</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0.35973440000000001</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0.3431148</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0.38222600000000001</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0.36424279999999998</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0.39876859999999997</v>
+      </c>
+      <c r="K17" s="2">
+        <v>0.40667799999999998</v>
+      </c>
+      <c r="L17" s="2">
+        <v>0.34946759999999999</v>
+      </c>
+      <c r="M17" s="2">
+        <v>0.44094070000000002</v>
+      </c>
+      <c r="N17" s="2">
+        <v>0.44702419999999998</v>
+      </c>
+      <c r="O17" s="2">
+        <v>0.47089540000000002</v>
+      </c>
+      <c r="P17" s="2">
+        <v>0.4895275</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>0.51173780000000002</v>
+      </c>
+      <c r="R17" s="2">
+        <v>0.53183000000000002</v>
+      </c>
+      <c r="S17" s="2">
+        <v>0.55343719999999996</v>
+      </c>
+      <c r="T17" s="2">
+        <v>0.57125610000000004</v>
+      </c>
+      <c r="U17" s="2">
+        <v>0.60395239999999994</v>
+      </c>
+      <c r="V17" s="2">
+        <v>0.66105959999999997</v>
+      </c>
+      <c r="W17" s="2">
+        <v>0.6828052</v>
+      </c>
+      <c r="X17" s="2">
+        <v>0.72124679999999997</v>
+      </c>
+      <c r="Y17" s="2">
+        <v>0.75218890000000005</v>
+      </c>
+      <c r="Z17" s="2">
+        <v>0.77375170000000004</v>
+      </c>
+      <c r="AA17" s="2">
+        <v>0.79037650000000004</v>
+      </c>
+      <c r="AB17" s="2">
+        <v>0.80134640000000001</v>
+      </c>
+      <c r="AC17" s="2">
+        <v>0.81794549999999999</v>
+      </c>
+      <c r="AD17" s="2">
+        <v>0.82234110000000005</v>
+      </c>
+      <c r="AE17" s="2">
+        <v>0.82653189999999999</v>
+      </c>
+      <c r="AF17" s="2">
+        <v>0.8356614</v>
+      </c>
+      <c r="AG17" s="2">
+        <v>0.84828619999999999</v>
+      </c>
+      <c r="AH17" s="2">
+        <v>0.86005489999999996</v>
+      </c>
+      <c r="AI17" s="2">
+        <v>0.87094090000000002</v>
+      </c>
+      <c r="AJ17" s="2">
+        <v>0.88100389999999995</v>
+      </c>
+      <c r="AK17" s="2">
+        <v>0.89030120000000001</v>
+      </c>
+      <c r="AL17" s="2">
+        <v>0.89888690000000004</v>
+      </c>
+      <c r="AM17" s="2">
+        <v>0.90681199999999995</v>
+      </c>
+      <c r="AN17" s="2">
+        <v>0.91412479999999996</v>
+      </c>
+      <c r="AO17" s="2">
+        <v>0.92087050000000004</v>
+      </c>
+      <c r="AP17" s="2">
+        <v>0.92709129999999995</v>
+      </c>
+      <c r="AQ17" s="2">
+        <v>0.93282679999999996</v>
+      </c>
+      <c r="AR17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0.21028369999999999</v>
+      </c>
+      <c r="E18" s="2">
+        <v>0.20295240000000001</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0.21602779999999999</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0.1991753</v>
+      </c>
+      <c r="H18" s="2">
+        <v>0.23347100000000001</v>
+      </c>
+      <c r="I18" s="2">
+        <v>0.21039240000000001</v>
+      </c>
+      <c r="J18" s="2">
+        <v>0.24479010000000001</v>
+      </c>
+      <c r="K18" s="2">
+        <v>0.2502199</v>
+      </c>
+      <c r="L18" s="2">
+        <v>0.19234850000000001</v>
+      </c>
+      <c r="M18" s="2">
+        <v>0.2773814</v>
+      </c>
+      <c r="N18" s="2">
+        <v>0.2790262</v>
+      </c>
+      <c r="O18" s="2">
+        <v>0.29735010000000001</v>
+      </c>
+      <c r="P18" s="2">
+        <v>0.3164344</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>0.33631349999999999</v>
+      </c>
+      <c r="R18" s="2">
+        <v>0.35768339999999998</v>
+      </c>
+      <c r="S18" s="2">
+        <v>0.37471130000000002</v>
+      </c>
+      <c r="T18" s="2">
+        <v>0.39159660000000002</v>
+      </c>
+      <c r="U18" s="2">
+        <v>0.42011929999999997</v>
+      </c>
+      <c r="V18" s="2">
+        <v>0.4813904</v>
+      </c>
+      <c r="W18" s="2">
+        <v>0.49814730000000002</v>
+      </c>
+      <c r="X18" s="2">
+        <v>0.54290430000000001</v>
+      </c>
+      <c r="Y18" s="2">
+        <v>0.57790580000000003</v>
+      </c>
+      <c r="Z18" s="2">
+        <v>0.60306349999999997</v>
+      </c>
+      <c r="AA18" s="2">
+        <v>0.61716320000000002</v>
+      </c>
+      <c r="AB18" s="2">
+        <v>0.63015160000000003</v>
+      </c>
+      <c r="AC18" s="2">
+        <v>0.65598140000000005</v>
+      </c>
+      <c r="AD18" s="2">
+        <v>0.6677303</v>
+      </c>
+      <c r="AE18" s="2">
+        <v>0.6746721</v>
+      </c>
+      <c r="AF18" s="2">
+        <v>0.68152199999999996</v>
+      </c>
+      <c r="AG18" s="2">
+        <v>0.69282290000000002</v>
+      </c>
+      <c r="AH18" s="2">
+        <v>0.706901</v>
+      </c>
+      <c r="AI18" s="2">
+        <v>0.72044799999999998</v>
+      </c>
+      <c r="AJ18" s="2">
+        <v>0.73342229999999997</v>
+      </c>
+      <c r="AK18" s="2">
+        <v>0.74584059999999996</v>
+      </c>
+      <c r="AL18" s="2">
+        <v>0.7577197</v>
+      </c>
+      <c r="AM18" s="2">
+        <v>0.76907709999999996</v>
+      </c>
+      <c r="AN18" s="2">
+        <v>0.77993049999999997</v>
+      </c>
+      <c r="AO18" s="2">
+        <v>0.79029769999999999</v>
+      </c>
+      <c r="AP18" s="2">
+        <v>0.80019680000000004</v>
+      </c>
+      <c r="AQ18" s="2">
+        <v>0.80964519999999995</v>
+      </c>
+      <c r="AR18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" t="s">
+        <v>0</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0.11865390000000001</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0.10412349999999999</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0.1175189</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0.10591250000000001</v>
+      </c>
+      <c r="H19" s="2">
+        <v>0.1223017</v>
+      </c>
+      <c r="I19" s="2">
+        <v>0.10710450000000001</v>
+      </c>
+      <c r="J19" s="2">
+        <v>0.13129469999999999</v>
+      </c>
+      <c r="K19" s="2">
+        <v>0.1314351</v>
+      </c>
+      <c r="L19" s="2">
+        <v>9.2467400000000005E-2</v>
+      </c>
+      <c r="M19" s="2">
+        <v>0.1552857</v>
+      </c>
+      <c r="N19" s="2">
+        <v>0.14928749999999999</v>
+      </c>
+      <c r="O19" s="2">
+        <v>0.16049079999999999</v>
+      </c>
+      <c r="P19" s="2">
+        <v>0.17640249999999999</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>0.19164239999999999</v>
+      </c>
+      <c r="R19" s="2">
+        <v>0.20360249999999999</v>
+      </c>
+      <c r="S19" s="2">
+        <v>0.21807480000000001</v>
+      </c>
+      <c r="T19" s="2">
+        <v>0.22670789999999999</v>
+      </c>
+      <c r="U19" s="2">
+        <v>0.2452638</v>
+      </c>
+      <c r="V19" s="2">
+        <v>0.2896553</v>
+      </c>
+      <c r="W19" s="2">
+        <v>0.31124030000000003</v>
+      </c>
+      <c r="X19" s="2">
+        <v>0.33848159999999999</v>
+      </c>
+      <c r="Y19" s="2">
+        <v>0.36539430000000001</v>
+      </c>
+      <c r="Z19" s="2">
+        <v>0.38354189999999999</v>
+      </c>
+      <c r="AA19" s="2">
+        <v>0.39121889999999998</v>
+      </c>
+      <c r="AB19" s="2">
+        <v>0.4013195</v>
+      </c>
+      <c r="AC19" s="2">
+        <v>0.42545529999999998</v>
+      </c>
+      <c r="AD19" s="2">
+        <v>0.43844889999999997</v>
+      </c>
+      <c r="AE19" s="2">
+        <v>0.44924229999999998</v>
+      </c>
+      <c r="AF19" s="2">
+        <v>0.45718890000000001</v>
+      </c>
+      <c r="AG19" s="2">
+        <v>0.4650649</v>
+      </c>
+      <c r="AH19" s="2">
+        <v>0.4755431</v>
+      </c>
+      <c r="AI19" s="2">
+        <v>0.48796780000000001</v>
+      </c>
+      <c r="AJ19" s="2">
+        <v>0.5002548</v>
+      </c>
+      <c r="AK19" s="2">
+        <v>0.51235459999999999</v>
+      </c>
+      <c r="AL19" s="2">
+        <v>0.52426220000000001</v>
+      </c>
+      <c r="AM19" s="2">
+        <v>0.53597300000000003</v>
+      </c>
+      <c r="AN19" s="2">
+        <v>0.5474831</v>
+      </c>
+      <c r="AO19" s="2">
+        <v>0.55878930000000004</v>
+      </c>
+      <c r="AP19" s="2">
+        <v>0.56988910000000004</v>
+      </c>
+      <c r="AQ19" s="2">
+        <v>0.58078059999999998</v>
+      </c>
+      <c r="AR19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B20" t="s">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1</v>
+      </c>
+      <c r="D20" s="2">
+        <v>5.9110500000000003E-2</v>
+      </c>
+      <c r="E20" s="2">
+        <v>5.1896299999999999E-2</v>
+      </c>
+      <c r="F20" s="2">
+        <v>5.70581E-2</v>
+      </c>
+      <c r="G20" s="2">
+        <v>5.0089700000000001E-2</v>
+      </c>
+      <c r="H20" s="2">
+        <v>6.0883E-2</v>
+      </c>
+      <c r="I20" s="2">
+        <v>5.13792E-2</v>
+      </c>
+      <c r="J20" s="2">
+        <v>6.3957100000000003E-2</v>
+      </c>
+      <c r="K20" s="2">
+        <v>6.4745399999999995E-2</v>
+      </c>
+      <c r="L20" s="2">
+        <v>4.2481499999999998E-2</v>
+      </c>
+      <c r="M20" s="2">
+        <v>7.7176499999999995E-2</v>
+      </c>
+      <c r="N20" s="2">
+        <v>7.0925500000000002E-2</v>
+      </c>
+      <c r="O20" s="2">
+        <v>7.6861499999999999E-2</v>
+      </c>
+      <c r="P20" s="2">
+        <v>8.3597099999999994E-2</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>9.4423400000000005E-2</v>
+      </c>
+      <c r="R20" s="2">
+        <v>0.1008283</v>
+      </c>
+      <c r="S20" s="2">
+        <v>0.1077524</v>
+      </c>
+      <c r="T20" s="2">
+        <v>0.111484</v>
+      </c>
+      <c r="U20" s="2">
+        <v>0.1197724</v>
+      </c>
+      <c r="V20" s="2">
+        <v>0.14766580000000001</v>
+      </c>
+      <c r="W20" s="2">
+        <v>0.159249</v>
+      </c>
+      <c r="X20" s="2">
+        <v>0.20809820000000001</v>
+      </c>
+      <c r="Y20" s="2">
+        <v>0.19157589999999999</v>
+      </c>
+      <c r="Z20" s="2">
+        <v>0.19986000000000001</v>
+      </c>
+      <c r="AA20" s="2">
+        <v>0.19816810000000001</v>
+      </c>
+      <c r="AB20" s="2">
+        <v>0.2098421</v>
+      </c>
+      <c r="AC20" s="2">
+        <v>0.22989509999999999</v>
+      </c>
+      <c r="AD20" s="2">
+        <v>0.24211640000000001</v>
+      </c>
+      <c r="AE20" s="2">
+        <v>0.25441809999999998</v>
+      </c>
+      <c r="AF20" s="2">
+        <v>0.26500259999999998</v>
+      </c>
+      <c r="AG20" s="2">
+        <v>0.2729453</v>
+      </c>
+      <c r="AH20" s="2">
+        <v>0.28088540000000001</v>
+      </c>
+      <c r="AI20" s="2">
+        <v>0.29130299999999998</v>
+      </c>
+      <c r="AJ20" s="2">
+        <v>0.30387930000000002</v>
+      </c>
+      <c r="AK20" s="2">
+        <v>0.31651820000000003</v>
+      </c>
+      <c r="AL20" s="2">
+        <v>0.32915729999999999</v>
+      </c>
+      <c r="AM20" s="2">
+        <v>0.34178049999999999</v>
+      </c>
+      <c r="AN20" s="2">
+        <v>0.35437299999999999</v>
+      </c>
+      <c r="AO20" s="2">
+        <v>0.36692079999999999</v>
+      </c>
+      <c r="AP20" s="2">
+        <v>0.37941049999999998</v>
+      </c>
+      <c r="AQ20" s="2">
+        <v>0.3918297</v>
+      </c>
+      <c r="AR20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2">
+        <v>3.1130999999999999E-2</v>
+      </c>
+      <c r="E21" s="2">
+        <v>2.6918299999999999E-2</v>
+      </c>
+      <c r="F21" s="2">
+        <v>2.9360299999999999E-2</v>
+      </c>
+      <c r="G21" s="2">
+        <v>2.5722999999999999E-2</v>
+      </c>
+      <c r="H21" s="2">
+        <v>3.0817500000000001E-2</v>
+      </c>
+      <c r="I21" s="2">
+        <v>2.5805499999999999E-2</v>
+      </c>
+      <c r="J21" s="2">
+        <v>3.2052400000000002E-2</v>
+      </c>
+      <c r="K21" s="2">
+        <v>3.2138800000000002E-2</v>
+      </c>
+      <c r="L21" s="2">
+        <v>2.12006E-2</v>
+      </c>
+      <c r="M21" s="2">
+        <v>3.8236600000000003E-2</v>
+      </c>
+      <c r="N21" s="2">
+        <v>3.4033599999999997E-2</v>
+      </c>
+      <c r="O21" s="2">
+        <v>3.6422099999999999E-2</v>
+      </c>
+      <c r="P21" s="2">
+        <v>3.9434900000000002E-2</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>4.4793600000000003E-2</v>
+      </c>
+      <c r="R21" s="2">
+        <v>4.7485600000000003E-2</v>
+      </c>
+      <c r="S21" s="2">
+        <v>5.0224600000000001E-2</v>
+      </c>
+      <c r="T21" s="2">
+        <v>5.1139200000000003E-2</v>
+      </c>
+      <c r="U21" s="2">
+        <v>5.3414900000000001E-2</v>
+      </c>
+      <c r="V21" s="2">
+        <v>8.2554199999999994E-2</v>
+      </c>
+      <c r="W21" s="2">
+        <v>0.101493</v>
+      </c>
+      <c r="X21" s="2">
+        <v>0.12404080000000001</v>
+      </c>
+      <c r="Y21" s="2">
+        <v>0.18596209999999999</v>
+      </c>
+      <c r="Z21" s="2">
+        <v>0.12676409999999999</v>
+      </c>
+      <c r="AA21" s="2">
+        <v>0.16148989999999999</v>
+      </c>
+      <c r="AB21" s="2">
+        <v>0.14134379999999999</v>
+      </c>
+      <c r="AC21" s="2">
+        <v>0.1341444</v>
+      </c>
+      <c r="AD21" s="2">
+        <v>0.1445777</v>
+      </c>
+      <c r="AE21" s="2">
+        <v>0.1553031</v>
+      </c>
+      <c r="AF21" s="2">
+        <v>0.16626669999999999</v>
+      </c>
+      <c r="AG21" s="2">
+        <v>0.1756877</v>
+      </c>
+      <c r="AH21" s="2">
+        <v>0.18282680000000001</v>
+      </c>
+      <c r="AI21" s="2">
+        <v>0.1900799</v>
+      </c>
+      <c r="AJ21" s="2">
+        <v>0.19984950000000001</v>
+      </c>
+      <c r="AK21" s="2">
+        <v>0.21170220000000001</v>
+      </c>
+      <c r="AL21" s="2">
+        <v>0.22375690000000001</v>
+      </c>
+      <c r="AM21" s="2">
+        <v>0.2359533</v>
+      </c>
+      <c r="AN21" s="2">
+        <v>0.2482702</v>
+      </c>
+      <c r="AO21" s="2">
+        <v>0.26068740000000001</v>
+      </c>
+      <c r="AP21" s="2">
+        <v>0.2731847</v>
+      </c>
+      <c r="AQ21" s="2">
+        <v>0.28574310000000003</v>
+      </c>
+      <c r="AR21" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
+      <c r="P22" s="2"/>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="2"/>
+      <c r="S22" s="2"/>
+      <c r="T22" s="2"/>
+      <c r="U22" s="2"/>
+      <c r="V22" s="2"/>
+    </row>
+    <row r="23" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
+      <c r="O23" s="2"/>
+      <c r="P23" s="2"/>
+      <c r="Q23" s="2"/>
+      <c r="R23" s="2"/>
+      <c r="S23" s="2"/>
+      <c r="T23" s="2"/>
+      <c r="U23" s="2"/>
+      <c r="V23" s="2"/>
+    </row>
+    <row r="24" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
+      <c r="O24" s="2"/>
+      <c r="P24" s="2"/>
+      <c r="Q24" s="2"/>
+      <c r="R24" s="2"/>
+      <c r="S24" s="2"/>
+      <c r="T24" s="2"/>
+      <c r="U24" s="2"/>
+      <c r="V24" s="2"/>
+    </row>
+    <row r="25" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B25" t="s">
+        <v>0</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0.93948989999999999</v>
+      </c>
+      <c r="E25" s="2">
+        <v>0.94297299999999995</v>
+      </c>
+      <c r="F25" s="2">
+        <v>0.90471290000000004</v>
+      </c>
+      <c r="G25" s="2">
+        <v>0.77590320000000002</v>
+      </c>
+      <c r="H25" s="2">
+        <v>0.95006199999999996</v>
+      </c>
+      <c r="I25" s="2">
+        <v>0.95427649999999997</v>
+      </c>
+      <c r="J25" s="2">
+        <v>0.96031330000000004</v>
+      </c>
+      <c r="K25" s="2">
+        <v>0.9645032</v>
+      </c>
+      <c r="L25" s="2">
+        <v>0.87848720000000002</v>
+      </c>
+      <c r="M25" s="2">
+        <v>0.96948210000000001</v>
+      </c>
+      <c r="N25" s="2">
+        <v>0.98619000000000001</v>
+      </c>
+      <c r="O25" s="2">
+        <v>0.98834540000000004</v>
+      </c>
+      <c r="P25" s="2">
+        <v>0.98920719999999995</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>0.98917869999999997</v>
+      </c>
+      <c r="R25" s="2">
+        <v>0.98923209999999995</v>
+      </c>
+      <c r="S25" s="2">
+        <v>0.98955170000000003</v>
+      </c>
+      <c r="T25" s="2">
+        <v>0.98905659999999995</v>
+      </c>
+      <c r="U25" s="2">
+        <v>0.98983200000000005</v>
+      </c>
+      <c r="V25" s="2">
+        <v>0.99013220000000002</v>
+      </c>
+      <c r="W25" s="2">
+        <v>0.99179430000000002</v>
+      </c>
+      <c r="X25" s="2">
+        <v>0.9886163</v>
+      </c>
+      <c r="Y25" s="2">
+        <v>0.99036069999999998</v>
+      </c>
+      <c r="Z25" s="2">
+        <v>0.99180179999999996</v>
+      </c>
+      <c r="AA25" s="2">
+        <v>0.99279919999999999</v>
+      </c>
+      <c r="AB25" s="2">
+        <v>0.99345119999999998</v>
+      </c>
+      <c r="AC25" s="2">
+        <v>0.99407210000000001</v>
+      </c>
+      <c r="AD25" s="2">
+        <v>0.99460139999999997</v>
+      </c>
+      <c r="AE25" s="2">
+        <v>0.99508260000000004</v>
+      </c>
+      <c r="AF25" s="2">
+        <v>0.99551979999999995</v>
+      </c>
+      <c r="AG25" s="2">
+        <v>0.99591730000000001</v>
+      </c>
+      <c r="AH25" s="2">
+        <v>0.99627860000000001</v>
+      </c>
+      <c r="AI25" s="2">
+        <v>0.99660709999999997</v>
+      </c>
+      <c r="AJ25" s="2">
+        <v>0.99690590000000001</v>
+      </c>
+      <c r="AK25" s="2">
+        <v>0.99717750000000005</v>
+      </c>
+      <c r="AL25" s="2">
+        <v>0.99742459999999999</v>
+      </c>
+      <c r="AM25" s="2">
+        <v>0.99764940000000002</v>
+      </c>
+      <c r="AN25" s="2">
+        <v>0.99785380000000001</v>
+      </c>
+      <c r="AO25" s="2">
+        <v>0.99803989999999998</v>
+      </c>
+      <c r="AP25" s="2">
+        <v>0.99820940000000002</v>
+      </c>
+      <c r="AQ25" s="2">
+        <v>0.99836369999999997</v>
+      </c>
+      <c r="AR25" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B26" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" s="2">
+        <v>0.93949099999999997</v>
+      </c>
+      <c r="E26" s="2">
+        <v>0.94073059999999997</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0.90780640000000001</v>
+      </c>
+      <c r="G26" s="2">
+        <v>0.79961349999999998</v>
+      </c>
+      <c r="H26" s="2">
+        <v>0.94946160000000002</v>
+      </c>
+      <c r="I26" s="2">
+        <v>0.95301800000000003</v>
+      </c>
+      <c r="J26" s="2">
+        <v>0.95776910000000004</v>
+      </c>
+      <c r="K26" s="2">
+        <v>0.96077749999999995</v>
+      </c>
+      <c r="L26" s="2">
+        <v>0.90532319999999999</v>
+      </c>
+      <c r="M26" s="2">
+        <v>0.96596040000000005</v>
+      </c>
+      <c r="N26" s="2">
+        <v>0.98366540000000002</v>
+      </c>
+      <c r="O26" s="2">
+        <v>0.98586359999999995</v>
+      </c>
+      <c r="P26" s="2">
+        <v>0.98736999999999997</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>0.98814270000000004</v>
+      </c>
+      <c r="R26" s="2">
+        <v>0.98858710000000005</v>
+      </c>
+      <c r="S26" s="2">
+        <v>0.98968060000000002</v>
+      </c>
+      <c r="T26" s="2">
+        <v>0.9894212</v>
+      </c>
+      <c r="U26" s="2">
+        <v>0.98944310000000002</v>
+      </c>
+      <c r="V26" s="2">
+        <v>0.98846239999999996</v>
+      </c>
+      <c r="W26" s="2">
+        <v>0.99082269999999995</v>
+      </c>
+      <c r="X26" s="2">
+        <v>0.9875081</v>
+      </c>
+      <c r="Y26" s="2">
+        <v>0.98954629999999999</v>
+      </c>
+      <c r="Z26" s="2">
+        <v>0.99047260000000004</v>
+      </c>
+      <c r="AA26" s="2">
+        <v>0.99127569999999998</v>
+      </c>
+      <c r="AB26" s="2">
+        <v>0.99169059999999998</v>
+      </c>
+      <c r="AC26" s="2">
+        <v>0.99239149999999998</v>
+      </c>
+      <c r="AD26" s="2">
+        <v>0.99306609999999995</v>
+      </c>
+      <c r="AE26" s="2">
+        <v>0.99368000000000001</v>
+      </c>
+      <c r="AF26" s="2">
+        <v>0.99423810000000001</v>
+      </c>
+      <c r="AG26" s="2">
+        <v>0.99474589999999996</v>
+      </c>
+      <c r="AH26" s="2">
+        <v>0.99520770000000003</v>
+      </c>
+      <c r="AI26" s="2">
+        <v>0.99562779999999995</v>
+      </c>
+      <c r="AJ26" s="2">
+        <v>0.99601010000000001</v>
+      </c>
+      <c r="AK26" s="2">
+        <v>0.99635810000000002</v>
+      </c>
+      <c r="AL26" s="2">
+        <v>0.99667459999999997</v>
+      </c>
+      <c r="AM26" s="2">
+        <v>0.99696280000000004</v>
+      </c>
+      <c r="AN26" s="2">
+        <v>0.99722520000000003</v>
+      </c>
+      <c r="AO26" s="2">
+        <v>0.99746429999999997</v>
+      </c>
+      <c r="AP26" s="2">
+        <v>0.99768179999999995</v>
+      </c>
+      <c r="AQ26" s="2">
+        <v>0.99787999999999999</v>
+      </c>
+      <c r="AR26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" s="2">
+        <v>0.93161919999999998</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0.93272820000000001</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0.91127089999999999</v>
+      </c>
+      <c r="G27" s="2">
+        <v>0.82108650000000005</v>
+      </c>
+      <c r="H27" s="2">
+        <v>0.94514849999999995</v>
+      </c>
+      <c r="I27" s="2">
+        <v>0.94743920000000004</v>
+      </c>
+      <c r="J27" s="2">
+        <v>0.95106740000000001</v>
+      </c>
+      <c r="K27" s="2">
+        <v>0.95269409999999999</v>
+      </c>
+      <c r="L27" s="2">
+        <v>0.92106429999999995</v>
+      </c>
+      <c r="M27" s="2">
+        <v>0.9688156</v>
+      </c>
+      <c r="N27" s="2">
+        <v>0.97883540000000002</v>
+      </c>
+      <c r="O27" s="2">
+        <v>0.98187020000000003</v>
+      </c>
+      <c r="P27" s="2">
+        <v>0.98326409999999997</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>0.98393450000000005</v>
+      </c>
+      <c r="R27" s="2">
+        <v>0.98528070000000001</v>
+      </c>
+      <c r="S27" s="2">
+        <v>0.98671589999999998</v>
+      </c>
+      <c r="T27" s="2">
+        <v>0.98705449999999995</v>
+      </c>
+      <c r="U27" s="2">
+        <v>0.98689610000000005</v>
+      </c>
+      <c r="V27" s="2">
+        <v>0.98603569999999996</v>
+      </c>
+      <c r="W27" s="2">
+        <v>0.98832960000000003</v>
+      </c>
+      <c r="X27" s="2">
+        <v>0.98380979999999996</v>
+      </c>
+      <c r="Y27" s="2">
+        <v>0.9864039</v>
+      </c>
+      <c r="Z27" s="2">
+        <v>0.98821720000000002</v>
+      </c>
+      <c r="AA27" s="2">
+        <v>0.98868769999999995</v>
+      </c>
+      <c r="AB27" s="2">
+        <v>0.98914420000000003</v>
+      </c>
+      <c r="AC27" s="2">
+        <v>0.99014060000000004</v>
+      </c>
+      <c r="AD27" s="2">
+        <v>0.99100639999999995</v>
+      </c>
+      <c r="AE27" s="2">
+        <v>0.99179439999999996</v>
+      </c>
+      <c r="AF27" s="2">
+        <v>0.99251180000000006</v>
+      </c>
+      <c r="AG27" s="2">
+        <v>0.99316499999999996</v>
+      </c>
+      <c r="AH27" s="2">
+        <v>0.99375970000000002</v>
+      </c>
+      <c r="AI27" s="2">
+        <v>0.9943014</v>
+      </c>
+      <c r="AJ27" s="2">
+        <v>0.99479450000000003</v>
+      </c>
+      <c r="AK27" s="2">
+        <v>0.99524380000000001</v>
+      </c>
+      <c r="AL27" s="2">
+        <v>0.9956528</v>
+      </c>
+      <c r="AM27" s="2">
+        <v>0.99602590000000002</v>
+      </c>
+      <c r="AN27" s="2">
+        <v>0.99636559999999996</v>
+      </c>
+      <c r="AO27" s="2">
+        <v>0.99667510000000004</v>
+      </c>
+      <c r="AP27" s="2">
+        <v>0.99695739999999999</v>
+      </c>
+      <c r="AQ27" s="2">
+        <v>0.99721470000000001</v>
+      </c>
+      <c r="AR27" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1</v>
+      </c>
+      <c r="D28" s="2">
+        <v>0.9258267</v>
+      </c>
+      <c r="E28" s="2">
+        <v>0.92652400000000001</v>
+      </c>
+      <c r="F28" s="2">
+        <v>0.91894580000000003</v>
+      </c>
+      <c r="G28" s="2">
+        <v>0.87593500000000002</v>
+      </c>
+      <c r="H28" s="2">
+        <v>0.93975129999999996</v>
+      </c>
+      <c r="I28" s="2">
+        <v>0.94033619999999996</v>
+      </c>
+      <c r="J28" s="2">
+        <v>0.94423509999999999</v>
+      </c>
+      <c r="K28" s="2">
+        <v>0.9445114</v>
+      </c>
+      <c r="L28" s="2">
+        <v>0.92678050000000001</v>
+      </c>
+      <c r="M28" s="2">
+        <v>0.96475900000000003</v>
+      </c>
+      <c r="N28" s="2">
+        <v>0.97298010000000001</v>
+      </c>
+      <c r="O28" s="2">
+        <v>0.97634869999999996</v>
+      </c>
+      <c r="P28" s="2">
+        <v>0.97793439999999998</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>0.97779039999999995</v>
+      </c>
+      <c r="R28" s="2">
+        <v>0.97875860000000003</v>
+      </c>
+      <c r="S28" s="2">
+        <v>0.98093280000000005</v>
+      </c>
+      <c r="T28" s="2">
+        <v>0.98248029999999997</v>
+      </c>
+      <c r="U28" s="2">
+        <v>0.98323970000000005</v>
+      </c>
+      <c r="V28" s="2">
+        <v>0.98304190000000002</v>
+      </c>
+      <c r="W28" s="2">
+        <v>0.98481830000000004</v>
+      </c>
+      <c r="X28" s="2">
+        <v>0.97968140000000004</v>
+      </c>
+      <c r="Y28" s="2">
+        <v>0.98287329999999995</v>
+      </c>
+      <c r="Z28" s="2">
+        <v>0.98508850000000003</v>
+      </c>
+      <c r="AA28" s="2">
+        <v>0.98658210000000002</v>
+      </c>
+      <c r="AB28" s="2">
+        <v>0.98736299999999999</v>
+      </c>
+      <c r="AC28" s="2">
+        <v>0.98845959999999999</v>
+      </c>
+      <c r="AD28" s="2">
+        <v>0.98945930000000004</v>
+      </c>
+      <c r="AE28" s="2">
+        <v>0.99037050000000004</v>
+      </c>
+      <c r="AF28" s="2">
+        <v>0.99120090000000005</v>
+      </c>
+      <c r="AG28" s="2">
+        <v>0.99195770000000005</v>
+      </c>
+      <c r="AH28" s="2">
+        <v>0.99264759999999996</v>
+      </c>
+      <c r="AI28" s="2">
+        <v>0.99327650000000001</v>
+      </c>
+      <c r="AJ28" s="2">
+        <v>0.99384980000000001</v>
+      </c>
+      <c r="AK28" s="2">
+        <v>0.9943727</v>
+      </c>
+      <c r="AL28" s="2">
+        <v>0.99484950000000005</v>
+      </c>
+      <c r="AM28" s="2">
+        <v>0.99528450000000002</v>
+      </c>
+      <c r="AN28" s="2">
+        <v>0.99568129999999999</v>
+      </c>
+      <c r="AO28" s="2">
+        <v>0.99604349999999997</v>
+      </c>
+      <c r="AP28" s="2">
+        <v>0.99637399999999998</v>
+      </c>
+      <c r="AQ28" s="2">
+        <v>0.99667570000000005</v>
+      </c>
+      <c r="AR28" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" t="s">
+        <v>0</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1</v>
+      </c>
+      <c r="D29" s="2">
+        <v>0.9168425</v>
+      </c>
+      <c r="E29" s="2">
+        <v>0.91528419999999999</v>
+      </c>
+      <c r="F29" s="2">
+        <v>0.91789080000000001</v>
+      </c>
+      <c r="G29" s="2">
+        <v>0.90036139999999998</v>
+      </c>
+      <c r="H29" s="2">
+        <v>0.93151050000000002</v>
+      </c>
+      <c r="I29" s="2">
+        <v>0.92972399999999999</v>
+      </c>
+      <c r="J29" s="2">
+        <v>0.93331719999999996</v>
+      </c>
+      <c r="K29" s="2">
+        <v>0.93374789999999996</v>
+      </c>
+      <c r="L29" s="2">
+        <v>0.92039139999999997</v>
+      </c>
+      <c r="M29" s="2">
+        <v>0.95520000000000005</v>
+      </c>
+      <c r="N29" s="2">
+        <v>0.96121650000000003</v>
+      </c>
+      <c r="O29" s="2">
+        <v>0.96611689999999995</v>
+      </c>
+      <c r="P29" s="2">
+        <v>0.96884550000000003</v>
+      </c>
+      <c r="Q29" s="2">
+        <v>0.96840000000000004</v>
+      </c>
+      <c r="R29" s="2">
+        <v>0.96889879999999995</v>
+      </c>
+      <c r="S29" s="2">
+        <v>0.9700299</v>
+      </c>
+      <c r="T29" s="2">
+        <v>0.97374910000000003</v>
+      </c>
+      <c r="U29" s="2">
+        <v>0.97592049999999997</v>
+      </c>
+      <c r="V29" s="2">
+        <v>0.97754969999999997</v>
+      </c>
+      <c r="W29" s="2">
+        <v>0.97825010000000001</v>
+      </c>
+      <c r="X29" s="2">
+        <v>0.97079269999999995</v>
+      </c>
+      <c r="Y29" s="2">
+        <v>0.9757171</v>
+      </c>
+      <c r="Z29" s="2">
+        <v>0.97920790000000002</v>
+      </c>
+      <c r="AA29" s="2">
+        <v>0.98138400000000003</v>
+      </c>
+      <c r="AB29" s="2">
+        <v>0.98301070000000002</v>
+      </c>
+      <c r="AC29" s="2">
+        <v>0.98470659999999999</v>
+      </c>
+      <c r="AD29" s="2">
+        <v>0.98602389999999995</v>
+      </c>
+      <c r="AE29" s="2">
+        <v>0.98722520000000002</v>
+      </c>
+      <c r="AF29" s="2">
+        <v>0.98832100000000001</v>
+      </c>
+      <c r="AG29" s="2">
+        <v>0.98932039999999999</v>
+      </c>
+      <c r="AH29" s="2">
+        <v>0.99023190000000005</v>
+      </c>
+      <c r="AI29" s="2">
+        <v>0.99106340000000004</v>
+      </c>
+      <c r="AJ29" s="2">
+        <v>0.99182190000000003</v>
+      </c>
+      <c r="AK29" s="2">
+        <v>0.99251400000000001</v>
+      </c>
+      <c r="AL29" s="2">
+        <v>0.99314539999999996</v>
+      </c>
+      <c r="AM29" s="2">
+        <v>0.99372170000000004</v>
+      </c>
+      <c r="AN29" s="2">
+        <v>0.99424769999999996</v>
+      </c>
+      <c r="AO29" s="2">
+        <v>0.99472799999999995</v>
+      </c>
+      <c r="AP29" s="2">
+        <v>0.99516660000000001</v>
+      </c>
+      <c r="AQ29" s="2">
+        <v>0.99556710000000004</v>
+      </c>
+      <c r="AR29" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B30" t="s">
+        <v>0</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1</v>
+      </c>
+      <c r="D30" s="2">
+        <v>0.90521810000000003</v>
+      </c>
+      <c r="E30" s="2">
+        <v>0.90139910000000001</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0.90693860000000004</v>
+      </c>
+      <c r="G30" s="2">
+        <v>0.9000283</v>
+      </c>
+      <c r="H30" s="2">
+        <v>0.91745129999999997</v>
+      </c>
+      <c r="I30" s="2">
+        <v>0.91563550000000005</v>
+      </c>
+      <c r="J30" s="2">
+        <v>0.91786389999999995</v>
+      </c>
+      <c r="K30" s="2">
+        <v>0.91763209999999995</v>
+      </c>
+      <c r="L30" s="2">
+        <v>0.91046609999999994</v>
+      </c>
+      <c r="M30" s="2">
+        <v>0.94075629999999999</v>
+      </c>
+      <c r="N30" s="2">
+        <v>0.94408110000000001</v>
+      </c>
+      <c r="O30" s="2">
+        <v>0.94993079999999996</v>
+      </c>
+      <c r="P30" s="2">
+        <v>0.95451850000000005</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>0.95463849999999995</v>
+      </c>
+      <c r="R30" s="2">
+        <v>0.9566268</v>
+      </c>
+      <c r="S30" s="2">
+        <v>0.95661490000000005</v>
+      </c>
+      <c r="T30" s="2">
+        <v>0.96013079999999995</v>
+      </c>
+      <c r="U30" s="2">
+        <v>0.96511539999999996</v>
+      </c>
+      <c r="V30" s="2">
+        <v>0.96954799999999997</v>
+      </c>
+      <c r="W30" s="2">
+        <v>0.97078249999999999</v>
+      </c>
+      <c r="X30" s="2">
+        <v>0.95980589999999999</v>
+      </c>
+      <c r="Y30" s="2">
+        <v>0.96404699999999999</v>
+      </c>
+      <c r="Z30" s="2">
+        <v>0.9694644</v>
+      </c>
+      <c r="AA30" s="2">
+        <v>0.97281700000000004</v>
+      </c>
+      <c r="AB30" s="2">
+        <v>0.97485049999999995</v>
+      </c>
+      <c r="AC30" s="2">
+        <v>0.97730649999999997</v>
+      </c>
+      <c r="AD30" s="2">
+        <v>0.97924730000000004</v>
+      </c>
+      <c r="AE30" s="2">
+        <v>0.98101970000000005</v>
+      </c>
+      <c r="AF30" s="2">
+        <v>0.98263809999999996</v>
+      </c>
+      <c r="AG30" s="2">
+        <v>0.98411579999999999</v>
+      </c>
+      <c r="AH30" s="2">
+        <v>0.98546489999999998</v>
+      </c>
+      <c r="AI30" s="2">
+        <v>0.98669649999999998</v>
+      </c>
+      <c r="AJ30" s="2">
+        <v>0.9878209</v>
+      </c>
+      <c r="AK30" s="2">
+        <v>0.98884760000000005</v>
+      </c>
+      <c r="AL30" s="2">
+        <v>0.98978509999999997</v>
+      </c>
+      <c r="AM30" s="2">
+        <v>0.99064090000000005</v>
+      </c>
+      <c r="AN30" s="2">
+        <v>0.99142280000000005</v>
+      </c>
+      <c r="AO30" s="2">
+        <v>0.99213689999999999</v>
+      </c>
+      <c r="AP30" s="2">
+        <v>0.99278929999999999</v>
+      </c>
+      <c r="AQ30" s="2">
+        <v>0.99338530000000003</v>
+      </c>
+      <c r="AR30" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B31" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1</v>
+      </c>
+      <c r="D31" s="2">
+        <v>0.88345790000000002</v>
+      </c>
+      <c r="E31" s="2">
+        <v>0.88070559999999998</v>
+      </c>
+      <c r="F31" s="2">
+        <v>0.88613830000000005</v>
+      </c>
+      <c r="G31" s="2">
+        <v>0.88326709999999997</v>
+      </c>
+      <c r="H31" s="2">
+        <v>0.89563159999999997</v>
+      </c>
+      <c r="I31" s="2">
+        <v>0.89508860000000001</v>
+      </c>
+      <c r="J31" s="2">
+        <v>0.89753139999999998</v>
+      </c>
+      <c r="K31" s="2">
+        <v>0.89721960000000001</v>
+      </c>
+      <c r="L31" s="2">
+        <v>0.89171929999999999</v>
+      </c>
+      <c r="M31" s="2">
+        <v>0.92242239999999998</v>
+      </c>
+      <c r="N31" s="2">
+        <v>0.92307870000000003</v>
+      </c>
+      <c r="O31" s="2">
+        <v>0.92866910000000003</v>
+      </c>
+      <c r="P31" s="2">
+        <v>0.93351499999999998</v>
+      </c>
+      <c r="Q31" s="2">
+        <v>0.93654919999999997</v>
+      </c>
+      <c r="R31" s="2">
+        <v>0.93957999999999997</v>
+      </c>
+      <c r="S31" s="2">
+        <v>0.94172489999999998</v>
+      </c>
+      <c r="T31" s="2">
+        <v>0.94454349999999998</v>
+      </c>
+      <c r="U31" s="2">
+        <v>0.94960809999999996</v>
+      </c>
+      <c r="V31" s="2">
+        <v>0.95810830000000002</v>
+      </c>
+      <c r="W31" s="2">
+        <v>0.96136909999999998</v>
+      </c>
+      <c r="X31" s="2">
+        <v>0.95030950000000003</v>
+      </c>
+      <c r="Y31" s="2">
+        <v>0.95237590000000005</v>
+      </c>
+      <c r="Z31" s="2">
+        <v>0.95666459999999998</v>
+      </c>
+      <c r="AA31" s="2">
+        <v>0.96204970000000001</v>
+      </c>
+      <c r="AB31" s="2">
+        <v>0.96510779999999996</v>
+      </c>
+      <c r="AC31" s="2">
+        <v>0.96841929999999998</v>
+      </c>
+      <c r="AD31" s="2">
+        <v>0.97110940000000001</v>
+      </c>
+      <c r="AE31" s="2">
+        <v>0.97356889999999996</v>
+      </c>
+      <c r="AF31" s="2">
+        <v>0.9758173</v>
+      </c>
+      <c r="AG31" s="2">
+        <v>0.97787179999999996</v>
+      </c>
+      <c r="AH31" s="2">
+        <v>0.97974910000000004</v>
+      </c>
+      <c r="AI31" s="2">
+        <v>0.98146409999999995</v>
+      </c>
+      <c r="AJ31" s="2">
+        <v>0.98303070000000004</v>
+      </c>
+      <c r="AK31" s="2">
+        <v>0.9844619</v>
+      </c>
+      <c r="AL31" s="2">
+        <v>0.98576900000000001</v>
+      </c>
+      <c r="AM31" s="2">
+        <v>0.98696309999999998</v>
+      </c>
+      <c r="AN31" s="2">
+        <v>0.98805390000000004</v>
+      </c>
+      <c r="AO31" s="2">
+        <v>0.9890504</v>
+      </c>
+      <c r="AP31" s="2">
+        <v>0.98996090000000003</v>
+      </c>
+      <c r="AQ31" s="2">
+        <v>0.99079289999999998</v>
+      </c>
+      <c r="AR31" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="32" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B32" t="s">
+        <v>0</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1</v>
+      </c>
+      <c r="D32" s="2">
+        <v>0.84343500000000005</v>
+      </c>
+      <c r="E32" s="2">
+        <v>0.83924840000000001</v>
+      </c>
+      <c r="F32" s="2">
+        <v>0.84788319999999995</v>
+      </c>
+      <c r="G32" s="2">
+        <v>0.84605779999999997</v>
+      </c>
+      <c r="H32" s="2">
+        <v>0.85739560000000004</v>
+      </c>
+      <c r="I32" s="2">
+        <v>0.85651259999999996</v>
+      </c>
+      <c r="J32" s="2">
+        <v>0.86072020000000005</v>
+      </c>
+      <c r="K32" s="2">
+        <v>0.8602495</v>
+      </c>
+      <c r="L32" s="2">
+        <v>0.85388260000000005</v>
+      </c>
+      <c r="M32" s="2">
+        <v>0.88936369999999998</v>
+      </c>
+      <c r="N32" s="2">
+        <v>0.89183959999999995</v>
+      </c>
+      <c r="O32" s="2">
+        <v>0.89666060000000003</v>
+      </c>
+      <c r="P32" s="2">
+        <v>0.90087729999999999</v>
+      </c>
+      <c r="Q32" s="2">
+        <v>0.90356429999999999</v>
+      </c>
+      <c r="R32" s="2">
+        <v>0.91263450000000002</v>
+      </c>
+      <c r="S32" s="2">
+        <v>0.91726229999999997</v>
+      </c>
+      <c r="T32" s="2">
+        <v>0.92294810000000005</v>
+      </c>
+      <c r="U32" s="2">
+        <v>0.92795439999999996</v>
+      </c>
+      <c r="V32" s="2">
+        <v>0.9386485</v>
+      </c>
+      <c r="W32" s="2">
+        <v>0.94476099999999996</v>
+      </c>
+      <c r="X32" s="2">
+        <v>0.93896789999999997</v>
+      </c>
+      <c r="Y32" s="2">
+        <v>0.94232309999999997</v>
+      </c>
+      <c r="Z32" s="2">
+        <v>0.9441832</v>
+      </c>
+      <c r="AA32" s="2">
+        <v>0.94772069999999997</v>
+      </c>
+      <c r="AB32" s="2">
+        <v>0.95219089999999995</v>
+      </c>
+      <c r="AC32" s="2">
+        <v>0.95688280000000003</v>
+      </c>
+      <c r="AD32" s="2">
+        <v>0.9605321</v>
+      </c>
+      <c r="AE32" s="2">
+        <v>0.96387389999999995</v>
+      </c>
+      <c r="AF32" s="2">
+        <v>0.96693269999999998</v>
+      </c>
+      <c r="AG32" s="2">
+        <v>0.96973140000000002</v>
+      </c>
+      <c r="AH32" s="2">
+        <v>0.97229120000000002</v>
+      </c>
+      <c r="AI32" s="2">
+        <v>0.97463200000000005</v>
+      </c>
+      <c r="AJ32" s="2">
+        <v>0.97677210000000003</v>
+      </c>
+      <c r="AK32" s="2">
+        <v>0.97872820000000005</v>
+      </c>
+      <c r="AL32" s="2">
+        <v>0.98051630000000001</v>
+      </c>
+      <c r="AM32" s="2">
+        <v>0.98215039999999998</v>
+      </c>
+      <c r="AN32" s="2">
+        <v>0.98364379999999996</v>
+      </c>
+      <c r="AO32" s="2">
+        <v>0.98500869999999996</v>
+      </c>
+      <c r="AP32" s="2">
+        <v>0.98625620000000003</v>
+      </c>
+      <c r="AQ32" s="2">
+        <v>0.98739650000000001</v>
+      </c>
+      <c r="AR32" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B33" t="s">
+        <v>0</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33" s="2">
+        <v>0.7850665</v>
+      </c>
+      <c r="E33" s="2">
+        <v>0.77841959999999999</v>
+      </c>
+      <c r="F33" s="2">
+        <v>0.79171210000000003</v>
+      </c>
+      <c r="G33" s="2">
+        <v>0.7891397</v>
+      </c>
+      <c r="H33" s="2">
+        <v>0.80492580000000002</v>
+      </c>
+      <c r="I33" s="2">
+        <v>0.80258580000000002</v>
+      </c>
+      <c r="J33" s="2">
+        <v>0.81053260000000005</v>
+      </c>
+      <c r="K33" s="2">
+        <v>0.81121900000000002</v>
+      </c>
+      <c r="L33" s="2">
+        <v>0.80051329999999998</v>
+      </c>
+      <c r="M33" s="2">
+        <v>0.84350539999999996</v>
+      </c>
+      <c r="N33" s="2">
+        <v>0.8490856</v>
+      </c>
+      <c r="O33" s="2">
+        <v>0.85656429999999995</v>
+      </c>
+      <c r="P33" s="2">
+        <v>0.8608112</v>
+      </c>
+      <c r="Q33" s="2">
+        <v>0.86219999999999997</v>
+      </c>
+      <c r="R33" s="2">
+        <v>0.87340609999999996</v>
+      </c>
+      <c r="S33" s="2">
+        <v>0.88432900000000003</v>
+      </c>
+      <c r="T33" s="2">
+        <v>0.89413050000000005</v>
+      </c>
+      <c r="U33" s="2">
+        <v>0.9032964</v>
+      </c>
+      <c r="V33" s="2">
+        <v>0.91490490000000002</v>
+      </c>
+      <c r="W33" s="2">
+        <v>0.9216647</v>
+      </c>
+      <c r="X33" s="2">
+        <v>0.92065779999999997</v>
+      </c>
+      <c r="Y33" s="2">
+        <v>0.92780609999999997</v>
+      </c>
+      <c r="Z33" s="2">
+        <v>0.93120440000000004</v>
+      </c>
+      <c r="AA33" s="2">
+        <v>0.9316854</v>
+      </c>
+      <c r="AB33" s="2">
+        <v>0.93506840000000002</v>
+      </c>
+      <c r="AC33" s="2">
+        <v>0.94167219999999996</v>
+      </c>
+      <c r="AD33" s="2">
+        <v>0.94656929999999995</v>
+      </c>
+      <c r="AE33" s="2">
+        <v>0.95106270000000004</v>
+      </c>
+      <c r="AF33" s="2">
+        <v>0.955183</v>
+      </c>
+      <c r="AG33" s="2">
+        <v>0.95895889999999995</v>
+      </c>
+      <c r="AH33" s="2">
+        <v>0.96241719999999997</v>
+      </c>
+      <c r="AI33" s="2">
+        <v>0.96558359999999999</v>
+      </c>
+      <c r="AJ33" s="2">
+        <v>0.96848140000000005</v>
+      </c>
+      <c r="AK33" s="2">
+        <v>0.97113289999999997</v>
+      </c>
+      <c r="AL33" s="2">
+        <v>0.97355809999999998</v>
+      </c>
+      <c r="AM33" s="2">
+        <v>0.97577610000000004</v>
+      </c>
+      <c r="AN33" s="2">
+        <v>0.97780409999999995</v>
+      </c>
+      <c r="AO33" s="2">
+        <v>0.97965869999999999</v>
+      </c>
+      <c r="AP33" s="2">
+        <v>0.98135419999999995</v>
+      </c>
+      <c r="AQ33" s="2">
+        <v>0.98290440000000001</v>
+      </c>
+      <c r="AR33" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="34" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B34" t="s">
+        <v>0</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1</v>
+      </c>
+      <c r="D34" s="2">
+        <v>0.7012005</v>
+      </c>
+      <c r="E34" s="2">
+        <v>0.69531489999999996</v>
+      </c>
+      <c r="F34" s="2">
+        <v>0.70582659999999997</v>
+      </c>
+      <c r="G34" s="2">
+        <v>0.70150179999999995</v>
+      </c>
+      <c r="H34" s="2">
+        <v>0.72642499999999999</v>
+      </c>
+      <c r="I34" s="2">
+        <v>0.72287950000000001</v>
+      </c>
+      <c r="J34" s="2">
+        <v>0.73401760000000005</v>
+      </c>
+      <c r="K34" s="2">
+        <v>0.73619590000000001</v>
+      </c>
+      <c r="L34" s="2">
+        <v>0.72082610000000003</v>
+      </c>
+      <c r="M34" s="2">
+        <v>0.77241689999999996</v>
+      </c>
+      <c r="N34" s="2">
+        <v>0.78179109999999996</v>
+      </c>
+      <c r="O34" s="2">
+        <v>0.79491339999999999</v>
+      </c>
+      <c r="P34" s="2">
+        <v>0.80406759999999999</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>0.80386069999999998</v>
+      </c>
+      <c r="R34" s="2">
+        <v>0.81703959999999998</v>
+      </c>
+      <c r="S34" s="2">
+        <v>0.83255080000000004</v>
+      </c>
+      <c r="T34" s="2">
+        <v>0.85006839999999995</v>
+      </c>
+      <c r="U34" s="2">
+        <v>0.86408059999999998</v>
+      </c>
+      <c r="V34" s="2">
+        <v>0.88288659999999997</v>
+      </c>
+      <c r="W34" s="2">
+        <v>0.88847580000000004</v>
+      </c>
+      <c r="X34" s="2">
+        <v>0.89275320000000002</v>
+      </c>
+      <c r="Y34" s="2">
+        <v>0.90706520000000002</v>
+      </c>
+      <c r="Z34" s="2">
+        <v>0.91414790000000001</v>
+      </c>
+      <c r="AA34" s="2">
+        <v>0.91619189999999995</v>
+      </c>
+      <c r="AB34" s="2">
+        <v>0.91603520000000005</v>
+      </c>
+      <c r="AC34" s="2">
+        <v>0.92252270000000003</v>
+      </c>
+      <c r="AD34" s="2">
+        <v>0.92888870000000001</v>
+      </c>
+      <c r="AE34" s="2">
+        <v>0.93478629999999996</v>
+      </c>
+      <c r="AF34" s="2">
+        <v>0.9402064</v>
+      </c>
+      <c r="AG34" s="2">
+        <v>0.94518400000000002</v>
+      </c>
+      <c r="AH34" s="2">
+        <v>0.94975189999999998</v>
+      </c>
+      <c r="AI34" s="2">
+        <v>0.95394129999999999</v>
+      </c>
+      <c r="AJ34" s="2">
+        <v>0.95778169999999996</v>
+      </c>
+      <c r="AK34" s="2">
+        <v>0.96130070000000001</v>
+      </c>
+      <c r="AL34" s="2">
+        <v>0.96452400000000005</v>
+      </c>
+      <c r="AM34" s="2">
+        <v>0.96747559999999999</v>
+      </c>
+      <c r="AN34" s="2">
+        <v>0.97017770000000003</v>
+      </c>
+      <c r="AO34" s="2">
+        <v>0.97265109999999999</v>
+      </c>
+      <c r="AP34" s="2">
+        <v>0.97491479999999997</v>
+      </c>
+      <c r="AQ34" s="2">
+        <v>0.97698629999999997</v>
+      </c>
+      <c r="AR34" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="35" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B35" t="s">
+        <v>0</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1</v>
+      </c>
+      <c r="D35" s="2">
+        <v>0.58211170000000001</v>
+      </c>
+      <c r="E35" s="2">
+        <v>0.57661600000000002</v>
+      </c>
+      <c r="F35" s="2">
+        <v>0.59163960000000004</v>
+      </c>
+      <c r="G35" s="2">
+        <v>0.58563100000000001</v>
+      </c>
+      <c r="H35" s="2">
+        <v>0.61504049999999999</v>
+      </c>
+      <c r="I35" s="2">
+        <v>0.61081269999999999</v>
+      </c>
+      <c r="J35" s="2">
+        <v>0.62892780000000004</v>
+      </c>
+      <c r="K35" s="2">
+        <v>0.63298140000000003</v>
+      </c>
+      <c r="L35" s="2">
+        <v>0.60962439999999996</v>
+      </c>
+      <c r="M35" s="2">
+        <v>0.67424569999999995</v>
+      </c>
+      <c r="N35" s="2">
+        <v>0.68271519999999997</v>
+      </c>
+      <c r="O35" s="2">
+        <v>0.70227980000000001</v>
+      </c>
+      <c r="P35" s="2">
+        <v>0.71881519999999999</v>
+      </c>
+      <c r="Q35" s="2">
+        <v>0.72609630000000003</v>
+      </c>
+      <c r="R35" s="2">
+        <v>0.73878770000000005</v>
+      </c>
+      <c r="S35" s="2">
+        <v>0.75633419999999996</v>
+      </c>
+      <c r="T35" s="2">
+        <v>0.77786509999999998</v>
+      </c>
+      <c r="U35" s="2">
+        <v>0.80298539999999996</v>
+      </c>
+      <c r="V35" s="2">
+        <v>0.83267259999999998</v>
+      </c>
+      <c r="W35" s="2">
+        <v>0.84266700000000005</v>
+      </c>
+      <c r="X35" s="2">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="Y35" s="2">
+        <v>0.86568060000000002</v>
+      </c>
+      <c r="Z35" s="2">
+        <v>0.8809612</v>
+      </c>
+      <c r="AA35" s="2">
+        <v>0.88639159999999995</v>
+      </c>
+      <c r="AB35" s="2">
+        <v>0.88664790000000004</v>
+      </c>
+      <c r="AC35" s="2">
+        <v>0.89228949999999996</v>
+      </c>
+      <c r="AD35" s="2">
+        <v>0.89821580000000001</v>
+      </c>
+      <c r="AE35" s="2">
+        <v>0.90637829999999997</v>
+      </c>
+      <c r="AF35" s="2">
+        <v>0.91396599999999995</v>
+      </c>
+      <c r="AG35" s="2">
+        <v>0.92096009999999995</v>
+      </c>
+      <c r="AH35" s="2">
+        <v>0.92740080000000003</v>
+      </c>
+      <c r="AI35" s="2">
+        <v>0.93332669999999995</v>
+      </c>
+      <c r="AJ35" s="2">
+        <v>0.93877520000000003</v>
+      </c>
+      <c r="AK35" s="2">
+        <v>0.94378139999999999</v>
+      </c>
+      <c r="AL35" s="2">
+        <v>0.94837859999999996</v>
+      </c>
+      <c r="AM35" s="2">
+        <v>0.95259859999999996</v>
+      </c>
+      <c r="AN35" s="2">
+        <v>0.95647059999999995</v>
+      </c>
+      <c r="AO35" s="2">
+        <v>0.96002240000000005</v>
+      </c>
+      <c r="AP35" s="2">
+        <v>0.96327940000000001</v>
+      </c>
+      <c r="AQ35" s="2">
+        <v>0.96626579999999995</v>
+      </c>
+      <c r="AR35" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="36" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B36" t="s">
+        <v>0</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1</v>
+      </c>
+      <c r="D36" s="2">
+        <v>0.43385200000000002</v>
+      </c>
+      <c r="E36" s="2">
+        <v>0.42837229999999998</v>
+      </c>
+      <c r="F36" s="2">
+        <v>0.4425828</v>
+      </c>
+      <c r="G36" s="2">
+        <v>0.43413859999999999</v>
+      </c>
+      <c r="H36" s="2">
+        <v>0.4663641</v>
+      </c>
+      <c r="I36" s="2">
+        <v>0.45413550000000003</v>
+      </c>
+      <c r="J36" s="2">
+        <v>0.48461670000000001</v>
+      </c>
+      <c r="K36" s="2">
+        <v>0.48811379999999999</v>
+      </c>
+      <c r="L36" s="2">
+        <v>0.44581989999999999</v>
+      </c>
+      <c r="M36" s="2">
+        <v>0.52641470000000001</v>
+      </c>
+      <c r="N36" s="2">
+        <v>0.53786900000000004</v>
+      </c>
+      <c r="O36" s="2">
+        <v>0.5607219</v>
+      </c>
+      <c r="P36" s="2">
+        <v>0.58000180000000001</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>0.59654039999999997</v>
+      </c>
+      <c r="R36" s="2">
+        <v>0.61376600000000003</v>
+      </c>
+      <c r="S36" s="2">
+        <v>0.63243780000000005</v>
+      </c>
+      <c r="T36" s="2">
+        <v>0.65468910000000002</v>
+      </c>
+      <c r="U36" s="2">
+        <v>0.68637060000000005</v>
+      </c>
+      <c r="V36" s="2">
+        <v>0.73627350000000003</v>
+      </c>
+      <c r="W36" s="2">
+        <v>0.75236709999999996</v>
+      </c>
+      <c r="X36" s="2">
+        <v>0.75709230000000005</v>
+      </c>
+      <c r="Y36" s="2">
+        <v>0.78356720000000002</v>
+      </c>
+      <c r="Z36" s="2">
+        <v>0.80734130000000004</v>
+      </c>
+      <c r="AA36" s="2">
+        <v>0.82058520000000001</v>
+      </c>
+      <c r="AB36" s="2">
+        <v>0.82327510000000004</v>
+      </c>
+      <c r="AC36" s="2">
+        <v>0.83252040000000005</v>
+      </c>
+      <c r="AD36" s="2">
+        <v>0.8365127</v>
+      </c>
+      <c r="AE36" s="2">
+        <v>0.84514739999999999</v>
+      </c>
+      <c r="AF36" s="2">
+        <v>0.85733400000000004</v>
+      </c>
+      <c r="AG36" s="2">
+        <v>0.86873330000000004</v>
+      </c>
+      <c r="AH36" s="2">
+        <v>0.87929619999999997</v>
+      </c>
+      <c r="AI36" s="2">
+        <v>0.88906909999999995</v>
+      </c>
+      <c r="AJ36" s="2">
+        <v>0.89809910000000004</v>
+      </c>
+      <c r="AK36" s="2">
+        <v>0.90643200000000002</v>
+      </c>
+      <c r="AL36" s="2">
+        <v>0.91411370000000003</v>
+      </c>
+      <c r="AM36" s="2">
+        <v>0.92118789999999995</v>
+      </c>
+      <c r="AN36" s="2">
+        <v>0.92769690000000005</v>
+      </c>
+      <c r="AO36" s="2">
+        <v>0.9336816</v>
+      </c>
+      <c r="AP36" s="2">
+        <v>0.93918020000000002</v>
+      </c>
+      <c r="AQ36" s="2">
+        <v>0.9442294</v>
+      </c>
+      <c r="AR36" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="37" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B37" t="s">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37" s="2">
+        <v>0.27882430000000002</v>
+      </c>
+      <c r="E37" s="2">
+        <v>0.27507759999999998</v>
+      </c>
+      <c r="F37" s="2">
+        <v>0.29231390000000002</v>
+      </c>
+      <c r="G37" s="2">
+        <v>0.27702680000000002</v>
+      </c>
+      <c r="H37" s="2">
+        <v>0.31223339999999999</v>
+      </c>
+      <c r="I37" s="2">
+        <v>0.29627049999999999</v>
+      </c>
+      <c r="J37" s="2">
+        <v>0.32747150000000003</v>
+      </c>
+      <c r="K37" s="2">
+        <v>0.33488089999999998</v>
+      </c>
+      <c r="L37" s="2">
+        <v>0.28378110000000001</v>
+      </c>
+      <c r="M37" s="2">
+        <v>0.36628840000000001</v>
+      </c>
+      <c r="N37" s="2">
+        <v>0.37220029999999998</v>
+      </c>
+      <c r="O37" s="2">
+        <v>0.3946095</v>
+      </c>
+      <c r="P37" s="2">
+        <v>0.41239510000000001</v>
+      </c>
+      <c r="Q37" s="2">
+        <v>0.43374289999999999</v>
+      </c>
+      <c r="R37" s="2">
+        <v>0.45331709999999997</v>
+      </c>
+      <c r="S37" s="2">
+        <v>0.47478599999999999</v>
+      </c>
+      <c r="T37" s="2">
+        <v>0.49261759999999999</v>
+      </c>
+      <c r="U37" s="2">
+        <v>0.52580159999999998</v>
+      </c>
+      <c r="V37" s="2">
+        <v>0.58497580000000005</v>
+      </c>
+      <c r="W37" s="2">
+        <v>0.60812029999999995</v>
+      </c>
+      <c r="X37" s="2">
+        <v>0.61376920000000001</v>
+      </c>
+      <c r="Y37" s="2">
+        <v>0.64961789999999997</v>
+      </c>
+      <c r="Z37" s="2">
+        <v>0.67543419999999998</v>
+      </c>
+      <c r="AA37" s="2">
+        <v>0.69584489999999999</v>
+      </c>
+      <c r="AB37" s="2">
+        <v>0.70967230000000003</v>
+      </c>
+      <c r="AC37" s="2">
+        <v>0.73082400000000003</v>
+      </c>
+      <c r="AD37" s="2">
+        <v>0.73664249999999998</v>
+      </c>
+      <c r="AE37" s="2">
+        <v>0.74225059999999998</v>
+      </c>
+      <c r="AF37" s="2">
+        <v>0.75439860000000003</v>
+      </c>
+      <c r="AG37" s="2">
+        <v>0.77135010000000004</v>
+      </c>
+      <c r="AH37" s="2">
+        <v>0.78742970000000001</v>
+      </c>
+      <c r="AI37" s="2">
+        <v>0.8025485</v>
+      </c>
+      <c r="AJ37" s="2">
+        <v>0.81673819999999997</v>
+      </c>
+      <c r="AK37" s="2">
+        <v>0.83003340000000003</v>
+      </c>
+      <c r="AL37" s="2">
+        <v>0.84247090000000002</v>
+      </c>
+      <c r="AM37" s="2">
+        <v>0.85408910000000005</v>
+      </c>
+      <c r="AN37" s="2">
+        <v>0.86492769999999997</v>
+      </c>
+      <c r="AO37" s="2">
+        <v>0.87502659999999999</v>
+      </c>
+      <c r="AP37" s="2">
+        <v>0.88442560000000003</v>
+      </c>
+      <c r="AQ37" s="2">
+        <v>0.89316419999999996</v>
+      </c>
+      <c r="AR37" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B38" t="s">
+        <v>0</v>
+      </c>
+      <c r="C38" t="s">
+        <v>1</v>
+      </c>
+      <c r="D38" s="2">
+        <v>0.16475049999999999</v>
+      </c>
+      <c r="E38" s="2">
+        <v>0.1590377</v>
+      </c>
+      <c r="F38" s="2">
+        <v>0.17004739999999999</v>
+      </c>
+      <c r="G38" s="2">
+        <v>0.1553002</v>
+      </c>
+      <c r="H38" s="2">
+        <v>0.18389639999999999</v>
+      </c>
+      <c r="I38" s="2">
+        <v>0.16523640000000001</v>
+      </c>
+      <c r="J38" s="2">
+        <v>0.19354589999999999</v>
+      </c>
+      <c r="K38" s="2">
+        <v>0.19806960000000001</v>
+      </c>
+      <c r="L38" s="2">
+        <v>0.15060200000000001</v>
+      </c>
+      <c r="M38" s="2">
+        <v>0.22118019999999999</v>
+      </c>
+      <c r="N38" s="2">
+        <v>0.22305990000000001</v>
+      </c>
+      <c r="O38" s="2">
+        <v>0.2385642</v>
+      </c>
+      <c r="P38" s="2">
+        <v>0.25512190000000001</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>0.27221250000000002</v>
+      </c>
+      <c r="R38" s="2">
+        <v>0.29087499999999999</v>
+      </c>
+      <c r="S38" s="2">
+        <v>0.30667250000000001</v>
+      </c>
+      <c r="T38" s="2">
+        <v>0.32181320000000002</v>
+      </c>
+      <c r="U38" s="2">
+        <v>0.34814509999999999</v>
+      </c>
+      <c r="V38" s="2">
+        <v>0.4050783</v>
+      </c>
+      <c r="W38" s="2">
+        <v>0.42117840000000001</v>
+      </c>
+      <c r="X38" s="2">
+        <v>0.42724990000000002</v>
+      </c>
+      <c r="Y38" s="2">
+        <v>0.46153690000000003</v>
+      </c>
+      <c r="Z38" s="2">
+        <v>0.48657080000000003</v>
+      </c>
+      <c r="AA38" s="2">
+        <v>0.50089680000000003</v>
+      </c>
+      <c r="AB38" s="2">
+        <v>0.51461460000000003</v>
+      </c>
+      <c r="AC38" s="2">
+        <v>0.54151539999999998</v>
+      </c>
+      <c r="AD38" s="2">
+        <v>0.55406569999999999</v>
+      </c>
+      <c r="AE38" s="2">
+        <v>0.56147630000000004</v>
+      </c>
+      <c r="AF38" s="2">
+        <v>0.56888590000000006</v>
+      </c>
+      <c r="AG38" s="2">
+        <v>0.58137570000000005</v>
+      </c>
+      <c r="AH38" s="2">
+        <v>0.59719029999999995</v>
+      </c>
+      <c r="AI38" s="2">
+        <v>0.61263900000000004</v>
+      </c>
+      <c r="AJ38" s="2">
+        <v>0.62765309999999996</v>
+      </c>
+      <c r="AK38" s="2">
+        <v>0.64222999999999997</v>
+      </c>
+      <c r="AL38" s="2">
+        <v>0.65636839999999996</v>
+      </c>
+      <c r="AM38" s="2">
+        <v>0.67006889999999997</v>
+      </c>
+      <c r="AN38" s="2">
+        <v>0.68333319999999997</v>
+      </c>
+      <c r="AO38" s="2">
+        <v>0.69616469999999997</v>
+      </c>
+      <c r="AP38" s="2">
+        <v>0.70856759999999996</v>
+      </c>
+      <c r="AQ38" s="2">
+        <v>0.7205473</v>
+      </c>
+      <c r="AR38" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B39" t="s">
+        <v>0</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2">
+        <v>9.14441E-2</v>
+      </c>
+      <c r="E39" s="2">
+        <v>8.0050700000000002E-2</v>
+      </c>
+      <c r="F39" s="2">
+        <v>9.0590299999999999E-2</v>
+      </c>
+      <c r="G39" s="2">
+        <v>8.0600099999999994E-2</v>
+      </c>
+      <c r="H39" s="2">
+        <v>9.4020900000000004E-2</v>
+      </c>
+      <c r="I39" s="2">
+        <v>8.2084900000000002E-2</v>
+      </c>
+      <c r="J39" s="2">
+        <v>0.1011011</v>
+      </c>
+      <c r="K39" s="2">
+        <v>0.10110189999999999</v>
+      </c>
+      <c r="L39" s="2">
+        <v>7.02874E-2</v>
+      </c>
+      <c r="M39" s="2">
+        <v>0.12015960000000001</v>
+      </c>
+      <c r="N39" s="2">
+        <v>0.1157934</v>
+      </c>
+      <c r="O39" s="2">
+        <v>0.12476230000000001</v>
+      </c>
+      <c r="P39" s="2">
+        <v>0.1373123</v>
+      </c>
+      <c r="Q39" s="2">
+        <v>0.1498101</v>
+      </c>
+      <c r="R39" s="2">
+        <v>0.15906880000000001</v>
+      </c>
+      <c r="S39" s="2">
+        <v>0.17136170000000001</v>
+      </c>
+      <c r="T39" s="2">
+        <v>0.17856749999999999</v>
+      </c>
+      <c r="U39" s="2">
+        <v>0.194711</v>
+      </c>
+      <c r="V39" s="2">
+        <v>0.2322988</v>
+      </c>
+      <c r="W39" s="2">
+        <v>0.25069010000000003</v>
+      </c>
+      <c r="X39" s="2">
+        <v>0.24570259999999999</v>
+      </c>
+      <c r="Y39" s="2">
+        <v>0.26877649999999997</v>
+      </c>
+      <c r="Z39" s="2">
+        <v>0.28375470000000003</v>
+      </c>
+      <c r="AA39" s="2">
+        <v>0.29031790000000002</v>
+      </c>
+      <c r="AB39" s="2">
+        <v>0.29946509999999998</v>
+      </c>
+      <c r="AC39" s="2">
+        <v>0.31975910000000002</v>
+      </c>
+      <c r="AD39" s="2">
+        <v>0.33112409999999998</v>
+      </c>
+      <c r="AE39" s="2">
+        <v>0.3404624</v>
+      </c>
+      <c r="AF39" s="2">
+        <v>0.34710999999999997</v>
+      </c>
+      <c r="AG39" s="2">
+        <v>0.3537747</v>
+      </c>
+      <c r="AH39" s="2">
+        <v>0.36309599999999997</v>
+      </c>
+      <c r="AI39" s="2">
+        <v>0.37445909999999999</v>
+      </c>
+      <c r="AJ39" s="2">
+        <v>0.38581739999999998</v>
+      </c>
+      <c r="AK39" s="2">
+        <v>0.39711980000000002</v>
+      </c>
+      <c r="AL39" s="2">
+        <v>0.40835850000000001</v>
+      </c>
+      <c r="AM39" s="2">
+        <v>0.4195258</v>
+      </c>
+      <c r="AN39" s="2">
+        <v>0.43061480000000002</v>
+      </c>
+      <c r="AO39" s="2">
+        <v>0.44161879999999998</v>
+      </c>
+      <c r="AP39" s="2">
+        <v>0.45253149999999998</v>
+      </c>
+      <c r="AQ39" s="2">
+        <v>0.46334720000000001</v>
+      </c>
+      <c r="AR39" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="40" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B40" t="s">
+        <v>0</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1</v>
+      </c>
+      <c r="D40" s="2">
+        <v>4.4845299999999998E-2</v>
+      </c>
+      <c r="E40" s="2">
+        <v>3.9527800000000002E-2</v>
+      </c>
+      <c r="F40" s="2">
+        <v>4.3489899999999998E-2</v>
+      </c>
+      <c r="G40" s="2">
+        <v>3.7648899999999999E-2</v>
+      </c>
+      <c r="H40" s="2">
+        <v>4.6156900000000001E-2</v>
+      </c>
+      <c r="I40" s="2">
+        <v>3.8879799999999999E-2</v>
+      </c>
+      <c r="J40" s="2">
+        <v>4.84809E-2</v>
+      </c>
+      <c r="K40" s="2">
+        <v>4.8920999999999999E-2</v>
+      </c>
+      <c r="L40" s="2">
+        <v>3.1858499999999998E-2</v>
+      </c>
+      <c r="M40" s="2">
+        <v>5.8611000000000003E-2</v>
+      </c>
+      <c r="N40" s="2">
+        <v>5.4017999999999997E-2</v>
+      </c>
+      <c r="O40" s="2">
+        <v>5.8373099999999997E-2</v>
+      </c>
+      <c r="P40" s="2">
+        <v>6.3513600000000003E-2</v>
+      </c>
+      <c r="Q40" s="2">
+        <v>7.1688199999999994E-2</v>
+      </c>
+      <c r="R40" s="2">
+        <v>7.6364000000000001E-2</v>
+      </c>
+      <c r="S40" s="2">
+        <v>8.1993899999999995E-2</v>
+      </c>
+      <c r="T40" s="2">
+        <v>8.4833400000000003E-2</v>
+      </c>
+      <c r="U40" s="2">
+        <v>9.1767100000000004E-2</v>
+      </c>
+      <c r="V40" s="2">
+        <v>0.1139389</v>
+      </c>
+      <c r="W40" s="2">
+        <v>0.1228871</v>
+      </c>
+      <c r="X40" s="2">
+        <v>0.14200840000000001</v>
+      </c>
+      <c r="Y40" s="2">
+        <v>0.1314459</v>
+      </c>
+      <c r="Z40" s="2">
+        <v>0.1378846</v>
+      </c>
+      <c r="AA40" s="2">
+        <v>0.13671939999999999</v>
+      </c>
+      <c r="AB40" s="2">
+        <v>0.1465641</v>
+      </c>
+      <c r="AC40" s="2">
+        <v>0.16105330000000001</v>
+      </c>
+      <c r="AD40" s="2">
+        <v>0.17024130000000001</v>
+      </c>
+      <c r="AE40" s="2">
+        <v>0.179566</v>
+      </c>
+      <c r="AF40" s="2">
+        <v>0.18746170000000001</v>
+      </c>
+      <c r="AG40" s="2">
+        <v>0.19310269999999999</v>
+      </c>
+      <c r="AH40" s="2">
+        <v>0.1987865</v>
+      </c>
+      <c r="AI40" s="2">
+        <v>0.20669850000000001</v>
+      </c>
+      <c r="AJ40" s="2">
+        <v>0.21658910000000001</v>
+      </c>
+      <c r="AK40" s="2">
+        <v>0.2266299</v>
+      </c>
+      <c r="AL40" s="2">
+        <v>0.23676929999999999</v>
+      </c>
+      <c r="AM40" s="2">
+        <v>0.2469964</v>
+      </c>
+      <c r="AN40" s="2">
+        <v>0.25730059999999999</v>
+      </c>
+      <c r="AO40" s="2">
+        <v>0.2676713</v>
+      </c>
+      <c r="AP40" s="2">
+        <v>0.27809859999999997</v>
+      </c>
+      <c r="AQ40" s="2">
+        <v>0.28857240000000001</v>
+      </c>
+      <c r="AR40" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="41" spans="1:44" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B41" t="s">
+        <v>0</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1</v>
+      </c>
+      <c r="D41" s="2">
+        <v>2.3437400000000001E-2</v>
+      </c>
+      <c r="E41" s="2">
+        <v>2.0357799999999999E-2</v>
+      </c>
+      <c r="F41" s="2">
+        <v>2.2212900000000001E-2</v>
+      </c>
+      <c r="G41" s="2">
+        <v>1.9176499999999999E-2</v>
+      </c>
+      <c r="H41" s="2">
+        <v>2.3160300000000002E-2</v>
+      </c>
+      <c r="I41" s="2">
+        <v>1.9357900000000001E-2</v>
+      </c>
+      <c r="J41" s="2">
+        <v>2.40462E-2</v>
+      </c>
+      <c r="K41" s="2">
+        <v>2.39971E-2</v>
+      </c>
+      <c r="L41" s="2">
+        <v>1.5728900000000001E-2</v>
+      </c>
+      <c r="M41" s="2">
+        <v>2.86947E-2</v>
+      </c>
+      <c r="N41" s="2">
+        <v>2.5615599999999999E-2</v>
+      </c>
+      <c r="O41" s="2">
+        <v>2.7272000000000001E-2</v>
+      </c>
+      <c r="P41" s="2">
+        <v>2.94886E-2</v>
+      </c>
+      <c r="Q41" s="2">
+        <v>3.3394699999999999E-2</v>
+      </c>
+      <c r="R41" s="2">
+        <v>3.5215999999999997E-2</v>
+      </c>
+      <c r="S41" s="2">
+        <v>3.7383899999999998E-2</v>
+      </c>
+      <c r="T41" s="2">
+        <v>3.79916E-2</v>
+      </c>
+      <c r="U41" s="2">
+        <v>3.9945000000000001E-2</v>
+      </c>
+      <c r="V41" s="2">
+        <v>6.2122700000000003E-2</v>
+      </c>
+      <c r="W41" s="2">
+        <v>7.6259199999999999E-2</v>
+      </c>
+      <c r="X41" s="2">
+        <v>7.9283800000000001E-2</v>
+      </c>
+      <c r="Y41" s="2">
+        <v>0.1212022</v>
+      </c>
+      <c r="Z41" s="2">
+        <v>8.1529000000000004E-2</v>
+      </c>
+      <c r="AA41" s="2">
+        <v>0.1037682</v>
+      </c>
+      <c r="AB41" s="2">
+        <v>9.4248499999999999E-2</v>
+      </c>
+      <c r="AC41" s="2">
+        <v>9.1167600000000001E-2</v>
+      </c>
+      <c r="AD41" s="2">
+        <v>9.8520099999999999E-2</v>
+      </c>
+      <c r="AE41" s="2">
+        <v>0.1061288</v>
+      </c>
+      <c r="AF41" s="2">
+        <v>0.113957</v>
+      </c>
+      <c r="AG41" s="2">
+        <v>0.12053850000000001</v>
+      </c>
+      <c r="AH41" s="2">
+        <v>0.12524950000000001</v>
+      </c>
+      <c r="AI41" s="2">
+        <v>0.13006719999999999</v>
+      </c>
+      <c r="AJ41" s="2">
+        <v>0.13699720000000001</v>
+      </c>
+      <c r="AK41" s="2">
+        <v>0.1457068</v>
+      </c>
+      <c r="AL41" s="2">
+        <v>0.15464559999999999</v>
+      </c>
+      <c r="AM41" s="2">
+        <v>0.16376979999999999</v>
+      </c>
+      <c r="AN41" s="2">
+        <v>0.17306769999999999</v>
+      </c>
+      <c r="AO41" s="2">
+        <v>0.18252779999999999</v>
+      </c>
+      <c r="AP41" s="2">
+        <v>0.19213839999999999</v>
+      </c>
+      <c r="AQ41" s="2">
+        <v>0.20188780000000001</v>
+      </c>
+      <c r="AR41" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
baseline pour tech et croissance
</commit_message>
<xml_diff>
--- a/all_shocks.xlsx
+++ b/all_shocks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\emanu\OneDrive\Matlab\cdc_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47DFB97A-B84D-4FCC-886D-1E6285D5A5E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FA5A2B0-7C73-44D9-9183-2CF1F1323721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1350" yWindow="1500" windowWidth="19395" windowHeight="10425" tabRatio="805" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15990" tabRatio="805" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_pop_shocks_norm2000" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2138" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2147" uniqueCount="376">
   <si>
     <t>=</t>
   </si>
@@ -1166,6 +1166,12 @@
   <si>
     <t>s_A_ctr</t>
   </si>
+  <si>
+    <t>s_dpib_des</t>
+  </si>
+  <si>
+    <t>s_A_des</t>
+  </si>
 </sst>
 </file>
 
@@ -12442,7 +12448,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D753D42-C95A-408F-AA7D-68FE79D9776F}">
-  <dimension ref="A1:AS26"/>
+  <dimension ref="A1:AS29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
@@ -13805,364 +13811,157 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="17" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>352</v>
-      </c>
-      <c r="C17">
+    <row r="15" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="B15" t="s">
+        <v>0</v>
+      </c>
+      <c r="C15" t="s">
         <v>1</v>
       </c>
-      <c r="D17">
-        <f>(1+D11)*C17</f>
-        <v>1.1222527472527473</v>
-      </c>
-      <c r="E17">
-        <f t="shared" ref="E17:AR20" si="0">(1+E11)*D17</f>
-        <v>1.1057692307692306</v>
-      </c>
-      <c r="F17">
-        <f t="shared" si="0"/>
-        <v>1.2376373626373625</v>
-      </c>
-      <c r="G17">
-        <f t="shared" si="0"/>
-        <v>1.2760989010989017</v>
-      </c>
-      <c r="H17">
-        <f t="shared" si="0"/>
-        <v>1.0343406593406592</v>
-      </c>
-      <c r="I17">
-        <f t="shared" si="0"/>
-        <v>1.6016483516483515</v>
-      </c>
-      <c r="J17">
-        <f t="shared" si="0"/>
-        <v>1.8461538461538465</v>
-      </c>
-      <c r="K17">
-        <f t="shared" si="0"/>
-        <v>1.671703296703297</v>
-      </c>
-      <c r="L17">
-        <f t="shared" si="0"/>
-        <v>1.9093406593406599</v>
-      </c>
-      <c r="M17">
-        <f t="shared" si="0"/>
-        <v>0.89560439560439609</v>
-      </c>
-      <c r="N17">
-        <f t="shared" si="0"/>
-        <v>1.9505494505494514</v>
-      </c>
-      <c r="O17">
-        <f t="shared" si="0"/>
-        <v>2.5231862264892282</v>
-      </c>
-      <c r="P17">
-        <f t="shared" si="0"/>
-        <v>3.1037651926187451</v>
-      </c>
-      <c r="Q17">
-        <f t="shared" si="0"/>
-        <v>4.2595837323909533</v>
-      </c>
-      <c r="R17">
-        <f t="shared" si="0"/>
-        <v>5.5205706406765271</v>
-      </c>
-      <c r="S17">
-        <f t="shared" si="0"/>
-        <v>7.1515304042995291</v>
-      </c>
-      <c r="T17">
-        <f t="shared" si="0"/>
-        <v>8.2340807604537929</v>
-      </c>
-      <c r="U17">
-        <f t="shared" si="0"/>
-        <v>8.9056022901293073</v>
-      </c>
-      <c r="V17">
-        <f t="shared" si="0"/>
-        <v>10.381660664279639</v>
-      </c>
-      <c r="W17">
-        <f t="shared" si="0"/>
-        <v>11.158021994533632</v>
-      </c>
-      <c r="X17">
-        <f t="shared" si="0"/>
-        <v>12.667385707353857</v>
-      </c>
-      <c r="Y17">
-        <f t="shared" si="0"/>
-        <v>14.077171137239191</v>
-      </c>
-      <c r="Z17">
-        <f t="shared" si="0"/>
-        <v>14.623032118944936</v>
-      </c>
-      <c r="AA17">
-        <f t="shared" si="0"/>
-        <v>15.51774799092483</v>
-      </c>
-      <c r="AB17">
-        <f t="shared" si="0"/>
-        <v>16.765632902853618</v>
-      </c>
-      <c r="AC17">
-        <f t="shared" si="0"/>
-        <v>17.468459765677682</v>
-      </c>
-      <c r="AD17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AE17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AF17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AG17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AH17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AI17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AJ17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AK17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AL17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AM17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AN17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AO17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AP17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AQ17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
-      </c>
-      <c r="AR17">
-        <f t="shared" si="0"/>
-        <v>18.212454463631964</v>
+      <c r="D15">
+        <v>0.12225274725274726</v>
+      </c>
+      <c r="E15">
+        <v>-1.4687882496940086E-2</v>
+      </c>
+      <c r="F15">
+        <v>0.11925465838509308</v>
+      </c>
+      <c r="G15">
+        <v>3.1076581576027218E-2</v>
+      </c>
+      <c r="H15">
+        <v>-0.18945102260495195</v>
+      </c>
+      <c r="I15">
+        <v>0.54847277556440899</v>
+      </c>
+      <c r="J15">
+        <v>0.15265866209262469</v>
+      </c>
+      <c r="K15">
+        <v>-9.4494047619047672E-2</v>
+      </c>
+      <c r="L15">
+        <v>0.14215283483977004</v>
+      </c>
+      <c r="M15">
+        <v>-0.53093525179856105</v>
+      </c>
+      <c r="N15">
+        <v>1.1779141104294477</v>
+      </c>
+      <c r="O15">
+        <v>0.29357716400292766</v>
+      </c>
+      <c r="P15">
+        <v>0.23009754889845646</v>
+      </c>
+      <c r="Q15">
+        <v>0.37239239054582196</v>
+      </c>
+      <c r="R15">
+        <v>0.29603524370156409</v>
+      </c>
+      <c r="S15">
+        <v>0.29543318431718024</v>
+      </c>
+      <c r="T15">
+        <v>0.15137324390083418</v>
+      </c>
+      <c r="U15">
+        <v>8.1553915878583849E-2</v>
+      </c>
+      <c r="V15">
+        <v>0.1657449239324722</v>
+      </c>
+      <c r="W15">
+        <v>7.4781998310273545E-2</v>
+      </c>
+      <c r="X15">
+        <v>0.13527162014554817</v>
+      </c>
+      <c r="Y15">
+        <v>0.111292532054732</v>
+      </c>
+      <c r="Z15">
+        <v>3.8776326321823706E-2</v>
+      </c>
+      <c r="AA15">
+        <v>6.1185386498655125E-2</v>
+      </c>
+      <c r="AB15">
+        <v>8.041662441345121E-2</v>
+      </c>
+      <c r="AC15">
+        <v>4.192068780800029E-2</v>
+      </c>
+      <c r="AD15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AE15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AF15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AG15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AH15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AI15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AJ15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AK15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AL15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AM15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AN15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AO15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AP15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AQ15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AR15" s="3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AS15" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>353</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18">
-        <f t="shared" ref="D18:S20" si="1">(1+D12)*C18</f>
-        <v>1.1222527472527473</v>
-      </c>
-      <c r="E18">
-        <f t="shared" si="1"/>
-        <v>1.1057692307692306</v>
-      </c>
-      <c r="F18">
-        <f t="shared" si="1"/>
-        <v>1.2376373626373625</v>
-      </c>
-      <c r="G18">
-        <f t="shared" si="1"/>
-        <v>1.2760989010989017</v>
-      </c>
-      <c r="H18">
-        <f t="shared" si="1"/>
-        <v>1.0343406593406592</v>
-      </c>
-      <c r="I18">
-        <f t="shared" si="1"/>
-        <v>1.6016483516483515</v>
-      </c>
-      <c r="J18">
-        <f t="shared" si="1"/>
-        <v>1.8461538461538465</v>
-      </c>
-      <c r="K18">
-        <f t="shared" si="1"/>
-        <v>1.671703296703297</v>
-      </c>
-      <c r="L18">
-        <f t="shared" si="1"/>
-        <v>1.9093406593406599</v>
-      </c>
-      <c r="M18">
-        <f t="shared" si="1"/>
-        <v>0.89560439560439609</v>
-      </c>
-      <c r="N18">
-        <f t="shared" si="1"/>
-        <v>1.9505494505494514</v>
-      </c>
-      <c r="O18">
-        <f t="shared" si="1"/>
-        <v>2.5231862264892282</v>
-      </c>
-      <c r="P18">
-        <f t="shared" si="1"/>
-        <v>3.1037651926187451</v>
-      </c>
-      <c r="Q18">
-        <f t="shared" si="1"/>
-        <v>4.2595837323909533</v>
-      </c>
-      <c r="R18">
-        <f t="shared" si="1"/>
-        <v>5.5205706406765271</v>
-      </c>
-      <c r="S18">
-        <f t="shared" si="1"/>
-        <v>7.1515304042995291</v>
-      </c>
-      <c r="T18">
-        <f t="shared" si="0"/>
-        <v>8.2340807604537929</v>
-      </c>
-      <c r="U18">
-        <f t="shared" si="0"/>
-        <v>8.9056022901293073</v>
-      </c>
-      <c r="V18">
-        <f t="shared" si="0"/>
-        <v>10.381660664279639</v>
-      </c>
-      <c r="W18">
-        <f t="shared" si="0"/>
-        <v>11.158021994533632</v>
-      </c>
-      <c r="X18">
-        <f t="shared" si="0"/>
-        <v>12.667385707353857</v>
-      </c>
-      <c r="Y18">
-        <f t="shared" si="0"/>
-        <v>14.077171137239191</v>
-      </c>
-      <c r="Z18">
-        <f t="shared" si="0"/>
-        <v>14.623032118944936</v>
-      </c>
-      <c r="AA18">
-        <f t="shared" si="0"/>
-        <v>15.51774799092483</v>
-      </c>
-      <c r="AB18">
-        <f t="shared" si="0"/>
-        <v>16.765632902853618</v>
-      </c>
-      <c r="AC18">
-        <f t="shared" si="0"/>
-        <v>17.468459765677682</v>
-      </c>
-      <c r="AD18">
-        <f t="shared" si="0"/>
-        <v>18.836941314735437</v>
-      </c>
-      <c r="AE18">
-        <f t="shared" si="0"/>
-        <v>20.614596693441005</v>
-      </c>
-      <c r="AF18">
-        <f t="shared" si="0"/>
-        <v>22.648829512186477</v>
-      </c>
-      <c r="AG18">
-        <f t="shared" si="0"/>
-        <v>24.6890147053807</v>
-      </c>
-      <c r="AH18">
-        <f t="shared" si="0"/>
-        <v>26.860155524439921</v>
-      </c>
-      <c r="AI18">
-        <f t="shared" si="0"/>
-        <v>29.222225487996671</v>
-      </c>
-      <c r="AJ18">
-        <f t="shared" si="0"/>
-        <v>31.792014818913756</v>
-      </c>
-      <c r="AK18">
-        <f t="shared" si="0"/>
-        <v>34.587790264680578</v>
-      </c>
-      <c r="AL18">
-        <f t="shared" si="0"/>
-        <v>37.629424942322899</v>
-      </c>
-      <c r="AM18">
-        <f t="shared" si="0"/>
-        <v>40.938539601815449</v>
-      </c>
-      <c r="AN18">
-        <f t="shared" si="0"/>
-        <v>44.538656312135316</v>
-      </c>
-      <c r="AO18">
-        <f t="shared" si="0"/>
-        <v>48.455365662397561</v>
-      </c>
-      <c r="AP18">
-        <f t="shared" si="0"/>
-        <v>52.716508666583309</v>
-      </c>
-      <c r="AQ18">
-        <f t="shared" si="0"/>
-        <v>57.35237466488757</v>
-      </c>
-      <c r="AR18">
-        <f t="shared" si="0"/>
-        <v>62.39591662842237</v>
+        <v>369</v>
       </c>
     </row>
     <row r="19" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
       <c r="D19">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="D19:AR19" si="0">(1+D11)*C19</f>
         <v>1.1222527472527473</v>
       </c>
       <c r="E19">
@@ -14267,596 +14066,756 @@
       </c>
       <c r="AD19">
         <f t="shared" si="0"/>
-        <v>18.799915394810874</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AE19">
         <f t="shared" si="0"/>
-        <v>20.053804532120097</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AF19">
         <f t="shared" si="0"/>
-        <v>21.181297272277327</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AG19">
         <f t="shared" si="0"/>
-        <v>22.195675968057021</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AH19">
         <f t="shared" si="0"/>
-        <v>23.212622420071288</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AI19">
         <f t="shared" si="0"/>
-        <v>24.276162636012941</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AJ19">
         <f t="shared" si="0"/>
-        <v>25.388431417407293</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AK19">
         <f t="shared" si="0"/>
-        <v>26.551661376670392</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AL19">
         <f t="shared" si="0"/>
-        <v>27.768187418542183</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AM19">
         <f t="shared" si="0"/>
-        <v>29.040451426846936</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AN19">
         <f t="shared" si="0"/>
-        <v>30.371007165988495</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AO19">
         <f t="shared" si="0"/>
-        <v>31.762525407018916</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AP19">
         <f t="shared" si="0"/>
-        <v>33.217799288569843</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AQ19">
         <f t="shared" si="0"/>
-        <v>34.739749923407402</v>
+        <v>18.212454463631964</v>
       </c>
       <c r="AR19">
         <f t="shared" si="0"/>
-        <v>36.331432261864457</v>
+        <v>18.212454463631964</v>
       </c>
     </row>
     <row r="20" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>355</v>
+      <c r="A20" s="3" t="s">
+        <v>353</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
       <c r="D20">
+        <f t="shared" ref="D20:AR20" si="1">(1+D12)*C20</f>
+        <v>1.1222527472527473</v>
+      </c>
+      <c r="E20">
         <f t="shared" si="1"/>
+        <v>1.1057692307692306</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="1"/>
+        <v>1.2376373626373625</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="1"/>
+        <v>1.2760989010989017</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="1"/>
+        <v>1.0343406593406592</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="1"/>
+        <v>1.6016483516483515</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="1"/>
+        <v>1.8461538461538465</v>
+      </c>
+      <c r="K20">
+        <f t="shared" si="1"/>
+        <v>1.671703296703297</v>
+      </c>
+      <c r="L20">
+        <f t="shared" si="1"/>
+        <v>1.9093406593406599</v>
+      </c>
+      <c r="M20">
+        <f t="shared" si="1"/>
+        <v>0.89560439560439609</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="1"/>
+        <v>1.9505494505494514</v>
+      </c>
+      <c r="O20">
+        <f t="shared" si="1"/>
+        <v>2.5231862264892282</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="1"/>
+        <v>3.1037651926187451</v>
+      </c>
+      <c r="Q20">
+        <f t="shared" si="1"/>
+        <v>4.2595837323909533</v>
+      </c>
+      <c r="R20">
+        <f t="shared" si="1"/>
+        <v>5.5205706406765271</v>
+      </c>
+      <c r="S20">
+        <f t="shared" si="1"/>
+        <v>7.1515304042995291</v>
+      </c>
+      <c r="T20">
+        <f t="shared" si="1"/>
+        <v>8.2340807604537929</v>
+      </c>
+      <c r="U20">
+        <f t="shared" si="1"/>
+        <v>8.9056022901293073</v>
+      </c>
+      <c r="V20">
+        <f t="shared" si="1"/>
+        <v>10.381660664279639</v>
+      </c>
+      <c r="W20">
+        <f t="shared" si="1"/>
+        <v>11.158021994533632</v>
+      </c>
+      <c r="X20">
+        <f t="shared" si="1"/>
+        <v>12.667385707353857</v>
+      </c>
+      <c r="Y20">
+        <f t="shared" si="1"/>
+        <v>14.077171137239191</v>
+      </c>
+      <c r="Z20">
+        <f t="shared" si="1"/>
+        <v>14.623032118944936</v>
+      </c>
+      <c r="AA20">
+        <f t="shared" si="1"/>
+        <v>15.51774799092483</v>
+      </c>
+      <c r="AB20">
+        <f t="shared" si="1"/>
+        <v>16.765632902853618</v>
+      </c>
+      <c r="AC20">
+        <f t="shared" si="1"/>
+        <v>17.468459765677682</v>
+      </c>
+      <c r="AD20">
+        <f t="shared" si="1"/>
+        <v>18.836941314735437</v>
+      </c>
+      <c r="AE20">
+        <f t="shared" si="1"/>
+        <v>20.614596693441005</v>
+      </c>
+      <c r="AF20">
+        <f t="shared" si="1"/>
+        <v>22.648829512186477</v>
+      </c>
+      <c r="AG20">
+        <f t="shared" si="1"/>
+        <v>24.6890147053807</v>
+      </c>
+      <c r="AH20">
+        <f t="shared" si="1"/>
+        <v>26.860155524439921</v>
+      </c>
+      <c r="AI20">
+        <f t="shared" si="1"/>
+        <v>29.222225487996671</v>
+      </c>
+      <c r="AJ20">
+        <f t="shared" si="1"/>
+        <v>31.792014818913756</v>
+      </c>
+      <c r="AK20">
+        <f t="shared" si="1"/>
+        <v>34.587790264680578</v>
+      </c>
+      <c r="AL20">
+        <f t="shared" si="1"/>
+        <v>37.629424942322899</v>
+      </c>
+      <c r="AM20">
+        <f t="shared" si="1"/>
+        <v>40.938539601815449</v>
+      </c>
+      <c r="AN20">
+        <f t="shared" si="1"/>
+        <v>44.538656312135316</v>
+      </c>
+      <c r="AO20">
+        <f t="shared" si="1"/>
+        <v>48.455365662397561</v>
+      </c>
+      <c r="AP20">
+        <f t="shared" si="1"/>
+        <v>52.716508666583309</v>
+      </c>
+      <c r="AQ20">
+        <f t="shared" si="1"/>
+        <v>57.35237466488757</v>
+      </c>
+      <c r="AR20">
+        <f t="shared" si="1"/>
+        <v>62.39591662842237</v>
+      </c>
+    </row>
+    <row r="21" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <f t="shared" ref="D21:AR21" si="2">(1+D13)*C21</f>
         <v>1.1222527472527473</v>
       </c>
-      <c r="E20">
-        <f t="shared" si="0"/>
+      <c r="E21">
+        <f t="shared" si="2"/>
         <v>1.1057692307692306</v>
       </c>
-      <c r="F20">
-        <f t="shared" si="0"/>
+      <c r="F21">
+        <f t="shared" si="2"/>
         <v>1.2376373626373625</v>
       </c>
-      <c r="G20">
-        <f t="shared" si="0"/>
+      <c r="G21">
+        <f t="shared" si="2"/>
         <v>1.2760989010989017</v>
       </c>
-      <c r="H20">
-        <f t="shared" si="0"/>
+      <c r="H21">
+        <f t="shared" si="2"/>
         <v>1.0343406593406592</v>
       </c>
-      <c r="I20">
-        <f t="shared" si="0"/>
+      <c r="I21">
+        <f t="shared" si="2"/>
         <v>1.6016483516483515</v>
       </c>
-      <c r="J20">
-        <f t="shared" si="0"/>
+      <c r="J21">
+        <f t="shared" si="2"/>
         <v>1.8461538461538465</v>
       </c>
-      <c r="K20">
-        <f t="shared" si="0"/>
+      <c r="K21">
+        <f t="shared" si="2"/>
         <v>1.671703296703297</v>
       </c>
-      <c r="L20">
-        <f t="shared" si="0"/>
+      <c r="L21">
+        <f t="shared" si="2"/>
         <v>1.9093406593406599</v>
       </c>
-      <c r="M20">
-        <f t="shared" si="0"/>
+      <c r="M21">
+        <f t="shared" si="2"/>
         <v>0.89560439560439609</v>
       </c>
-      <c r="N20">
-        <f t="shared" si="0"/>
+      <c r="N21">
+        <f t="shared" si="2"/>
         <v>1.9505494505494514</v>
       </c>
-      <c r="O20">
-        <f t="shared" si="0"/>
+      <c r="O21">
+        <f t="shared" si="2"/>
         <v>2.5231862264892282</v>
       </c>
-      <c r="P20">
-        <f t="shared" si="0"/>
+      <c r="P21">
+        <f t="shared" si="2"/>
         <v>3.1037651926187451</v>
       </c>
-      <c r="Q20">
-        <f t="shared" si="0"/>
+      <c r="Q21">
+        <f t="shared" si="2"/>
         <v>4.2595837323909533</v>
       </c>
-      <c r="R20">
-        <f t="shared" si="0"/>
+      <c r="R21">
+        <f t="shared" si="2"/>
         <v>5.5205706406765271</v>
       </c>
-      <c r="S20">
-        <f t="shared" si="0"/>
+      <c r="S21">
+        <f t="shared" si="2"/>
         <v>7.1515304042995291</v>
       </c>
-      <c r="T20">
-        <f t="shared" si="0"/>
+      <c r="T21">
+        <f t="shared" si="2"/>
         <v>8.2340807604537929</v>
       </c>
-      <c r="U20">
-        <f t="shared" si="0"/>
+      <c r="U21">
+        <f t="shared" si="2"/>
         <v>8.9056022901293073</v>
       </c>
-      <c r="V20">
-        <f t="shared" si="0"/>
+      <c r="V21">
+        <f t="shared" si="2"/>
         <v>10.381660664279639</v>
       </c>
-      <c r="W20">
-        <f t="shared" si="0"/>
+      <c r="W21">
+        <f t="shared" si="2"/>
         <v>11.158021994533632</v>
       </c>
-      <c r="X20">
-        <f t="shared" si="0"/>
+      <c r="X21">
+        <f t="shared" si="2"/>
         <v>12.667385707353857</v>
       </c>
-      <c r="Y20">
-        <f t="shared" si="0"/>
+      <c r="Y21">
+        <f t="shared" si="2"/>
         <v>14.077171137239191</v>
       </c>
-      <c r="Z20">
-        <f t="shared" si="0"/>
+      <c r="Z21">
+        <f t="shared" si="2"/>
         <v>14.623032118944936</v>
       </c>
-      <c r="AA20">
-        <f t="shared" si="0"/>
+      <c r="AA21">
+        <f t="shared" si="2"/>
         <v>15.51774799092483</v>
       </c>
-      <c r="AB20">
-        <f t="shared" si="0"/>
+      <c r="AB21">
+        <f t="shared" si="2"/>
         <v>16.765632902853618</v>
       </c>
-      <c r="AC20">
-        <f t="shared" si="0"/>
+      <c r="AC21">
+        <f t="shared" si="2"/>
         <v>17.468459765677682</v>
       </c>
-      <c r="AD20">
-        <f t="shared" si="0"/>
+      <c r="AD21">
+        <f t="shared" si="2"/>
+        <v>18.799915394810874</v>
+      </c>
+      <c r="AE21">
+        <f t="shared" si="2"/>
+        <v>20.053804532120097</v>
+      </c>
+      <c r="AF21">
+        <f t="shared" si="2"/>
+        <v>21.181297272277327</v>
+      </c>
+      <c r="AG21">
+        <f t="shared" si="2"/>
+        <v>22.195675968057021</v>
+      </c>
+      <c r="AH21">
+        <f t="shared" si="2"/>
+        <v>23.212622420071288</v>
+      </c>
+      <c r="AI21">
+        <f t="shared" si="2"/>
+        <v>24.276162636012941</v>
+      </c>
+      <c r="AJ21">
+        <f t="shared" si="2"/>
+        <v>25.388431417407293</v>
+      </c>
+      <c r="AK21">
+        <f t="shared" si="2"/>
+        <v>26.551661376670392</v>
+      </c>
+      <c r="AL21">
+        <f t="shared" si="2"/>
+        <v>27.768187418542183</v>
+      </c>
+      <c r="AM21">
+        <f t="shared" si="2"/>
+        <v>29.040451426846936</v>
+      </c>
+      <c r="AN21">
+        <f t="shared" si="2"/>
+        <v>30.371007165988495</v>
+      </c>
+      <c r="AO21">
+        <f t="shared" si="2"/>
+        <v>31.762525407018916</v>
+      </c>
+      <c r="AP21">
+        <f t="shared" si="2"/>
+        <v>33.217799288569843</v>
+      </c>
+      <c r="AQ21">
+        <f t="shared" si="2"/>
+        <v>34.739749923407402</v>
+      </c>
+      <c r="AR21">
+        <f t="shared" si="2"/>
+        <v>36.331432261864457</v>
+      </c>
+    </row>
+    <row r="22" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>355</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <f t="shared" ref="D22:AR22" si="3">(1+D14)*C22</f>
+        <v>1.1222527472527473</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="3"/>
+        <v>1.1057692307692306</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="3"/>
+        <v>1.2376373626373625</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="3"/>
+        <v>1.2760989010989017</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="3"/>
+        <v>1.0343406593406592</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="3"/>
+        <v>1.6016483516483515</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="3"/>
+        <v>1.8461538461538465</v>
+      </c>
+      <c r="K22">
+        <f t="shared" si="3"/>
+        <v>1.671703296703297</v>
+      </c>
+      <c r="L22">
+        <f t="shared" si="3"/>
+        <v>1.9093406593406599</v>
+      </c>
+      <c r="M22">
+        <f t="shared" si="3"/>
+        <v>0.89560439560439609</v>
+      </c>
+      <c r="N22">
+        <f t="shared" si="3"/>
+        <v>1.9505494505494514</v>
+      </c>
+      <c r="O22">
+        <f t="shared" si="3"/>
+        <v>2.5231862264892282</v>
+      </c>
+      <c r="P22">
+        <f t="shared" si="3"/>
+        <v>3.1037651926187451</v>
+      </c>
+      <c r="Q22">
+        <f t="shared" si="3"/>
+        <v>4.2595837323909533</v>
+      </c>
+      <c r="R22">
+        <f t="shared" si="3"/>
+        <v>5.5205706406765271</v>
+      </c>
+      <c r="S22">
+        <f t="shared" si="3"/>
+        <v>7.1515304042995291</v>
+      </c>
+      <c r="T22">
+        <f t="shared" si="3"/>
+        <v>8.2340807604537929</v>
+      </c>
+      <c r="U22">
+        <f t="shared" si="3"/>
+        <v>8.9056022901293073</v>
+      </c>
+      <c r="V22">
+        <f t="shared" si="3"/>
+        <v>10.381660664279639</v>
+      </c>
+      <c r="W22">
+        <f t="shared" si="3"/>
+        <v>11.158021994533632</v>
+      </c>
+      <c r="X22">
+        <f t="shared" si="3"/>
+        <v>12.667385707353857</v>
+      </c>
+      <c r="Y22">
+        <f t="shared" si="3"/>
+        <v>14.077171137239191</v>
+      </c>
+      <c r="Z22">
+        <f t="shared" si="3"/>
+        <v>14.623032118944936</v>
+      </c>
+      <c r="AA22">
+        <f t="shared" si="3"/>
+        <v>15.51774799092483</v>
+      </c>
+      <c r="AB22">
+        <f t="shared" si="3"/>
+        <v>16.765632902853618</v>
+      </c>
+      <c r="AC22">
+        <f t="shared" si="3"/>
+        <v>17.468459765677682</v>
+      </c>
+      <c r="AD22">
+        <f t="shared" si="3"/>
         <v>18.818428354773157</v>
       </c>
-      <c r="AE20">
-        <f t="shared" si="0"/>
+      <c r="AE22">
+        <f t="shared" si="3"/>
         <v>20.332878951738923</v>
       </c>
-      <c r="AF20">
-        <f t="shared" si="0"/>
+      <c r="AF22">
+        <f t="shared" si="3"/>
         <v>21.904497864247048</v>
       </c>
-      <c r="AG20">
-        <f t="shared" si="0"/>
+      <c r="AG22">
+        <f t="shared" si="3"/>
         <v>23.412153046022741</v>
       </c>
-      <c r="AH20">
-        <f t="shared" si="0"/>
+      <c r="AH22">
+        <f t="shared" si="3"/>
         <v>24.974270621332423</v>
       </c>
-      <c r="AI20">
-        <f t="shared" si="0"/>
+      <c r="AI22">
+        <f t="shared" si="3"/>
         <v>26.640616599484613</v>
       </c>
-      <c r="AJ20">
-        <f t="shared" si="0"/>
+      <c r="AJ22">
+        <f t="shared" si="3"/>
         <v>28.418145360950291</v>
       </c>
-      <c r="AK20">
-        <f t="shared" si="0"/>
+      <c r="AK22">
+        <f t="shared" si="3"/>
         <v>30.314275299908942</v>
       </c>
-      <c r="AL20">
-        <f t="shared" si="0"/>
+      <c r="AL22">
+        <f t="shared" si="3"/>
         <v>32.336919784407065</v>
       </c>
-      <c r="AM20">
-        <f t="shared" si="0"/>
+      <c r="AM22">
+        <f t="shared" si="3"/>
         <v>34.494520182256117</v>
       </c>
-      <c r="AN20">
-        <f t="shared" si="0"/>
+      <c r="AN22">
+        <f t="shared" si="3"/>
         <v>36.79608109050119</v>
       </c>
-      <c r="AO20">
-        <f t="shared" si="0"/>
+      <c r="AO22">
+        <f t="shared" si="3"/>
         <v>39.251207915488216</v>
       </c>
-      <c r="AP20">
-        <f t="shared" si="0"/>
+      <c r="AP22">
+        <f t="shared" si="3"/>
         <v>41.870146960367506</v>
       </c>
-      <c r="AQ20">
-        <f t="shared" si="0"/>
+      <c r="AQ22">
+        <f t="shared" si="3"/>
         <v>44.663828187336101</v>
       </c>
-      <c r="AR20">
-        <f t="shared" si="0"/>
+      <c r="AR22">
+        <f t="shared" si="3"/>
         <v>47.643910833084149</v>
       </c>
     </row>
     <row r="23" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="B23" t="s">
-        <v>0</v>
-      </c>
-      <c r="C23" t="s">
+        <v>374</v>
+      </c>
+      <c r="C23">
         <v>1</v>
       </c>
       <c r="D23">
-        <f t="shared" ref="D23:W26" si="2">D17/$X17</f>
-        <v>8.8593871946382796E-2</v>
+        <f>(1+D15)*C23</f>
+        <v>1.1222527472527473</v>
       </c>
       <c r="E23">
-        <f t="shared" si="2"/>
-        <v>8.7292615565285364E-2</v>
+        <f t="shared" ref="E23:AR23" si="4">(1+E15)*D23</f>
+        <v>1.1057692307692306</v>
       </c>
       <c r="F23">
-        <f t="shared" si="2"/>
-        <v>9.7702666614064737E-2</v>
+        <f t="shared" si="4"/>
+        <v>1.2376373626373625</v>
       </c>
       <c r="G23">
-        <f t="shared" si="2"/>
-        <v>0.10073893150329211</v>
+        <f t="shared" si="4"/>
+        <v>1.2760989010989017</v>
       </c>
       <c r="H23">
-        <f t="shared" si="2"/>
-        <v>8.16538379138632E-2</v>
+        <f t="shared" si="4"/>
+        <v>1.0343406593406592</v>
       </c>
       <c r="I23">
-        <f t="shared" si="2"/>
-        <v>0.12643874502996613</v>
+        <f t="shared" si="4"/>
+        <v>1.6016483516483515</v>
       </c>
       <c r="J23">
-        <f t="shared" si="2"/>
-        <v>0.14574071468291125</v>
+        <f t="shared" si="4"/>
+        <v>1.8461538461538465</v>
       </c>
       <c r="K23">
-        <f t="shared" si="2"/>
-        <v>0.1319690846496302</v>
+        <f t="shared" si="4"/>
+        <v>1.671703296703297</v>
       </c>
       <c r="L23">
-        <f t="shared" si="2"/>
-        <v>0.15072886414378472</v>
+        <f t="shared" si="4"/>
+        <v>1.9093406593406599</v>
       </c>
       <c r="M23">
-        <f t="shared" si="2"/>
-        <v>7.0701596706293293E-2</v>
+        <f t="shared" si="4"/>
+        <v>0.89560439560439609</v>
       </c>
       <c r="N23">
-        <f t="shared" si="2"/>
-        <v>0.15398200509652832</v>
+        <f t="shared" si="4"/>
+        <v>1.9505494505494514</v>
       </c>
       <c r="O23">
-        <f t="shared" si="2"/>
-        <v>0.19918760546025144</v>
+        <f t="shared" si="4"/>
+        <v>2.5231862264892282</v>
       </c>
       <c r="P23">
-        <f t="shared" si="2"/>
-        <v>0.2450201852476081</v>
+        <f t="shared" si="4"/>
+        <v>3.1037651926187451</v>
       </c>
       <c r="Q23">
-        <f t="shared" si="2"/>
-        <v>0.33626383776394503</v>
+        <f t="shared" si="4"/>
+        <v>4.2595837323909533</v>
       </c>
       <c r="R23">
-        <f t="shared" si="2"/>
-        <v>0.43580978492441769</v>
+        <f t="shared" si="4"/>
+        <v>5.5205706406765271</v>
       </c>
       <c r="S23">
-        <f t="shared" si="2"/>
-        <v>0.56456245744122391</v>
+        <f t="shared" si="4"/>
+        <v>7.1515304042995291</v>
       </c>
       <c r="T23">
-        <f t="shared" si="2"/>
-        <v>0.65002210800872851</v>
+        <f t="shared" si="4"/>
+        <v>8.2340807604537929</v>
       </c>
       <c r="U23">
-        <f t="shared" si="2"/>
-        <v>0.70303395632449217</v>
+        <f t="shared" si="4"/>
+        <v>8.9056022901293073</v>
       </c>
       <c r="V23">
-        <f t="shared" si="2"/>
-        <v>0.81955826593744008</v>
+        <f t="shared" si="4"/>
+        <v>10.381660664279639</v>
       </c>
       <c r="W23">
-        <f t="shared" si="2"/>
-        <v>0.88084647079594436</v>
+        <f t="shared" si="4"/>
+        <v>11.158021994533632</v>
       </c>
       <c r="X23">
-        <f>X17/$X17</f>
-        <v>1</v>
+        <f t="shared" si="4"/>
+        <v>12.667385707353857</v>
       </c>
       <c r="Y23">
-        <f t="shared" ref="Y23:AR23" si="3">Y17/$X17</f>
-        <v>1.111292532054732</v>
+        <f t="shared" si="4"/>
+        <v>14.077171137239191</v>
       </c>
       <c r="Z23">
-        <f t="shared" si="3"/>
-        <v>1.1543843739166921</v>
+        <f t="shared" si="4"/>
+        <v>14.623032118944936</v>
       </c>
       <c r="AA23">
-        <f t="shared" si="3"/>
-        <v>1.225015828002793</v>
+        <f t="shared" si="4"/>
+        <v>15.51774799092483</v>
       </c>
       <c r="AB23">
-        <f t="shared" si="3"/>
-        <v>1.3235274657438263</v>
+        <f t="shared" si="4"/>
+        <v>16.765632902853618</v>
       </c>
       <c r="AC23">
-        <f t="shared" si="3"/>
-        <v>1.3790106474405872</v>
+        <f t="shared" si="4"/>
+        <v>17.468459765677682</v>
       </c>
       <c r="AD23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>17.905171259819621</v>
       </c>
       <c r="AE23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>18.352800541315109</v>
       </c>
       <c r="AF23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>18.811620554847984</v>
       </c>
       <c r="AG23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>19.281911068719182</v>
       </c>
       <c r="AH23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>19.763958845437159</v>
       </c>
       <c r="AI23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>20.258057816573086</v>
       </c>
       <c r="AJ23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>20.76450926198741</v>
       </c>
       <c r="AK23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>21.283621993537093</v>
       </c>
       <c r="AL23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>21.815712543375518</v>
       </c>
       <c r="AM23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>22.361105356959904</v>
       </c>
       <c r="AN23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>22.9201329908839</v>
       </c>
       <c r="AO23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>23.493136315655995</v>
       </c>
       <c r="AP23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>24.080464723547394</v>
       </c>
       <c r="AQ23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
+        <f t="shared" si="4"/>
+        <v>24.682476341636075</v>
       </c>
       <c r="AR23">
-        <f t="shared" si="3"/>
-        <v>1.4377437368990038</v>
-      </c>
-      <c r="AS23" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="B24" t="s">
-        <v>0</v>
-      </c>
-      <c r="C24" t="s">
-        <v>1</v>
-      </c>
-      <c r="D24">
-        <f t="shared" si="2"/>
-        <v>8.8593871946382796E-2</v>
-      </c>
-      <c r="E24">
-        <f t="shared" si="2"/>
-        <v>8.7292615565285364E-2</v>
-      </c>
-      <c r="F24">
-        <f t="shared" si="2"/>
-        <v>9.7702666614064737E-2</v>
-      </c>
-      <c r="G24">
-        <f t="shared" si="2"/>
-        <v>0.10073893150329211</v>
-      </c>
-      <c r="H24">
-        <f t="shared" si="2"/>
-        <v>8.16538379138632E-2</v>
-      </c>
-      <c r="I24">
-        <f t="shared" si="2"/>
-        <v>0.12643874502996613</v>
-      </c>
-      <c r="J24">
-        <f t="shared" si="2"/>
-        <v>0.14574071468291125</v>
-      </c>
-      <c r="K24">
-        <f t="shared" si="2"/>
-        <v>0.1319690846496302</v>
-      </c>
-      <c r="L24">
-        <f t="shared" si="2"/>
-        <v>0.15072886414378472</v>
-      </c>
-      <c r="M24">
-        <f t="shared" si="2"/>
-        <v>7.0701596706293293E-2</v>
-      </c>
-      <c r="N24">
-        <f t="shared" si="2"/>
-        <v>0.15398200509652832</v>
-      </c>
-      <c r="O24">
-        <f t="shared" si="2"/>
-        <v>0.19918760546025144</v>
-      </c>
-      <c r="P24">
-        <f t="shared" si="2"/>
-        <v>0.2450201852476081</v>
-      </c>
-      <c r="Q24">
-        <f t="shared" si="2"/>
-        <v>0.33626383776394503</v>
-      </c>
-      <c r="R24">
-        <f t="shared" si="2"/>
-        <v>0.43580978492441769</v>
-      </c>
-      <c r="S24">
-        <f t="shared" si="2"/>
-        <v>0.56456245744122391</v>
-      </c>
-      <c r="T24">
-        <f t="shared" si="2"/>
-        <v>0.65002210800872851</v>
-      </c>
-      <c r="U24">
-        <f t="shared" si="2"/>
-        <v>0.70303395632449217</v>
-      </c>
-      <c r="V24">
-        <f t="shared" si="2"/>
-        <v>0.81955826593744008</v>
-      </c>
-      <c r="W24">
-        <f t="shared" si="2"/>
-        <v>0.88084647079594436</v>
-      </c>
-      <c r="X24">
-        <f t="shared" ref="X24:AM26" si="4">X18/$X18</f>
-        <v>1</v>
-      </c>
-      <c r="Y24">
         <f t="shared" si="4"/>
-        <v>1.111292532054732</v>
-      </c>
-      <c r="Z24">
-        <f t="shared" si="4"/>
-        <v>1.1543843739166921</v>
-      </c>
-      <c r="AA24">
-        <f t="shared" si="4"/>
-        <v>1.225015828002793</v>
-      </c>
-      <c r="AB24">
-        <f t="shared" si="4"/>
-        <v>1.3235274657438263</v>
-      </c>
-      <c r="AC24">
-        <f t="shared" si="4"/>
-        <v>1.3790106474405872</v>
-      </c>
-      <c r="AD24">
-        <f t="shared" si="4"/>
-        <v>1.4870425318935334</v>
-      </c>
-      <c r="AE24">
-        <f t="shared" si="4"/>
-        <v>1.6273757797927884</v>
-      </c>
-      <c r="AF24">
-        <f t="shared" si="4"/>
-        <v>1.7879639915786292</v>
-      </c>
-      <c r="AG24">
-        <f t="shared" si="4"/>
-        <v>1.9490221009886728</v>
-      </c>
-      <c r="AH24">
-        <f t="shared" si="4"/>
-        <v>2.1204182255890944</v>
-      </c>
-      <c r="AI24">
-        <f t="shared" si="4"/>
-        <v>2.3068868480914855</v>
-      </c>
-      <c r="AJ24">
-        <f t="shared" si="4"/>
-        <v>2.5097534371640227</v>
-      </c>
-      <c r="AK24">
-        <f t="shared" si="4"/>
-        <v>2.7304600225918096</v>
-      </c>
-      <c r="AL24">
-        <f t="shared" si="4"/>
-        <v>2.9705754456089322</v>
-      </c>
-      <c r="AM24">
-        <f t="shared" si="4"/>
-        <v>3.2318065106400926</v>
-      </c>
-      <c r="AN24">
-        <f t="shared" ref="AN24:AR24" si="5">AN18/$X18</f>
-        <v>3.5160101177213767</v>
-      </c>
-      <c r="AO24">
-        <f t="shared" si="5"/>
-        <v>3.8252064618406258</v>
-      </c>
-      <c r="AP24">
-        <f t="shared" si="5"/>
-        <v>4.1615933930218567</v>
-      </c>
-      <c r="AQ24">
-        <f t="shared" si="5"/>
-        <v>4.5275620392290197</v>
-      </c>
-      <c r="AR24">
-        <f t="shared" si="5"/>
-        <v>4.9257138031408783</v>
-      </c>
-      <c r="AS24" t="s">
-        <v>46</v>
+        <v>25.299538250176976</v>
       </c>
     </row>
     <row r="25" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B25" t="s">
         <v>0</v>
@@ -14865,176 +14824,176 @@
         <v>1</v>
       </c>
       <c r="D25">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D25:AR25" si="5">D19/$X19</f>
         <v>8.8593871946382796E-2</v>
       </c>
       <c r="E25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>8.7292615565285364E-2</v>
       </c>
       <c r="F25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>9.7702666614064737E-2</v>
       </c>
       <c r="G25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.10073893150329211</v>
       </c>
       <c r="H25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>8.16538379138632E-2</v>
       </c>
       <c r="I25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.12643874502996613</v>
       </c>
       <c r="J25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.14574071468291125</v>
       </c>
       <c r="K25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.1319690846496302</v>
       </c>
       <c r="L25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.15072886414378472</v>
       </c>
       <c r="M25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>7.0701596706293293E-2</v>
       </c>
       <c r="N25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.15398200509652832</v>
       </c>
       <c r="O25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.19918760546025144</v>
       </c>
       <c r="P25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.2450201852476081</v>
       </c>
       <c r="Q25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.33626383776394503</v>
       </c>
       <c r="R25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.43580978492441769</v>
       </c>
       <c r="S25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.56456245744122391</v>
       </c>
       <c r="T25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.65002210800872851</v>
       </c>
       <c r="U25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.70303395632449217</v>
       </c>
       <c r="V25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.81955826593744008</v>
       </c>
       <c r="W25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.88084647079594436</v>
       </c>
       <c r="X25">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="Y25">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1.111292532054732</v>
       </c>
       <c r="Z25">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1.1543843739166921</v>
       </c>
       <c r="AA25">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1.225015828002793</v>
       </c>
       <c r="AB25">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1.3235274657438263</v>
       </c>
       <c r="AC25">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1.3790106474405872</v>
       </c>
       <c r="AD25">
-        <f t="shared" si="4"/>
-        <v>1.4841195988764178</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AE25">
-        <f t="shared" si="4"/>
-        <v>1.5831052275039015</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AF25">
-        <f t="shared" si="4"/>
-        <v>1.672112759618652</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AG25">
-        <f t="shared" si="4"/>
-        <v>1.75219074249643</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AH25">
-        <f t="shared" si="4"/>
-        <v>1.8324714314647856</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AI25">
-        <f t="shared" si="4"/>
-        <v>1.9164303666793525</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AJ25">
-        <f t="shared" si="4"/>
-        <v>2.0042360755359669</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AK25">
-        <f t="shared" si="4"/>
-        <v>2.0960648069045718</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AL25">
-        <f t="shared" si="4"/>
-        <v>2.1921008849064876</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AM25">
-        <f t="shared" si="4"/>
-        <v>2.2925370789008142</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AN25">
-        <f t="shared" ref="AN25:AR25" si="6">AN19/$X19</f>
-        <v>2.3975749904226151</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AO25">
-        <f t="shared" si="6"/>
-        <v>2.5074254578495756</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AP25">
-        <f t="shared" si="6"/>
-        <v>2.6223089796094041</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AQ25">
-        <f t="shared" si="6"/>
-        <v>2.7424561567774615</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AR25">
-        <f t="shared" si="6"/>
-        <v>2.8681081559530313</v>
+        <f t="shared" si="5"/>
+        <v>1.4377437368990038</v>
       </c>
       <c r="AS25" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>373</v>
+      <c r="A26" s="3" t="s">
+        <v>371</v>
       </c>
       <c r="B26" t="s">
         <v>0</v>
@@ -15043,170 +15002,704 @@
         <v>1</v>
       </c>
       <c r="D26">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D26:AR26" si="6">D20/$X20</f>
         <v>8.8593871946382796E-2</v>
       </c>
       <c r="E26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>8.7292615565285364E-2</v>
       </c>
       <c r="F26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>9.7702666614064737E-2</v>
       </c>
       <c r="G26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.10073893150329211</v>
       </c>
       <c r="H26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>8.16538379138632E-2</v>
       </c>
       <c r="I26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.12643874502996613</v>
       </c>
       <c r="J26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.14574071468291125</v>
       </c>
       <c r="K26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.1319690846496302</v>
       </c>
       <c r="L26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.15072886414378472</v>
       </c>
       <c r="M26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>7.0701596706293293E-2</v>
       </c>
       <c r="N26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.15398200509652832</v>
       </c>
       <c r="O26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.19918760546025144</v>
       </c>
       <c r="P26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.2450201852476081</v>
       </c>
       <c r="Q26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.33626383776394503</v>
       </c>
       <c r="R26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.43580978492441769</v>
       </c>
       <c r="S26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.56456245744122391</v>
       </c>
       <c r="T26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.65002210800872851</v>
       </c>
       <c r="U26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.70303395632449217</v>
       </c>
       <c r="V26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.81955826593744008</v>
       </c>
       <c r="W26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0.88084647079594436</v>
       </c>
       <c r="X26">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="Y26">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.111292532054732</v>
       </c>
       <c r="Z26">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.1543843739166921</v>
       </c>
       <c r="AA26">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.225015828002793</v>
       </c>
       <c r="AB26">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.3235274657438263</v>
       </c>
       <c r="AC26">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.3790106474405872</v>
       </c>
       <c r="AD26">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
+        <v>1.4870425318935334</v>
+      </c>
+      <c r="AE26">
+        <f t="shared" si="6"/>
+        <v>1.6273757797927884</v>
+      </c>
+      <c r="AF26">
+        <f t="shared" si="6"/>
+        <v>1.7879639915786292</v>
+      </c>
+      <c r="AG26">
+        <f t="shared" si="6"/>
+        <v>1.9490221009886728</v>
+      </c>
+      <c r="AH26">
+        <f t="shared" si="6"/>
+        <v>2.1204182255890944</v>
+      </c>
+      <c r="AI26">
+        <f t="shared" si="6"/>
+        <v>2.3068868480914855</v>
+      </c>
+      <c r="AJ26">
+        <f t="shared" si="6"/>
+        <v>2.5097534371640227</v>
+      </c>
+      <c r="AK26">
+        <f t="shared" si="6"/>
+        <v>2.7304600225918096</v>
+      </c>
+      <c r="AL26">
+        <f t="shared" si="6"/>
+        <v>2.9705754456089322</v>
+      </c>
+      <c r="AM26">
+        <f t="shared" si="6"/>
+        <v>3.2318065106400926</v>
+      </c>
+      <c r="AN26">
+        <f t="shared" si="6"/>
+        <v>3.5160101177213767</v>
+      </c>
+      <c r="AO26">
+        <f t="shared" si="6"/>
+        <v>3.8252064618406258</v>
+      </c>
+      <c r="AP26">
+        <f t="shared" si="6"/>
+        <v>4.1615933930218567</v>
+      </c>
+      <c r="AQ26">
+        <f t="shared" si="6"/>
+        <v>4.5275620392290197</v>
+      </c>
+      <c r="AR26">
+        <f t="shared" si="6"/>
+        <v>4.9257138031408783</v>
+      </c>
+      <c r="AS26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="B27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <f t="shared" ref="D27:AR27" si="7">D21/$X21</f>
+        <v>8.8593871946382796E-2</v>
+      </c>
+      <c r="E27">
+        <f t="shared" si="7"/>
+        <v>8.7292615565285364E-2</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="7"/>
+        <v>9.7702666614064737E-2</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="7"/>
+        <v>0.10073893150329211</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="7"/>
+        <v>8.16538379138632E-2</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="7"/>
+        <v>0.12643874502996613</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="7"/>
+        <v>0.14574071468291125</v>
+      </c>
+      <c r="K27">
+        <f t="shared" si="7"/>
+        <v>0.1319690846496302</v>
+      </c>
+      <c r="L27">
+        <f t="shared" si="7"/>
+        <v>0.15072886414378472</v>
+      </c>
+      <c r="M27">
+        <f t="shared" si="7"/>
+        <v>7.0701596706293293E-2</v>
+      </c>
+      <c r="N27">
+        <f t="shared" si="7"/>
+        <v>0.15398200509652832</v>
+      </c>
+      <c r="O27">
+        <f t="shared" si="7"/>
+        <v>0.19918760546025144</v>
+      </c>
+      <c r="P27">
+        <f t="shared" si="7"/>
+        <v>0.2450201852476081</v>
+      </c>
+      <c r="Q27">
+        <f t="shared" si="7"/>
+        <v>0.33626383776394503</v>
+      </c>
+      <c r="R27">
+        <f t="shared" si="7"/>
+        <v>0.43580978492441769</v>
+      </c>
+      <c r="S27">
+        <f t="shared" si="7"/>
+        <v>0.56456245744122391</v>
+      </c>
+      <c r="T27">
+        <f t="shared" si="7"/>
+        <v>0.65002210800872851</v>
+      </c>
+      <c r="U27">
+        <f t="shared" si="7"/>
+        <v>0.70303395632449217</v>
+      </c>
+      <c r="V27">
+        <f t="shared" si="7"/>
+        <v>0.81955826593744008</v>
+      </c>
+      <c r="W27">
+        <f t="shared" si="7"/>
+        <v>0.88084647079594436</v>
+      </c>
+      <c r="X27">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="Y27">
+        <f t="shared" si="7"/>
+        <v>1.111292532054732</v>
+      </c>
+      <c r="Z27">
+        <f t="shared" si="7"/>
+        <v>1.1543843739166921</v>
+      </c>
+      <c r="AA27">
+        <f t="shared" si="7"/>
+        <v>1.225015828002793</v>
+      </c>
+      <c r="AB27">
+        <f t="shared" si="7"/>
+        <v>1.3235274657438263</v>
+      </c>
+      <c r="AC27">
+        <f t="shared" si="7"/>
+        <v>1.3790106474405872</v>
+      </c>
+      <c r="AD27">
+        <f t="shared" si="7"/>
+        <v>1.4841195988764178</v>
+      </c>
+      <c r="AE27">
+        <f t="shared" si="7"/>
+        <v>1.5831052275039015</v>
+      </c>
+      <c r="AF27">
+        <f t="shared" si="7"/>
+        <v>1.672112759618652</v>
+      </c>
+      <c r="AG27">
+        <f t="shared" si="7"/>
+        <v>1.75219074249643</v>
+      </c>
+      <c r="AH27">
+        <f t="shared" si="7"/>
+        <v>1.8324714314647856</v>
+      </c>
+      <c r="AI27">
+        <f t="shared" si="7"/>
+        <v>1.9164303666793525</v>
+      </c>
+      <c r="AJ27">
+        <f t="shared" si="7"/>
+        <v>2.0042360755359669</v>
+      </c>
+      <c r="AK27">
+        <f t="shared" si="7"/>
+        <v>2.0960648069045718</v>
+      </c>
+      <c r="AL27">
+        <f t="shared" si="7"/>
+        <v>2.1921008849064876</v>
+      </c>
+      <c r="AM27">
+        <f t="shared" si="7"/>
+        <v>2.2925370789008142</v>
+      </c>
+      <c r="AN27">
+        <f t="shared" si="7"/>
+        <v>2.3975749904226151</v>
+      </c>
+      <c r="AO27">
+        <f t="shared" si="7"/>
+        <v>2.5074254578495756</v>
+      </c>
+      <c r="AP27">
+        <f t="shared" si="7"/>
+        <v>2.6223089796094041</v>
+      </c>
+      <c r="AQ27">
+        <f t="shared" si="7"/>
+        <v>2.7424561567774615</v>
+      </c>
+      <c r="AR27">
+        <f t="shared" si="7"/>
+        <v>2.8681081559530313</v>
+      </c>
+      <c r="AS27" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>373</v>
+      </c>
+      <c r="B28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <f t="shared" ref="D28:AR28" si="8">D22/$X22</f>
+        <v>8.8593871946382796E-2</v>
+      </c>
+      <c r="E28">
+        <f t="shared" si="8"/>
+        <v>8.7292615565285364E-2</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="8"/>
+        <v>9.7702666614064737E-2</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="8"/>
+        <v>0.10073893150329211</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="8"/>
+        <v>8.16538379138632E-2</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="8"/>
+        <v>0.12643874502996613</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="8"/>
+        <v>0.14574071468291125</v>
+      </c>
+      <c r="K28">
+        <f t="shared" si="8"/>
+        <v>0.1319690846496302</v>
+      </c>
+      <c r="L28">
+        <f t="shared" si="8"/>
+        <v>0.15072886414378472</v>
+      </c>
+      <c r="M28">
+        <f t="shared" si="8"/>
+        <v>7.0701596706293293E-2</v>
+      </c>
+      <c r="N28">
+        <f t="shared" si="8"/>
+        <v>0.15398200509652832</v>
+      </c>
+      <c r="O28">
+        <f t="shared" si="8"/>
+        <v>0.19918760546025144</v>
+      </c>
+      <c r="P28">
+        <f t="shared" si="8"/>
+        <v>0.2450201852476081</v>
+      </c>
+      <c r="Q28">
+        <f t="shared" si="8"/>
+        <v>0.33626383776394503</v>
+      </c>
+      <c r="R28">
+        <f t="shared" si="8"/>
+        <v>0.43580978492441769</v>
+      </c>
+      <c r="S28">
+        <f t="shared" si="8"/>
+        <v>0.56456245744122391</v>
+      </c>
+      <c r="T28">
+        <f t="shared" si="8"/>
+        <v>0.65002210800872851</v>
+      </c>
+      <c r="U28">
+        <f t="shared" si="8"/>
+        <v>0.70303395632449217</v>
+      </c>
+      <c r="V28">
+        <f t="shared" si="8"/>
+        <v>0.81955826593744008</v>
+      </c>
+      <c r="W28">
+        <f t="shared" si="8"/>
+        <v>0.88084647079594436</v>
+      </c>
+      <c r="X28">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="Y28">
+        <f t="shared" si="8"/>
+        <v>1.111292532054732</v>
+      </c>
+      <c r="Z28">
+        <f t="shared" si="8"/>
+        <v>1.1543843739166921</v>
+      </c>
+      <c r="AA28">
+        <f t="shared" si="8"/>
+        <v>1.225015828002793</v>
+      </c>
+      <c r="AB28">
+        <f t="shared" si="8"/>
+        <v>1.3235274657438263</v>
+      </c>
+      <c r="AC28">
+        <f t="shared" si="8"/>
+        <v>1.3790106474405872</v>
+      </c>
+      <c r="AD28">
+        <f t="shared" si="8"/>
         <v>1.4855810653849757</v>
       </c>
-      <c r="AE26">
-        <f t="shared" si="4"/>
+      <c r="AE28">
+        <f t="shared" si="8"/>
         <v>1.605136167909925</v>
       </c>
-      <c r="AF26">
-        <f t="shared" si="4"/>
+      <c r="AF28">
+        <f t="shared" si="8"/>
         <v>1.7292043023155699</v>
       </c>
-      <c r="AG26">
-        <f t="shared" si="4"/>
+      <c r="AG28">
+        <f t="shared" si="8"/>
         <v>1.8482229551462361</v>
       </c>
-      <c r="AH26">
-        <f t="shared" si="4"/>
+      <c r="AH28">
+        <f t="shared" si="8"/>
         <v>1.9715410265619364</v>
       </c>
-      <c r="AI26">
-        <f t="shared" si="4"/>
+      <c r="AI28">
+        <f t="shared" si="8"/>
         <v>2.1030871890179212</v>
       </c>
-      <c r="AJ26">
-        <f t="shared" si="4"/>
+      <c r="AJ28">
+        <f t="shared" si="8"/>
         <v>2.2434104413867</v>
       </c>
-      <c r="AK26">
-        <f t="shared" si="4"/>
+      <c r="AK28">
+        <f t="shared" si="8"/>
         <v>2.3930964131225951</v>
       </c>
-      <c r="AL26">
-        <f t="shared" si="4"/>
+      <c r="AL28">
+        <f t="shared" si="8"/>
         <v>2.5527698083460395</v>
       </c>
-      <c r="AM26">
-        <f t="shared" si="4"/>
+      <c r="AM28">
+        <f t="shared" si="8"/>
         <v>2.7230970130033105</v>
       </c>
-      <c r="AN26">
-        <f t="shared" ref="AN26:AR26" si="7">AN20/$X20</f>
+      <c r="AN28">
+        <f t="shared" si="8"/>
         <v>2.9047888759824994</v>
       </c>
-      <c r="AO26">
-        <f t="shared" si="7"/>
+      <c r="AO28">
+        <f t="shared" si="8"/>
         <v>3.0986036757925142</v>
       </c>
-      <c r="AP26">
-        <f t="shared" si="7"/>
+      <c r="AP28">
+        <f t="shared" si="8"/>
         <v>3.3053502851863454</v>
       </c>
-      <c r="AQ26">
-        <f t="shared" si="7"/>
+      <c r="AQ28">
+        <f t="shared" si="8"/>
         <v>3.5258915469359398</v>
       </c>
-      <c r="AR26">
-        <f t="shared" si="7"/>
+      <c r="AR28">
+        <f t="shared" si="8"/>
         <v>3.7611478748472313</v>
       </c>
-      <c r="AS26" t="s">
+      <c r="AS28" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="B29" t="s">
+        <v>0</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1</v>
+      </c>
+      <c r="D29">
+        <f>D23/$X23</f>
+        <v>8.8593871946382796E-2</v>
+      </c>
+      <c r="E29">
+        <f t="shared" ref="E29:AR29" si="9">E23/$X23</f>
+        <v>8.7292615565285364E-2</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="9"/>
+        <v>9.7702666614064737E-2</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="9"/>
+        <v>0.10073893150329211</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="9"/>
+        <v>8.16538379138632E-2</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="9"/>
+        <v>0.12643874502996613</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="9"/>
+        <v>0.14574071468291125</v>
+      </c>
+      <c r="K29">
+        <f t="shared" si="9"/>
+        <v>0.1319690846496302</v>
+      </c>
+      <c r="L29">
+        <f t="shared" si="9"/>
+        <v>0.15072886414378472</v>
+      </c>
+      <c r="M29">
+        <f t="shared" si="9"/>
+        <v>7.0701596706293293E-2</v>
+      </c>
+      <c r="N29">
+        <f t="shared" si="9"/>
+        <v>0.15398200509652832</v>
+      </c>
+      <c r="O29">
+        <f t="shared" si="9"/>
+        <v>0.19918760546025144</v>
+      </c>
+      <c r="P29">
+        <f t="shared" si="9"/>
+        <v>0.2450201852476081</v>
+      </c>
+      <c r="Q29">
+        <f t="shared" si="9"/>
+        <v>0.33626383776394503</v>
+      </c>
+      <c r="R29">
+        <f t="shared" si="9"/>
+        <v>0.43580978492441769</v>
+      </c>
+      <c r="S29">
+        <f t="shared" si="9"/>
+        <v>0.56456245744122391</v>
+      </c>
+      <c r="T29">
+        <f t="shared" si="9"/>
+        <v>0.65002210800872851</v>
+      </c>
+      <c r="U29">
+        <f t="shared" si="9"/>
+        <v>0.70303395632449217</v>
+      </c>
+      <c r="V29">
+        <f t="shared" si="9"/>
+        <v>0.81955826593744008</v>
+      </c>
+      <c r="W29">
+        <f t="shared" si="9"/>
+        <v>0.88084647079594436</v>
+      </c>
+      <c r="X29">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="Y29">
+        <f t="shared" si="9"/>
+        <v>1.111292532054732</v>
+      </c>
+      <c r="Z29">
+        <f t="shared" si="9"/>
+        <v>1.1543843739166921</v>
+      </c>
+      <c r="AA29">
+        <f t="shared" si="9"/>
+        <v>1.225015828002793</v>
+      </c>
+      <c r="AB29">
+        <f t="shared" si="9"/>
+        <v>1.3235274657438263</v>
+      </c>
+      <c r="AC29">
+        <f t="shared" si="9"/>
+        <v>1.3790106474405872</v>
+      </c>
+      <c r="AD29">
+        <f t="shared" si="9"/>
+        <v>1.4134859136266016</v>
+      </c>
+      <c r="AE29">
+        <f t="shared" si="9"/>
+        <v>1.4488230614672664</v>
+      </c>
+      <c r="AF29">
+        <f t="shared" si="9"/>
+        <v>1.4850436380039478</v>
+      </c>
+      <c r="AG29">
+        <f t="shared" si="9"/>
+        <v>1.5221697289540466</v>
+      </c>
+      <c r="AH29">
+        <f t="shared" si="9"/>
+        <v>1.5602239721778974</v>
+      </c>
+      <c r="AI29">
+        <f t="shared" si="9"/>
+        <v>1.5992295714823446</v>
+      </c>
+      <c r="AJ29">
+        <f t="shared" si="9"/>
+        <v>1.6392103107694029</v>
+      </c>
+      <c r="AK29">
+        <f t="shared" si="9"/>
+        <v>1.680190568538638</v>
+      </c>
+      <c r="AL29">
+        <f t="shared" si="9"/>
+        <v>1.7221953327521038</v>
+      </c>
+      <c r="AM29">
+        <f t="shared" si="9"/>
+        <v>1.765250216070906</v>
+      </c>
+      <c r="AN29">
+        <f t="shared" si="9"/>
+        <v>1.8093814714726786</v>
+      </c>
+      <c r="AO29">
+        <f t="shared" si="9"/>
+        <v>1.8546160082594956</v>
+      </c>
+      <c r="AP29">
+        <f t="shared" si="9"/>
+        <v>1.9009814084659828</v>
+      </c>
+      <c r="AQ29">
+        <f t="shared" si="9"/>
+        <v>1.948505943677632</v>
+      </c>
+      <c r="AR29">
+        <f t="shared" si="9"/>
+        <v>1.9972185922695729</v>
+      </c>
+      <c r="AS29" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
mig med modified shocks
</commit_message>
<xml_diff>
--- a/all_shocks.xlsx
+++ b/all_shocks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\emanu\OneDrive\Matlab\cdc_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F5F89A3-787D-4A71-89A3-020826AC8D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB8C3A2-4153-4764-8A65-BD990F66725E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15990" tabRatio="805" firstSheet="6" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34107,60 +34107,60 @@
         <v>-81.114524782440284</v>
       </c>
       <c r="AD46">
-        <f>AD9+ABS(AD9*0.3)</f>
-        <v>-64.42730538153296</v>
+        <f>AD9+ABS(AD9*0.5)</f>
+        <v>-46.019503843952116</v>
       </c>
       <c r="AE46">
-        <f t="shared" ref="AE46:AQ46" si="4">AE9+ABS(AE9*0.3)</f>
-        <v>-70.380388859541995</v>
+        <f t="shared" ref="AE46:AQ46" si="4">AE9+ABS(AE9*0.5)</f>
+        <v>-50.271706328244285</v>
       </c>
       <c r="AF46">
         <f t="shared" si="4"/>
-        <v>-76.861643235532384</v>
+        <v>-54.901173739665985</v>
       </c>
       <c r="AG46">
         <f t="shared" si="4"/>
-        <v>-83.906231026322828</v>
+        <v>-59.93302216165916</v>
       </c>
       <c r="AH46">
         <f t="shared" si="4"/>
-        <v>-91.564730703860363</v>
+        <v>-65.403379074185978</v>
       </c>
       <c r="AI46">
         <f t="shared" si="4"/>
-        <v>-99.875183758332895</v>
+        <v>-71.339416970237778</v>
       </c>
       <c r="AJ46">
         <f t="shared" si="4"/>
-        <v>-108.89793604728482</v>
+        <v>-77.784240033774864</v>
       </c>
       <c r="AK46">
         <f t="shared" si="4"/>
-        <v>-118.69616811316295</v>
+        <v>-84.782977223687823</v>
       </c>
       <c r="AL46">
         <f t="shared" si="4"/>
-        <v>-129.33426544722511</v>
+        <v>-92.38161817658937</v>
       </c>
       <c r="AM46">
         <f t="shared" si="4"/>
-        <v>-140.85087113675098</v>
+        <v>-100.60776509767928</v>
       </c>
       <c r="AN46">
         <f t="shared" si="4"/>
-        <v>-153.33643929531871</v>
+        <v>-109.5260280680848</v>
       </c>
       <c r="AO46">
         <f t="shared" si="4"/>
-        <v>-166.84016460373556</v>
+        <v>-119.17154614552538</v>
       </c>
       <c r="AP46">
         <f t="shared" si="4"/>
-        <v>-181.48921874776644</v>
+        <v>-129.6351562484046</v>
       </c>
       <c r="AQ46">
         <f t="shared" si="4"/>
-        <v>-197.37715065999669</v>
+        <v>-140.98367904285476</v>
       </c>
       <c r="AR46" t="s">
         <v>46</v>
@@ -34255,60 +34255,60 @@
         <v>-40.463689809324435</v>
       </c>
       <c r="AD47">
-        <f t="shared" ref="AD46:AQ48" si="5">AD10+ABS(AD10*0.3)</f>
-        <v>-32.113119980104543</v>
+        <f>AD10+ABS(AD10*0.5)</f>
+        <v>-22.937942842931818</v>
       </c>
       <c r="AE47">
-        <f t="shared" si="5"/>
-        <v>-35.018954526465777</v>
+        <f t="shared" ref="AE47:AQ47" si="5">AE10+ABS(AE10*0.5)</f>
+        <v>-25.013538947475553</v>
       </c>
       <c r="AF47">
         <f t="shared" si="5"/>
-        <v>-38.171812818597459</v>
+        <v>-27.265580584712474</v>
       </c>
       <c r="AG47">
         <f t="shared" si="5"/>
-        <v>-41.592575174886342</v>
+        <v>-29.708982267775959</v>
       </c>
       <c r="AH47">
         <f t="shared" si="5"/>
-        <v>-45.299427103980889</v>
+        <v>-32.356733645700636</v>
       </c>
       <c r="AI47">
         <f t="shared" si="5"/>
-        <v>-49.319785602930068</v>
+        <v>-35.228418287807195</v>
       </c>
       <c r="AJ47">
         <f t="shared" si="5"/>
-        <v>-53.675486708134798</v>
+        <v>-38.339633362953428</v>
       </c>
       <c r="AK47">
         <f t="shared" si="5"/>
-        <v>-58.387515256526328</v>
+        <v>-41.705368040375951</v>
       </c>
       <c r="AL47">
         <f t="shared" si="5"/>
-        <v>-63.495783196731438</v>
+        <v>-45.354130854808169</v>
       </c>
       <c r="AM47">
         <f t="shared" si="5"/>
-        <v>-69.015708788180859</v>
+        <v>-49.296934848700609</v>
       </c>
       <c r="AN47">
         <f t="shared" si="5"/>
-        <v>-74.985599357878996</v>
+        <v>-53.561142398484996</v>
       </c>
       <c r="AO47">
         <f t="shared" si="5"/>
-        <v>-81.442531016803372</v>
+        <v>-58.173236440573838</v>
       </c>
       <c r="AP47">
         <f t="shared" si="5"/>
-        <v>-88.423218147484477</v>
+        <v>-63.15944153391748</v>
       </c>
       <c r="AQ47">
         <f t="shared" si="5"/>
-        <v>-95.976800295666663</v>
+        <v>-68.554857354047613</v>
       </c>
       <c r="AR47" t="s">
         <v>46</v>
@@ -34403,60 +34403,60 @@
         <v>-23.674200109742657</v>
       </c>
       <c r="AD48">
-        <f t="shared" si="5"/>
-        <v>-18.711627670570714</v>
+        <f t="shared" ref="AD48:AL49" si="6">AD11+ABS(AD11*0.5)</f>
+        <v>-13.36544833612194</v>
       </c>
       <c r="AE48">
-        <f t="shared" si="5"/>
-        <v>-20.408489212667874</v>
+        <f t="shared" ref="AE48:AQ48" si="7">AE11+ABS(AE11*0.5)</f>
+        <v>-14.577492294762767</v>
       </c>
       <c r="AF48">
-        <f t="shared" si="5"/>
-        <v>-22.25066042842186</v>
+        <f t="shared" si="7"/>
+        <v>-15.893328877444187</v>
       </c>
       <c r="AG48">
-        <f t="shared" si="5"/>
-        <v>-24.250205630003769</v>
+        <f t="shared" si="7"/>
+        <v>-17.321575450002694</v>
       </c>
       <c r="AH48">
-        <f t="shared" si="5"/>
-        <v>-26.417265986663836</v>
+        <f>AH11+ABS(AH11*0.5)</f>
+        <v>-18.869475704759882</v>
       </c>
       <c r="AI48">
-        <f t="shared" si="5"/>
-        <v>-28.768160989078311</v>
+        <f t="shared" si="7"/>
+        <v>-20.54868642077022</v>
       </c>
       <c r="AJ48">
-        <f t="shared" si="5"/>
-        <v>-31.316233777229371</v>
+        <f t="shared" si="7"/>
+        <v>-22.368738412306694</v>
       </c>
       <c r="AK48">
-        <f t="shared" si="5"/>
-        <v>-34.072699090209881</v>
+        <f t="shared" si="7"/>
+        <v>-24.33764220729277</v>
       </c>
       <c r="AL48">
-        <f t="shared" si="5"/>
-        <v>-37.060858174449365</v>
+        <f t="shared" si="7"/>
+        <v>-26.472041553178119</v>
       </c>
       <c r="AM48">
-        <f t="shared" si="5"/>
-        <v>-40.291179534158211</v>
+        <f t="shared" si="7"/>
+        <v>-28.779413952970149</v>
       </c>
       <c r="AN48">
-        <f t="shared" si="5"/>
-        <v>-43.7885800046271</v>
+        <f t="shared" si="7"/>
+        <v>-31.277557146162213</v>
       </c>
       <c r="AO48">
-        <f t="shared" si="5"/>
-        <v>-47.570982422628688</v>
+        <f t="shared" si="7"/>
+        <v>-33.979273159020494</v>
       </c>
       <c r="AP48">
-        <f t="shared" si="5"/>
-        <v>-51.656983232176614</v>
+        <f t="shared" si="7"/>
+        <v>-36.897845165840437</v>
       </c>
       <c r="AQ48">
-        <f t="shared" si="5"/>
-        <v>-56.073830500421394</v>
+        <f t="shared" si="7"/>
+        <v>-40.052736071729569</v>
       </c>
       <c r="AR48" t="s">
         <v>46</v>
@@ -34551,60 +34551,60 @@
         <v>-14.303633531713665</v>
       </c>
       <c r="AD49">
-        <f>AD12+ABS(AD12*0.3)</f>
-        <v>-11.511192035150875</v>
+        <f t="shared" si="6"/>
+        <v>-8.2222800251077679</v>
       </c>
       <c r="AE49">
-        <f t="shared" ref="AE49:AQ49" si="6">AE12+ABS(AE12*0.3)</f>
-        <v>-12.552855269892813</v>
+        <f t="shared" ref="AE49:AQ49" si="8">AE12+ABS(AE12*0.5)</f>
+        <v>-8.9663251927805803</v>
       </c>
       <c r="AF49">
-        <f t="shared" si="6"/>
-        <v>-13.68281542918599</v>
+        <f t="shared" si="8"/>
+        <v>-9.7734395922757074</v>
       </c>
       <c r="AG49">
-        <f t="shared" si="6"/>
-        <v>-14.908104868023344</v>
+        <f t="shared" si="8"/>
+        <v>-10.648646334302388</v>
       </c>
       <c r="AH49">
-        <f t="shared" si="6"/>
-        <v>-16.236133699776275</v>
+        <f t="shared" si="8"/>
+        <v>-11.597238356983052</v>
       </c>
       <c r="AI49">
-        <f t="shared" si="6"/>
-        <v>-17.674944566488065</v>
+        <f t="shared" si="8"/>
+        <v>-12.624960404634333</v>
       </c>
       <c r="AJ49">
-        <f t="shared" si="6"/>
-        <v>-19.232872666600585</v>
+        <f t="shared" si="8"/>
+        <v>-13.737766190428989</v>
       </c>
       <c r="AK49">
-        <f t="shared" si="6"/>
-        <v>-20.91848411160332</v>
+        <f t="shared" si="8"/>
+        <v>-14.941774365430941</v>
       </c>
       <c r="AL49">
-        <f t="shared" si="6"/>
-        <v>-22.743815130791688</v>
+        <f t="shared" si="8"/>
+        <v>-16.245582236279777</v>
       </c>
       <c r="AM49">
-        <f t="shared" si="6"/>
-        <v>-24.717249524945068</v>
+        <f t="shared" si="8"/>
+        <v>-17.655178232103619</v>
       </c>
       <c r="AN49">
-        <f t="shared" si="6"/>
-        <v>-26.850070563624115</v>
+        <f t="shared" si="8"/>
+        <v>-19.178621831160083</v>
       </c>
       <c r="AO49">
-        <f t="shared" si="6"/>
-        <v>-29.155277885677464</v>
+        <f t="shared" si="8"/>
+        <v>-20.825198489769615</v>
       </c>
       <c r="AP49">
-        <f t="shared" si="6"/>
-        <v>-31.644584226319552</v>
+        <f t="shared" si="8"/>
+        <v>-22.60327444737111</v>
       </c>
       <c r="AQ49">
-        <f t="shared" si="6"/>
-        <v>-34.332261965911606</v>
+        <f t="shared" si="8"/>
+        <v>-24.523044261365431</v>
       </c>
       <c r="AR49" t="s">
         <v>46</v>
@@ -34699,59 +34699,59 @@
         <v>-8.2871033823576603</v>
       </c>
       <c r="AD50">
-        <f t="shared" ref="AD50:AQ56" si="7">AD13</f>
+        <f t="shared" ref="AD50:AQ56" si="9">AD13</f>
         <v>-9.8188892500974099</v>
       </c>
       <c r="AE50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-10.740632502532307</v>
       </c>
       <c r="AF50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-11.744019990504757</v>
       </c>
       <c r="AG50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-12.836202838172486</v>
       </c>
       <c r="AH50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-14.024181595832932</v>
       </c>
       <c r="AI50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-15.316355941584742</v>
       </c>
       <c r="AJ50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-16.720402635268254</v>
       </c>
       <c r="AK50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-18.246247334054299</v>
       </c>
       <c r="AL50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-19.904203844803195</v>
       </c>
       <c r="AM50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-21.702893831931878</v>
       </c>
       <c r="AN50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-23.654691382574317</v>
       </c>
       <c r="AO50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-25.772634749681988</v>
       </c>
       <c r="AP50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-28.068016479015245</v>
       </c>
       <c r="AQ50">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-30.55693831764194</v>
       </c>
       <c r="AR50" t="s">
@@ -34847,59 +34847,59 @@
         <v>-6.7225750932718054</v>
       </c>
       <c r="AD51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-7.6895421686767325</v>
       </c>
       <c r="AE51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-8.4181083595319226</v>
       </c>
       <c r="AF51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-9.2171052305017032</v>
       </c>
       <c r="AG51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-10.087865534643354</v>
       </c>
       <c r="AH51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-11.036131544691676</v>
       </c>
       <c r="AI51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-12.068651365626467</v>
       </c>
       <c r="AJ51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-13.192259497306354</v>
       </c>
       <c r="AK51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-14.414622186472537</v>
       </c>
       <c r="AL51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-15.743889714564718</v>
       </c>
       <c r="AM51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-17.18816697718546</v>
       </c>
       <c r="AN51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-18.757739142612671</v>
       </c>
       <c r="AO51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-20.461614733836285</v>
       </c>
       <c r="AP51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-22.311076658720495</v>
       </c>
       <c r="AQ51">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-24.317859912008515</v>
       </c>
       <c r="AR51" t="s">
@@ -34995,59 +34995,59 @@
         <v>-4.6974263531520091</v>
       </c>
       <c r="AD52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-5.2098000263997637</v>
       </c>
       <c r="AE52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-5.526172307484881</v>
       </c>
       <c r="AF52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-6.0086706738866429</v>
       </c>
       <c r="AG52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-6.532635693105842</v>
       </c>
       <c r="AH52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-7.0976821647975719</v>
       </c>
       <c r="AI52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-7.706597150850655</v>
       </c>
       <c r="AJ52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-8.3621236554562781</v>
       </c>
       <c r="AK52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-9.0673534568478669</v>
       </c>
       <c r="AL52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-9.8252539768406759</v>
       </c>
       <c r="AM52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-10.638929328201813</v>
       </c>
       <c r="AN52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-11.511989037751521</v>
       </c>
       <c r="AO52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-12.447455599242465</v>
       </c>
       <c r="AP52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-13.449494745072093</v>
       </c>
       <c r="AQ52">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-14.521041973206797</v>
       </c>
       <c r="AR52" t="s">
@@ -35143,59 +35143,59 @@
         <v>-3.1690507996876063</v>
       </c>
       <c r="AD53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-3.5472660784970982</v>
       </c>
       <c r="AE53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-3.6453350918154976</v>
       </c>
       <c r="AF53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-3.8824656701572557</v>
       </c>
       <c r="AG53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-4.2816078320970883</v>
       </c>
       <c r="AH53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-4.7230006935293911</v>
       </c>
       <c r="AI53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-5.2067777308347569</v>
       </c>
       <c r="AJ53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-5.7366755410540318</v>
       </c>
       <c r="AK53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-6.3168363136229804</v>
       </c>
       <c r="AL53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-6.9515820975016105</v>
       </c>
       <c r="AM53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-7.6458078166823817</v>
       </c>
       <c r="AN53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-8.4045814741367284</v>
       </c>
       <c r="AO53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-9.2335337101860873</v>
       </c>
       <c r="AP53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-10.138654976432225</v>
       </c>
       <c r="AQ53">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-11.126366728746675</v>
       </c>
       <c r="AR53" t="s">
@@ -35291,59 +35291,59 @@
         <v>-2.0263907990980918</v>
       </c>
       <c r="AD54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-2.3734000979690371</v>
       </c>
       <c r="AE54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-2.442366779221405</v>
       </c>
       <c r="AF54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-2.5095193910174305</v>
       </c>
       <c r="AG54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-2.707846719428566</v>
       </c>
       <c r="AH54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-3.047714552831744</v>
       </c>
       <c r="AI54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-3.4255940622024075</v>
       </c>
       <c r="AJ54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-3.8421688674402641</v>
       </c>
       <c r="AK54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-4.3010253040712856</v>
       </c>
       <c r="AL54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-4.8061018749316995</v>
       </c>
       <c r="AM54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-5.3616673582833796</v>
       </c>
       <c r="AN54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-5.9723564504634297</v>
       </c>
       <c r="AO54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-6.6432444633498964</v>
       </c>
       <c r="AP54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-7.3798368420703353</v>
       </c>
       <c r="AQ54">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-8.1881206177984076</v>
       </c>
       <c r="AR54" t="s">
@@ -35439,59 +35439,59 @@
         <v>-0.90922570866843833</v>
       </c>
       <c r="AD55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.0679013436454499</v>
       </c>
       <c r="AE55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.133730805701417</v>
       </c>
       <c r="AF55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.170083874581578</v>
       </c>
       <c r="AG55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.2077499756147887</v>
       </c>
       <c r="AH55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.2836076123083824</v>
       </c>
       <c r="AI55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.3905779810379741</v>
       </c>
       <c r="AJ55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.5045892547098407</v>
       </c>
       <c r="AK55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.6255560553774744</v>
       </c>
       <c r="AL55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.7538497427125253</v>
       </c>
       <c r="AM55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.8898546986015747</v>
       </c>
       <c r="AN55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-2.0339784758484845</v>
       </c>
       <c r="AO55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-2.1866478503581641</v>
       </c>
       <c r="AP55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-2.3483098475430744</v>
       </c>
       <c r="AQ55">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-2.5194405582982062</v>
       </c>
       <c r="AR55" t="s">
@@ -35587,59 +35587,59 @@
         <v>-0.33840882647909187</v>
       </c>
       <c r="AD56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.38623460937785792</v>
       </c>
       <c r="AE56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.40393192505171638</v>
       </c>
       <c r="AF56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.41881783081219259</v>
       </c>
       <c r="AG56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.43000395427803073</v>
       </c>
       <c r="AH56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.44139899838699681</v>
       </c>
       <c r="AI56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.45755942734223387</v>
       </c>
       <c r="AJ56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.47740964459108226</v>
       </c>
       <c r="AK56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.49790257564262741</v>
       </c>
       <c r="AL56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.51899460107614681</v>
       </c>
       <c r="AM56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.54070820008819953</v>
       </c>
       <c r="AN56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.56306413253164256</v>
       </c>
       <c r="AO56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.58608377679462653</v>
       </c>
       <c r="AP56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.60978987710909593</v>
       </c>
       <c r="AQ56">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.63420584852182693</v>
       </c>
       <c r="AR56" t="s">
@@ -35739,55 +35739,55 @@
         <v>-0.10354066147586227</v>
       </c>
       <c r="AE57">
-        <f t="shared" ref="AE57:AQ57" si="8">AE20</f>
+        <f t="shared" ref="AE57:AQ57" si="10">AE20</f>
         <v>-0.10921795664419576</v>
       </c>
       <c r="AF57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.11498526638215645</v>
       </c>
       <c r="AG57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.1202055999811098</v>
       </c>
       <c r="AH57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.12417330165217377</v>
       </c>
       <c r="AI57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.12809726705579383</v>
       </c>
       <c r="AJ57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.13305456800708915</v>
       </c>
       <c r="AK57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.13924571485342696</v>
       </c>
       <c r="AL57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.14557859694923714</v>
       </c>
       <c r="AM57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.15202864672132388</v>
       </c>
       <c r="AN57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.15859982700951369</v>
       </c>
       <c r="AO57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.16529648644051242</v>
       </c>
       <c r="AP57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.17212420451542987</v>
       </c>
       <c r="AQ57">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-0.17908722299279622</v>
       </c>
       <c r="AR57" t="s">
@@ -35892,55 +35892,55 @@
         <v>46.218982102423325</v>
       </c>
       <c r="AE60">
-        <f t="shared" ref="AE60:AQ60" si="9">AE23</f>
+        <f t="shared" ref="AE60:AQ60" si="11">AE23</f>
         <v>60.227848101266005</v>
       </c>
       <c r="AF60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>75.553862441209048</v>
       </c>
       <c r="AG60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>92.3275537199506</v>
       </c>
       <c r="AH60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>110.66807169835067</v>
       </c>
       <c r="AI60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>130.7178079685259</v>
       </c>
       <c r="AJ60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>152.63284794105175</v>
       </c>
       <c r="AK60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>176.58194898267573</v>
       </c>
       <c r="AL60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>202.7157033740271</v>
       </c>
       <c r="AM60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>231.2506255761927</v>
       </c>
       <c r="AN60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>262.38633415021343</v>
       </c>
       <c r="AO60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>296.36841897700373</v>
       </c>
       <c r="AP60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>333.36916573202456</v>
       </c>
       <c r="AQ60">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>373.69811320754479</v>
       </c>
       <c r="AR60" t="s">
@@ -36036,59 +36036,59 @@
         <v>-16.512669737099856</v>
       </c>
       <c r="AD61">
-        <f t="shared" ref="AD61:AQ63" si="10">AD24</f>
+        <f t="shared" ref="AD61:AQ63" si="12">AD24</f>
         <v>-17.613132401837788</v>
       </c>
       <c r="AE61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-19.466609869949338</v>
       </c>
       <c r="AF61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-21.519849457660683</v>
       </c>
       <c r="AG61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-23.777006114112055</v>
       </c>
       <c r="AH61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-26.272296653851868</v>
       </c>
       <c r="AI61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-29.013013005407714</v>
       </c>
       <c r="AJ61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-32.03894695851568</v>
       </c>
       <c r="AK61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-35.368309227888489</v>
       </c>
       <c r="AL61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-39.057185233055066</v>
       </c>
       <c r="AM61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-43.072089590886435</v>
       </c>
       <c r="AN61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-47.517032831345659</v>
       </c>
       <c r="AO61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-52.417682326600129</v>
       </c>
       <c r="AP61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-57.814778330324373</v>
       </c>
       <c r="AQ61">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-63.714029572087895</v>
       </c>
       <c r="AR61" t="s">
@@ -36184,59 +36184,59 @@
         <v>-3.6222142908222565</v>
       </c>
       <c r="AD62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-4.527169607882044</v>
       </c>
       <c r="AE62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-5.1188242956962853</v>
       </c>
       <c r="AF62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-5.7826460127012069</v>
       </c>
       <c r="AG62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-6.5300340219898203</v>
       </c>
       <c r="AH62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-7.3696531599472621</v>
       </c>
       <c r="AI62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-8.3116726765060207</v>
       </c>
       <c r="AJ62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-9.3757249833354592</v>
       </c>
       <c r="AK62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-10.557298623333566</v>
       </c>
       <c r="AL62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-11.890936925777027</v>
       </c>
       <c r="AM62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-13.365873365649634</v>
       </c>
       <c r="AN62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-15.045552492273828</v>
       </c>
       <c r="AO62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-16.896967152606521</v>
       </c>
       <c r="AP62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-18.959716566093846</v>
       </c>
       <c r="AQ62">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-21.277737604813638</v>
       </c>
       <c r="AR62" t="s">
@@ -36332,59 +36332,59 @@
         <v>-12.162367860336971</v>
       </c>
       <c r="AD63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-13.368348203119652</v>
       </c>
       <c r="AE63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-14.693840458709545</v>
       </c>
       <c r="AF63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-16.146831599769186</v>
       </c>
       <c r="AG63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-17.738561206162188</v>
       </c>
       <c r="AH63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-19.481633729765605</v>
       </c>
       <c r="AI63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-21.390430052590048</v>
       </c>
       <c r="AJ63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-23.479627326574089</v>
       </c>
       <c r="AK63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-25.76172388017541</v>
       </c>
       <c r="AL63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-28.263580551189094</v>
       </c>
       <c r="AM63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-30.994003391069597</v>
       </c>
       <c r="AN63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-33.981751054910532</v>
       </c>
       <c r="AO63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-37.238802647892683</v>
       </c>
       <c r="AP63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-40.79997062857025</v>
       </c>
       <c r="AQ63">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>-44.68431074038817</v>
       </c>
       <c r="AR63" t="s">
@@ -36480,60 +36480,60 @@
         <v>-13.617884107128326</v>
       </c>
       <c r="AD64">
-        <f>AD27+ABS(AD27*0.3)</f>
-        <v>-11.125400209561827</v>
+        <f>AD27+ABS(AD27*0.5)</f>
+        <v>-7.9467144354013044</v>
       </c>
       <c r="AE64">
-        <f t="shared" ref="AE64:AQ64" si="11">AE27+ABS(AE27*0.3)</f>
-        <v>-12.203448689657012</v>
+        <f t="shared" ref="AE64:AQ64" si="13">AE27+ABS(AE27*0.5)</f>
+        <v>-8.716749064040723</v>
       </c>
       <c r="AF64">
-        <f t="shared" si="11"/>
-        <v>-13.381302890754373</v>
+        <f t="shared" si="13"/>
+        <v>-9.5580734933959803</v>
       </c>
       <c r="AG64">
-        <f t="shared" si="11"/>
-        <v>-14.668956624084903</v>
+        <f t="shared" si="13"/>
+        <v>-10.477826160060644</v>
       </c>
       <c r="AH64">
-        <f t="shared" si="11"/>
-        <v>-16.075332138808339</v>
+        <f t="shared" si="13"/>
+        <v>-11.482380099148813</v>
       </c>
       <c r="AI64">
-        <f t="shared" si="11"/>
-        <v>-17.610869087553084</v>
+        <f t="shared" si="13"/>
+        <v>-12.57919220539506</v>
       </c>
       <c r="AJ64">
-        <f t="shared" si="11"/>
-        <v>-19.287463406339178</v>
+        <f t="shared" si="13"/>
+        <v>-13.776759575956554</v>
       </c>
       <c r="AK64">
-        <f t="shared" si="11"/>
-        <v>-21.115805685246848</v>
+        <f t="shared" si="13"/>
+        <v>-15.082718346604892</v>
       </c>
       <c r="AL64">
-        <f t="shared" si="11"/>
-        <v>-23.110376444616385</v>
+        <f t="shared" si="13"/>
+        <v>-16.50741174615456</v>
       </c>
       <c r="AM64">
-        <f t="shared" si="11"/>
-        <v>-25.285262743356693</v>
+        <f t="shared" si="13"/>
+        <v>-18.060901959540494</v>
       </c>
       <c r="AN64">
-        <f t="shared" si="11"/>
-        <v>-27.653532183041769</v>
+        <f t="shared" si="13"/>
+        <v>-19.752522987886977</v>
       </c>
       <c r="AO64">
-        <f t="shared" si="11"/>
-        <v>-30.23323201035852</v>
+        <f t="shared" si="13"/>
+        <v>-21.595165721684658</v>
       </c>
       <c r="AP64">
-        <f t="shared" si="11"/>
-        <v>-33.043442457888894</v>
+        <f t="shared" si="13"/>
+        <v>-23.602458898492067</v>
       </c>
       <c r="AQ64">
-        <f t="shared" si="11"/>
-        <v>-36.104171704787923</v>
+        <f t="shared" si="13"/>
+        <v>-25.788694074848515</v>
       </c>
       <c r="AR64" t="s">
         <v>46</v>
@@ -36628,60 +36628,60 @@
         <v>-7.3020682104987245</v>
       </c>
       <c r="AD65">
-        <f t="shared" ref="AD65:AQ67" si="12">AD28+ABS(AD28*0.3)</f>
-        <v>-5.9995860667085354</v>
+        <f t="shared" ref="AD65:AQ67" si="14">AD28+ABS(AD28*0.5)</f>
+        <v>-4.2854186190775252</v>
       </c>
       <c r="AE65">
-        <f t="shared" si="12"/>
-        <v>-6.5719870926246724</v>
+        <f t="shared" si="14"/>
+        <v>-4.6942764947319091</v>
       </c>
       <c r="AF65">
-        <f t="shared" si="12"/>
-        <v>-7.1964246098833415</v>
+        <f t="shared" si="14"/>
+        <v>-5.1403032927738153</v>
       </c>
       <c r="AG65">
-        <f t="shared" si="12"/>
-        <v>-7.8779617947601084</v>
+        <f t="shared" si="14"/>
+        <v>-5.6271155676857916</v>
       </c>
       <c r="AH65">
-        <f t="shared" si="12"/>
-        <v>-8.6212050864698533</v>
+        <f t="shared" si="14"/>
+        <v>-6.1580036331927523</v>
       </c>
       <c r="AI65">
-        <f t="shared" si="12"/>
-        <v>-9.4315435326281332</v>
+        <f t="shared" si="14"/>
+        <v>-6.7368168090200946</v>
       </c>
       <c r="AJ65">
-        <f t="shared" si="12"/>
-        <v>-10.314412554297455</v>
+        <f t="shared" si="14"/>
+        <v>-7.3674375387838964</v>
       </c>
       <c r="AK65">
-        <f t="shared" si="12"/>
-        <v>-11.27544794381069</v>
+        <f t="shared" si="14"/>
+        <v>-8.053891388436206</v>
       </c>
       <c r="AL65">
-        <f t="shared" si="12"/>
-        <v>-12.323032010491463</v>
+        <f t="shared" si="14"/>
+        <v>-8.8021657217796161</v>
       </c>
       <c r="AM65">
-        <f t="shared" si="12"/>
-        <v>-13.463054147584682</v>
+        <f t="shared" si="14"/>
+        <v>-9.6164672482747733</v>
       </c>
       <c r="AN65">
-        <f t="shared" si="12"/>
-        <v>-14.701116729916658</v>
+        <f t="shared" si="14"/>
+        <v>-10.500797664226184</v>
       </c>
       <c r="AO65">
-        <f t="shared" si="12"/>
-        <v>-16.050204527855776</v>
+        <f t="shared" si="14"/>
+        <v>-11.46443180561127</v>
       </c>
       <c r="AP65">
-        <f t="shared" si="12"/>
-        <v>-17.515578895562765</v>
+        <f t="shared" si="14"/>
+        <v>-12.511127782544833</v>
       </c>
       <c r="AQ65">
-        <f t="shared" si="12"/>
-        <v>-19.108112003705568</v>
+        <f t="shared" si="14"/>
+        <v>-13.648651431218262</v>
       </c>
       <c r="AR65" t="s">
         <v>46</v>
@@ -36776,60 +36776,60 @@
         <v>-4.8939058071404951</v>
       </c>
       <c r="AD66">
-        <f t="shared" si="12"/>
-        <v>-3.9861955166388734</v>
+        <f t="shared" si="14"/>
+        <v>-2.8472825118849094</v>
       </c>
       <c r="AE66">
-        <f t="shared" si="12"/>
-        <v>-4.3681748100246596</v>
+        <f t="shared" si="14"/>
+        <v>-3.1201248643033281</v>
       </c>
       <c r="AF66">
-        <f t="shared" si="12"/>
-        <v>-4.7853241790547951</v>
+        <f t="shared" si="14"/>
+        <v>-3.4180886993248532</v>
       </c>
       <c r="AG66">
-        <f t="shared" si="12"/>
-        <v>-5.2411105279430767</v>
+        <f t="shared" si="14"/>
+        <v>-3.7436503771021972</v>
       </c>
       <c r="AH66">
-        <f t="shared" si="12"/>
-        <v>-5.7384335159244717</v>
+        <f t="shared" si="14"/>
+        <v>-4.0988810828031941</v>
       </c>
       <c r="AI66">
-        <f t="shared" si="12"/>
-        <v>-6.2812186681000792</v>
+        <f t="shared" si="14"/>
+        <v>-4.4865847629286275</v>
       </c>
       <c r="AJ66">
-        <f t="shared" si="12"/>
-        <v>-6.8730906578598105</v>
+        <f t="shared" si="14"/>
+        <v>-4.9093504698998647</v>
       </c>
       <c r="AK66">
-        <f t="shared" si="12"/>
-        <v>-7.5185283465055264</v>
+        <f t="shared" si="14"/>
+        <v>-5.3703773903610905</v>
       </c>
       <c r="AL66">
-        <f t="shared" si="12"/>
-        <v>-8.2220745178456003</v>
+        <f t="shared" si="14"/>
+        <v>-5.8729103698897145</v>
       </c>
       <c r="AM66">
-        <f t="shared" si="12"/>
-        <v>-8.9880586317162212</v>
+        <f t="shared" si="14"/>
+        <v>-6.4200418797973011</v>
       </c>
       <c r="AN66">
-        <f t="shared" si="12"/>
-        <v>-9.8226445487125673</v>
+        <f t="shared" si="14"/>
+        <v>-7.0161746776518346</v>
       </c>
       <c r="AO66">
-        <f t="shared" si="12"/>
-        <v>-10.730849781936666</v>
+        <f t="shared" si="14"/>
+        <v>-7.6648927013833319</v>
       </c>
       <c r="AP66">
-        <f t="shared" si="12"/>
-        <v>-11.718633799733224</v>
+        <f t="shared" si="14"/>
+        <v>-8.3704527140951601</v>
       </c>
       <c r="AQ66">
-        <f t="shared" si="12"/>
-        <v>-12.792690936671629</v>
+        <f t="shared" si="14"/>
+        <v>-9.1376363833368774</v>
       </c>
       <c r="AR66" t="s">
         <v>46</v>
@@ -36924,60 +36924,60 @@
         <v>-3.3537062556172632</v>
       </c>
       <c r="AD67">
-        <f t="shared" si="12"/>
-        <v>-2.8090416974688903</v>
+        <f t="shared" si="14"/>
+        <v>-2.0064583553349218</v>
       </c>
       <c r="AE67">
-        <f t="shared" si="12"/>
-        <v>-3.077196003977162</v>
+        <f t="shared" si="14"/>
+        <v>-2.1979971456979728</v>
       </c>
       <c r="AF67">
-        <f t="shared" si="12"/>
-        <v>-3.3699680445692941</v>
+        <f t="shared" si="14"/>
+        <v>-2.40712003183521</v>
       </c>
       <c r="AG67">
-        <f t="shared" si="12"/>
-        <v>-3.6894973388705337</v>
+        <f t="shared" si="14"/>
+        <v>-2.6353552420503812</v>
       </c>
       <c r="AH67">
-        <f t="shared" si="12"/>
-        <v>-4.0382090822803018</v>
+        <f t="shared" si="14"/>
+        <v>-2.8844350587716443</v>
       </c>
       <c r="AI67">
-        <f t="shared" si="12"/>
-        <v>-4.4183371265435492</v>
+        <f t="shared" si="14"/>
+        <v>-3.1559550903882494</v>
       </c>
       <c r="AJ67">
-        <f t="shared" si="12"/>
-        <v>-4.8328343322809753</v>
+        <f t="shared" si="14"/>
+        <v>-3.4520245230578395</v>
       </c>
       <c r="AK67">
-        <f t="shared" si="12"/>
-        <v>-5.2843903819303879</v>
+        <f t="shared" si="14"/>
+        <v>-3.774564558521706</v>
       </c>
       <c r="AL67">
-        <f t="shared" si="12"/>
-        <v>-5.7761335448865703</v>
+        <f t="shared" si="14"/>
+        <v>-4.1258096749189788</v>
       </c>
       <c r="AM67">
-        <f t="shared" si="12"/>
-        <v>-6.3118372419458995</v>
+        <f t="shared" si="14"/>
+        <v>-4.5084551728184996</v>
       </c>
       <c r="AN67">
-        <f t="shared" si="12"/>
-        <v>-6.8948777773669692</v>
+        <f t="shared" si="14"/>
+        <v>-4.9249126981192637</v>
       </c>
       <c r="AO67">
-        <f t="shared" si="12"/>
-        <v>-7.5285357236163488</v>
+        <f t="shared" si="14"/>
+        <v>-5.377525516868821</v>
       </c>
       <c r="AP67">
-        <f t="shared" si="12"/>
-        <v>-8.217907504817326</v>
+        <f t="shared" si="14"/>
+        <v>-5.8699339320123753</v>
       </c>
       <c r="AQ67">
-        <f t="shared" si="12"/>
-        <v>-8.9672071226142016</v>
+        <f t="shared" si="14"/>
+        <v>-6.4051479447244288</v>
       </c>
       <c r="AR67" t="s">
         <v>46</v>
@@ -37072,59 +37072,59 @@
         <v>-2.1857990418582016</v>
       </c>
       <c r="AD68">
-        <f t="shared" ref="AD68:AQ74" si="13">AD31</f>
+        <f t="shared" ref="AD68:AQ74" si="15">AD31</f>
         <v>-2.7391311045950744</v>
       </c>
       <c r="AE68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.0073140220590027</v>
       </c>
       <c r="AF68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.3014267183283401</v>
       </c>
       <c r="AG68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.6238535641361018</v>
       </c>
       <c r="AH68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.9772522843465481</v>
       </c>
       <c r="AI68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.3643332907102526</v>
       </c>
       <c r="AJ68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.7883860299325214</v>
       </c>
       <c r="AK68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-5.252490905056117</v>
       </c>
       <c r="AL68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-5.76061125523022</v>
       </c>
       <c r="AM68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-6.3162421087626015</v>
       </c>
       <c r="AN68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-6.9239590989803972</v>
       </c>
       <c r="AO68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-7.5877564963149098</v>
       </c>
       <c r="AP68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-8.3137020731616005</v>
       </c>
       <c r="AQ68">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-9.1063748117293741</v>
       </c>
       <c r="AR68" t="s">
@@ -37220,59 +37220,59 @@
         <v>-2.3874116768859692</v>
       </c>
       <c r="AD69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.8241586164514305</v>
       </c>
       <c r="AE69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.0999290332953016</v>
       </c>
       <c r="AF69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.4042055101680062</v>
       </c>
       <c r="AG69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.7378760800909254</v>
       </c>
       <c r="AH69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.1037353615677539</v>
       </c>
       <c r="AI69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.5047173490731236</v>
       </c>
       <c r="AJ69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.9439456952539746</v>
       </c>
       <c r="AK69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-5.4249753805768162</v>
       </c>
       <c r="AL69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-5.9516445473907158</v>
       </c>
       <c r="AM69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-6.5278860798736336</v>
       </c>
       <c r="AN69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-7.1582453756766942</v>
       </c>
       <c r="AO69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-7.8473073459177503</v>
       </c>
       <c r="AP69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-8.6005805729804319</v>
       </c>
       <c r="AQ69">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-9.4233529580188975</v>
       </c>
       <c r="AR69" t="s">
@@ -37368,59 +37368,59 @@
         <v>-2.6747507563640167</v>
       </c>
       <c r="AD70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.9817799400698184</v>
       </c>
       <c r="AE70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.1704593972444521</v>
       </c>
       <c r="AF70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.4582801246515982</v>
       </c>
       <c r="AG70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.772767170419892</v>
       </c>
       <c r="AH70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.1140577980455966</v>
       </c>
       <c r="AI70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.4841505228258622</v>
       </c>
       <c r="AJ70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.885081480901059</v>
       </c>
       <c r="AK70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-5.3191710659491385</v>
       </c>
       <c r="AL70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-5.7886526227267776</v>
       </c>
       <c r="AM70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-6.2959677141237798</v>
       </c>
       <c r="AN70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-6.8438292176990601</v>
       </c>
       <c r="AO70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-7.4347480959203516</v>
       </c>
       <c r="AP70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-8.0717137381003958</v>
       </c>
       <c r="AQ70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-8.7574228245761141</v>
       </c>
       <c r="AR70" t="s">
@@ -37516,59 +37516,59 @@
         <v>-1.830300481199377</v>
       </c>
       <c r="AD71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.0543390393849768</v>
       </c>
       <c r="AE71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.1146119577730733</v>
       </c>
       <c r="AF71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.2569609104815589</v>
       </c>
       <c r="AG71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.4956924542397108</v>
       </c>
       <c r="AH71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.761390691895274</v>
       </c>
       <c r="AI71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.0545136123852199</v>
       </c>
       <c r="AJ71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.3776538474849609</v>
       </c>
       <c r="AK71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.7336780166992192</v>
       </c>
       <c r="AL71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.1256327362201981</v>
       </c>
       <c r="AM71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.5569369133575464</v>
       </c>
       <c r="AN71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-5.0311963908561834</v>
       </c>
       <c r="AO71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-5.5523495535279865</v>
       </c>
       <c r="AP71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-6.1247609309354152</v>
       </c>
       <c r="AQ71">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-6.753015371419397</v>
       </c>
       <c r="AR71" t="s">
@@ -37664,59 +37664,59 @@
         <v>-1.1943976942555206</v>
       </c>
       <c r="AD72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.3982578254629683</v>
       </c>
       <c r="AE72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.4407990261453469</v>
       </c>
       <c r="AF72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.4825711540987552</v>
       </c>
       <c r="AG72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.6014285051976898</v>
       </c>
       <c r="AH72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.8034666880014294</v>
       </c>
       <c r="AI72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.0286683343083238</v>
       </c>
       <c r="AJ72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.2775765526423588</v>
       </c>
       <c r="AK72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.5524492399814021</v>
       </c>
       <c r="AL72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-2.8557454490458798</v>
       </c>
       <c r="AM72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.1901369519906022</v>
       </c>
       <c r="AN72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.55853422089081</v>
       </c>
       <c r="AO72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-3.9641167944192777</v>
       </c>
       <c r="AP72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.410341236304899</v>
       </c>
       <c r="AQ72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-4.9009633279177161</v>
       </c>
       <c r="AR72" t="s">
@@ -37812,59 +37812,59 @@
         <v>-0.54894672666293554</v>
       </c>
       <c r="AD73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.64243073025627329</v>
       </c>
       <c r="AE73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.68141936538085868</v>
       </c>
       <c r="AF73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.70311931161763486</v>
       </c>
       <c r="AG73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.7257321906850811</v>
       </c>
       <c r="AH73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.77090589092580974</v>
       </c>
       <c r="AI73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.83429413418260778</v>
       </c>
       <c r="AJ73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.90175948810007567</v>
       </c>
       <c r="AK73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.97324990110882315</v>
       </c>
       <c r="AL73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.0489772437645737</v>
       </c>
       <c r="AM73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.1291619348106032</v>
       </c>
       <c r="AN73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.2140368532483292</v>
       </c>
       <c r="AO73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.303844298451049</v>
       </c>
       <c r="AP73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.3988425633218831</v>
       </c>
       <c r="AQ73">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-1.4992987365782582</v>
       </c>
       <c r="AR73" t="s">
@@ -37960,59 +37960,59 @@
         <v>-0.20696018009111428</v>
       </c>
       <c r="AD74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.23549644592518182</v>
       </c>
       <c r="AE74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.24627764271645347</v>
       </c>
       <c r="AF74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.25517829110734436</v>
       </c>
       <c r="AG74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.26170345826377184</v>
       </c>
       <c r="AH74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.26839218912480778</v>
       </c>
       <c r="AI74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.27813864669959409</v>
       </c>
       <c r="AJ74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.29017481641859155</v>
       </c>
       <c r="AK74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.30257470511947204</v>
       </c>
       <c r="AL74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.31531041369346569</v>
       </c>
       <c r="AM74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.32839358458906265</v>
       </c>
       <c r="AN74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.34183510471530232</v>
       </c>
       <c r="AO74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.35564763078833406</v>
       </c>
       <c r="AP74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.36984269038066175</v>
       </c>
       <c r="AQ74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>-0.38443291821286563</v>
       </c>
       <c r="AR74" t="s">
@@ -38112,55 +38112,55 @@
         <v>-5.8844346629341571E-2</v>
       </c>
       <c r="AE75">
-        <f t="shared" ref="AE75:AQ75" si="14">AE38</f>
+        <f t="shared" ref="AE75:AQ75" si="16">AE38</f>
         <v>-6.2336844777710176E-2</v>
       </c>
       <c r="AF75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-6.5876348804450036E-2</v>
       </c>
       <c r="AG75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-6.9037553383493933E-2</v>
       </c>
       <c r="AH75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-7.1345674879800702E-2</v>
       </c>
       <c r="AI75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-7.3630565061254982E-2</v>
       </c>
       <c r="AJ75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-7.6598895088601626E-2</v>
       </c>
       <c r="AK75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-8.0381655308611188E-2</v>
       </c>
       <c r="AL75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-8.424531400610169E-2</v>
       </c>
       <c r="AM75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-8.8172473103100169E-2</v>
       </c>
       <c r="AN75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-9.216576348705785E-2</v>
       </c>
       <c r="AO75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-9.6227772984214477E-2</v>
       </c>
       <c r="AP75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-0.10036111758262778</v>
       </c>
       <c r="AQ75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-0.10456944641753063</v>
       </c>
       <c r="AR75" t="s">
@@ -38797,46 +38797,46 @@
         <v>-81.114524782440284</v>
       </c>
       <c r="AD82">
-        <v>-64.42730538153296</v>
+        <v>-46.019503843952116</v>
       </c>
       <c r="AE82">
-        <v>-70.380388859541995</v>
+        <v>-50.271706328244285</v>
       </c>
       <c r="AF82">
-        <v>-76.861643235532384</v>
+        <v>-54.901173739665985</v>
       </c>
       <c r="AG82">
-        <v>-83.906231026322828</v>
+        <v>-59.93302216165916</v>
       </c>
       <c r="AH82">
-        <v>-91.564730703860363</v>
+        <v>-65.403379074185978</v>
       </c>
       <c r="AI82">
-        <v>-99.875183758332895</v>
+        <v>-71.339416970237778</v>
       </c>
       <c r="AJ82">
-        <v>-108.89793604728482</v>
+        <v>-77.784240033774864</v>
       </c>
       <c r="AK82">
-        <v>-118.69616811316295</v>
+        <v>-84.782977223687823</v>
       </c>
       <c r="AL82">
-        <v>-129.33426544722511</v>
+        <v>-92.38161817658937</v>
       </c>
       <c r="AM82">
-        <v>-140.85087113675098</v>
+        <v>-100.60776509767928</v>
       </c>
       <c r="AN82">
-        <v>-153.33643929531871</v>
+        <v>-109.5260280680848</v>
       </c>
       <c r="AO82">
-        <v>-166.84016460373556</v>
+        <v>-119.17154614552538</v>
       </c>
       <c r="AP82">
-        <v>-181.48921874776644</v>
+        <v>-129.6351562484046</v>
       </c>
       <c r="AQ82">
-        <v>-197.37715065999669</v>
+        <v>-140.98367904285476</v>
       </c>
       <c r="AR82" t="s">
         <v>46</v>
@@ -38931,46 +38931,46 @@
         <v>-40.463689809324435</v>
       </c>
       <c r="AD83">
-        <v>-32.113119980104543</v>
+        <v>-22.937942842931818</v>
       </c>
       <c r="AE83">
-        <v>-35.018954526465777</v>
+        <v>-25.013538947475553</v>
       </c>
       <c r="AF83">
-        <v>-38.171812818597459</v>
+        <v>-27.265580584712474</v>
       </c>
       <c r="AG83">
-        <v>-41.592575174886342</v>
+        <v>-29.708982267775959</v>
       </c>
       <c r="AH83">
-        <v>-45.299427103980889</v>
+        <v>-32.356733645700636</v>
       </c>
       <c r="AI83">
-        <v>-49.319785602930068</v>
+        <v>-35.228418287807195</v>
       </c>
       <c r="AJ83">
-        <v>-53.675486708134798</v>
+        <v>-38.339633362953428</v>
       </c>
       <c r="AK83">
-        <v>-58.387515256526328</v>
+        <v>-41.705368040375951</v>
       </c>
       <c r="AL83">
-        <v>-63.495783196731438</v>
+        <v>-45.354130854808169</v>
       </c>
       <c r="AM83">
-        <v>-69.015708788180859</v>
+        <v>-49.296934848700609</v>
       </c>
       <c r="AN83">
-        <v>-74.985599357878996</v>
+        <v>-53.561142398484996</v>
       </c>
       <c r="AO83">
-        <v>-81.442531016803372</v>
+        <v>-58.173236440573838</v>
       </c>
       <c r="AP83">
-        <v>-88.423218147484477</v>
+        <v>-63.15944153391748</v>
       </c>
       <c r="AQ83">
-        <v>-95.976800295666663</v>
+        <v>-68.554857354047613</v>
       </c>
       <c r="AR83" t="s">
         <v>46</v>
@@ -39065,46 +39065,46 @@
         <v>-23.674200109742657</v>
       </c>
       <c r="AD84">
-        <v>-18.711627670570714</v>
+        <v>-13.36544833612194</v>
       </c>
       <c r="AE84">
-        <v>-20.408489212667874</v>
+        <v>-14.577492294762767</v>
       </c>
       <c r="AF84">
-        <v>-22.25066042842186</v>
+        <v>-15.893328877444187</v>
       </c>
       <c r="AG84">
-        <v>-24.250205630003769</v>
+        <v>-17.321575450002694</v>
       </c>
       <c r="AH84">
-        <v>-26.417265986663836</v>
+        <v>-18.869475704759882</v>
       </c>
       <c r="AI84">
-        <v>-28.768160989078311</v>
+        <v>-20.54868642077022</v>
       </c>
       <c r="AJ84">
-        <v>-31.316233777229371</v>
+        <v>-22.368738412306694</v>
       </c>
       <c r="AK84">
-        <v>-34.072699090209881</v>
+        <v>-24.33764220729277</v>
       </c>
       <c r="AL84">
-        <v>-37.060858174449365</v>
+        <v>-26.472041553178119</v>
       </c>
       <c r="AM84">
-        <v>-40.291179534158211</v>
+        <v>-28.779413952970149</v>
       </c>
       <c r="AN84">
-        <v>-43.7885800046271</v>
+        <v>-31.277557146162213</v>
       </c>
       <c r="AO84">
-        <v>-47.570982422628688</v>
+        <v>-33.979273159020494</v>
       </c>
       <c r="AP84">
-        <v>-51.656983232176614</v>
+        <v>-36.897845165840437</v>
       </c>
       <c r="AQ84">
-        <v>-56.073830500421394</v>
+        <v>-40.052736071729569</v>
       </c>
       <c r="AR84" t="s">
         <v>46</v>
@@ -39199,46 +39199,46 @@
         <v>-14.303633531713665</v>
       </c>
       <c r="AD85">
-        <v>-11.511192035150875</v>
+        <v>-8.2222800251077679</v>
       </c>
       <c r="AE85">
-        <v>-12.552855269892813</v>
+        <v>-8.9663251927805803</v>
       </c>
       <c r="AF85">
-        <v>-13.68281542918599</v>
+        <v>-9.7734395922757074</v>
       </c>
       <c r="AG85">
-        <v>-14.908104868023344</v>
+        <v>-10.648646334302388</v>
       </c>
       <c r="AH85">
-        <v>-16.236133699776275</v>
+        <v>-11.597238356983052</v>
       </c>
       <c r="AI85">
-        <v>-17.674944566488065</v>
+        <v>-12.624960404634333</v>
       </c>
       <c r="AJ85">
-        <v>-19.232872666600585</v>
+        <v>-13.737766190428989</v>
       </c>
       <c r="AK85">
-        <v>-20.91848411160332</v>
+        <v>-14.941774365430941</v>
       </c>
       <c r="AL85">
-        <v>-22.743815130791688</v>
+        <v>-16.245582236279777</v>
       </c>
       <c r="AM85">
-        <v>-24.717249524945068</v>
+        <v>-17.655178232103619</v>
       </c>
       <c r="AN85">
-        <v>-26.850070563624115</v>
+        <v>-19.178621831160083</v>
       </c>
       <c r="AO85">
-        <v>-29.155277885677464</v>
+        <v>-20.825198489769615</v>
       </c>
       <c r="AP85">
-        <v>-31.644584226319552</v>
+        <v>-22.60327444737111</v>
       </c>
       <c r="AQ85">
-        <v>-34.332261965911606</v>
+        <v>-24.523044261365431</v>
       </c>
       <c r="AR85" t="s">
         <v>46</v>
@@ -40946,46 +40946,46 @@
         <v>-13.617884107128326</v>
       </c>
       <c r="AD100">
-        <v>-11.125400209561827</v>
+        <v>-7.9467144354013044</v>
       </c>
       <c r="AE100">
-        <v>-12.203448689657012</v>
+        <v>-8.716749064040723</v>
       </c>
       <c r="AF100">
-        <v>-13.381302890754373</v>
+        <v>-9.5580734933959803</v>
       </c>
       <c r="AG100">
-        <v>-14.668956624084903</v>
+        <v>-10.477826160060644</v>
       </c>
       <c r="AH100">
-        <v>-16.075332138808339</v>
+        <v>-11.482380099148813</v>
       </c>
       <c r="AI100">
-        <v>-17.610869087553084</v>
+        <v>-12.57919220539506</v>
       </c>
       <c r="AJ100">
-        <v>-19.287463406339178</v>
+        <v>-13.776759575956554</v>
       </c>
       <c r="AK100">
-        <v>-21.115805685246848</v>
+        <v>-15.082718346604892</v>
       </c>
       <c r="AL100">
-        <v>-23.110376444616385</v>
+        <v>-16.50741174615456</v>
       </c>
       <c r="AM100">
-        <v>-25.285262743356693</v>
+        <v>-18.060901959540494</v>
       </c>
       <c r="AN100">
-        <v>-27.653532183041769</v>
+        <v>-19.752522987886977</v>
       </c>
       <c r="AO100">
-        <v>-30.23323201035852</v>
+        <v>-21.595165721684658</v>
       </c>
       <c r="AP100">
-        <v>-33.043442457888894</v>
+        <v>-23.602458898492067</v>
       </c>
       <c r="AQ100">
-        <v>-36.104171704787923</v>
+        <v>-25.788694074848515</v>
       </c>
       <c r="AR100" t="s">
         <v>46</v>
@@ -41080,46 +41080,46 @@
         <v>-7.3020682104987245</v>
       </c>
       <c r="AD101">
-        <v>-5.9995860667085354</v>
+        <v>-4.2854186190775252</v>
       </c>
       <c r="AE101">
-        <v>-6.5719870926246724</v>
+        <v>-4.6942764947319091</v>
       </c>
       <c r="AF101">
-        <v>-7.1964246098833415</v>
+        <v>-5.1403032927738153</v>
       </c>
       <c r="AG101">
-        <v>-7.8779617947601084</v>
+        <v>-5.6271155676857916</v>
       </c>
       <c r="AH101">
-        <v>-8.6212050864698533</v>
+        <v>-6.1580036331927523</v>
       </c>
       <c r="AI101">
-        <v>-9.4315435326281332</v>
+        <v>-6.7368168090200946</v>
       </c>
       <c r="AJ101">
-        <v>-10.314412554297455</v>
+        <v>-7.3674375387838964</v>
       </c>
       <c r="AK101">
-        <v>-11.27544794381069</v>
+        <v>-8.053891388436206</v>
       </c>
       <c r="AL101">
-        <v>-12.323032010491463</v>
+        <v>-8.8021657217796161</v>
       </c>
       <c r="AM101">
-        <v>-13.463054147584682</v>
+        <v>-9.6164672482747733</v>
       </c>
       <c r="AN101">
-        <v>-14.701116729916658</v>
+        <v>-10.500797664226184</v>
       </c>
       <c r="AO101">
-        <v>-16.050204527855776</v>
+        <v>-11.46443180561127</v>
       </c>
       <c r="AP101">
-        <v>-17.515578895562765</v>
+        <v>-12.511127782544833</v>
       </c>
       <c r="AQ101">
-        <v>-19.108112003705568</v>
+        <v>-13.648651431218262</v>
       </c>
       <c r="AR101" t="s">
         <v>46</v>
@@ -41214,46 +41214,46 @@
         <v>-4.8939058071404951</v>
       </c>
       <c r="AD102">
-        <v>-3.9861955166388734</v>
+        <v>-2.8472825118849094</v>
       </c>
       <c r="AE102">
-        <v>-4.3681748100246596</v>
+        <v>-3.1201248643033281</v>
       </c>
       <c r="AF102">
-        <v>-4.7853241790547951</v>
+        <v>-3.4180886993248532</v>
       </c>
       <c r="AG102">
-        <v>-5.2411105279430767</v>
+        <v>-3.7436503771021972</v>
       </c>
       <c r="AH102">
-        <v>-5.7384335159244717</v>
+        <v>-4.0988810828031941</v>
       </c>
       <c r="AI102">
-        <v>-6.2812186681000792</v>
+        <v>-4.4865847629286275</v>
       </c>
       <c r="AJ102">
-        <v>-6.8730906578598105</v>
+        <v>-4.9093504698998647</v>
       </c>
       <c r="AK102">
-        <v>-7.5185283465055264</v>
+        <v>-5.3703773903610905</v>
       </c>
       <c r="AL102">
-        <v>-8.2220745178456003</v>
+        <v>-5.8729103698897145</v>
       </c>
       <c r="AM102">
-        <v>-8.9880586317162212</v>
+        <v>-6.4200418797973011</v>
       </c>
       <c r="AN102">
-        <v>-9.8226445487125673</v>
+        <v>-7.0161746776518346</v>
       </c>
       <c r="AO102">
-        <v>-10.730849781936666</v>
+        <v>-7.6648927013833319</v>
       </c>
       <c r="AP102">
-        <v>-11.718633799733224</v>
+        <v>-8.3704527140951601</v>
       </c>
       <c r="AQ102">
-        <v>-12.792690936671629</v>
+        <v>-9.1376363833368774</v>
       </c>
       <c r="AR102" t="s">
         <v>46</v>
@@ -41348,46 +41348,46 @@
         <v>-3.3537062556172632</v>
       </c>
       <c r="AD103">
-        <v>-2.8090416974688903</v>
+        <v>-2.0064583553349218</v>
       </c>
       <c r="AE103">
-        <v>-3.077196003977162</v>
+        <v>-2.1979971456979728</v>
       </c>
       <c r="AF103">
-        <v>-3.3699680445692941</v>
+        <v>-2.40712003183521</v>
       </c>
       <c r="AG103">
-        <v>-3.6894973388705337</v>
+        <v>-2.6353552420503812</v>
       </c>
       <c r="AH103">
-        <v>-4.0382090822803018</v>
+        <v>-2.8844350587716443</v>
       </c>
       <c r="AI103">
-        <v>-4.4183371265435492</v>
+        <v>-3.1559550903882494</v>
       </c>
       <c r="AJ103">
-        <v>-4.8328343322809753</v>
+        <v>-3.4520245230578395</v>
       </c>
       <c r="AK103">
-        <v>-5.2843903819303879</v>
+        <v>-3.774564558521706</v>
       </c>
       <c r="AL103">
-        <v>-5.7761335448865703</v>
+        <v>-4.1258096749189788</v>
       </c>
       <c r="AM103">
-        <v>-6.3118372419458995</v>
+        <v>-4.5084551728184996</v>
       </c>
       <c r="AN103">
-        <v>-6.8948777773669692</v>
+        <v>-4.9249126981192637</v>
       </c>
       <c r="AO103">
-        <v>-7.5285357236163488</v>
+        <v>-5.377525516868821</v>
       </c>
       <c r="AP103">
-        <v>-8.217907504817326</v>
+        <v>-5.8699339320123753</v>
       </c>
       <c r="AQ103">
-        <v>-8.9672071226142016</v>
+        <v>-6.4051479447244288</v>
       </c>
       <c r="AR103" t="s">
         <v>46</v>

</xml_diff>